<commit_message>
Template: lighter chart gridlines, legends on top, axis label in caption
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -910,21 +910,6 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>x (m)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="high"/>
@@ -937,7 +922,16 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+              <a:solidFill>
+                <a:srgbClr val="E3E3E3"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
         <title>
           <tx>
             <rich>
@@ -960,7 +954,7 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="b"/>
+      <legendPos val="t"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1057,21 +1051,6 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>x (m)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="high"/>
@@ -1084,7 +1063,16 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+              <a:solidFill>
+                <a:srgbClr val="E3E3E3"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
         <title>
           <tx>
             <rich>
@@ -1107,7 +1095,7 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="b"/>
+      <legendPos val="t"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1204,21 +1192,6 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>x (m)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
@@ -1231,7 +1204,16 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+              <a:solidFill>
+                <a:srgbClr val="E3E3E3"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
         <title>
           <tx>
             <rich>
@@ -1254,7 +1236,7 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="b"/>
+      <legendPos val="t"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -4278,7 +4260,7 @@
     <row r="92" ht="14" customHeight="1">
       <c r="B92" s="66" t="inlineStr">
         <is>
-          <t>Deflected shapes (mm, plotted downward)</t>
+          <t>Deflected shapes (mm, plotted downward;  x in m)</t>
         </is>
       </c>
     </row>
@@ -4312,12 +4294,12 @@
     <row r="106" ht="14" customHeight="1">
       <c r="B106" s="66" t="inlineStr">
         <is>
-          <t>Bending moment envelope (kN·m, sagging plotted down)</t>
+          <t>Bending moment envelope (kN·m, sagging down;  x in m)</t>
         </is>
       </c>
       <c r="F106" s="66" t="inlineStr">
         <is>
-          <t>Shear force envelope (kN)</t>
+          <t>Shear force envelope (kN;  x in m)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v0.2.2: OAR.SECTIONLIST, section size dropdown filtered by type, section properties wired
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -1684,7 +1684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AF201"/>
+  <dimension ref="B1:AL201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.5" customWidth="1" min="1" max="1"/>
@@ -1722,6 +1722,7 @@
     <col width="9" customWidth="1" min="34" max="34"/>
     <col width="9" customWidth="1" min="35" max="35"/>
     <col width="9" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1" ht="17" customHeight="1">
@@ -1870,6 +1871,11 @@
           <t>Governing (OAR.GOVERNING)</t>
         </is>
       </c>
+      <c r="AL7" s="15" t="inlineStr">
+        <is>
+          <t>Sections (OAR.SECTIONLIST)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="B8" s="10" t="inlineStr">
@@ -1900,6 +1906,10 @@
       <c r="T8" s="18" t="n"/>
       <c r="Z8" s="19" cm="1">
         <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1,$I$77:$J$78)</f>
+        <v/>
+      </c>
+      <c r="AL8" s="19" cm="1">
+        <f t="array" ref="AL8">OAR.SECTIONLIST(SectionType)</f>
         <v/>
       </c>
     </row>
@@ -2517,7 +2527,10 @@
           <t>Mass</t>
         </is>
       </c>
-      <c r="H27" s="38" t="n"/>
+      <c r="H27" s="38" cm="1">
+        <f t="array" ref="H27">OAR.SECTION(SectionSize,"Mass",Grade)</f>
+        <v/>
+      </c>
       <c r="I27" s="42" t="inlineStr">
         <is>
           <t>kg/m</t>
@@ -2551,7 +2564,10 @@
           <t>Ix</t>
         </is>
       </c>
-      <c r="H28" s="38" t="n"/>
+      <c r="H28" s="38" cm="1">
+        <f t="array" ref="H28">OAR.SECTION(SectionSize,"Ix",Grade)</f>
+        <v/>
+      </c>
       <c r="I28" s="42" t="inlineStr">
         <is>
           <t>×10⁶ mm⁴</t>
@@ -2585,7 +2601,10 @@
           <t>Iy</t>
         </is>
       </c>
-      <c r="H29" s="33" t="n"/>
+      <c r="H29" s="33" cm="1">
+        <f t="array" ref="H29">OAR.SECTION(SectionSize,"Iy",Grade)</f>
+        <v/>
+      </c>
       <c r="I29" s="42" t="inlineStr">
         <is>
           <t>×10⁶ mm⁴</t>
@@ -2617,7 +2636,10 @@
           <t>J</t>
         </is>
       </c>
-      <c r="H30" s="38" t="n"/>
+      <c r="H30" s="38" cm="1">
+        <f t="array" ref="H30">OAR.SECTION(SectionSize,"J",Grade)</f>
+        <v/>
+      </c>
       <c r="I30" s="42" t="inlineStr">
         <is>
           <t>×10³ mm⁴</t>
@@ -2651,7 +2673,10 @@
           <t>Iw</t>
         </is>
       </c>
-      <c r="H31" s="38" t="n"/>
+      <c r="H31" s="38" cm="1">
+        <f t="array" ref="H31">OAR.SECTION(SectionSize,"Iw",Grade)</f>
+        <v/>
+      </c>
       <c r="I31" s="42" t="inlineStr">
         <is>
           <t>×10⁹ mm⁶</t>
@@ -2682,7 +2707,10 @@
           <t>Zex</t>
         </is>
       </c>
-      <c r="H32" s="46" t="n"/>
+      <c r="H32" s="46" cm="1">
+        <f t="array" ref="H32">OAR.SECTION(SectionSize,"Ze",Grade)</f>
+        <v/>
+      </c>
       <c r="I32" s="42" t="inlineStr">
         <is>
           <t>×10³ mm³</t>
@@ -2703,7 +2731,10 @@
           <t>φMsx</t>
         </is>
       </c>
-      <c r="H33" s="38" t="n"/>
+      <c r="H33" s="38" cm="1">
+        <f t="array" ref="H33">OAR.SECTION(SectionSize,"phiMsx",Grade)</f>
+        <v/>
+      </c>
       <c r="I33" s="42" t="inlineStr">
         <is>
           <t>kN·m</t>
@@ -5203,9 +5234,9 @@
       <formula>$B188&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="11">
+  <dataValidations count="12">
     <dataValidation sqref="E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"UB,UC,PFC,WB,WC,RHS,SHS,CHS,TFB"</formula1>
+      <formula1>"UB,UC,WB,PFC"</formula1>
     </dataValidation>
     <dataValidation sqref="E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
@@ -5237,6 +5268,9 @@
     <dataValidation sqref="E77:F81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"F,P,L,U,–"</formula1>
     </dataValidation>
+    <dataValidation sqref="E27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Section size" error="Pick a section from the list for the selected Section type." type="list">
+      <formula1>OFFSET($AL$8,0,0,MAX(1,COUNTA($AL$8:$AL$300)),1)</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.6" header="0.2" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Sheet: explicit Restraints_B1[#Data] reference; section dropdown falls back to full list if add-in not loaded
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -407,7 +407,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -452,6 +452,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1684,7 +1685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AL201"/>
+  <dimension ref="B1:AN201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.5" customWidth="1" min="1" max="1"/>
@@ -1723,6 +1724,7 @@
     <col width="9" customWidth="1" min="35" max="35"/>
     <col width="9" customWidth="1" min="36" max="36"/>
     <col width="12" customWidth="1" min="38" max="38"/>
+    <col width="12" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1" ht="17" customHeight="1">
@@ -1876,6 +1878,11 @@
           <t>Sections (OAR.SECTIONLIST)</t>
         </is>
       </c>
+      <c r="AN7" s="15" t="inlineStr">
+        <is>
+          <t>All sections (fallback)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="B8" s="10" t="inlineStr">
@@ -1905,13 +1912,18 @@
       <c r="S8" s="17" t="n"/>
       <c r="T8" s="18" t="n"/>
       <c r="Z8" s="19" cm="1">
-        <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1,$I$77:$J$78)</f>
+        <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
         <v/>
       </c>
       <c r="AL8" s="19" cm="1">
         <f t="array" ref="AL8">OAR.SECTIONLIST(SectionType)</f>
         <v/>
       </c>
+      <c r="AN8" s="20" t="inlineStr">
+        <is>
+          <t>1200WB455</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="14" customHeight="1">
       <c r="B9" s="6" t="inlineStr">
@@ -1924,42 +1936,52 @@
           <t>Max utilisation</t>
         </is>
       </c>
-      <c r="I9" s="20" t="inlineStr">
+      <c r="I9" s="21" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="M9" s="21" t="n"/>
-      <c r="N9" s="22" t="n"/>
-      <c r="O9" s="22" t="n"/>
-      <c r="P9" s="22" t="n"/>
-      <c r="Q9" s="22" t="n"/>
-      <c r="R9" s="22" t="n"/>
-      <c r="S9" s="22" t="n"/>
-      <c r="T9" s="23" t="n"/>
+      <c r="M9" s="22" t="n"/>
+      <c r="N9" s="23" t="n"/>
+      <c r="O9" s="23" t="n"/>
+      <c r="P9" s="23" t="n"/>
+      <c r="Q9" s="23" t="n"/>
+      <c r="R9" s="23" t="n"/>
+      <c r="S9" s="23" t="n"/>
+      <c r="T9" s="24" t="n"/>
+      <c r="AN9" s="20" t="inlineStr">
+        <is>
+          <t>1200WB423</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="24">
+      <c r="B10" s="25">
         <f>IF(SectionSize="","–",SectionSize&amp;"  Gr "&amp;Grade)</f>
         <v/>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="26">
         <f>IF(COUNT(I14:I23)=0,"–",MAX(I14:I23))</f>
         <v/>
       </c>
-      <c r="I10" s="26">
+      <c r="I10" s="27">
         <f>IF(COUNT(I14:I23)=0,"PENDING",IF(MAX(I14:I23)&lt;=1,"PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="J10" s="27" t="n"/>
-      <c r="M10" s="21" t="n"/>
-      <c r="N10" s="22" t="n"/>
-      <c r="O10" s="22" t="n"/>
-      <c r="P10" s="22" t="n"/>
-      <c r="Q10" s="22" t="n"/>
-      <c r="R10" s="22" t="n"/>
-      <c r="S10" s="22" t="n"/>
-      <c r="T10" s="23" t="n"/>
+      <c r="J10" s="28" t="n"/>
+      <c r="M10" s="22" t="n"/>
+      <c r="N10" s="23" t="n"/>
+      <c r="O10" s="23" t="n"/>
+      <c r="P10" s="23" t="n"/>
+      <c r="Q10" s="23" t="n"/>
+      <c r="R10" s="23" t="n"/>
+      <c r="S10" s="23" t="n"/>
+      <c r="T10" s="24" t="n"/>
+      <c r="AN10" s="20" t="inlineStr">
+        <is>
+          <t>1200WB392</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="14" customHeight="1">
       <c r="B11" s="6">
@@ -1970,24 +1992,29 @@
         <f>IF(COUNT(I14:I23)=0,"","Governs: "&amp;INDEX(D14:D23,MATCH(MAX(I14:I23),I14:I23,0)))</f>
         <v/>
       </c>
-      <c r="M11" s="21" t="n"/>
-      <c r="N11" s="22" t="n"/>
-      <c r="O11" s="22" t="n"/>
-      <c r="P11" s="22" t="n"/>
-      <c r="Q11" s="22" t="n"/>
-      <c r="R11" s="22" t="n"/>
-      <c r="S11" s="22" t="n"/>
-      <c r="T11" s="23" t="n"/>
+      <c r="M11" s="22" t="n"/>
+      <c r="N11" s="23" t="n"/>
+      <c r="O11" s="23" t="n"/>
+      <c r="P11" s="23" t="n"/>
+      <c r="Q11" s="23" t="n"/>
+      <c r="R11" s="23" t="n"/>
+      <c r="S11" s="23" t="n"/>
+      <c r="T11" s="24" t="n"/>
+      <c r="AN11" s="20" t="inlineStr">
+        <is>
+          <t>1200WB342</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="14" customHeight="1">
-      <c r="M12" s="21" t="n"/>
-      <c r="N12" s="22" t="n"/>
-      <c r="O12" s="22" t="n"/>
-      <c r="P12" s="22" t="n"/>
-      <c r="Q12" s="22" t="n"/>
-      <c r="R12" s="22" t="n"/>
-      <c r="S12" s="22" t="n"/>
-      <c r="T12" s="23" t="n"/>
+      <c r="M12" s="22" t="n"/>
+      <c r="N12" s="23" t="n"/>
+      <c r="O12" s="23" t="n"/>
+      <c r="P12" s="23" t="n"/>
+      <c r="Q12" s="23" t="n"/>
+      <c r="R12" s="23" t="n"/>
+      <c r="S12" s="23" t="n"/>
+      <c r="T12" s="24" t="n"/>
       <c r="Z12" s="15" t="inlineStr">
         <is>
           <t>Envelope (OAR.ENVELOPE)</t>
@@ -1998,56 +2025,61 @@
           <t>Deflected shapes (OAR.DEFLECTIONS)</t>
         </is>
       </c>
+      <c r="AN12" s="20" t="inlineStr">
+        <is>
+          <t>1200WB317</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="D13" s="28" t="inlineStr">
+      <c r="D13" s="29" t="inlineStr">
         <is>
           <t>Basis</t>
         </is>
       </c>
-      <c r="E13" s="28" t="inlineStr">
+      <c r="E13" s="29" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="F13" s="28" t="inlineStr">
+      <c r="F13" s="29" t="inlineStr">
         <is>
           <t>Limit</t>
         </is>
       </c>
-      <c r="G13" s="28" t="inlineStr">
+      <c r="G13" s="29" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="H13" s="28" t="inlineStr">
+      <c r="H13" s="29" t="inlineStr">
         <is>
           <t>L / x</t>
         </is>
       </c>
-      <c r="I13" s="28" t="inlineStr">
+      <c r="I13" s="29" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
-      <c r="J13" s="28" t="inlineStr">
+      <c r="J13" s="29" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="M13" s="21" t="n"/>
-      <c r="N13" s="22" t="n"/>
-      <c r="O13" s="22" t="n"/>
-      <c r="P13" s="22" t="n"/>
-      <c r="Q13" s="22" t="n"/>
-      <c r="R13" s="22" t="n"/>
-      <c r="S13" s="22" t="n"/>
-      <c r="T13" s="23" t="n"/>
+      <c r="M13" s="22" t="n"/>
+      <c r="N13" s="23" t="n"/>
+      <c r="O13" s="23" t="n"/>
+      <c r="P13" s="23" t="n"/>
+      <c r="Q13" s="23" t="n"/>
+      <c r="R13" s="23" t="n"/>
+      <c r="S13" s="23" t="n"/>
+      <c r="T13" s="24" t="n"/>
       <c r="Z13" s="19" cm="1">
         <f t="array" ref="Z13">OAR.ENVELOPE(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),60)</f>
         <v/>
@@ -2056,412 +2088,472 @@
         <f t="array" ref="AF13">OAR.DEFLECTIONS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],PsiL,PsiS,60)</f>
         <v/>
       </c>
+      <c r="AN13" s="20" t="inlineStr">
+        <is>
+          <t>1200WB278</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="14" customHeight="1">
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>Serviceability</t>
         </is>
       </c>
-      <c r="C14" s="30" t="n"/>
-      <c r="D14" s="30" t="n"/>
-      <c r="E14" s="30" t="n"/>
-      <c r="F14" s="30" t="n"/>
-      <c r="G14" s="30" t="n"/>
-      <c r="H14" s="30" t="n"/>
-      <c r="I14" s="30" t="n"/>
-      <c r="J14" s="30" t="n"/>
-      <c r="M14" s="21" t="n"/>
-      <c r="N14" s="22" t="n"/>
-      <c r="O14" s="22" t="n"/>
-      <c r="P14" s="22" t="n"/>
-      <c r="Q14" s="22" t="n"/>
-      <c r="R14" s="22" t="n"/>
-      <c r="S14" s="22" t="n"/>
-      <c r="T14" s="23" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
+      <c r="H14" s="31" t="n"/>
+      <c r="I14" s="31" t="n"/>
+      <c r="J14" s="31" t="n"/>
+      <c r="M14" s="22" t="n"/>
+      <c r="N14" s="23" t="n"/>
+      <c r="O14" s="23" t="n"/>
+      <c r="P14" s="23" t="n"/>
+      <c r="Q14" s="23" t="n"/>
+      <c r="R14" s="23" t="n"/>
+      <c r="S14" s="23" t="n"/>
+      <c r="T14" s="24" t="n"/>
+      <c r="AN14" s="20" t="inlineStr">
+        <is>
+          <t>1200WB249</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="14" customHeight="1">
-      <c r="B15" s="31" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>Δg</t>
         </is>
       </c>
-      <c r="D15" s="32" t="inlineStr">
+      <c r="D15" s="33" t="inlineStr">
         <is>
           <t>Dead load</t>
         </is>
       </c>
-      <c r="E15" s="33" cm="1">
+      <c r="E15" s="34" cm="1">
         <f t="array" ref="E15">INDEX(_xlfn.ANCHORARRAY(B86),1,2)</f>
         <v/>
       </c>
-      <c r="F15" s="33">
+      <c r="F15" s="34">
         <f>IF(N(E37)=0,"",IF(N(F37)=0,Span/E37,MIN(Span/E37,F37)))</f>
         <v/>
       </c>
-      <c r="G15" s="34" t="inlineStr">
+      <c r="G15" s="35" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="H15" s="35">
+      <c r="H15" s="36">
         <f>IF(N(E15)=0,"",Span/E15)</f>
         <v/>
       </c>
-      <c r="I15" s="36">
+      <c r="I15" s="37">
         <f>IF(OR(E15="",N(F15)=0),"",ABS(E15)/F15)</f>
         <v/>
       </c>
-      <c r="J15" s="37">
+      <c r="J15" s="38">
         <f>IF(I15="","–",IF(I15&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
-      <c r="M15" s="21" t="n"/>
-      <c r="N15" s="22" t="n"/>
-      <c r="O15" s="22" t="n"/>
-      <c r="P15" s="22" t="n"/>
-      <c r="Q15" s="22" t="n"/>
-      <c r="R15" s="22" t="n"/>
-      <c r="S15" s="22" t="n"/>
-      <c r="T15" s="23" t="n"/>
+      <c r="M15" s="22" t="n"/>
+      <c r="N15" s="23" t="n"/>
+      <c r="O15" s="23" t="n"/>
+      <c r="P15" s="23" t="n"/>
+      <c r="Q15" s="23" t="n"/>
+      <c r="R15" s="23" t="n"/>
+      <c r="S15" s="23" t="n"/>
+      <c r="T15" s="24" t="n"/>
+      <c r="AN15" s="20" t="inlineStr">
+        <is>
+          <t>1000WB322</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="14" customHeight="1">
-      <c r="B16" s="31" t="inlineStr">
+      <c r="B16" s="32" t="inlineStr">
         <is>
           <t>Δg+ψl·q</t>
         </is>
       </c>
-      <c r="D16" s="32" t="inlineStr">
+      <c r="D16" s="33" t="inlineStr">
         <is>
           <t>Long term</t>
         </is>
       </c>
-      <c r="E16" s="33" cm="1">
+      <c r="E16" s="34" cm="1">
         <f t="array" ref="E16">INDEX(_xlfn.ANCHORARRAY(B86),2,2)</f>
         <v/>
       </c>
-      <c r="F16" s="33">
+      <c r="F16" s="34">
         <f>IF(N(E38)=0,"",IF(N(F38)=0,Span/E38,MIN(Span/E38,F38)))</f>
         <v/>
       </c>
-      <c r="G16" s="34" t="inlineStr">
+      <c r="G16" s="35" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="H16" s="35">
+      <c r="H16" s="36">
         <f>IF(N(E16)=0,"",Span/E16)</f>
         <v/>
       </c>
-      <c r="I16" s="36">
+      <c r="I16" s="37">
         <f>IF(OR(E16="",N(F16)=0),"",ABS(E16)/F16)</f>
         <v/>
       </c>
-      <c r="J16" s="37">
+      <c r="J16" s="38">
         <f>IF(I16="","–",IF(I16&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
-      <c r="M16" s="21" t="n"/>
-      <c r="N16" s="22" t="n"/>
-      <c r="O16" s="22" t="n"/>
-      <c r="P16" s="22" t="n"/>
-      <c r="Q16" s="22" t="n"/>
-      <c r="R16" s="22" t="n"/>
-      <c r="S16" s="22" t="n"/>
-      <c r="T16" s="23" t="n"/>
+      <c r="M16" s="22" t="n"/>
+      <c r="N16" s="23" t="n"/>
+      <c r="O16" s="23" t="n"/>
+      <c r="P16" s="23" t="n"/>
+      <c r="Q16" s="23" t="n"/>
+      <c r="R16" s="23" t="n"/>
+      <c r="S16" s="23" t="n"/>
+      <c r="T16" s="24" t="n"/>
+      <c r="AN16" s="20" t="inlineStr">
+        <is>
+          <t>1000WB296</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="14" customHeight="1">
-      <c r="B17" s="31" t="inlineStr">
+      <c r="B17" s="32" t="inlineStr">
         <is>
           <t>Δg+ψs·q</t>
         </is>
       </c>
-      <c r="D17" s="32" t="inlineStr">
+      <c r="D17" s="33" t="inlineStr">
         <is>
           <t>Short term</t>
         </is>
       </c>
-      <c r="E17" s="33" cm="1">
+      <c r="E17" s="34" cm="1">
         <f t="array" ref="E17">INDEX(_xlfn.ANCHORARRAY(B86),3,2)</f>
         <v/>
       </c>
-      <c r="F17" s="33">
+      <c r="F17" s="34">
         <f>IF(N(E39)=0,"",IF(N(F39)=0,Span/E39,MIN(Span/E39,F39)))</f>
         <v/>
       </c>
-      <c r="G17" s="34" t="inlineStr">
+      <c r="G17" s="35" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="H17" s="35">
+      <c r="H17" s="36">
         <f>IF(N(E17)=0,"",Span/E17)</f>
         <v/>
       </c>
-      <c r="I17" s="36">
+      <c r="I17" s="37">
         <f>IF(OR(E17="",N(F17)=0),"",ABS(E17)/F17)</f>
         <v/>
       </c>
-      <c r="J17" s="37">
+      <c r="J17" s="38">
         <f>IF(I17="","–",IF(I17&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
-      <c r="M17" s="21" t="n"/>
-      <c r="N17" s="22" t="n"/>
-      <c r="O17" s="22" t="n"/>
-      <c r="P17" s="22" t="n"/>
-      <c r="Q17" s="22" t="n"/>
-      <c r="R17" s="22" t="n"/>
-      <c r="S17" s="22" t="n"/>
-      <c r="T17" s="23" t="n"/>
+      <c r="M17" s="22" t="n"/>
+      <c r="N17" s="23" t="n"/>
+      <c r="O17" s="23" t="n"/>
+      <c r="P17" s="23" t="n"/>
+      <c r="Q17" s="23" t="n"/>
+      <c r="R17" s="23" t="n"/>
+      <c r="S17" s="23" t="n"/>
+      <c r="T17" s="24" t="n"/>
+      <c r="AN17" s="20" t="inlineStr">
+        <is>
+          <t>1000WB258</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="14" customHeight="1">
-      <c r="B18" s="31" t="inlineStr">
+      <c r="B18" s="32" t="inlineStr">
         <is>
           <t>Δq</t>
         </is>
       </c>
-      <c r="D18" s="32" t="inlineStr">
+      <c r="D18" s="33" t="inlineStr">
         <is>
           <t>Live load only</t>
         </is>
       </c>
-      <c r="E18" s="33" cm="1">
+      <c r="E18" s="34" cm="1">
         <f t="array" ref="E18">INDEX(_xlfn.ANCHORARRAY(B86),4,2)</f>
         <v/>
       </c>
-      <c r="F18" s="33">
+      <c r="F18" s="34">
         <f>IF(N(E40)=0,"",IF(N(F40)=0,Span/E40,MIN(Span/E40,F40)))</f>
         <v/>
       </c>
-      <c r="G18" s="34" t="inlineStr">
+      <c r="G18" s="35" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="H18" s="35">
+      <c r="H18" s="36">
         <f>IF(N(E18)=0,"",Span/E18)</f>
         <v/>
       </c>
-      <c r="I18" s="36">
+      <c r="I18" s="37">
         <f>IF(OR(E18="",N(F18)=0),"",ABS(E18)/F18)</f>
         <v/>
       </c>
-      <c r="J18" s="37">
+      <c r="J18" s="38">
         <f>IF(I18="","–",IF(I18&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
-      <c r="M18" s="21" t="n"/>
-      <c r="N18" s="22" t="n"/>
-      <c r="O18" s="22" t="n"/>
-      <c r="P18" s="22" t="n"/>
-      <c r="Q18" s="22" t="n"/>
-      <c r="R18" s="22" t="n"/>
-      <c r="S18" s="22" t="n"/>
-      <c r="T18" s="23" t="n"/>
+      <c r="M18" s="22" t="n"/>
+      <c r="N18" s="23" t="n"/>
+      <c r="O18" s="23" t="n"/>
+      <c r="P18" s="23" t="n"/>
+      <c r="Q18" s="23" t="n"/>
+      <c r="R18" s="23" t="n"/>
+      <c r="S18" s="23" t="n"/>
+      <c r="T18" s="24" t="n"/>
+      <c r="AN18" s="20" t="inlineStr">
+        <is>
+          <t>1000WB215</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="14" customHeight="1">
-      <c r="B19" s="31" t="inlineStr">
+      <c r="B19" s="32" t="inlineStr">
         <is>
           <t>Δ1kN</t>
         </is>
       </c>
-      <c r="D19" s="32" t="inlineStr">
+      <c r="D19" s="33" t="inlineStr">
         <is>
           <t>1 kN at midspan</t>
         </is>
       </c>
-      <c r="E19" s="33" cm="1">
+      <c r="E19" s="34" cm="1">
         <f t="array" ref="E19">INDEX(_xlfn.ANCHORARRAY(B86),5,2)</f>
         <v/>
       </c>
-      <c r="F19" s="33">
+      <c r="F19" s="34">
         <f>IF(N(E41)=0,"",IF(N(F41)=0,Span/E41,MIN(Span/E41,F41)))</f>
         <v/>
       </c>
-      <c r="G19" s="34" t="inlineStr">
+      <c r="G19" s="35" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="H19" s="35">
+      <c r="H19" s="36">
         <f>IF(N(E19)=0,"",Span/E19)</f>
         <v/>
       </c>
-      <c r="I19" s="36">
+      <c r="I19" s="37">
         <f>IF(OR(E19="",N(F19)=0),"",ABS(E19)/F19)</f>
         <v/>
       </c>
-      <c r="J19" s="37">
+      <c r="J19" s="38">
         <f>IF(I19="","–",IF(I19&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
-      <c r="M19" s="21" t="n"/>
-      <c r="N19" s="22" t="n"/>
-      <c r="O19" s="22" t="n"/>
-      <c r="P19" s="22" t="n"/>
-      <c r="Q19" s="22" t="n"/>
-      <c r="R19" s="22" t="n"/>
-      <c r="S19" s="22" t="n"/>
-      <c r="T19" s="23" t="n"/>
+      <c r="M19" s="22" t="n"/>
+      <c r="N19" s="23" t="n"/>
+      <c r="O19" s="23" t="n"/>
+      <c r="P19" s="23" t="n"/>
+      <c r="Q19" s="23" t="n"/>
+      <c r="R19" s="23" t="n"/>
+      <c r="S19" s="23" t="n"/>
+      <c r="T19" s="24" t="n"/>
+      <c r="AN19" s="20" t="inlineStr">
+        <is>
+          <t>900WB282</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="14" customHeight="1">
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="30" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
-      <c r="C20" s="30" t="n"/>
-      <c r="D20" s="30" t="n"/>
-      <c r="E20" s="30" t="n"/>
-      <c r="F20" s="30" t="n"/>
-      <c r="G20" s="30" t="n"/>
-      <c r="H20" s="30" t="n"/>
-      <c r="I20" s="30" t="n"/>
-      <c r="J20" s="30" t="n"/>
-      <c r="M20" s="21" t="n"/>
-      <c r="N20" s="22" t="n"/>
-      <c r="O20" s="22" t="n"/>
-      <c r="P20" s="22" t="n"/>
-      <c r="Q20" s="22" t="n"/>
-      <c r="R20" s="22" t="n"/>
-      <c r="S20" s="22" t="n"/>
-      <c r="T20" s="23" t="n"/>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="31" t="n"/>
+      <c r="E20" s="31" t="n"/>
+      <c r="F20" s="31" t="n"/>
+      <c r="G20" s="31" t="n"/>
+      <c r="H20" s="31" t="n"/>
+      <c r="I20" s="31" t="n"/>
+      <c r="J20" s="31" t="n"/>
+      <c r="M20" s="22" t="n"/>
+      <c r="N20" s="23" t="n"/>
+      <c r="O20" s="23" t="n"/>
+      <c r="P20" s="23" t="n"/>
+      <c r="Q20" s="23" t="n"/>
+      <c r="R20" s="23" t="n"/>
+      <c r="S20" s="23" t="n"/>
+      <c r="T20" s="24" t="n"/>
+      <c r="AN20" s="20" t="inlineStr">
+        <is>
+          <t>900WB257</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="14" customHeight="1">
-      <c r="B21" s="31" t="inlineStr">
+      <c r="B21" s="32" t="inlineStr">
         <is>
           <t>M* / φMbx</t>
         </is>
       </c>
-      <c r="D21" s="32" t="inlineStr">
+      <c r="D21" s="33" t="inlineStr">
         <is>
           <t>Bending – gravity (top flange critical)</t>
         </is>
       </c>
-      <c r="E21" s="38" cm="1">
+      <c r="E21" s="39" cm="1">
         <f t="array" ref="E21">INDEX(_xlfn.ANCHORARRAY(Z8),1,2)</f>
         <v/>
       </c>
-      <c r="F21" s="38" cm="1">
+      <c r="F21" s="39" cm="1">
         <f t="array" ref="F21">INDEX(_xlfn.ANCHORARRAY(Z8),1,3)</f>
         <v/>
       </c>
-      <c r="G21" s="34" t="inlineStr">
+      <c r="G21" s="35" t="inlineStr">
         <is>
           <t>kN·m</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr"/>
-      <c r="I21" s="36">
+      <c r="I21" s="37">
         <f>IF(OR(E21="",N(F21)=0),"",ABS(E21)/F21)</f>
         <v/>
       </c>
-      <c r="J21" s="37">
+      <c r="J21" s="38">
         <f>IF(I21="","–",IF(I21&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
-      <c r="M21" s="21" t="n"/>
-      <c r="N21" s="22" t="n"/>
-      <c r="O21" s="22" t="n"/>
-      <c r="P21" s="22" t="n"/>
-      <c r="Q21" s="22" t="n"/>
-      <c r="R21" s="22" t="n"/>
-      <c r="S21" s="22" t="n"/>
-      <c r="T21" s="23" t="n"/>
+      <c r="M21" s="22" t="n"/>
+      <c r="N21" s="23" t="n"/>
+      <c r="O21" s="23" t="n"/>
+      <c r="P21" s="23" t="n"/>
+      <c r="Q21" s="23" t="n"/>
+      <c r="R21" s="23" t="n"/>
+      <c r="S21" s="23" t="n"/>
+      <c r="T21" s="24" t="n"/>
+      <c r="AN21" s="20" t="inlineStr">
+        <is>
+          <t>900WB218</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="14" customHeight="1">
-      <c r="B22" s="31" t="inlineStr">
+      <c r="B22" s="32" t="inlineStr">
         <is>
           <t>M* / φMbx</t>
         </is>
       </c>
-      <c r="D22" s="32">
+      <c r="D22" s="33">
         <f>IF(NumUpliftCombos=0,"Bending – uplift (no uplift combinations)","Bending – uplift (bottom flange critical)")</f>
         <v/>
       </c>
-      <c r="E22" s="38" cm="1">
+      <c r="E22" s="39" cm="1">
         <f t="array" ref="E22">INDEX(_xlfn.ANCHORARRAY(Z8),2,2)</f>
         <v/>
       </c>
-      <c r="F22" s="38" cm="1">
+      <c r="F22" s="39" cm="1">
         <f t="array" ref="F22">INDEX(_xlfn.ANCHORARRAY(Z8),2,3)</f>
         <v/>
       </c>
-      <c r="G22" s="34" t="inlineStr">
+      <c r="G22" s="35" t="inlineStr">
         <is>
           <t>kN·m</t>
         </is>
       </c>
       <c r="H22" s="19" t="inlineStr"/>
-      <c r="I22" s="36">
+      <c r="I22" s="37">
         <f>IF(OR(E22="",N(F22)=0),"",ABS(E22)/F22)</f>
         <v/>
       </c>
-      <c r="J22" s="37">
+      <c r="J22" s="38">
         <f>IF(I22="","–",IF(I22&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
-      <c r="M22" s="21" t="n"/>
-      <c r="N22" s="22" t="n"/>
-      <c r="O22" s="22" t="n"/>
-      <c r="P22" s="22" t="n"/>
-      <c r="Q22" s="22" t="n"/>
-      <c r="R22" s="22" t="n"/>
-      <c r="S22" s="22" t="n"/>
-      <c r="T22" s="23" t="n"/>
+      <c r="M22" s="22" t="n"/>
+      <c r="N22" s="23" t="n"/>
+      <c r="O22" s="23" t="n"/>
+      <c r="P22" s="23" t="n"/>
+      <c r="Q22" s="23" t="n"/>
+      <c r="R22" s="23" t="n"/>
+      <c r="S22" s="23" t="n"/>
+      <c r="T22" s="24" t="n"/>
+      <c r="AN22" s="20" t="inlineStr">
+        <is>
+          <t>900WB175</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="14" customHeight="1">
-      <c r="B23" s="31" t="inlineStr">
+      <c r="B23" s="32" t="inlineStr">
         <is>
           <t>V* / φVv</t>
         </is>
       </c>
-      <c r="D23" s="32" t="inlineStr">
+      <c r="D23" s="33" t="inlineStr">
         <is>
           <t>Shear</t>
         </is>
       </c>
-      <c r="E23" s="38" cm="1">
+      <c r="E23" s="39" cm="1">
         <f t="array" ref="E23">INDEX(_xlfn.ANCHORARRAY(Z8),3,2)</f>
         <v/>
       </c>
-      <c r="F23" s="38" cm="1">
+      <c r="F23" s="39" cm="1">
         <f t="array" ref="F23">INDEX(_xlfn.ANCHORARRAY(Z8),3,3)</f>
         <v/>
       </c>
-      <c r="G23" s="34" t="inlineStr">
+      <c r="G23" s="35" t="inlineStr">
         <is>
           <t>kN</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr"/>
-      <c r="I23" s="36">
+      <c r="I23" s="37">
         <f>IF(OR(E23="",N(F23)=0),"",ABS(E23)/F23)</f>
         <v/>
       </c>
-      <c r="J23" s="37">
+      <c r="J23" s="38">
         <f>IF(I23="","–",IF(I23&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
-      <c r="M23" s="21" t="n"/>
-      <c r="N23" s="22" t="n"/>
-      <c r="O23" s="22" t="n"/>
-      <c r="P23" s="22" t="n"/>
-      <c r="Q23" s="22" t="n"/>
-      <c r="R23" s="22" t="n"/>
-      <c r="S23" s="22" t="n"/>
-      <c r="T23" s="23" t="n"/>
+      <c r="M23" s="22" t="n"/>
+      <c r="N23" s="23" t="n"/>
+      <c r="O23" s="23" t="n"/>
+      <c r="P23" s="23" t="n"/>
+      <c r="Q23" s="23" t="n"/>
+      <c r="R23" s="23" t="n"/>
+      <c r="S23" s="23" t="n"/>
+      <c r="T23" s="24" t="n"/>
+      <c r="AN23" s="20" t="inlineStr">
+        <is>
+          <t>800WB192</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="14" customHeight="1">
-      <c r="M24" s="21" t="n"/>
-      <c r="N24" s="22" t="n"/>
-      <c r="O24" s="22" t="n"/>
-      <c r="P24" s="22" t="n"/>
-      <c r="Q24" s="22" t="n"/>
-      <c r="R24" s="22" t="n"/>
-      <c r="S24" s="22" t="n"/>
-      <c r="T24" s="23" t="n"/>
+      <c r="M24" s="22" t="n"/>
+      <c r="N24" s="23" t="n"/>
+      <c r="O24" s="23" t="n"/>
+      <c r="P24" s="23" t="n"/>
+      <c r="Q24" s="23" t="n"/>
+      <c r="R24" s="23" t="n"/>
+      <c r="S24" s="23" t="n"/>
+      <c r="T24" s="24" t="n"/>
+      <c r="AN24" s="20" t="inlineStr">
+        <is>
+          <t>800WB168</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="10" t="inlineStr">
@@ -2477,17 +2569,22 @@
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="11" t="n"/>
       <c r="J25" s="11" t="n"/>
-      <c r="M25" s="21" t="n"/>
-      <c r="N25" s="22" t="n"/>
-      <c r="O25" s="22" t="n"/>
-      <c r="P25" s="22" t="n"/>
-      <c r="Q25" s="22" t="n"/>
-      <c r="R25" s="22" t="n"/>
-      <c r="S25" s="22" t="n"/>
-      <c r="T25" s="23" t="n"/>
+      <c r="M25" s="22" t="n"/>
+      <c r="N25" s="23" t="n"/>
+      <c r="O25" s="23" t="n"/>
+      <c r="P25" s="23" t="n"/>
+      <c r="Q25" s="23" t="n"/>
+      <c r="R25" s="23" t="n"/>
+      <c r="S25" s="23" t="n"/>
+      <c r="T25" s="24" t="n"/>
+      <c r="AN25" s="20" t="inlineStr">
+        <is>
+          <t>800WB146</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="14" customHeight="1">
-      <c r="B26" s="39" t="inlineStr">
+      <c r="B26" s="40" t="inlineStr">
         <is>
           <t>Section type</t>
         </is>
@@ -2497,22 +2594,27 @@
           <t>UB</t>
         </is>
       </c>
-      <c r="G26" s="40" t="inlineStr">
+      <c r="G26" s="41" t="inlineStr">
         <is>
           <t>Section properties (add-in)</t>
         </is>
       </c>
-      <c r="M26" s="21" t="n"/>
-      <c r="N26" s="22" t="n"/>
-      <c r="O26" s="22" t="n"/>
-      <c r="P26" s="22" t="n"/>
-      <c r="Q26" s="22" t="n"/>
-      <c r="R26" s="22" t="n"/>
-      <c r="S26" s="22" t="n"/>
-      <c r="T26" s="23" t="n"/>
+      <c r="M26" s="22" t="n"/>
+      <c r="N26" s="23" t="n"/>
+      <c r="O26" s="23" t="n"/>
+      <c r="P26" s="23" t="n"/>
+      <c r="Q26" s="23" t="n"/>
+      <c r="R26" s="23" t="n"/>
+      <c r="S26" s="23" t="n"/>
+      <c r="T26" s="24" t="n"/>
+      <c r="AN26" s="20" t="inlineStr">
+        <is>
+          <t>800WB122</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="14" customHeight="1">
-      <c r="B27" s="39" t="inlineStr">
+      <c r="B27" s="40" t="inlineStr">
         <is>
           <t>Section size</t>
         </is>
@@ -2522,105 +2624,120 @@
           <t>310UB40.4</t>
         </is>
       </c>
-      <c r="G27" s="41" t="inlineStr">
+      <c r="G27" s="42" t="inlineStr">
         <is>
           <t>Mass</t>
         </is>
       </c>
-      <c r="H27" s="38" cm="1">
+      <c r="H27" s="39" cm="1">
         <f t="array" ref="H27">OAR.SECTION(SectionSize,"Mass",Grade)</f>
         <v/>
       </c>
-      <c r="I27" s="42" t="inlineStr">
+      <c r="I27" s="43" t="inlineStr">
         <is>
           <t>kg/m</t>
         </is>
       </c>
-      <c r="M27" s="21" t="n"/>
-      <c r="N27" s="22" t="n"/>
-      <c r="O27" s="22" t="n"/>
-      <c r="P27" s="22" t="n"/>
-      <c r="Q27" s="22" t="n"/>
-      <c r="R27" s="22" t="n"/>
-      <c r="S27" s="22" t="n"/>
-      <c r="T27" s="23" t="n"/>
+      <c r="M27" s="22" t="n"/>
+      <c r="N27" s="23" t="n"/>
+      <c r="O27" s="23" t="n"/>
+      <c r="P27" s="23" t="n"/>
+      <c r="Q27" s="23" t="n"/>
+      <c r="R27" s="23" t="n"/>
+      <c r="S27" s="23" t="n"/>
+      <c r="T27" s="24" t="n"/>
+      <c r="AN27" s="20" t="inlineStr">
+        <is>
+          <t>700WB173</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="14" customHeight="1">
-      <c r="B28" s="39" t="inlineStr">
+      <c r="B28" s="40" t="inlineStr">
         <is>
           <t>Steel grade</t>
         </is>
       </c>
-      <c r="E28" s="43" t="n">
+      <c r="E28" s="44" t="n">
         <v>300</v>
       </c>
-      <c r="F28" s="42" t="inlineStr">
+      <c r="F28" s="43" t="inlineStr">
         <is>
           <t>MPa</t>
         </is>
       </c>
-      <c r="G28" s="41" t="inlineStr">
+      <c r="G28" s="42" t="inlineStr">
         <is>
           <t>Ix</t>
         </is>
       </c>
-      <c r="H28" s="38" cm="1">
+      <c r="H28" s="39" cm="1">
         <f t="array" ref="H28">OAR.SECTION(SectionSize,"Ix",Grade)</f>
         <v/>
       </c>
-      <c r="I28" s="42" t="inlineStr">
+      <c r="I28" s="43" t="inlineStr">
         <is>
           <t>×10⁶ mm⁴</t>
         </is>
       </c>
-      <c r="M28" s="21" t="n"/>
-      <c r="N28" s="22" t="n"/>
-      <c r="O28" s="22" t="n"/>
-      <c r="P28" s="22" t="n"/>
-      <c r="Q28" s="22" t="n"/>
-      <c r="R28" s="22" t="n"/>
-      <c r="S28" s="22" t="n"/>
-      <c r="T28" s="23" t="n"/>
+      <c r="M28" s="22" t="n"/>
+      <c r="N28" s="23" t="n"/>
+      <c r="O28" s="23" t="n"/>
+      <c r="P28" s="23" t="n"/>
+      <c r="Q28" s="23" t="n"/>
+      <c r="R28" s="23" t="n"/>
+      <c r="S28" s="23" t="n"/>
+      <c r="T28" s="24" t="n"/>
+      <c r="AN28" s="20" t="inlineStr">
+        <is>
+          <t>700WB150</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="14" customHeight="1">
-      <c r="B29" s="39" t="inlineStr">
+      <c r="B29" s="40" t="inlineStr">
         <is>
           <t>Span (centre to centre of supports)</t>
         </is>
       </c>
-      <c r="E29" s="44" t="n">
+      <c r="E29" s="45" t="n">
         <v>8300</v>
       </c>
-      <c r="F29" s="42" t="inlineStr">
+      <c r="F29" s="43" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="G29" s="41" t="inlineStr">
+      <c r="G29" s="42" t="inlineStr">
         <is>
           <t>Iy</t>
         </is>
       </c>
-      <c r="H29" s="33" cm="1">
+      <c r="H29" s="34" cm="1">
         <f t="array" ref="H29">OAR.SECTION(SectionSize,"Iy",Grade)</f>
         <v/>
       </c>
-      <c r="I29" s="42" t="inlineStr">
+      <c r="I29" s="43" t="inlineStr">
         <is>
           <t>×10⁶ mm⁴</t>
         </is>
       </c>
-      <c r="M29" s="21" t="n"/>
-      <c r="N29" s="22" t="n"/>
-      <c r="O29" s="22" t="n"/>
-      <c r="P29" s="22" t="n"/>
-      <c r="Q29" s="22" t="n"/>
-      <c r="R29" s="22" t="n"/>
-      <c r="S29" s="22" t="n"/>
-      <c r="T29" s="23" t="n"/>
+      <c r="M29" s="22" t="n"/>
+      <c r="N29" s="23" t="n"/>
+      <c r="O29" s="23" t="n"/>
+      <c r="P29" s="23" t="n"/>
+      <c r="Q29" s="23" t="n"/>
+      <c r="R29" s="23" t="n"/>
+      <c r="S29" s="23" t="n"/>
+      <c r="T29" s="24" t="n"/>
+      <c r="AN29" s="20" t="inlineStr">
+        <is>
+          <t>700WB130</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="14" customHeight="1">
-      <c r="B30" s="39" t="inlineStr">
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t>Support condition</t>
         </is>
@@ -2630,69 +2747,79 @@
           <t>Simply supported</t>
         </is>
       </c>
-      <c r="F30" s="45" t="n"/>
-      <c r="G30" s="41" t="inlineStr">
+      <c r="F30" s="46" t="n"/>
+      <c r="G30" s="42" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="H30" s="38" cm="1">
+      <c r="H30" s="39" cm="1">
         <f t="array" ref="H30">OAR.SECTION(SectionSize,"J",Grade)</f>
         <v/>
       </c>
-      <c r="I30" s="42" t="inlineStr">
+      <c r="I30" s="43" t="inlineStr">
         <is>
           <t>×10³ mm⁴</t>
         </is>
       </c>
-      <c r="M30" s="21" t="n"/>
-      <c r="N30" s="22" t="n"/>
-      <c r="O30" s="22" t="n"/>
-      <c r="P30" s="22" t="n"/>
-      <c r="Q30" s="22" t="n"/>
-      <c r="R30" s="22" t="n"/>
-      <c r="S30" s="22" t="n"/>
-      <c r="T30" s="23" t="n"/>
+      <c r="M30" s="22" t="n"/>
+      <c r="N30" s="23" t="n"/>
+      <c r="O30" s="23" t="n"/>
+      <c r="P30" s="23" t="n"/>
+      <c r="Q30" s="23" t="n"/>
+      <c r="R30" s="23" t="n"/>
+      <c r="S30" s="23" t="n"/>
+      <c r="T30" s="24" t="n"/>
+      <c r="AN30" s="20" t="inlineStr">
+        <is>
+          <t>700WB115</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="14" customHeight="1">
-      <c r="B31" s="39" t="inlineStr">
+      <c r="B31" s="40" t="inlineStr">
         <is>
           <t>Elastic modulus</t>
         </is>
       </c>
-      <c r="E31" s="44" t="n">
+      <c r="E31" s="45" t="n">
         <v>200000</v>
       </c>
-      <c r="F31" s="42" t="inlineStr">
+      <c r="F31" s="43" t="inlineStr">
         <is>
           <t>MPa</t>
         </is>
       </c>
-      <c r="G31" s="41" t="inlineStr">
+      <c r="G31" s="42" t="inlineStr">
         <is>
           <t>Iw</t>
         </is>
       </c>
-      <c r="H31" s="38" cm="1">
+      <c r="H31" s="39" cm="1">
         <f t="array" ref="H31">OAR.SECTION(SectionSize,"Iw",Grade)</f>
         <v/>
       </c>
-      <c r="I31" s="42" t="inlineStr">
+      <c r="I31" s="43" t="inlineStr">
         <is>
           <t>×10⁹ mm⁶</t>
         </is>
       </c>
-      <c r="M31" s="21" t="n"/>
-      <c r="N31" s="22" t="n"/>
-      <c r="O31" s="22" t="n"/>
-      <c r="P31" s="22" t="n"/>
-      <c r="Q31" s="22" t="n"/>
-      <c r="R31" s="22" t="n"/>
-      <c r="S31" s="22" t="n"/>
-      <c r="T31" s="23" t="n"/>
+      <c r="M31" s="22" t="n"/>
+      <c r="N31" s="23" t="n"/>
+      <c r="O31" s="23" t="n"/>
+      <c r="P31" s="23" t="n"/>
+      <c r="Q31" s="23" t="n"/>
+      <c r="R31" s="23" t="n"/>
+      <c r="S31" s="23" t="n"/>
+      <c r="T31" s="24" t="n"/>
+      <c r="AN31" s="20" t="inlineStr">
+        <is>
+          <t>760UB244</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="14" customHeight="1">
-      <c r="B32" s="39" t="inlineStr">
+      <c r="B32" s="40" t="inlineStr">
         <is>
           <t>Include self-weight</t>
         </is>
@@ -2702,62 +2829,77 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G32" s="41" t="inlineStr">
+      <c r="G32" s="42" t="inlineStr">
         <is>
           <t>Zex</t>
         </is>
       </c>
-      <c r="H32" s="46" cm="1">
+      <c r="H32" s="47" cm="1">
         <f t="array" ref="H32">OAR.SECTION(SectionSize,"Ze",Grade)</f>
         <v/>
       </c>
-      <c r="I32" s="42" t="inlineStr">
+      <c r="I32" s="43" t="inlineStr">
         <is>
           <t>×10³ mm³</t>
         </is>
       </c>
-      <c r="M32" s="21" t="n"/>
-      <c r="N32" s="22" t="n"/>
-      <c r="O32" s="22" t="n"/>
-      <c r="P32" s="22" t="n"/>
-      <c r="Q32" s="22" t="n"/>
-      <c r="R32" s="22" t="n"/>
-      <c r="S32" s="22" t="n"/>
-      <c r="T32" s="23" t="n"/>
+      <c r="M32" s="22" t="n"/>
+      <c r="N32" s="23" t="n"/>
+      <c r="O32" s="23" t="n"/>
+      <c r="P32" s="23" t="n"/>
+      <c r="Q32" s="23" t="n"/>
+      <c r="R32" s="23" t="n"/>
+      <c r="S32" s="23" t="n"/>
+      <c r="T32" s="24" t="n"/>
+      <c r="AN32" s="20" t="inlineStr">
+        <is>
+          <t>760UB220</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="14" customHeight="1">
-      <c r="G33" s="41" t="inlineStr">
+      <c r="G33" s="42" t="inlineStr">
         <is>
           <t>φMsx</t>
         </is>
       </c>
-      <c r="H33" s="38" cm="1">
+      <c r="H33" s="39" cm="1">
         <f t="array" ref="H33">OAR.SECTION(SectionSize,"phiMsx",Grade)</f>
         <v/>
       </c>
-      <c r="I33" s="42" t="inlineStr">
+      <c r="I33" s="43" t="inlineStr">
         <is>
           <t>kN·m</t>
         </is>
       </c>
-      <c r="M33" s="21" t="n"/>
-      <c r="N33" s="22" t="n"/>
-      <c r="O33" s="22" t="n"/>
-      <c r="P33" s="22" t="n"/>
-      <c r="Q33" s="22" t="n"/>
-      <c r="R33" s="22" t="n"/>
-      <c r="S33" s="22" t="n"/>
-      <c r="T33" s="23" t="n"/>
+      <c r="M33" s="22" t="n"/>
+      <c r="N33" s="23" t="n"/>
+      <c r="O33" s="23" t="n"/>
+      <c r="P33" s="23" t="n"/>
+      <c r="Q33" s="23" t="n"/>
+      <c r="R33" s="23" t="n"/>
+      <c r="S33" s="23" t="n"/>
+      <c r="T33" s="24" t="n"/>
+      <c r="AN33" s="20" t="inlineStr">
+        <is>
+          <t>760UB197</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="14" customHeight="1">
-      <c r="M34" s="21" t="n"/>
-      <c r="N34" s="22" t="n"/>
-      <c r="O34" s="22" t="n"/>
-      <c r="P34" s="22" t="n"/>
-      <c r="Q34" s="22" t="n"/>
-      <c r="R34" s="22" t="n"/>
-      <c r="S34" s="22" t="n"/>
-      <c r="T34" s="23" t="n"/>
+      <c r="M34" s="22" t="n"/>
+      <c r="N34" s="23" t="n"/>
+      <c r="O34" s="23" t="n"/>
+      <c r="P34" s="23" t="n"/>
+      <c r="Q34" s="23" t="n"/>
+      <c r="R34" s="23" t="n"/>
+      <c r="S34" s="23" t="n"/>
+      <c r="T34" s="24" t="n"/>
+      <c r="AN34" s="20" t="inlineStr">
+        <is>
+          <t>760UB173</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="10" t="inlineStr">
@@ -2773,70 +2915,80 @@
       <c r="H35" s="11" t="n"/>
       <c r="I35" s="11" t="n"/>
       <c r="J35" s="11" t="n"/>
-      <c r="M35" s="21" t="n"/>
-      <c r="N35" s="22" t="n"/>
-      <c r="O35" s="22" t="n"/>
-      <c r="P35" s="22" t="n"/>
-      <c r="Q35" s="22" t="n"/>
-      <c r="R35" s="22" t="n"/>
-      <c r="S35" s="22" t="n"/>
-      <c r="T35" s="23" t="n"/>
+      <c r="M35" s="22" t="n"/>
+      <c r="N35" s="23" t="n"/>
+      <c r="O35" s="23" t="n"/>
+      <c r="P35" s="23" t="n"/>
+      <c r="Q35" s="23" t="n"/>
+      <c r="R35" s="23" t="n"/>
+      <c r="S35" s="23" t="n"/>
+      <c r="T35" s="24" t="n"/>
+      <c r="AN35" s="20" t="inlineStr">
+        <is>
+          <t>760UB147</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="14" customHeight="1">
-      <c r="B36" s="47" t="inlineStr">
+      <c r="B36" s="48" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C36" s="45" t="n"/>
-      <c r="D36" s="47" t="inlineStr">
+      <c r="C36" s="46" t="n"/>
+      <c r="D36" s="48" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E36" s="47" t="inlineStr">
+      <c r="E36" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">Span / </t>
         </is>
       </c>
-      <c r="F36" s="47" t="inlineStr">
+      <c r="F36" s="48" t="inlineStr">
         <is>
           <t>Max (mm)</t>
         </is>
       </c>
-      <c r="G36" s="47" t="inlineStr">
+      <c r="G36" s="48" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="M36" s="21" t="n"/>
-      <c r="N36" s="22" t="n"/>
-      <c r="O36" s="22" t="n"/>
-      <c r="P36" s="22" t="n"/>
-      <c r="Q36" s="22" t="n"/>
-      <c r="R36" s="22" t="n"/>
-      <c r="S36" s="22" t="n"/>
-      <c r="T36" s="23" t="n"/>
+      <c r="M36" s="22" t="n"/>
+      <c r="N36" s="23" t="n"/>
+      <c r="O36" s="23" t="n"/>
+      <c r="P36" s="23" t="n"/>
+      <c r="Q36" s="23" t="n"/>
+      <c r="R36" s="23" t="n"/>
+      <c r="S36" s="23" t="n"/>
+      <c r="T36" s="24" t="n"/>
+      <c r="AN36" s="20" t="inlineStr">
+        <is>
+          <t>690UB140</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="14" customHeight="1">
-      <c r="B37" s="48" t="inlineStr">
+      <c r="B37" s="49" t="inlineStr">
         <is>
           <t>Δg</t>
         </is>
       </c>
-      <c r="C37" s="49" t="n"/>
-      <c r="D37" s="50" t="inlineStr">
+      <c r="C37" s="50" t="n"/>
+      <c r="D37" s="51" t="inlineStr">
         <is>
           <t>Dead load</t>
         </is>
       </c>
-      <c r="E37" s="43" t="n">
+      <c r="E37" s="44" t="n">
         <v>500</v>
       </c>
-      <c r="F37" s="51" t="n">
+      <c r="F37" s="52" t="n">
         <v>20</v>
       </c>
-      <c r="G37" s="52" t="inlineStr">
+      <c r="G37" s="53" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -2846,34 +2998,39 @@
           <t>Limit = lesser of L/ratio and max</t>
         </is>
       </c>
-      <c r="M37" s="21" t="n"/>
-      <c r="N37" s="22" t="n"/>
-      <c r="O37" s="22" t="n"/>
-      <c r="P37" s="22" t="n"/>
-      <c r="Q37" s="22" t="n"/>
-      <c r="R37" s="22" t="n"/>
-      <c r="S37" s="22" t="n"/>
-      <c r="T37" s="23" t="n"/>
+      <c r="M37" s="22" t="n"/>
+      <c r="N37" s="23" t="n"/>
+      <c r="O37" s="23" t="n"/>
+      <c r="P37" s="23" t="n"/>
+      <c r="Q37" s="23" t="n"/>
+      <c r="R37" s="23" t="n"/>
+      <c r="S37" s="23" t="n"/>
+      <c r="T37" s="24" t="n"/>
+      <c r="AN37" s="20" t="inlineStr">
+        <is>
+          <t>690UB125</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="14" customHeight="1">
-      <c r="B38" s="48" t="inlineStr">
+      <c r="B38" s="49" t="inlineStr">
         <is>
           <t>Δg+ψl·q</t>
         </is>
       </c>
-      <c r="C38" s="49" t="n"/>
-      <c r="D38" s="50" t="inlineStr">
+      <c r="C38" s="50" t="n"/>
+      <c r="D38" s="51" t="inlineStr">
         <is>
           <t>Long term (ψl)</t>
         </is>
       </c>
-      <c r="E38" s="43" t="n">
+      <c r="E38" s="44" t="n">
         <v>360</v>
       </c>
-      <c r="F38" s="51" t="n">
+      <c r="F38" s="52" t="n">
         <v>25</v>
       </c>
-      <c r="G38" s="51" t="n">
+      <c r="G38" s="52" t="n">
         <v>0.4</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
@@ -2881,102 +3038,128 @@
           <t>Blank max = ratio only</t>
         </is>
       </c>
-      <c r="M38" s="21" t="n"/>
-      <c r="N38" s="22" t="n"/>
-      <c r="O38" s="22" t="n"/>
-      <c r="P38" s="22" t="n"/>
-      <c r="Q38" s="22" t="n"/>
-      <c r="R38" s="22" t="n"/>
-      <c r="S38" s="22" t="n"/>
-      <c r="T38" s="23" t="n"/>
+      <c r="M38" s="22" t="n"/>
+      <c r="N38" s="23" t="n"/>
+      <c r="O38" s="23" t="n"/>
+      <c r="P38" s="23" t="n"/>
+      <c r="Q38" s="23" t="n"/>
+      <c r="R38" s="23" t="n"/>
+      <c r="S38" s="23" t="n"/>
+      <c r="T38" s="24" t="n"/>
+      <c r="AN38" s="20" t="inlineStr">
+        <is>
+          <t>610UB125</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="14" customHeight="1">
-      <c r="B39" s="48" t="inlineStr">
+      <c r="B39" s="49" t="inlineStr">
         <is>
           <t>Δg+ψs·q</t>
         </is>
       </c>
-      <c r="C39" s="49" t="n"/>
-      <c r="D39" s="50" t="inlineStr">
+      <c r="C39" s="50" t="n"/>
+      <c r="D39" s="51" t="inlineStr">
         <is>
           <t>Short term (ψs)</t>
         </is>
       </c>
-      <c r="E39" s="43" t="n">
+      <c r="E39" s="44" t="n">
         <v>300</v>
       </c>
-      <c r="F39" s="51" t="n">
+      <c r="F39" s="52" t="n">
         <v>30</v>
       </c>
-      <c r="G39" s="51" t="n">
+      <c r="G39" s="52" t="n">
         <v>0.7</v>
       </c>
-      <c r="M39" s="21" t="n"/>
-      <c r="N39" s="22" t="n"/>
-      <c r="O39" s="22" t="n"/>
-      <c r="P39" s="22" t="n"/>
-      <c r="Q39" s="22" t="n"/>
-      <c r="R39" s="22" t="n"/>
-      <c r="S39" s="22" t="n"/>
-      <c r="T39" s="23" t="n"/>
+      <c r="M39" s="22" t="n"/>
+      <c r="N39" s="23" t="n"/>
+      <c r="O39" s="23" t="n"/>
+      <c r="P39" s="23" t="n"/>
+      <c r="Q39" s="23" t="n"/>
+      <c r="R39" s="23" t="n"/>
+      <c r="S39" s="23" t="n"/>
+      <c r="T39" s="24" t="n"/>
+      <c r="AN39" s="20" t="inlineStr">
+        <is>
+          <t>610UB113</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="14" customHeight="1">
-      <c r="B40" s="48" t="inlineStr">
+      <c r="B40" s="49" t="inlineStr">
         <is>
           <t>Δq</t>
         </is>
       </c>
-      <c r="C40" s="49" t="n"/>
-      <c r="D40" s="50" t="inlineStr">
+      <c r="C40" s="50" t="n"/>
+      <c r="D40" s="51" t="inlineStr">
         <is>
           <t>Live load only</t>
         </is>
       </c>
-      <c r="E40" s="43" t="n">
+      <c r="E40" s="44" t="n">
         <v>250</v>
       </c>
-      <c r="F40" s="51" t="n">
+      <c r="F40" s="52" t="n">
         <v>30</v>
       </c>
-      <c r="G40" s="52" t="inlineStr">
+      <c r="G40" s="53" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="M40" s="53" t="n"/>
-      <c r="N40" s="54" t="n"/>
-      <c r="O40" s="54" t="n"/>
-      <c r="P40" s="54" t="n"/>
-      <c r="Q40" s="54" t="n"/>
-      <c r="R40" s="54" t="n"/>
-      <c r="S40" s="54" t="n"/>
-      <c r="T40" s="55" t="n"/>
+      <c r="M40" s="54" t="n"/>
+      <c r="N40" s="55" t="n"/>
+      <c r="O40" s="55" t="n"/>
+      <c r="P40" s="55" t="n"/>
+      <c r="Q40" s="55" t="n"/>
+      <c r="R40" s="55" t="n"/>
+      <c r="S40" s="55" t="n"/>
+      <c r="T40" s="56" t="n"/>
+      <c r="AN40" s="20" t="inlineStr">
+        <is>
+          <t>610UB101</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="14" customHeight="1">
-      <c r="B41" s="48" t="inlineStr">
+      <c r="B41" s="49" t="inlineStr">
         <is>
           <t>Δ1kN</t>
         </is>
       </c>
-      <c r="C41" s="49" t="n"/>
-      <c r="D41" s="50" t="inlineStr">
+      <c r="C41" s="50" t="n"/>
+      <c r="D41" s="51" t="inlineStr">
         <is>
           <t>1 kN point load at midspan</t>
         </is>
       </c>
-      <c r="E41" s="43" t="n">
+      <c r="E41" s="44" t="n">
         <v>1000</v>
       </c>
-      <c r="F41" s="51" t="n">
+      <c r="F41" s="52" t="n">
         <v>1.5</v>
       </c>
-      <c r="G41" s="52" t="inlineStr">
+      <c r="G41" s="53" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-    </row>
-    <row r="42" ht="14" customHeight="1"/>
+      <c r="AN41" s="20" t="inlineStr">
+        <is>
+          <t>530UB92.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="14" customHeight="1">
+      <c r="AN42" s="20" t="inlineStr">
+        <is>
+          <t>530UB82</t>
+        </is>
+      </c>
+    </row>
     <row r="43" ht="20" customHeight="1">
       <c r="B43" s="10" t="inlineStr">
         <is>
@@ -3007,6 +3190,11 @@
       <c r="V43" s="11" t="n"/>
       <c r="W43" s="11" t="n"/>
       <c r="X43" s="11" t="n"/>
+      <c r="AN43" s="20" t="inlineStr">
+        <is>
+          <t>460UB82.1</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="14" customHeight="1">
       <c r="B44" s="15" t="inlineStr">
@@ -3019,6 +3207,11 @@
           <t>Include: blank = follow the Combination set;  Yes / No = force on or off.  Active rows appear in the calc.</t>
         </is>
       </c>
+      <c r="AN44" s="20" t="inlineStr">
+        <is>
+          <t>460UB74.6</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="14" customHeight="1">
       <c r="B45" s="15" t="inlineStr">
@@ -3031,111 +3224,121 @@
           <t>Groups: Gravity (Floor, Roof, All), Wind (Roof, All), Storage (All only), Custom (always, unless Include = No).  Add rows at the bottom for custom combinations.</t>
         </is>
       </c>
+      <c r="AN45" s="20" t="inlineStr">
+        <is>
+          <t>460UB67.1</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="26" customHeight="1">
-      <c r="B46" s="56" t="inlineStr">
+      <c r="B46" s="57" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C46" s="56" t="inlineStr">
+      <c r="C46" s="57" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D46" s="56" t="inlineStr">
+      <c r="D46" s="57" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E46" s="56" t="inlineStr">
+      <c r="E46" s="57" t="inlineStr">
         <is>
           <t>Trib (m | m²)</t>
         </is>
       </c>
-      <c r="F46" s="56" t="inlineStr">
+      <c r="F46" s="57" t="inlineStr">
         <is>
           <t>Press. (kPa)</t>
         </is>
       </c>
-      <c r="G46" s="56" t="inlineStr">
+      <c r="G46" s="57" t="inlineStr">
         <is>
           <t>+ Direct (kN/m | kN)</t>
         </is>
       </c>
-      <c r="H46" s="56" t="inlineStr">
+      <c r="H46" s="57" t="inlineStr">
         <is>
           <t>Start (mm)</t>
         </is>
       </c>
-      <c r="I46" s="56" t="inlineStr">
+      <c r="I46" s="57" t="inlineStr">
         <is>
           <t>End (mm)</t>
         </is>
       </c>
-      <c r="J46" s="56" t="inlineStr">
+      <c r="J46" s="57" t="inlineStr">
         <is>
           <t>Load</t>
         </is>
       </c>
-      <c r="M46" s="28" t="inlineStr">
+      <c r="M46" s="29" t="inlineStr">
         <is>
           <t>Include</t>
         </is>
       </c>
-      <c r="N46" s="28" t="inlineStr">
+      <c r="N46" s="29" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="O46" s="28" t="inlineStr">
+      <c r="O46" s="29" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="P46" s="28" t="inlineStr">
+      <c r="P46" s="29" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="Q46" s="28" t="inlineStr">
+      <c r="Q46" s="29" t="inlineStr">
         <is>
           <t>Crit. flange</t>
         </is>
       </c>
-      <c r="R46" s="28" t="inlineStr">
+      <c r="R46" s="29" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="S46" s="28" t="inlineStr">
+      <c r="S46" s="29" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="T46" s="28" t="inlineStr">
+      <c r="T46" s="29" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="U46" s="28" t="inlineStr">
+      <c r="U46" s="29" t="inlineStr">
         <is>
           <t>Wd</t>
         </is>
       </c>
-      <c r="V46" s="28" t="inlineStr">
+      <c r="V46" s="29" t="inlineStr">
         <is>
           <t>Wu</t>
         </is>
       </c>
-      <c r="W46" s="28" t="inlineStr">
+      <c r="W46" s="29" t="inlineStr">
         <is>
           <t>Wid</t>
         </is>
       </c>
-      <c r="X46" s="28" t="inlineStr">
+      <c r="X46" s="29" t="inlineStr">
         <is>
           <t>Wiu</t>
+        </is>
+      </c>
+      <c r="AN46" s="20" t="inlineStr">
+        <is>
+          <t>410UB59.7</t>
         </is>
       </c>
     </row>
@@ -3155,21 +3358,21 @@
           <t>Roof sheeting + purlins</t>
         </is>
       </c>
-      <c r="E47" s="57" t="n">
+      <c r="E47" s="58" t="n">
         <v>5.65</v>
       </c>
-      <c r="F47" s="58" t="n">
+      <c r="F47" s="59" t="n">
         <v>0.1</v>
       </c>
-      <c r="G47" s="58" t="n"/>
-      <c r="H47" s="44" t="n"/>
-      <c r="I47" s="44" t="n"/>
-      <c r="J47" s="59">
+      <c r="G47" s="59" t="n"/>
+      <c r="H47" s="45" t="n"/>
+      <c r="I47" s="45" t="n"/>
+      <c r="J47" s="60">
         <f>IF(B47="","",N(E47)*N(F47)+N(G47))</f>
         <v/>
       </c>
       <c r="M47" s="2" t="n"/>
-      <c r="N47" s="60">
+      <c r="N47" s="61">
         <f>IF(M47="No",0,IF(P47="",0,IF(M47="Yes",1,IF(OR(CombSet="All",O47="Custom",AND(O47="Gravity",CombSet&lt;&gt;"Custom"),AND(O47="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3193,23 +3396,28 @@
           <t>1.35G</t>
         </is>
       </c>
-      <c r="S47" s="58" t="n">
+      <c r="S47" s="59" t="n">
         <v>1.35</v>
       </c>
-      <c r="T47" s="58" t="n">
+      <c r="T47" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="U47" s="58" t="n">
+      <c r="U47" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="V47" s="58" t="n">
+      <c r="V47" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="W47" s="58" t="n">
+      <c r="W47" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="X47" s="58" t="n">
+      <c r="X47" s="59" t="n">
         <v>0</v>
+      </c>
+      <c r="AN47" s="20" t="inlineStr">
+        <is>
+          <t>410UB53.7</t>
+        </is>
       </c>
     </row>
     <row r="48" ht="14" customHeight="1">
@@ -3228,21 +3436,21 @@
           <t>Ceiling + services</t>
         </is>
       </c>
-      <c r="E48" s="57" t="n">
+      <c r="E48" s="58" t="n">
         <v>5.65</v>
       </c>
-      <c r="F48" s="58" t="n">
+      <c r="F48" s="59" t="n">
         <v>0.15</v>
       </c>
-      <c r="G48" s="58" t="n"/>
-      <c r="H48" s="44" t="n"/>
-      <c r="I48" s="44" t="n"/>
-      <c r="J48" s="59">
+      <c r="G48" s="59" t="n"/>
+      <c r="H48" s="45" t="n"/>
+      <c r="I48" s="45" t="n"/>
+      <c r="J48" s="60">
         <f>IF(B48="","",N(E48)*N(F48)+N(G48))</f>
         <v/>
       </c>
       <c r="M48" s="2" t="n"/>
-      <c r="N48" s="60">
+      <c r="N48" s="61">
         <f>IF(M48="No",0,IF(P48="",0,IF(M48="Yes",1,IF(OR(CombSet="All",O48="Custom",AND(O48="Gravity",CombSet&lt;&gt;"Custom"),AND(O48="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3266,23 +3474,28 @@
           <t>1.2G + 1.5Q</t>
         </is>
       </c>
-      <c r="S48" s="58" t="n">
+      <c r="S48" s="59" t="n">
         <v>1.2</v>
       </c>
-      <c r="T48" s="58" t="n">
+      <c r="T48" s="59" t="n">
         <v>1.5</v>
       </c>
-      <c r="U48" s="58" t="n">
+      <c r="U48" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="V48" s="58" t="n">
+      <c r="V48" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="W48" s="58" t="n">
+      <c r="W48" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="X48" s="58" t="n">
+      <c r="X48" s="59" t="n">
         <v>0</v>
+      </c>
+      <c r="AN48" s="20" t="inlineStr">
+        <is>
+          <t>360UB56.7</t>
+        </is>
       </c>
     </row>
     <row r="49" ht="14" customHeight="1">
@@ -3301,19 +3514,19 @@
           <t>Beam bracket / misc.</t>
         </is>
       </c>
-      <c r="E49" s="57" t="n"/>
-      <c r="F49" s="58" t="n"/>
-      <c r="G49" s="58" t="n">
+      <c r="E49" s="58" t="n"/>
+      <c r="F49" s="59" t="n"/>
+      <c r="G49" s="59" t="n">
         <v>0.05</v>
       </c>
-      <c r="H49" s="44" t="n"/>
-      <c r="I49" s="44" t="n"/>
-      <c r="J49" s="59">
+      <c r="H49" s="45" t="n"/>
+      <c r="I49" s="45" t="n"/>
+      <c r="J49" s="60">
         <f>IF(B49="","",N(E49)*N(F49)+N(G49))</f>
         <v/>
       </c>
       <c r="M49" s="2" t="n"/>
-      <c r="N49" s="60">
+      <c r="N49" s="61">
         <f>IF(M49="No",0,IF(P49="",0,IF(M49="Yes",1,IF(OR(CombSet="All",O49="Custom",AND(O49="Gravity",CombSet&lt;&gt;"Custom"),AND(O49="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3337,24 +3550,29 @@
           <t>1.2G + 1.5ψlQ</t>
         </is>
       </c>
-      <c r="S49" s="58" t="n">
+      <c r="S49" s="59" t="n">
         <v>1.2</v>
       </c>
-      <c r="T49" s="58">
+      <c r="T49" s="59">
         <f>1.5*PsiL</f>
         <v/>
       </c>
-      <c r="U49" s="58" t="n">
+      <c r="U49" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="V49" s="58" t="n">
+      <c r="V49" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="W49" s="58" t="n">
+      <c r="W49" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="X49" s="58" t="n">
+      <c r="X49" s="59" t="n">
         <v>0</v>
+      </c>
+      <c r="AN49" s="20" t="inlineStr">
+        <is>
+          <t>360UB50.7</t>
+        </is>
       </c>
     </row>
     <row r="50" ht="14" customHeight="1">
@@ -3373,21 +3591,21 @@
           <t>Roof live (non-trafficable)</t>
         </is>
       </c>
-      <c r="E50" s="57" t="n">
+      <c r="E50" s="58" t="n">
         <v>5.65</v>
       </c>
-      <c r="F50" s="58" t="n">
+      <c r="F50" s="59" t="n">
         <v>0.25</v>
       </c>
-      <c r="G50" s="58" t="n"/>
-      <c r="H50" s="44" t="n"/>
-      <c r="I50" s="44" t="n"/>
-      <c r="J50" s="59">
+      <c r="G50" s="59" t="n"/>
+      <c r="H50" s="45" t="n"/>
+      <c r="I50" s="45" t="n"/>
+      <c r="J50" s="60">
         <f>IF(B50="","",N(E50)*N(F50)+N(G50))</f>
         <v/>
       </c>
       <c r="M50" s="2" t="n"/>
-      <c r="N50" s="60">
+      <c r="N50" s="61">
         <f>IF(M50="No",0,IF(P50="",0,IF(M50="Yes",1,IF(OR(CombSet="All",O50="Custom",AND(O50="Gravity",CombSet&lt;&gt;"Custom"),AND(O50="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3411,24 +3629,29 @@
           <t>1.2G + ψcQ + Wd + Wi(−cpi)</t>
         </is>
       </c>
-      <c r="S50" s="58" t="n">
+      <c r="S50" s="59" t="n">
         <v>1.2</v>
       </c>
-      <c r="T50" s="58">
+      <c r="T50" s="59">
         <f>PsiC</f>
         <v/>
       </c>
-      <c r="U50" s="58" t="n">
+      <c r="U50" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="V50" s="58" t="n">
+      <c r="V50" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="W50" s="58" t="n">
+      <c r="W50" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="X50" s="58" t="n">
+      <c r="X50" s="59" t="n">
         <v>0</v>
+      </c>
+      <c r="AN50" s="20" t="inlineStr">
+        <is>
+          <t>360UB44.7</t>
+        </is>
       </c>
     </row>
     <row r="51" ht="14" customHeight="1">
@@ -3447,21 +3670,21 @@
           <t>External wind – net uplift</t>
         </is>
       </c>
-      <c r="E51" s="57" t="n">
+      <c r="E51" s="58" t="n">
         <v>5.65</v>
       </c>
-      <c r="F51" s="58" t="n">
+      <c r="F51" s="59" t="n">
         <v>1.72</v>
       </c>
-      <c r="G51" s="58" t="n"/>
-      <c r="H51" s="44" t="n"/>
-      <c r="I51" s="44" t="n"/>
-      <c r="J51" s="59">
+      <c r="G51" s="59" t="n"/>
+      <c r="H51" s="45" t="n"/>
+      <c r="I51" s="45" t="n"/>
+      <c r="J51" s="60">
         <f>IF(B51="","",N(E51)*N(F51)+N(G51))</f>
         <v/>
       </c>
       <c r="M51" s="2" t="n"/>
-      <c r="N51" s="60">
+      <c r="N51" s="61">
         <f>IF(M51="No",0,IF(P51="",0,IF(M51="Yes",1,IF(OR(CombSet="All",O51="Custom",AND(O51="Gravity",CombSet&lt;&gt;"Custom"),AND(O51="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3485,23 +3708,28 @@
           <t>0.9G + Wu + Wi(+cpi)</t>
         </is>
       </c>
-      <c r="S51" s="58" t="n">
+      <c r="S51" s="59" t="n">
         <v>0.9</v>
       </c>
-      <c r="T51" s="58" t="n">
+      <c r="T51" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="U51" s="58" t="n">
+      <c r="U51" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="V51" s="58" t="n">
+      <c r="V51" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="W51" s="58" t="n">
+      <c r="W51" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="X51" s="58" t="n">
+      <c r="X51" s="59" t="n">
         <v>1</v>
+      </c>
+      <c r="AN51" s="20" t="inlineStr">
+        <is>
+          <t>310UB46.2</t>
+        </is>
       </c>
     </row>
     <row r="52" ht="14" customHeight="1">
@@ -3520,21 +3748,21 @@
           <t>External wind – downward</t>
         </is>
       </c>
-      <c r="E52" s="57" t="n">
+      <c r="E52" s="58" t="n">
         <v>5.65</v>
       </c>
-      <c r="F52" s="58" t="n">
+      <c r="F52" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G52" s="58" t="n"/>
-      <c r="H52" s="44" t="n"/>
-      <c r="I52" s="44" t="n"/>
-      <c r="J52" s="59">
+      <c r="G52" s="59" t="n"/>
+      <c r="H52" s="45" t="n"/>
+      <c r="I52" s="45" t="n"/>
+      <c r="J52" s="60">
         <f>IF(B52="","",N(E52)*N(F52)+N(G52))</f>
         <v/>
       </c>
       <c r="M52" s="2" t="n"/>
-      <c r="N52" s="60">
+      <c r="N52" s="61">
         <f>IF(M52="No",0,IF(P52="",0,IF(M52="Yes",1,IF(OR(CombSet="All",O52="Custom",AND(O52="Gravity",CombSet&lt;&gt;"Custom"),AND(O52="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3546,12 +3774,17 @@
       <c r="P52" s="2" t="n"/>
       <c r="Q52" s="2" t="n"/>
       <c r="R52" s="5" t="n"/>
-      <c r="S52" s="58" t="n"/>
-      <c r="T52" s="58" t="n"/>
-      <c r="U52" s="58" t="n"/>
-      <c r="V52" s="58" t="n"/>
-      <c r="W52" s="58" t="n"/>
-      <c r="X52" s="58" t="n"/>
+      <c r="S52" s="59" t="n"/>
+      <c r="T52" s="59" t="n"/>
+      <c r="U52" s="59" t="n"/>
+      <c r="V52" s="59" t="n"/>
+      <c r="W52" s="59" t="n"/>
+      <c r="X52" s="59" t="n"/>
+      <c r="AN52" s="20" t="inlineStr">
+        <is>
+          <t>310UB40.4</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="14" customHeight="1">
       <c r="B53" s="2" t="inlineStr">
@@ -3569,21 +3802,21 @@
           <t>Internal pressure (+cpi)</t>
         </is>
       </c>
-      <c r="E53" s="57" t="n">
+      <c r="E53" s="58" t="n">
         <v>5.65</v>
       </c>
-      <c r="F53" s="58" t="n">
+      <c r="F53" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G53" s="58" t="n"/>
-      <c r="H53" s="44" t="n"/>
-      <c r="I53" s="44" t="n"/>
-      <c r="J53" s="59">
+      <c r="G53" s="59" t="n"/>
+      <c r="H53" s="45" t="n"/>
+      <c r="I53" s="45" t="n"/>
+      <c r="J53" s="60">
         <f>IF(B53="","",N(E53)*N(F53)+N(G53))</f>
         <v/>
       </c>
       <c r="M53" s="2" t="n"/>
-      <c r="N53" s="60">
+      <c r="N53" s="61">
         <f>IF(M53="No",0,IF(P53="",0,IF(M53="Yes",1,IF(OR(CombSet="All",O53="Custom",AND(O53="Gravity",CombSet&lt;&gt;"Custom"),AND(O53="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3595,12 +3828,17 @@
       <c r="P53" s="2" t="n"/>
       <c r="Q53" s="2" t="n"/>
       <c r="R53" s="5" t="n"/>
-      <c r="S53" s="58" t="n"/>
-      <c r="T53" s="58" t="n"/>
-      <c r="U53" s="58" t="n"/>
-      <c r="V53" s="58" t="n"/>
-      <c r="W53" s="58" t="n"/>
-      <c r="X53" s="58" t="n"/>
+      <c r="S53" s="59" t="n"/>
+      <c r="T53" s="59" t="n"/>
+      <c r="U53" s="59" t="n"/>
+      <c r="V53" s="59" t="n"/>
+      <c r="W53" s="59" t="n"/>
+      <c r="X53" s="59" t="n"/>
+      <c r="AN53" s="20" t="inlineStr">
+        <is>
+          <t>310UB32</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="14" customHeight="1">
       <c r="B54" s="2" t="inlineStr">
@@ -3618,21 +3856,21 @@
           <t>Internal suction (−cpi)</t>
         </is>
       </c>
-      <c r="E54" s="57" t="n">
+      <c r="E54" s="58" t="n">
         <v>5.65</v>
       </c>
-      <c r="F54" s="58" t="n">
+      <c r="F54" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G54" s="58" t="n"/>
-      <c r="H54" s="44" t="n"/>
-      <c r="I54" s="44" t="n"/>
-      <c r="J54" s="59">
+      <c r="G54" s="59" t="n"/>
+      <c r="H54" s="45" t="n"/>
+      <c r="I54" s="45" t="n"/>
+      <c r="J54" s="60">
         <f>IF(B54="","",N(E54)*N(F54)+N(G54))</f>
         <v/>
       </c>
       <c r="M54" s="2" t="n"/>
-      <c r="N54" s="60">
+      <c r="N54" s="61">
         <f>IF(M54="No",0,IF(P54="",0,IF(M54="Yes",1,IF(OR(CombSet="All",O54="Custom",AND(O54="Gravity",CombSet&lt;&gt;"Custom"),AND(O54="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3644,12 +3882,17 @@
       <c r="P54" s="2" t="n"/>
       <c r="Q54" s="2" t="n"/>
       <c r="R54" s="5" t="n"/>
-      <c r="S54" s="58" t="n"/>
-      <c r="T54" s="58" t="n"/>
-      <c r="U54" s="58" t="n"/>
-      <c r="V54" s="58" t="n"/>
-      <c r="W54" s="58" t="n"/>
-      <c r="X54" s="58" t="n"/>
+      <c r="S54" s="59" t="n"/>
+      <c r="T54" s="59" t="n"/>
+      <c r="U54" s="59" t="n"/>
+      <c r="V54" s="59" t="n"/>
+      <c r="W54" s="59" t="n"/>
+      <c r="X54" s="59" t="n"/>
+      <c r="AN54" s="20" t="inlineStr">
+        <is>
+          <t>250UB37.3</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="14" customHeight="1">
       <c r="B55" s="2" t="inlineStr">
@@ -3667,34 +3910,39 @@
           <t>Mech. unit on platform (example)</t>
         </is>
       </c>
-      <c r="E55" s="57" t="n">
+      <c r="E55" s="58" t="n">
         <v>1.5</v>
       </c>
-      <c r="F55" s="58" t="n">
+      <c r="F55" s="59" t="n">
         <v>0.5</v>
       </c>
-      <c r="G55" s="58" t="n">
+      <c r="G55" s="59" t="n">
         <v>2</v>
       </c>
-      <c r="H55" s="44" t="n">
+      <c r="H55" s="45" t="n">
         <v>4150</v>
       </c>
-      <c r="I55" s="44" t="n"/>
-      <c r="J55" s="59">
+      <c r="I55" s="45" t="n"/>
+      <c r="J55" s="60">
         <f>IF(B55="","",N(E55)*N(F55)+N(G55))</f>
         <v/>
+      </c>
+      <c r="AN55" s="20" t="inlineStr">
+        <is>
+          <t>250UB31.4</t>
+        </is>
       </c>
     </row>
     <row r="56" ht="14" customHeight="1">
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="5" t="n"/>
-      <c r="E56" s="57" t="n"/>
-      <c r="F56" s="58" t="n"/>
-      <c r="G56" s="58" t="n"/>
-      <c r="H56" s="44" t="n"/>
-      <c r="I56" s="44" t="n"/>
-      <c r="J56" s="59">
+      <c r="E56" s="58" t="n"/>
+      <c r="F56" s="59" t="n"/>
+      <c r="G56" s="59" t="n"/>
+      <c r="H56" s="45" t="n"/>
+      <c r="I56" s="45" t="n"/>
+      <c r="J56" s="60">
         <f>IF(B56="","",N(E56)*N(F56)+N(G56))</f>
         <v/>
       </c>
@@ -3703,90 +3951,122 @@
           <t>Active uplift (bottom flange) combinations:</t>
         </is>
       </c>
-      <c r="S56" s="46">
+      <c r="S56" s="47">
         <f>COUNTIFS(CombLib_B1[Active],1,CombLib_B1[Crit. flange],"Bottom")</f>
         <v/>
+      </c>
+      <c r="AN56" s="20" t="inlineStr">
+        <is>
+          <t>250UB25.7</t>
+        </is>
       </c>
     </row>
     <row r="57" ht="14" customHeight="1">
       <c r="B57" s="2" t="n"/>
       <c r="C57" s="2" t="n"/>
       <c r="D57" s="5" t="n"/>
-      <c r="E57" s="57" t="n"/>
-      <c r="F57" s="58" t="n"/>
-      <c r="G57" s="58" t="n"/>
-      <c r="H57" s="44" t="n"/>
-      <c r="I57" s="44" t="n"/>
-      <c r="J57" s="59">
+      <c r="E57" s="58" t="n"/>
+      <c r="F57" s="59" t="n"/>
+      <c r="G57" s="59" t="n"/>
+      <c r="H57" s="45" t="n"/>
+      <c r="I57" s="45" t="n"/>
+      <c r="J57" s="60">
         <f>IF(B57="","",N(E57)*N(F57)+N(G57))</f>
         <v/>
       </c>
-    </row>
-    <row r="58" ht="14" customHeight="1"/>
+      <c r="AN57" s="20" t="inlineStr">
+        <is>
+          <t>200UB29.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="14" customHeight="1">
+      <c r="AN58" s="20" t="inlineStr">
+        <is>
+          <t>200UB25.4</t>
+        </is>
+      </c>
+    </row>
     <row r="59" ht="14" customHeight="1">
-      <c r="E59" s="47" t="inlineStr">
+      <c r="E59" s="48" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="F59" s="47" t="inlineStr">
+      <c r="F59" s="48" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="G59" s="47" t="inlineStr">
+      <c r="G59" s="48" t="inlineStr">
         <is>
           <t>Wd</t>
         </is>
       </c>
-      <c r="H59" s="47" t="inlineStr">
+      <c r="H59" s="48" t="inlineStr">
         <is>
           <t>Wu</t>
         </is>
       </c>
-      <c r="I59" s="47" t="inlineStr">
+      <c r="I59" s="48" t="inlineStr">
         <is>
           <t>Wid</t>
         </is>
       </c>
-      <c r="J59" s="47" t="inlineStr">
+      <c r="J59" s="48" t="inlineStr">
         <is>
           <t>Wiu</t>
         </is>
       </c>
+      <c r="AN59" s="20" t="inlineStr">
+        <is>
+          <t>200UB22.3</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="14" customHeight="1">
-      <c r="B60" s="40" t="inlineStr">
+      <c r="B60" s="41" t="inlineStr">
         <is>
           <t>Full-span UDL totals (excl. self-weight):</t>
         </is>
       </c>
-      <c r="E60" s="59">
+      <c r="E60" s="60">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"G",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-      <c r="F60" s="59">
+      <c r="F60" s="60">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"Q",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-      <c r="G60" s="59">
+      <c r="G60" s="60">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"Wd",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-      <c r="H60" s="59">
+      <c r="H60" s="60">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"Wu",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-      <c r="I60" s="59">
+      <c r="I60" s="60">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"Wid",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-      <c r="J60" s="59">
+      <c r="J60" s="60">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"Wiu",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-    </row>
-    <row r="61" ht="14" customHeight="1"/>
+      <c r="AN60" s="20" t="inlineStr">
+        <is>
+          <t>200UB18.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="14" customHeight="1">
+      <c r="AN61" s="20" t="inlineStr">
+        <is>
+          <t>180UB22.2</t>
+        </is>
+      </c>
+    </row>
     <row r="62" ht="20" customHeight="1">
       <c r="B62" s="10" t="inlineStr">
         <is>
@@ -3801,9 +4081,14 @@
       <c r="H62" s="11" t="n"/>
       <c r="I62" s="11" t="n"/>
       <c r="J62" s="11" t="n"/>
+      <c r="AN62" s="20" t="inlineStr">
+        <is>
+          <t>180UB18.1</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="14" customHeight="1">
-      <c r="B63" s="39" t="inlineStr">
+      <c r="B63" s="40" t="inlineStr">
         <is>
           <t>Combination set</t>
         </is>
@@ -3813,17 +4098,22 @@
           <t>Roof</t>
         </is>
       </c>
-      <c r="F63" s="41" t="inlineStr">
+      <c r="F63" s="42" t="inlineStr">
         <is>
           <t>ψc</t>
         </is>
       </c>
-      <c r="G63" s="51" t="n">
+      <c r="G63" s="52" t="n">
         <v>0.4</v>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
           <t>Table 4.1 (roofs 0.0)</t>
+        </is>
+      </c>
+      <c r="AN63" s="20" t="inlineStr">
+        <is>
+          <t>180UB16.1</t>
         </is>
       </c>
     </row>
@@ -3833,144 +4123,194 @@
           <t>Floor = gravity only.  Roof = gravity + wind.  All = every library row.  Custom = only rows set to Yes / Custom.  Edit in the library to the right →</t>
         </is>
       </c>
+      <c r="AN64" s="20" t="inlineStr">
+        <is>
+          <t>150UB18</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="14" customHeight="1">
-      <c r="B65" s="28" t="inlineStr">
+      <c r="B65" s="29" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C65" s="28" t="inlineStr">
+      <c r="C65" s="29" t="inlineStr">
         <is>
           <t>Crit. flange</t>
         </is>
       </c>
-      <c r="D65" s="28" t="inlineStr">
+      <c r="D65" s="29" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="E65" s="28" t="inlineStr">
+      <c r="E65" s="29" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="F65" s="28" t="inlineStr">
+      <c r="F65" s="29" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="G65" s="28" t="inlineStr">
+      <c r="G65" s="29" t="inlineStr">
         <is>
           <t>Wd</t>
         </is>
       </c>
-      <c r="H65" s="28" t="inlineStr">
+      <c r="H65" s="29" t="inlineStr">
         <is>
           <t>Wu</t>
         </is>
       </c>
-      <c r="I65" s="28" t="inlineStr">
+      <c r="I65" s="29" t="inlineStr">
         <is>
           <t>Wid</t>
         </is>
       </c>
-      <c r="J65" s="28" t="inlineStr">
+      <c r="J65" s="29" t="inlineStr">
         <is>
           <t>Wiu</t>
         </is>
       </c>
+      <c r="AN65" s="20" t="inlineStr">
+        <is>
+          <t>150UB14</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="14" customHeight="1">
-      <c r="B66" s="31" cm="1">
+      <c r="B66" s="32" cm="1">
         <f t="array" ref="B66">_xlfn._xlws.FILTER(CombLib_B1[[ID]:[Wiu]],CombLib_B1[Active]=1,"No combinations selected")</f>
         <v/>
       </c>
-      <c r="C66" s="31" t="n"/>
-      <c r="D66" s="39" t="n"/>
-      <c r="E66" s="61" t="n"/>
-      <c r="F66" s="61" t="n"/>
-      <c r="G66" s="61" t="n"/>
-      <c r="H66" s="61" t="n"/>
-      <c r="I66" s="61" t="n"/>
-      <c r="J66" s="61" t="n"/>
+      <c r="C66" s="32" t="n"/>
+      <c r="D66" s="40" t="n"/>
+      <c r="E66" s="62" t="n"/>
+      <c r="F66" s="62" t="n"/>
+      <c r="G66" s="62" t="n"/>
+      <c r="H66" s="62" t="n"/>
+      <c r="I66" s="62" t="n"/>
+      <c r="J66" s="62" t="n"/>
+      <c r="AN66" s="20" t="inlineStr">
+        <is>
+          <t>380PFC</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="14" customHeight="1">
-      <c r="B67" s="31" t="n"/>
-      <c r="C67" s="31" t="n"/>
-      <c r="D67" s="39" t="n"/>
-      <c r="E67" s="61" t="n"/>
-      <c r="F67" s="61" t="n"/>
-      <c r="G67" s="61" t="n"/>
-      <c r="H67" s="61" t="n"/>
-      <c r="I67" s="61" t="n"/>
-      <c r="J67" s="61" t="n"/>
+      <c r="B67" s="32" t="n"/>
+      <c r="C67" s="32" t="n"/>
+      <c r="D67" s="40" t="n"/>
+      <c r="E67" s="62" t="n"/>
+      <c r="F67" s="62" t="n"/>
+      <c r="G67" s="62" t="n"/>
+      <c r="H67" s="62" t="n"/>
+      <c r="I67" s="62" t="n"/>
+      <c r="J67" s="62" t="n"/>
+      <c r="AN67" s="20" t="inlineStr">
+        <is>
+          <t>300PFC</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="14" customHeight="1">
-      <c r="B68" s="31" t="n"/>
-      <c r="C68" s="31" t="n"/>
-      <c r="D68" s="39" t="n"/>
-      <c r="E68" s="61" t="n"/>
-      <c r="F68" s="61" t="n"/>
-      <c r="G68" s="61" t="n"/>
-      <c r="H68" s="61" t="n"/>
-      <c r="I68" s="61" t="n"/>
-      <c r="J68" s="61" t="n"/>
+      <c r="B68" s="32" t="n"/>
+      <c r="C68" s="32" t="n"/>
+      <c r="D68" s="40" t="n"/>
+      <c r="E68" s="62" t="n"/>
+      <c r="F68" s="62" t="n"/>
+      <c r="G68" s="62" t="n"/>
+      <c r="H68" s="62" t="n"/>
+      <c r="I68" s="62" t="n"/>
+      <c r="J68" s="62" t="n"/>
+      <c r="AN68" s="20" t="inlineStr">
+        <is>
+          <t>250PFC</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="14" customHeight="1">
-      <c r="B69" s="31" t="n"/>
-      <c r="C69" s="31" t="n"/>
-      <c r="D69" s="39" t="n"/>
-      <c r="E69" s="61" t="n"/>
-      <c r="F69" s="61" t="n"/>
-      <c r="G69" s="61" t="n"/>
-      <c r="H69" s="61" t="n"/>
-      <c r="I69" s="61" t="n"/>
-      <c r="J69" s="61" t="n"/>
+      <c r="B69" s="32" t="n"/>
+      <c r="C69" s="32" t="n"/>
+      <c r="D69" s="40" t="n"/>
+      <c r="E69" s="62" t="n"/>
+      <c r="F69" s="62" t="n"/>
+      <c r="G69" s="62" t="n"/>
+      <c r="H69" s="62" t="n"/>
+      <c r="I69" s="62" t="n"/>
+      <c r="J69" s="62" t="n"/>
+      <c r="AN69" s="20" t="inlineStr">
+        <is>
+          <t>230PFC</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="14" customHeight="1">
-      <c r="B70" s="31" t="n"/>
-      <c r="C70" s="31" t="n"/>
-      <c r="D70" s="39" t="n"/>
-      <c r="E70" s="61" t="n"/>
-      <c r="F70" s="61" t="n"/>
-      <c r="G70" s="61" t="n"/>
-      <c r="H70" s="61" t="n"/>
-      <c r="I70" s="61" t="n"/>
-      <c r="J70" s="61" t="n"/>
+      <c r="B70" s="32" t="n"/>
+      <c r="C70" s="32" t="n"/>
+      <c r="D70" s="40" t="n"/>
+      <c r="E70" s="62" t="n"/>
+      <c r="F70" s="62" t="n"/>
+      <c r="G70" s="62" t="n"/>
+      <c r="H70" s="62" t="n"/>
+      <c r="I70" s="62" t="n"/>
+      <c r="J70" s="62" t="n"/>
+      <c r="AN70" s="20" t="inlineStr">
+        <is>
+          <t>200PFC</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="14" customHeight="1">
-      <c r="B71" s="31" t="n"/>
-      <c r="C71" s="31" t="n"/>
-      <c r="D71" s="39" t="n"/>
-      <c r="E71" s="61" t="n"/>
-      <c r="F71" s="61" t="n"/>
-      <c r="G71" s="61" t="n"/>
-      <c r="H71" s="61" t="n"/>
-      <c r="I71" s="61" t="n"/>
-      <c r="J71" s="61" t="n"/>
+      <c r="B71" s="32" t="n"/>
+      <c r="C71" s="32" t="n"/>
+      <c r="D71" s="40" t="n"/>
+      <c r="E71" s="62" t="n"/>
+      <c r="F71" s="62" t="n"/>
+      <c r="G71" s="62" t="n"/>
+      <c r="H71" s="62" t="n"/>
+      <c r="I71" s="62" t="n"/>
+      <c r="J71" s="62" t="n"/>
+      <c r="AN71" s="20" t="inlineStr">
+        <is>
+          <t>180PFC</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="14" customHeight="1">
-      <c r="B72" s="31" t="n"/>
-      <c r="C72" s="31" t="n"/>
-      <c r="D72" s="39" t="n"/>
-      <c r="E72" s="61" t="n"/>
-      <c r="F72" s="61" t="n"/>
-      <c r="G72" s="61" t="n"/>
-      <c r="H72" s="61" t="n"/>
-      <c r="I72" s="61" t="n"/>
-      <c r="J72" s="61" t="n"/>
+      <c r="B72" s="32" t="n"/>
+      <c r="C72" s="32" t="n"/>
+      <c r="D72" s="40" t="n"/>
+      <c r="E72" s="62" t="n"/>
+      <c r="F72" s="62" t="n"/>
+      <c r="G72" s="62" t="n"/>
+      <c r="H72" s="62" t="n"/>
+      <c r="I72" s="62" t="n"/>
+      <c r="J72" s="62" t="n"/>
+      <c r="AN72" s="20" t="inlineStr">
+        <is>
+          <t>150PFC</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="14" customHeight="1">
-      <c r="B73" s="31" t="n"/>
-      <c r="C73" s="31" t="n"/>
-      <c r="D73" s="39" t="n"/>
-      <c r="E73" s="61" t="n"/>
-      <c r="F73" s="61" t="n"/>
-      <c r="G73" s="61" t="n"/>
-      <c r="H73" s="61" t="n"/>
-      <c r="I73" s="61" t="n"/>
-      <c r="J73" s="61" t="n"/>
+      <c r="B73" s="32" t="n"/>
+      <c r="C73" s="32" t="n"/>
+      <c r="D73" s="40" t="n"/>
+      <c r="E73" s="62" t="n"/>
+      <c r="F73" s="62" t="n"/>
+      <c r="G73" s="62" t="n"/>
+      <c r="H73" s="62" t="n"/>
+      <c r="I73" s="62" t="n"/>
+      <c r="J73" s="62" t="n"/>
+      <c r="AN73" s="20" t="inlineStr">
+        <is>
+          <t>125PFC</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="20" customHeight="1">
       <c r="B74" s="10" t="inlineStr">
@@ -3986,6 +4326,11 @@
       <c r="H74" s="11" t="n"/>
       <c r="I74" s="11" t="n"/>
       <c r="J74" s="11" t="n"/>
+      <c r="AN74" s="20" t="inlineStr">
+        <is>
+          <t>100PFC</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="14" customHeight="1">
       <c r="B75" s="15" t="inlineStr">
@@ -3993,56 +4338,66 @@
           <t>Restraint type at each cross-section for the critical flange: F, P, L or U (– = none). Supports must be F or P.</t>
         </is>
       </c>
+      <c r="AN75" s="20" t="inlineStr">
+        <is>
+          <t>75PFC</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="14" customHeight="1">
-      <c r="B76" s="28" t="inlineStr">
+      <c r="B76" s="29" t="inlineStr">
         <is>
           <t>x (mm)</t>
         </is>
       </c>
-      <c r="C76" s="28" t="inlineStr">
+      <c r="C76" s="29" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
       </c>
-      <c r="D76" s="28" t="inlineStr">
+      <c r="D76" s="29" t="inlineStr">
         <is>
           <t>Restraint provided by</t>
         </is>
       </c>
-      <c r="E76" s="28" t="inlineStr">
+      <c r="E76" s="29" t="inlineStr">
         <is>
           <t>Top flange</t>
         </is>
       </c>
-      <c r="F76" s="28" t="inlineStr">
+      <c r="F76" s="29" t="inlineStr">
         <is>
           <t>Bottom fl.</t>
         </is>
       </c>
-      <c r="G76" s="28" t="inlineStr">
+      <c r="G76" s="29" t="inlineStr">
         <is>
           <t>αm override</t>
         </is>
       </c>
-      <c r="H76" s="28" t="inlineStr">
+      <c r="H76" s="29" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="I76" s="28" t="inlineStr">
+      <c r="I76" s="29" t="inlineStr">
         <is>
           <t>Top</t>
         </is>
       </c>
-      <c r="J76" s="28" t="inlineStr">
+      <c r="J76" s="29" t="inlineStr">
         <is>
           <t>Bottom</t>
         </is>
       </c>
+      <c r="AN76" s="20" t="inlineStr">
+        <is>
+          <t>310UC158</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="14" customHeight="1">
-      <c r="B77" s="62">
+      <c r="B77" s="63">
         <f>0</f>
         <v/>
       </c>
@@ -4066,21 +4421,26 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G77" s="58" t="n"/>
-      <c r="H77" s="31" t="inlineStr">
+      <c r="G77" s="59" t="n"/>
+      <c r="H77" s="32" t="inlineStr">
         <is>
           <t>kl</t>
         </is>
       </c>
-      <c r="I77" s="58" t="n">
+      <c r="I77" s="59" t="n">
         <v>1.4</v>
       </c>
-      <c r="J77" s="58" t="n">
+      <c r="J77" s="59" t="n">
         <v>1</v>
       </c>
+      <c r="AN77" s="20" t="inlineStr">
+        <is>
+          <t>310UC137</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="14" customHeight="1">
-      <c r="B78" s="44" t="n">
+      <c r="B78" s="45" t="n">
         <v>2767</v>
       </c>
       <c r="C78" s="2" t="inlineStr"/>
@@ -4099,21 +4459,26 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G78" s="58" t="n"/>
-      <c r="H78" s="31" t="inlineStr">
+      <c r="G78" s="59" t="n"/>
+      <c r="H78" s="32" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="I78" s="58" t="n">
+      <c r="I78" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="J78" s="58" t="n">
+      <c r="J78" s="59" t="n">
         <v>1</v>
       </c>
+      <c r="AN78" s="20" t="inlineStr">
+        <is>
+          <t>310UC118</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="14" customHeight="1">
-      <c r="B79" s="44" t="n">
+      <c r="B79" s="45" t="n">
         <v>5533</v>
       </c>
       <c r="C79" s="2" t="inlineStr"/>
@@ -4132,15 +4497,20 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G79" s="58" t="n"/>
+      <c r="G79" s="59" t="n"/>
       <c r="H79" s="15" t="inlineStr">
         <is>
           <t>kt from restraint</t>
         </is>
       </c>
+      <c r="AN79" s="20" t="inlineStr">
+        <is>
+          <t>310UC97</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="14" customHeight="1">
-      <c r="B80" s="62">
+      <c r="B80" s="63">
         <f>Span</f>
         <v/>
       </c>
@@ -4164,20 +4534,30 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G80" s="58" t="n"/>
+      <c r="G80" s="59" t="n"/>
       <c r="H80" s="15" t="inlineStr">
         <is>
           <t>types (add-in)</t>
         </is>
       </c>
+      <c r="AN80" s="20" t="inlineStr">
+        <is>
+          <t>250UC89.5</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="14" customHeight="1">
-      <c r="B81" s="44" t="n"/>
+      <c r="B81" s="45" t="n"/>
       <c r="C81" s="2" t="n"/>
       <c r="D81" s="5" t="n"/>
       <c r="E81" s="2" t="n"/>
       <c r="F81" s="2" t="n"/>
-      <c r="G81" s="58" t="n"/>
+      <c r="G81" s="59" t="n"/>
+      <c r="AN81" s="20" t="inlineStr">
+        <is>
+          <t>250UC73</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="14" customHeight="1">
       <c r="B82" s="15" t="inlineStr">
@@ -4185,8 +4565,19 @@
           <t>αm override applies to the segment starting at that row (blank = Cl. 5.6.1.1(a)(iii)); flagged * in the output.</t>
         </is>
       </c>
-    </row>
-    <row r="83" ht="14" customHeight="1"/>
+      <c r="AN82" s="20" t="inlineStr">
+        <is>
+          <t>200UC59.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="14" customHeight="1">
+      <c r="AN83" s="20" t="inlineStr">
+        <is>
+          <t>200UC52</t>
+        </is>
+      </c>
+    </row>
     <row r="84" ht="20" customHeight="1">
       <c r="B84" s="10" t="inlineStr">
         <is>
@@ -4201,95 +4592,120 @@
       <c r="H84" s="11" t="n"/>
       <c r="I84" s="11" t="n"/>
       <c r="J84" s="11" t="n"/>
+      <c r="AN84" s="20" t="inlineStr">
+        <is>
+          <t>200UC46</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="14" customHeight="1">
-      <c r="B85" s="56" t="inlineStr">
+      <c r="B85" s="57" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C85" s="56" t="inlineStr">
+      <c r="C85" s="57" t="inlineStr">
         <is>
           <t>Δ max (mm)</t>
         </is>
       </c>
-      <c r="D85" s="56" t="inlineStr">
+      <c r="D85" s="57" t="inlineStr">
         <is>
           <t>at x (mm)</t>
         </is>
       </c>
-      <c r="E85" s="56" t="inlineStr">
+      <c r="E85" s="57" t="inlineStr">
         <is>
           <t>Limit (mm)</t>
         </is>
       </c>
-      <c r="F85" s="56" t="inlineStr">
+      <c r="F85" s="57" t="inlineStr">
         <is>
           <t>L / Δ</t>
         </is>
       </c>
-      <c r="G85" s="56" t="inlineStr">
+      <c r="G85" s="57" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
+      <c r="AN85" s="20" t="inlineStr">
+        <is>
+          <t>150UC37</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="14" customHeight="1">
-      <c r="B86" s="31" cm="1">
+      <c r="B86" s="32" cm="1">
         <f t="array" ref="B86">OAR.SLS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],$E$37:$F$41,PsiL,PsiS)</f>
         <v/>
       </c>
-      <c r="C86" s="61" t="n"/>
-      <c r="D86" s="63" t="n"/>
-      <c r="E86" s="61" t="n"/>
-      <c r="F86" s="64" t="n"/>
-      <c r="G86" s="65" t="n"/>
+      <c r="C86" s="62" t="n"/>
+      <c r="D86" s="64" t="n"/>
+      <c r="E86" s="62" t="n"/>
+      <c r="F86" s="65" t="n"/>
+      <c r="G86" s="66" t="n"/>
       <c r="H86" s="6" t="inlineStr">
         <is>
           <t>Δ1kN: 1 kN at midspan,</t>
         </is>
       </c>
+      <c r="AN86" s="20" t="inlineStr">
+        <is>
+          <t>150UC30</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="14" customHeight="1">
-      <c r="B87" s="31" t="n"/>
-      <c r="C87" s="61" t="n"/>
-      <c r="D87" s="63" t="n"/>
-      <c r="E87" s="61" t="n"/>
-      <c r="F87" s="64" t="n"/>
-      <c r="G87" s="65" t="n"/>
+      <c r="B87" s="32" t="n"/>
+      <c r="C87" s="62" t="n"/>
+      <c r="D87" s="64" t="n"/>
+      <c r="E87" s="62" t="n"/>
+      <c r="F87" s="65" t="n"/>
+      <c r="G87" s="66" t="n"/>
       <c r="H87" s="6" t="inlineStr">
         <is>
           <t>beam alone</t>
         </is>
       </c>
+      <c r="AN87" s="20" t="inlineStr">
+        <is>
+          <t>150UC23</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="14" customHeight="1">
-      <c r="B88" s="31" t="n"/>
-      <c r="C88" s="61" t="n"/>
-      <c r="D88" s="63" t="n"/>
-      <c r="E88" s="61" t="n"/>
-      <c r="F88" s="64" t="n"/>
-      <c r="G88" s="65" t="n"/>
+      <c r="B88" s="32" t="n"/>
+      <c r="C88" s="62" t="n"/>
+      <c r="D88" s="64" t="n"/>
+      <c r="E88" s="62" t="n"/>
+      <c r="F88" s="65" t="n"/>
+      <c r="G88" s="66" t="n"/>
+      <c r="AN88" s="20" t="inlineStr">
+        <is>
+          <t>100UC15</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="14" customHeight="1">
-      <c r="B89" s="31" t="n"/>
-      <c r="C89" s="61" t="n"/>
-      <c r="D89" s="63" t="n"/>
-      <c r="E89" s="61" t="n"/>
-      <c r="F89" s="64" t="n"/>
-      <c r="G89" s="65" t="n"/>
+      <c r="B89" s="32" t="n"/>
+      <c r="C89" s="62" t="n"/>
+      <c r="D89" s="64" t="n"/>
+      <c r="E89" s="62" t="n"/>
+      <c r="F89" s="65" t="n"/>
+      <c r="G89" s="66" t="n"/>
     </row>
     <row r="90" ht="14" customHeight="1">
-      <c r="B90" s="31" t="n"/>
-      <c r="C90" s="61" t="n"/>
-      <c r="D90" s="63" t="n"/>
-      <c r="E90" s="61" t="n"/>
-      <c r="F90" s="64" t="n"/>
-      <c r="G90" s="65" t="n"/>
+      <c r="B90" s="32" t="n"/>
+      <c r="C90" s="62" t="n"/>
+      <c r="D90" s="64" t="n"/>
+      <c r="E90" s="62" t="n"/>
+      <c r="F90" s="65" t="n"/>
+      <c r="G90" s="66" t="n"/>
     </row>
     <row r="91" ht="14" customHeight="1"/>
     <row r="92" ht="14" customHeight="1">
-      <c r="B92" s="66" t="inlineStr">
+      <c r="B92" s="67" t="inlineStr">
         <is>
           <t>Deflected shapes (mm, plotted downward;  x in m)</t>
         </is>
@@ -4323,12 +4739,12 @@
       <c r="J105" s="11" t="n"/>
     </row>
     <row r="106" ht="14" customHeight="1">
-      <c r="B106" s="66" t="inlineStr">
+      <c r="B106" s="67" t="inlineStr">
         <is>
           <t>Bending moment envelope (kN·m, sagging down;  x in m)</t>
         </is>
       </c>
-      <c r="F106" s="66" t="inlineStr">
+      <c r="F106" s="67" t="inlineStr">
         <is>
           <t>Shear force envelope (kN;  x in m)</t>
         </is>
@@ -4349,230 +4765,230 @@
     <row r="119" ht="14" customHeight="1"/>
     <row r="120" ht="14" customHeight="1"/>
     <row r="121" ht="16" customHeight="1">
-      <c r="B121" s="56" t="inlineStr">
+      <c r="B121" s="57" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="C121" s="56" t="inlineStr">
+      <c r="C121" s="57" t="inlineStr">
         <is>
           <t>Segment (m)</t>
         </is>
       </c>
-      <c r="D121" s="56" t="inlineStr">
+      <c r="D121" s="57" t="inlineStr">
         <is>
           <t>Ends</t>
         </is>
       </c>
-      <c r="E121" s="56" t="inlineStr">
+      <c r="E121" s="57" t="inlineStr">
         <is>
           <t>Le (m)</t>
         </is>
       </c>
-      <c r="F121" s="56" t="inlineStr">
+      <c r="F121" s="57" t="inlineStr">
         <is>
           <t>αm</t>
         </is>
       </c>
-      <c r="G121" s="56" t="inlineStr">
+      <c r="G121" s="57" t="inlineStr">
         <is>
           <t>αs</t>
         </is>
       </c>
-      <c r="H121" s="56" t="inlineStr">
+      <c r="H121" s="57" t="inlineStr">
         <is>
           <t>φMb (kN·m)</t>
         </is>
       </c>
-      <c r="I121" s="56" t="inlineStr">
+      <c r="I121" s="57" t="inlineStr">
         <is>
           <t>M* (kN·m)</t>
         </is>
       </c>
-      <c r="J121" s="56" t="inlineStr">
+      <c r="J121" s="57" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
     </row>
     <row r="122" ht="14" customHeight="1">
-      <c r="B122" s="31" cm="1">
-        <f t="array" ref="B122">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1,$I$77:$J$78)</f>
-        <v/>
-      </c>
-      <c r="C122" s="31" t="n"/>
-      <c r="D122" s="31" t="n"/>
-      <c r="E122" s="61" t="n"/>
-      <c r="F122" s="67" t="n"/>
-      <c r="G122" s="67" t="n"/>
-      <c r="H122" s="68" t="n"/>
-      <c r="I122" s="68" t="n"/>
-      <c r="J122" s="65" t="n"/>
+      <c r="B122" s="32" cm="1">
+        <f t="array" ref="B122">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
+        <v/>
+      </c>
+      <c r="C122" s="32" t="n"/>
+      <c r="D122" s="32" t="n"/>
+      <c r="E122" s="62" t="n"/>
+      <c r="F122" s="68" t="n"/>
+      <c r="G122" s="68" t="n"/>
+      <c r="H122" s="69" t="n"/>
+      <c r="I122" s="69" t="n"/>
+      <c r="J122" s="66" t="n"/>
     </row>
     <row r="123" ht="14" customHeight="1">
-      <c r="B123" s="31" t="n"/>
-      <c r="C123" s="31" t="n"/>
-      <c r="D123" s="31" t="n"/>
-      <c r="E123" s="61" t="n"/>
-      <c r="F123" s="67" t="n"/>
-      <c r="G123" s="67" t="n"/>
-      <c r="H123" s="68" t="n"/>
-      <c r="I123" s="68" t="n"/>
-      <c r="J123" s="65" t="n"/>
+      <c r="B123" s="32" t="n"/>
+      <c r="C123" s="32" t="n"/>
+      <c r="D123" s="32" t="n"/>
+      <c r="E123" s="62" t="n"/>
+      <c r="F123" s="68" t="n"/>
+      <c r="G123" s="68" t="n"/>
+      <c r="H123" s="69" t="n"/>
+      <c r="I123" s="69" t="n"/>
+      <c r="J123" s="66" t="n"/>
     </row>
     <row r="124" ht="14" customHeight="1">
-      <c r="B124" s="31" t="n"/>
-      <c r="C124" s="31" t="n"/>
-      <c r="D124" s="31" t="n"/>
-      <c r="E124" s="61" t="n"/>
-      <c r="F124" s="67" t="n"/>
-      <c r="G124" s="67" t="n"/>
-      <c r="H124" s="68" t="n"/>
-      <c r="I124" s="68" t="n"/>
-      <c r="J124" s="65" t="n"/>
+      <c r="B124" s="32" t="n"/>
+      <c r="C124" s="32" t="n"/>
+      <c r="D124" s="32" t="n"/>
+      <c r="E124" s="62" t="n"/>
+      <c r="F124" s="68" t="n"/>
+      <c r="G124" s="68" t="n"/>
+      <c r="H124" s="69" t="n"/>
+      <c r="I124" s="69" t="n"/>
+      <c r="J124" s="66" t="n"/>
     </row>
     <row r="125" ht="14" customHeight="1">
-      <c r="B125" s="31" t="n"/>
-      <c r="C125" s="31" t="n"/>
-      <c r="D125" s="31" t="n"/>
-      <c r="E125" s="61" t="n"/>
-      <c r="F125" s="67" t="n"/>
-      <c r="G125" s="67" t="n"/>
-      <c r="H125" s="68" t="n"/>
-      <c r="I125" s="68" t="n"/>
-      <c r="J125" s="65" t="n"/>
+      <c r="B125" s="32" t="n"/>
+      <c r="C125" s="32" t="n"/>
+      <c r="D125" s="32" t="n"/>
+      <c r="E125" s="62" t="n"/>
+      <c r="F125" s="68" t="n"/>
+      <c r="G125" s="68" t="n"/>
+      <c r="H125" s="69" t="n"/>
+      <c r="I125" s="69" t="n"/>
+      <c r="J125" s="66" t="n"/>
     </row>
     <row r="126" ht="14" customHeight="1">
-      <c r="B126" s="31" t="n"/>
-      <c r="C126" s="31" t="n"/>
-      <c r="D126" s="31" t="n"/>
-      <c r="E126" s="61" t="n"/>
-      <c r="F126" s="67" t="n"/>
-      <c r="G126" s="67" t="n"/>
-      <c r="H126" s="68" t="n"/>
-      <c r="I126" s="68" t="n"/>
-      <c r="J126" s="65" t="n"/>
+      <c r="B126" s="32" t="n"/>
+      <c r="C126" s="32" t="n"/>
+      <c r="D126" s="32" t="n"/>
+      <c r="E126" s="62" t="n"/>
+      <c r="F126" s="68" t="n"/>
+      <c r="G126" s="68" t="n"/>
+      <c r="H126" s="69" t="n"/>
+      <c r="I126" s="69" t="n"/>
+      <c r="J126" s="66" t="n"/>
     </row>
     <row r="127" ht="14" customHeight="1">
-      <c r="B127" s="31" t="n"/>
-      <c r="C127" s="31" t="n"/>
-      <c r="D127" s="31" t="n"/>
-      <c r="E127" s="61" t="n"/>
-      <c r="F127" s="67" t="n"/>
-      <c r="G127" s="67" t="n"/>
-      <c r="H127" s="68" t="n"/>
-      <c r="I127" s="68" t="n"/>
-      <c r="J127" s="65" t="n"/>
+      <c r="B127" s="32" t="n"/>
+      <c r="C127" s="32" t="n"/>
+      <c r="D127" s="32" t="n"/>
+      <c r="E127" s="62" t="n"/>
+      <c r="F127" s="68" t="n"/>
+      <c r="G127" s="68" t="n"/>
+      <c r="H127" s="69" t="n"/>
+      <c r="I127" s="69" t="n"/>
+      <c r="J127" s="66" t="n"/>
     </row>
     <row r="128" ht="14" customHeight="1">
-      <c r="B128" s="31" t="n"/>
-      <c r="C128" s="31" t="n"/>
-      <c r="D128" s="31" t="n"/>
-      <c r="E128" s="61" t="n"/>
-      <c r="F128" s="67" t="n"/>
-      <c r="G128" s="67" t="n"/>
-      <c r="H128" s="68" t="n"/>
-      <c r="I128" s="68" t="n"/>
-      <c r="J128" s="65" t="n"/>
+      <c r="B128" s="32" t="n"/>
+      <c r="C128" s="32" t="n"/>
+      <c r="D128" s="32" t="n"/>
+      <c r="E128" s="62" t="n"/>
+      <c r="F128" s="68" t="n"/>
+      <c r="G128" s="68" t="n"/>
+      <c r="H128" s="69" t="n"/>
+      <c r="I128" s="69" t="n"/>
+      <c r="J128" s="66" t="n"/>
     </row>
     <row r="129" ht="14" customHeight="1">
-      <c r="B129" s="31" t="n"/>
-      <c r="C129" s="31" t="n"/>
-      <c r="D129" s="31" t="n"/>
-      <c r="E129" s="61" t="n"/>
-      <c r="F129" s="67" t="n"/>
-      <c r="G129" s="67" t="n"/>
-      <c r="H129" s="68" t="n"/>
-      <c r="I129" s="68" t="n"/>
-      <c r="J129" s="65" t="n"/>
+      <c r="B129" s="32" t="n"/>
+      <c r="C129" s="32" t="n"/>
+      <c r="D129" s="32" t="n"/>
+      <c r="E129" s="62" t="n"/>
+      <c r="F129" s="68" t="n"/>
+      <c r="G129" s="68" t="n"/>
+      <c r="H129" s="69" t="n"/>
+      <c r="I129" s="69" t="n"/>
+      <c r="J129" s="66" t="n"/>
     </row>
     <row r="130" ht="14" customHeight="1">
-      <c r="B130" s="31" t="n"/>
-      <c r="C130" s="31" t="n"/>
-      <c r="D130" s="31" t="n"/>
-      <c r="E130" s="61" t="n"/>
-      <c r="F130" s="67" t="n"/>
-      <c r="G130" s="67" t="n"/>
-      <c r="H130" s="68" t="n"/>
-      <c r="I130" s="68" t="n"/>
-      <c r="J130" s="65" t="n"/>
+      <c r="B130" s="32" t="n"/>
+      <c r="C130" s="32" t="n"/>
+      <c r="D130" s="32" t="n"/>
+      <c r="E130" s="62" t="n"/>
+      <c r="F130" s="68" t="n"/>
+      <c r="G130" s="68" t="n"/>
+      <c r="H130" s="69" t="n"/>
+      <c r="I130" s="69" t="n"/>
+      <c r="J130" s="66" t="n"/>
     </row>
     <row r="131" ht="14" customHeight="1">
-      <c r="B131" s="31" t="n"/>
-      <c r="C131" s="31" t="n"/>
-      <c r="D131" s="31" t="n"/>
-      <c r="E131" s="61" t="n"/>
-      <c r="F131" s="67" t="n"/>
-      <c r="G131" s="67" t="n"/>
-      <c r="H131" s="68" t="n"/>
-      <c r="I131" s="68" t="n"/>
-      <c r="J131" s="65" t="n"/>
+      <c r="B131" s="32" t="n"/>
+      <c r="C131" s="32" t="n"/>
+      <c r="D131" s="32" t="n"/>
+      <c r="E131" s="62" t="n"/>
+      <c r="F131" s="68" t="n"/>
+      <c r="G131" s="68" t="n"/>
+      <c r="H131" s="69" t="n"/>
+      <c r="I131" s="69" t="n"/>
+      <c r="J131" s="66" t="n"/>
     </row>
     <row r="132" ht="14" customHeight="1">
-      <c r="B132" s="31" t="n"/>
-      <c r="C132" s="31" t="n"/>
-      <c r="D132" s="31" t="n"/>
-      <c r="E132" s="61" t="n"/>
-      <c r="F132" s="67" t="n"/>
-      <c r="G132" s="67" t="n"/>
-      <c r="H132" s="68" t="n"/>
-      <c r="I132" s="68" t="n"/>
-      <c r="J132" s="65" t="n"/>
+      <c r="B132" s="32" t="n"/>
+      <c r="C132" s="32" t="n"/>
+      <c r="D132" s="32" t="n"/>
+      <c r="E132" s="62" t="n"/>
+      <c r="F132" s="68" t="n"/>
+      <c r="G132" s="68" t="n"/>
+      <c r="H132" s="69" t="n"/>
+      <c r="I132" s="69" t="n"/>
+      <c r="J132" s="66" t="n"/>
     </row>
     <row r="133" ht="14" customHeight="1">
-      <c r="B133" s="31" t="n"/>
-      <c r="C133" s="31" t="n"/>
-      <c r="D133" s="31" t="n"/>
-      <c r="E133" s="61" t="n"/>
-      <c r="F133" s="67" t="n"/>
-      <c r="G133" s="67" t="n"/>
-      <c r="H133" s="68" t="n"/>
-      <c r="I133" s="68" t="n"/>
-      <c r="J133" s="65" t="n"/>
+      <c r="B133" s="32" t="n"/>
+      <c r="C133" s="32" t="n"/>
+      <c r="D133" s="32" t="n"/>
+      <c r="E133" s="62" t="n"/>
+      <c r="F133" s="68" t="n"/>
+      <c r="G133" s="68" t="n"/>
+      <c r="H133" s="69" t="n"/>
+      <c r="I133" s="69" t="n"/>
+      <c r="J133" s="66" t="n"/>
     </row>
     <row r="134" ht="14" customHeight="1">
-      <c r="B134" s="31" t="n"/>
-      <c r="C134" s="31" t="n"/>
-      <c r="D134" s="31" t="n"/>
-      <c r="E134" s="61" t="n"/>
-      <c r="F134" s="67" t="n"/>
-      <c r="G134" s="67" t="n"/>
-      <c r="H134" s="68" t="n"/>
-      <c r="I134" s="68" t="n"/>
-      <c r="J134" s="65" t="n"/>
+      <c r="B134" s="32" t="n"/>
+      <c r="C134" s="32" t="n"/>
+      <c r="D134" s="32" t="n"/>
+      <c r="E134" s="62" t="n"/>
+      <c r="F134" s="68" t="n"/>
+      <c r="G134" s="68" t="n"/>
+      <c r="H134" s="69" t="n"/>
+      <c r="I134" s="69" t="n"/>
+      <c r="J134" s="66" t="n"/>
     </row>
     <row r="135" ht="14" customHeight="1">
-      <c r="B135" s="31" t="n"/>
-      <c r="C135" s="31" t="n"/>
-      <c r="D135" s="31" t="n"/>
-      <c r="E135" s="61" t="n"/>
-      <c r="F135" s="67" t="n"/>
-      <c r="G135" s="67" t="n"/>
-      <c r="H135" s="68" t="n"/>
-      <c r="I135" s="68" t="n"/>
-      <c r="J135" s="65" t="n"/>
+      <c r="B135" s="32" t="n"/>
+      <c r="C135" s="32" t="n"/>
+      <c r="D135" s="32" t="n"/>
+      <c r="E135" s="62" t="n"/>
+      <c r="F135" s="68" t="n"/>
+      <c r="G135" s="68" t="n"/>
+      <c r="H135" s="69" t="n"/>
+      <c r="I135" s="69" t="n"/>
+      <c r="J135" s="66" t="n"/>
     </row>
     <row r="136" ht="14" customHeight="1">
-      <c r="B136" s="31" t="n"/>
-      <c r="C136" s="31" t="n"/>
-      <c r="D136" s="31" t="n"/>
-      <c r="E136" s="61" t="n"/>
-      <c r="F136" s="67" t="n"/>
-      <c r="G136" s="67" t="n"/>
-      <c r="H136" s="68" t="n"/>
-      <c r="I136" s="68" t="n"/>
-      <c r="J136" s="65" t="n"/>
+      <c r="B136" s="32" t="n"/>
+      <c r="C136" s="32" t="n"/>
+      <c r="D136" s="32" t="n"/>
+      <c r="E136" s="62" t="n"/>
+      <c r="F136" s="68" t="n"/>
+      <c r="G136" s="68" t="n"/>
+      <c r="H136" s="69" t="n"/>
+      <c r="I136" s="69" t="n"/>
+      <c r="J136" s="66" t="n"/>
     </row>
     <row r="137" ht="14" customHeight="1">
-      <c r="B137" s="31" t="n"/>
-      <c r="C137" s="31" t="n"/>
-      <c r="D137" s="31" t="n"/>
-      <c r="E137" s="61" t="n"/>
-      <c r="F137" s="67" t="n"/>
-      <c r="G137" s="67" t="n"/>
-      <c r="H137" s="68" t="n"/>
-      <c r="I137" s="68" t="n"/>
-      <c r="J137" s="65" t="n"/>
+      <c r="B137" s="32" t="n"/>
+      <c r="C137" s="32" t="n"/>
+      <c r="D137" s="32" t="n"/>
+      <c r="E137" s="62" t="n"/>
+      <c r="F137" s="68" t="n"/>
+      <c r="G137" s="68" t="n"/>
+      <c r="H137" s="69" t="n"/>
+      <c r="I137" s="69" t="n"/>
+      <c r="J137" s="66" t="n"/>
     </row>
     <row r="138" ht="14" customHeight="1">
       <c r="B138" s="15" t="inlineStr">
@@ -4605,117 +5021,117 @@
       </c>
     </row>
     <row r="142">
-      <c r="D142" s="69" cm="1">
-        <f t="array" ref="D142">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1,$I$77:$J$78)</f>
-        <v/>
-      </c>
-      <c r="E142" s="70" t="n"/>
-      <c r="F142" s="32" t="n"/>
+      <c r="D142" s="70" cm="1">
+        <f t="array" ref="D142">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
+        <v/>
+      </c>
+      <c r="E142" s="71" t="n"/>
+      <c r="F142" s="33" t="n"/>
     </row>
     <row r="143">
-      <c r="D143" s="69" t="n"/>
-      <c r="E143" s="70" t="n"/>
-      <c r="F143" s="32" t="n"/>
+      <c r="D143" s="70" t="n"/>
+      <c r="E143" s="71" t="n"/>
+      <c r="F143" s="33" t="n"/>
     </row>
     <row r="144">
-      <c r="D144" s="69" t="n"/>
-      <c r="E144" s="70" t="n"/>
-      <c r="F144" s="32" t="n"/>
+      <c r="D144" s="70" t="n"/>
+      <c r="E144" s="71" t="n"/>
+      <c r="F144" s="33" t="n"/>
     </row>
     <row r="145">
-      <c r="D145" s="69" t="n"/>
-      <c r="E145" s="70" t="n"/>
-      <c r="F145" s="32" t="n"/>
+      <c r="D145" s="70" t="n"/>
+      <c r="E145" s="71" t="n"/>
+      <c r="F145" s="33" t="n"/>
     </row>
     <row r="146">
-      <c r="D146" s="69" t="n"/>
-      <c r="E146" s="70" t="n"/>
-      <c r="F146" s="32" t="n"/>
+      <c r="D146" s="70" t="n"/>
+      <c r="E146" s="71" t="n"/>
+      <c r="F146" s="33" t="n"/>
     </row>
     <row r="147">
-      <c r="D147" s="69" t="n"/>
-      <c r="E147" s="70" t="n"/>
-      <c r="F147" s="32" t="n"/>
+      <c r="D147" s="70" t="n"/>
+      <c r="E147" s="71" t="n"/>
+      <c r="F147" s="33" t="n"/>
     </row>
     <row r="148">
-      <c r="D148" s="69" t="n"/>
-      <c r="E148" s="70" t="n"/>
-      <c r="F148" s="32" t="n"/>
+      <c r="D148" s="70" t="n"/>
+      <c r="E148" s="71" t="n"/>
+      <c r="F148" s="33" t="n"/>
     </row>
     <row r="149">
-      <c r="D149" s="69" t="n"/>
-      <c r="E149" s="70" t="n"/>
-      <c r="F149" s="32" t="n"/>
+      <c r="D149" s="70" t="n"/>
+      <c r="E149" s="71" t="n"/>
+      <c r="F149" s="33" t="n"/>
     </row>
     <row r="150">
-      <c r="D150" s="69" t="n"/>
-      <c r="E150" s="70" t="n"/>
-      <c r="F150" s="32" t="n"/>
+      <c r="D150" s="70" t="n"/>
+      <c r="E150" s="71" t="n"/>
+      <c r="F150" s="33" t="n"/>
     </row>
     <row r="151">
-      <c r="D151" s="69" t="n"/>
-      <c r="E151" s="70" t="n"/>
-      <c r="F151" s="32" t="n"/>
+      <c r="D151" s="70" t="n"/>
+      <c r="E151" s="71" t="n"/>
+      <c r="F151" s="33" t="n"/>
     </row>
     <row r="152">
-      <c r="D152" s="69" t="n"/>
-      <c r="E152" s="70" t="n"/>
-      <c r="F152" s="32" t="n"/>
+      <c r="D152" s="70" t="n"/>
+      <c r="E152" s="71" t="n"/>
+      <c r="F152" s="33" t="n"/>
     </row>
     <row r="153">
-      <c r="D153" s="69" t="n"/>
-      <c r="E153" s="70" t="n"/>
-      <c r="F153" s="32" t="n"/>
+      <c r="D153" s="70" t="n"/>
+      <c r="E153" s="71" t="n"/>
+      <c r="F153" s="33" t="n"/>
     </row>
     <row r="154">
-      <c r="D154" s="69" t="n"/>
-      <c r="E154" s="70" t="n"/>
-      <c r="F154" s="32" t="n"/>
+      <c r="D154" s="70" t="n"/>
+      <c r="E154" s="71" t="n"/>
+      <c r="F154" s="33" t="n"/>
     </row>
     <row r="155">
-      <c r="D155" s="69" t="n"/>
-      <c r="E155" s="70" t="n"/>
-      <c r="F155" s="32" t="n"/>
+      <c r="D155" s="70" t="n"/>
+      <c r="E155" s="71" t="n"/>
+      <c r="F155" s="33" t="n"/>
     </row>
     <row r="156">
-      <c r="D156" s="69" t="n"/>
-      <c r="E156" s="70" t="n"/>
-      <c r="F156" s="32" t="n"/>
+      <c r="D156" s="70" t="n"/>
+      <c r="E156" s="71" t="n"/>
+      <c r="F156" s="33" t="n"/>
     </row>
     <row r="157">
-      <c r="D157" s="69" t="n"/>
-      <c r="E157" s="70" t="n"/>
-      <c r="F157" s="32" t="n"/>
+      <c r="D157" s="70" t="n"/>
+      <c r="E157" s="71" t="n"/>
+      <c r="F157" s="33" t="n"/>
     </row>
     <row r="158">
-      <c r="D158" s="69" t="n"/>
-      <c r="E158" s="70" t="n"/>
-      <c r="F158" s="32" t="n"/>
+      <c r="D158" s="70" t="n"/>
+      <c r="E158" s="71" t="n"/>
+      <c r="F158" s="33" t="n"/>
     </row>
     <row r="159">
-      <c r="D159" s="69" t="n"/>
-      <c r="E159" s="70" t="n"/>
-      <c r="F159" s="32" t="n"/>
+      <c r="D159" s="70" t="n"/>
+      <c r="E159" s="71" t="n"/>
+      <c r="F159" s="33" t="n"/>
     </row>
     <row r="160">
-      <c r="D160" s="69" t="n"/>
-      <c r="E160" s="70" t="n"/>
-      <c r="F160" s="32" t="n"/>
+      <c r="D160" s="70" t="n"/>
+      <c r="E160" s="71" t="n"/>
+      <c r="F160" s="33" t="n"/>
     </row>
     <row r="161">
-      <c r="D161" s="69" t="n"/>
-      <c r="E161" s="70" t="n"/>
-      <c r="F161" s="32" t="n"/>
+      <c r="D161" s="70" t="n"/>
+      <c r="E161" s="71" t="n"/>
+      <c r="F161" s="33" t="n"/>
     </row>
     <row r="162">
-      <c r="D162" s="69" t="n"/>
-      <c r="E162" s="70" t="n"/>
-      <c r="F162" s="32" t="n"/>
+      <c r="D162" s="70" t="n"/>
+      <c r="E162" s="71" t="n"/>
+      <c r="F162" s="33" t="n"/>
     </row>
     <row r="163">
-      <c r="D163" s="69" t="n"/>
-      <c r="E163" s="70" t="n"/>
-      <c r="F163" s="32" t="n"/>
+      <c r="D163" s="70" t="n"/>
+      <c r="E163" s="71" t="n"/>
+      <c r="F163" s="33" t="n"/>
     </row>
     <row r="165" ht="20" customHeight="1">
       <c r="B165" s="10" t="inlineStr">
@@ -4733,103 +5149,103 @@
       <c r="J165" s="11" t="n"/>
     </row>
     <row r="166">
-      <c r="B166" s="56" t="inlineStr">
+      <c r="B166" s="57" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="C166" s="56" t="inlineStr">
+      <c r="C166" s="57" t="inlineStr">
         <is>
           <t>V* (kN)</t>
         </is>
       </c>
-      <c r="D166" s="56" t="inlineStr">
+      <c r="D166" s="57" t="inlineStr">
         <is>
           <t>at x (m)</t>
         </is>
       </c>
-      <c r="E166" s="56" t="inlineStr">
+      <c r="E166" s="57" t="inlineStr">
         <is>
           <t>φVv (kN)</t>
         </is>
       </c>
-      <c r="F166" s="56" t="inlineStr">
+      <c r="F166" s="57" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
-      <c r="G166" s="56" t="inlineStr">
+      <c r="G166" s="57" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="B167" s="31" cm="1">
+      <c r="B167" s="32" cm="1">
         <f t="array" ref="B167">OAR.SHEAR(SectionSize,Grade,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
         <v/>
       </c>
-      <c r="C167" s="68" t="n"/>
-      <c r="D167" s="61" t="n"/>
-      <c r="E167" s="68" t="n"/>
-      <c r="F167" s="65" t="n"/>
-      <c r="G167" s="71" t="n"/>
+      <c r="C167" s="69" t="n"/>
+      <c r="D167" s="62" t="n"/>
+      <c r="E167" s="69" t="n"/>
+      <c r="F167" s="66" t="n"/>
+      <c r="G167" s="72" t="n"/>
     </row>
     <row r="168">
-      <c r="B168" s="31" t="n"/>
-      <c r="C168" s="68" t="n"/>
-      <c r="D168" s="61" t="n"/>
-      <c r="E168" s="68" t="n"/>
-      <c r="F168" s="65" t="n"/>
-      <c r="G168" s="71" t="n"/>
+      <c r="B168" s="32" t="n"/>
+      <c r="C168" s="69" t="n"/>
+      <c r="D168" s="62" t="n"/>
+      <c r="E168" s="69" t="n"/>
+      <c r="F168" s="66" t="n"/>
+      <c r="G168" s="72" t="n"/>
     </row>
     <row r="169">
-      <c r="B169" s="31" t="n"/>
-      <c r="C169" s="68" t="n"/>
-      <c r="D169" s="61" t="n"/>
-      <c r="E169" s="68" t="n"/>
-      <c r="F169" s="65" t="n"/>
-      <c r="G169" s="71" t="n"/>
+      <c r="B169" s="32" t="n"/>
+      <c r="C169" s="69" t="n"/>
+      <c r="D169" s="62" t="n"/>
+      <c r="E169" s="69" t="n"/>
+      <c r="F169" s="66" t="n"/>
+      <c r="G169" s="72" t="n"/>
     </row>
     <row r="170">
-      <c r="B170" s="31" t="n"/>
-      <c r="C170" s="68" t="n"/>
-      <c r="D170" s="61" t="n"/>
-      <c r="E170" s="68" t="n"/>
-      <c r="F170" s="65" t="n"/>
-      <c r="G170" s="71" t="n"/>
+      <c r="B170" s="32" t="n"/>
+      <c r="C170" s="69" t="n"/>
+      <c r="D170" s="62" t="n"/>
+      <c r="E170" s="69" t="n"/>
+      <c r="F170" s="66" t="n"/>
+      <c r="G170" s="72" t="n"/>
     </row>
     <row r="171">
-      <c r="B171" s="31" t="n"/>
-      <c r="C171" s="68" t="n"/>
-      <c r="D171" s="61" t="n"/>
-      <c r="E171" s="68" t="n"/>
-      <c r="F171" s="65" t="n"/>
-      <c r="G171" s="71" t="n"/>
+      <c r="B171" s="32" t="n"/>
+      <c r="C171" s="69" t="n"/>
+      <c r="D171" s="62" t="n"/>
+      <c r="E171" s="69" t="n"/>
+      <c r="F171" s="66" t="n"/>
+      <c r="G171" s="72" t="n"/>
     </row>
     <row r="172">
-      <c r="B172" s="31" t="n"/>
-      <c r="C172" s="68" t="n"/>
-      <c r="D172" s="61" t="n"/>
-      <c r="E172" s="68" t="n"/>
-      <c r="F172" s="65" t="n"/>
-      <c r="G172" s="71" t="n"/>
+      <c r="B172" s="32" t="n"/>
+      <c r="C172" s="69" t="n"/>
+      <c r="D172" s="62" t="n"/>
+      <c r="E172" s="69" t="n"/>
+      <c r="F172" s="66" t="n"/>
+      <c r="G172" s="72" t="n"/>
     </row>
     <row r="173">
-      <c r="B173" s="31" t="n"/>
-      <c r="C173" s="68" t="n"/>
-      <c r="D173" s="61" t="n"/>
-      <c r="E173" s="68" t="n"/>
-      <c r="F173" s="65" t="n"/>
-      <c r="G173" s="71" t="n"/>
+      <c r="B173" s="32" t="n"/>
+      <c r="C173" s="69" t="n"/>
+      <c r="D173" s="62" t="n"/>
+      <c r="E173" s="69" t="n"/>
+      <c r="F173" s="66" t="n"/>
+      <c r="G173" s="72" t="n"/>
     </row>
     <row r="174">
-      <c r="B174" s="31" t="n"/>
-      <c r="C174" s="68" t="n"/>
-      <c r="D174" s="61" t="n"/>
-      <c r="E174" s="68" t="n"/>
-      <c r="F174" s="65" t="n"/>
-      <c r="G174" s="71" t="n"/>
+      <c r="B174" s="32" t="n"/>
+      <c r="C174" s="69" t="n"/>
+      <c r="D174" s="62" t="n"/>
+      <c r="E174" s="69" t="n"/>
+      <c r="F174" s="66" t="n"/>
+      <c r="G174" s="72" t="n"/>
     </row>
     <row r="176" ht="20" customHeight="1">
       <c r="B176" s="10" t="inlineStr">
@@ -4854,148 +5270,148 @@
       </c>
     </row>
     <row r="178">
-      <c r="B178" s="28" t="inlineStr">
+      <c r="B178" s="29" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="D178" s="28" t="inlineStr">
+      <c r="D178" s="29" t="inlineStr">
         <is>
           <t>Left (kN)</t>
         </is>
       </c>
-      <c r="E178" s="28" t="inlineStr">
+      <c r="E178" s="29" t="inlineStr">
         <is>
           <t>Right (kN)</t>
         </is>
       </c>
-      <c r="F178" s="28" t="inlineStr">
+      <c r="F178" s="29" t="inlineStr">
         <is>
           <t>Transfer names</t>
         </is>
       </c>
     </row>
     <row r="179">
-      <c r="B179" s="48" t="inlineStr">
+      <c r="B179" s="49" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="C179" s="49" t="n"/>
-      <c r="D179" s="33" cm="1">
+      <c r="C179" s="50" t="n"/>
+      <c r="D179" s="34" cm="1">
         <f t="array" ref="D179">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,2)</f>
         <v/>
       </c>
-      <c r="E179" s="33" cm="1">
+      <c r="E179" s="34" cm="1">
         <f t="array" ref="E179">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,3)</f>
         <v/>
       </c>
-      <c r="F179" s="20" t="inlineStr">
+      <c r="F179" s="21" t="inlineStr">
         <is>
           <t>RxnL_G  ·  RxnR_G</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="B180" s="48" t="inlineStr">
+      <c r="B180" s="49" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C180" s="49" t="n"/>
-      <c r="D180" s="33" cm="1">
+      <c r="C180" s="50" t="n"/>
+      <c r="D180" s="34" cm="1">
         <f t="array" ref="D180">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,2)</f>
         <v/>
       </c>
-      <c r="E180" s="33" cm="1">
+      <c r="E180" s="34" cm="1">
         <f t="array" ref="E180">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,3)</f>
         <v/>
       </c>
-      <c r="F180" s="20" t="inlineStr">
+      <c r="F180" s="21" t="inlineStr">
         <is>
           <t>RxnL_Q  ·  RxnR_Q</t>
         </is>
       </c>
     </row>
     <row r="181">
-      <c r="B181" s="48" t="inlineStr">
+      <c r="B181" s="49" t="inlineStr">
         <is>
           <t>Wd</t>
         </is>
       </c>
-      <c r="C181" s="49" t="n"/>
-      <c r="D181" s="33" cm="1">
+      <c r="C181" s="50" t="n"/>
+      <c r="D181" s="34" cm="1">
         <f t="array" ref="D181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,2)</f>
         <v/>
       </c>
-      <c r="E181" s="33" cm="1">
+      <c r="E181" s="34" cm="1">
         <f t="array" ref="E181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,3)</f>
         <v/>
       </c>
-      <c r="F181" s="20" t="inlineStr">
+      <c r="F181" s="21" t="inlineStr">
         <is>
           <t>RxnL_Wd  ·  RxnR_Wd</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="B182" s="48" t="inlineStr">
+      <c r="B182" s="49" t="inlineStr">
         <is>
           <t>Wu</t>
         </is>
       </c>
-      <c r="C182" s="49" t="n"/>
-      <c r="D182" s="33" cm="1">
+      <c r="C182" s="50" t="n"/>
+      <c r="D182" s="34" cm="1">
         <f t="array" ref="D182">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,2)</f>
         <v/>
       </c>
-      <c r="E182" s="33" cm="1">
+      <c r="E182" s="34" cm="1">
         <f t="array" ref="E182">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,3)</f>
         <v/>
       </c>
-      <c r="F182" s="20" t="inlineStr">
+      <c r="F182" s="21" t="inlineStr">
         <is>
           <t>RxnL_Wu  ·  RxnR_Wu</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="B183" s="48" t="inlineStr">
+      <c r="B183" s="49" t="inlineStr">
         <is>
           <t>Wid</t>
         </is>
       </c>
-      <c r="C183" s="49" t="n"/>
-      <c r="D183" s="33" cm="1">
+      <c r="C183" s="50" t="n"/>
+      <c r="D183" s="34" cm="1">
         <f t="array" ref="D183">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,2)</f>
         <v/>
       </c>
-      <c r="E183" s="33" cm="1">
+      <c r="E183" s="34" cm="1">
         <f t="array" ref="E183">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,3)</f>
         <v/>
       </c>
-      <c r="F183" s="20" t="inlineStr">
+      <c r="F183" s="21" t="inlineStr">
         <is>
           <t>RxnL_Wid  ·  RxnR_Wid</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="B184" s="48" t="inlineStr">
+      <c r="B184" s="49" t="inlineStr">
         <is>
           <t>Wiu</t>
         </is>
       </c>
-      <c r="C184" s="49" t="n"/>
-      <c r="D184" s="33" cm="1">
+      <c r="C184" s="50" t="n"/>
+      <c r="D184" s="34" cm="1">
         <f t="array" ref="D184">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,2)</f>
         <v/>
       </c>
-      <c r="E184" s="33" cm="1">
+      <c r="E184" s="34" cm="1">
         <f t="array" ref="E184">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,3)</f>
         <v/>
       </c>
-      <c r="F184" s="20" t="inlineStr">
+      <c r="F184" s="21" t="inlineStr">
         <is>
           <t>RxnL_Wiu  ·  RxnR_Wiu</t>
         </is>
@@ -5009,94 +5425,94 @@
       </c>
     </row>
     <row r="187">
-      <c r="B187" s="56" t="inlineStr">
+      <c r="B187" s="57" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C187" s="56" t="inlineStr">
+      <c r="C187" s="57" t="inlineStr">
         <is>
           <t>Left (kN)</t>
         </is>
       </c>
-      <c r="D187" s="56" t="inlineStr">
+      <c r="D187" s="57" t="inlineStr">
         <is>
           <t>Right (kN)</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="B188" s="31" cm="1">
+      <c r="B188" s="32" cm="1">
         <f t="array" ref="B188">OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
         <v/>
       </c>
-      <c r="C188" s="61" t="n"/>
-      <c r="D188" s="61" t="n"/>
+      <c r="C188" s="62" t="n"/>
+      <c r="D188" s="62" t="n"/>
     </row>
     <row r="189">
-      <c r="B189" s="31" t="n"/>
-      <c r="C189" s="61" t="n"/>
-      <c r="D189" s="61" t="n"/>
+      <c r="B189" s="32" t="n"/>
+      <c r="C189" s="62" t="n"/>
+      <c r="D189" s="62" t="n"/>
     </row>
     <row r="190">
-      <c r="B190" s="31" t="n"/>
-      <c r="C190" s="61" t="n"/>
-      <c r="D190" s="61" t="n"/>
+      <c r="B190" s="32" t="n"/>
+      <c r="C190" s="62" t="n"/>
+      <c r="D190" s="62" t="n"/>
     </row>
     <row r="191">
-      <c r="B191" s="31" t="n"/>
-      <c r="C191" s="61" t="n"/>
-      <c r="D191" s="61" t="n"/>
+      <c r="B191" s="32" t="n"/>
+      <c r="C191" s="62" t="n"/>
+      <c r="D191" s="62" t="n"/>
     </row>
     <row r="192">
-      <c r="B192" s="31" t="n"/>
-      <c r="C192" s="61" t="n"/>
-      <c r="D192" s="61" t="n"/>
+      <c r="B192" s="32" t="n"/>
+      <c r="C192" s="62" t="n"/>
+      <c r="D192" s="62" t="n"/>
     </row>
     <row r="193">
-      <c r="B193" s="31" t="n"/>
-      <c r="C193" s="61" t="n"/>
-      <c r="D193" s="61" t="n"/>
+      <c r="B193" s="32" t="n"/>
+      <c r="C193" s="62" t="n"/>
+      <c r="D193" s="62" t="n"/>
     </row>
     <row r="194">
-      <c r="B194" s="31" t="n"/>
-      <c r="C194" s="61" t="n"/>
-      <c r="D194" s="61" t="n"/>
+      <c r="B194" s="32" t="n"/>
+      <c r="C194" s="62" t="n"/>
+      <c r="D194" s="62" t="n"/>
     </row>
     <row r="195">
-      <c r="B195" s="31" t="n"/>
-      <c r="C195" s="61" t="n"/>
-      <c r="D195" s="61" t="n"/>
+      <c r="B195" s="32" t="n"/>
+      <c r="C195" s="62" t="n"/>
+      <c r="D195" s="62" t="n"/>
     </row>
     <row r="196">
-      <c r="B196" s="31" t="n"/>
-      <c r="C196" s="61" t="n"/>
-      <c r="D196" s="61" t="n"/>
+      <c r="B196" s="32" t="n"/>
+      <c r="C196" s="62" t="n"/>
+      <c r="D196" s="62" t="n"/>
     </row>
     <row r="197">
-      <c r="B197" s="31" t="n"/>
-      <c r="C197" s="61" t="n"/>
-      <c r="D197" s="61" t="n"/>
+      <c r="B197" s="32" t="n"/>
+      <c r="C197" s="62" t="n"/>
+      <c r="D197" s="62" t="n"/>
     </row>
     <row r="198">
-      <c r="B198" s="31" t="n"/>
-      <c r="C198" s="61" t="n"/>
-      <c r="D198" s="61" t="n"/>
+      <c r="B198" s="32" t="n"/>
+      <c r="C198" s="62" t="n"/>
+      <c r="D198" s="62" t="n"/>
     </row>
     <row r="199">
-      <c r="B199" s="31" t="n"/>
-      <c r="C199" s="61" t="n"/>
-      <c r="D199" s="61" t="n"/>
+      <c r="B199" s="32" t="n"/>
+      <c r="C199" s="62" t="n"/>
+      <c r="D199" s="62" t="n"/>
     </row>
     <row r="200">
-      <c r="B200" s="31" t="n"/>
-      <c r="C200" s="61" t="n"/>
-      <c r="D200" s="61" t="n"/>
+      <c r="B200" s="32" t="n"/>
+      <c r="C200" s="62" t="n"/>
+      <c r="D200" s="62" t="n"/>
     </row>
     <row r="201">
-      <c r="B201" s="31" t="n"/>
-      <c r="C201" s="61" t="n"/>
-      <c r="D201" s="61" t="n"/>
+      <c r="B201" s="32" t="n"/>
+      <c r="C201" s="62" t="n"/>
+      <c r="D201" s="62" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="40">
@@ -5269,7 +5685,7 @@
       <formula1>"F,P,L,U,–"</formula1>
     </dataValidation>
     <dataValidation sqref="E27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Section size" error="Pick a section from the list for the selected Section type." type="list">
-      <formula1>OFFSET($AL$8,0,0,MAX(1,COUNTA($AL$8:$AL$300)),1)</formula1>
+      <formula1>IF(ISERROR($AL$8),$AN$8:$AN$88,OFFSET($AL$8,0,0,MAX(1,COUNTA($AL$8:$AL$300)),1))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.6" header="0.2" footer="0.25"/>

</xml_diff>

<commit_message>
Sheet: load library with case-filtered description dropdown and pressure lookup
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -407,7 +407,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -459,6 +459,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -469,8 +472,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -545,9 +551,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1360,7 +1363,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CombLib_B1" displayName="CombLib_B1" ref="M46:X54" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="LoadLib_B1" displayName="LoadLib_B1" ref="AP9:AS31" headerRowCount="1">
+  <autoFilter ref="AP9:AS31"/>
+  <tableColumns count="4">
+    <tableColumn id="42" name="Case"/>
+    <tableColumn id="43" name="Description"/>
+    <tableColumn id="44" name="kPa"/>
+    <tableColumn id="45" name="Source / note"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight15" showRowStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CombLib_B1" displayName="CombLib_B1" ref="M46:X54" headerRowCount="1">
   <autoFilter ref="M46:X54"/>
   <tableColumns count="12">
     <tableColumn id="13" name="Include"/>
@@ -1380,8 +1396,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Restraints_B1" displayName="Restraints_B1" ref="B76:G81" headerRowCount="1">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Restraints_B1" displayName="Restraints_B1" ref="B76:G81" headerRowCount="1">
   <autoFilter ref="B76:G81"/>
   <tableColumns count="6">
     <tableColumn id="2" name="x (mm)"/>
@@ -1685,7 +1701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AN201"/>
+  <dimension ref="B1:AS201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.5" customWidth="1" min="1" max="1"/>
@@ -1725,6 +1741,10 @@
     <col width="9" customWidth="1" min="36" max="36"/>
     <col width="12" customWidth="1" min="38" max="38"/>
     <col width="12" customWidth="1" min="40" max="40"/>
+    <col width="7" customWidth="1" min="42" max="42"/>
+    <col width="38" customWidth="1" min="43" max="43"/>
+    <col width="8" customWidth="1" min="44" max="44"/>
+    <col width="46" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1" ht="17" customHeight="1">
@@ -1851,6 +1871,11 @@
           <t>Add-in data for summary and charts  (not printed)</t>
         </is>
       </c>
+      <c r="AP6" s="12" t="inlineStr">
+        <is>
+          <t>Load Library  (not printed)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="14" customHeight="1">
       <c r="G7" s="1" t="inlineStr">
@@ -1881,6 +1906,11 @@
       <c r="AN7" s="15" t="inlineStr">
         <is>
           <t>All sections (fallback)</t>
+        </is>
+      </c>
+      <c r="AP7" s="15" t="inlineStr">
+        <is>
+          <t>Typical starting values only – verify for each job. Picking a Description in the loads table fills Press. (kPa); type over it to change. Keep rows grouped by case (insert new rows inside the case's block).</t>
         </is>
       </c>
     </row>
@@ -1954,21 +1984,41 @@
           <t>1200WB423</t>
         </is>
       </c>
+      <c r="AP9" s="25" t="inlineStr">
+        <is>
+          <t>Case</t>
+        </is>
+      </c>
+      <c r="AQ9" s="25" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="AR9" s="25" t="inlineStr">
+        <is>
+          <t>kPa</t>
+        </is>
+      </c>
+      <c r="AS9" s="25" t="inlineStr">
+        <is>
+          <t>Source / note</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="25">
+      <c r="B10" s="26">
         <f>IF(SectionSize="","–",SectionSize&amp;"  Gr "&amp;Grade)</f>
         <v/>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="27">
         <f>IF(COUNT(I14:I23)=0,"–",MAX(I14:I23))</f>
         <v/>
       </c>
-      <c r="I10" s="27">
+      <c r="I10" s="28">
         <f>IF(COUNT(I14:I23)=0,"PENDING",IF(MAX(I14:I23)&lt;=1,"PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="J10" s="28" t="n"/>
+      <c r="J10" s="29" t="n"/>
       <c r="M10" s="22" t="n"/>
       <c r="N10" s="23" t="n"/>
       <c r="O10" s="23" t="n"/>
@@ -1982,6 +2032,24 @@
           <t>1200WB392</t>
         </is>
       </c>
+      <c r="AP10" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AQ10" s="5" t="inlineStr">
+        <is>
+          <t>Roof sheeting + purlins</t>
+        </is>
+      </c>
+      <c r="AR10" s="30" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AS10" s="31" t="inlineStr">
+        <is>
+          <t>allowance – check sheeting and purlin weights</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="14" customHeight="1">
       <c r="B11" s="6">
@@ -2003,6 +2071,24 @@
       <c r="AN11" s="20" t="inlineStr">
         <is>
           <t>1200WB342</t>
+        </is>
+      </c>
+      <c r="AP11" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AQ11" s="5" t="inlineStr">
+        <is>
+          <t>Light sheet roof (20 kg/m²)</t>
+        </is>
+      </c>
+      <c r="AR11" s="30" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="AS11" s="31" t="inlineStr">
+        <is>
+          <t>20 kg/m² x 9.81</t>
         </is>
       </c>
     </row>
@@ -2030,44 +2116,62 @@
           <t>1200WB317</t>
         </is>
       </c>
+      <c r="AP12" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AQ12" s="5" t="inlineStr">
+        <is>
+          <t>Sheet roof (40 kg/m²)</t>
+        </is>
+      </c>
+      <c r="AR12" s="30" t="n">
+        <v>0.392</v>
+      </c>
+      <c r="AS12" s="31" t="inlineStr">
+        <is>
+          <t>40 kg/m² x 9.81</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="D13" s="29" t="inlineStr">
+      <c r="D13" s="25" t="inlineStr">
         <is>
           <t>Basis</t>
         </is>
       </c>
-      <c r="E13" s="29" t="inlineStr">
+      <c r="E13" s="25" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="F13" s="29" t="inlineStr">
+      <c r="F13" s="25" t="inlineStr">
         <is>
           <t>Limit</t>
         </is>
       </c>
-      <c r="G13" s="29" t="inlineStr">
+      <c r="G13" s="25" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="H13" s="29" t="inlineStr">
+      <c r="H13" s="25" t="inlineStr">
         <is>
           <t>L / x</t>
         </is>
       </c>
-      <c r="I13" s="29" t="inlineStr">
+      <c r="I13" s="25" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
-      <c r="J13" s="29" t="inlineStr">
+      <c r="J13" s="25" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2093,21 +2197,39 @@
           <t>1200WB278</t>
         </is>
       </c>
+      <c r="AP13" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AQ13" s="5" t="inlineStr">
+        <is>
+          <t>Tiled roof (90 kg/m²)</t>
+        </is>
+      </c>
+      <c r="AR13" s="30" t="n">
+        <v>0.883</v>
+      </c>
+      <c r="AS13" s="31" t="inlineStr">
+        <is>
+          <t>90 kg/m² x 9.81</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="14" customHeight="1">
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="32" t="inlineStr">
         <is>
           <t>Serviceability</t>
         </is>
       </c>
-      <c r="C14" s="31" t="n"/>
-      <c r="D14" s="31" t="n"/>
-      <c r="E14" s="31" t="n"/>
-      <c r="F14" s="31" t="n"/>
-      <c r="G14" s="31" t="n"/>
-      <c r="H14" s="31" t="n"/>
-      <c r="I14" s="31" t="n"/>
-      <c r="J14" s="31" t="n"/>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="33" t="n"/>
+      <c r="E14" s="33" t="n"/>
+      <c r="F14" s="33" t="n"/>
+      <c r="G14" s="33" t="n"/>
+      <c r="H14" s="33" t="n"/>
+      <c r="I14" s="33" t="n"/>
+      <c r="J14" s="33" t="n"/>
       <c r="M14" s="22" t="n"/>
       <c r="N14" s="23" t="n"/>
       <c r="O14" s="23" t="n"/>
@@ -2121,40 +2243,58 @@
           <t>1200WB249</t>
         </is>
       </c>
+      <c r="AP14" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AQ14" s="5" t="inlineStr">
+        <is>
+          <t>Ceiling + services</t>
+        </is>
+      </c>
+      <c r="AR14" s="30" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AS14" s="31" t="inlineStr">
+        <is>
+          <t>allowance</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="14" customHeight="1">
-      <c r="B15" s="32" t="inlineStr">
+      <c r="B15" s="34" t="inlineStr">
         <is>
           <t>Δg</t>
         </is>
       </c>
-      <c r="D15" s="33" t="inlineStr">
+      <c r="D15" s="35" t="inlineStr">
         <is>
           <t>Dead load</t>
         </is>
       </c>
-      <c r="E15" s="34" cm="1">
+      <c r="E15" s="36" cm="1">
         <f t="array" ref="E15">INDEX(_xlfn.ANCHORARRAY(B86),1,2)</f>
         <v/>
       </c>
-      <c r="F15" s="34">
+      <c r="F15" s="36">
         <f>IF(N(E37)=0,"",IF(N(F37)=0,Span/E37,MIN(Span/E37,F37)))</f>
         <v/>
       </c>
-      <c r="G15" s="35" t="inlineStr">
+      <c r="G15" s="37" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="H15" s="36">
+      <c r="H15" s="38">
         <f>IF(N(E15)=0,"",Span/E15)</f>
         <v/>
       </c>
-      <c r="I15" s="37">
+      <c r="I15" s="39">
         <f>IF(OR(E15="",N(F15)=0),"",ABS(E15)/F15)</f>
         <v/>
       </c>
-      <c r="J15" s="38">
+      <c r="J15" s="40">
         <f>IF(I15="","–",IF(I15&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
@@ -2171,40 +2311,58 @@
           <t>1000WB322</t>
         </is>
       </c>
+      <c r="AP15" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AQ15" s="5" t="inlineStr">
+        <is>
+          <t>Services allowance</t>
+        </is>
+      </c>
+      <c r="AR15" s="30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AS15" s="31" t="inlineStr">
+        <is>
+          <t>allowance</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="14" customHeight="1">
-      <c r="B16" s="32" t="inlineStr">
+      <c r="B16" s="34" t="inlineStr">
         <is>
           <t>Δg+ψl·q</t>
         </is>
       </c>
-      <c r="D16" s="33" t="inlineStr">
+      <c r="D16" s="35" t="inlineStr">
         <is>
           <t>Long term</t>
         </is>
       </c>
-      <c r="E16" s="34" cm="1">
+      <c r="E16" s="36" cm="1">
         <f t="array" ref="E16">INDEX(_xlfn.ANCHORARRAY(B86),2,2)</f>
         <v/>
       </c>
-      <c r="F16" s="34">
+      <c r="F16" s="36">
         <f>IF(N(E38)=0,"",IF(N(F38)=0,Span/E38,MIN(Span/E38,F38)))</f>
         <v/>
       </c>
-      <c r="G16" s="35" t="inlineStr">
+      <c r="G16" s="37" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="H16" s="36">
+      <c r="H16" s="38">
         <f>IF(N(E16)=0,"",Span/E16)</f>
         <v/>
       </c>
-      <c r="I16" s="37">
+      <c r="I16" s="39">
         <f>IF(OR(E16="",N(F16)=0),"",ABS(E16)/F16)</f>
         <v/>
       </c>
-      <c r="J16" s="38">
+      <c r="J16" s="40">
         <f>IF(I16="","–",IF(I16&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
@@ -2221,40 +2379,58 @@
           <t>1000WB296</t>
         </is>
       </c>
+      <c r="AP16" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AQ16" s="5" t="inlineStr">
+        <is>
+          <t>Typical floor (60 kg/m²)</t>
+        </is>
+      </c>
+      <c r="AR16" s="30" t="n">
+        <v>0.589</v>
+      </c>
+      <c r="AS16" s="31" t="inlineStr">
+        <is>
+          <t>60 kg/m² x 9.81</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="14" customHeight="1">
-      <c r="B17" s="32" t="inlineStr">
+      <c r="B17" s="34" t="inlineStr">
         <is>
           <t>Δg+ψs·q</t>
         </is>
       </c>
-      <c r="D17" s="33" t="inlineStr">
+      <c r="D17" s="35" t="inlineStr">
         <is>
           <t>Short term</t>
         </is>
       </c>
-      <c r="E17" s="34" cm="1">
+      <c r="E17" s="36" cm="1">
         <f t="array" ref="E17">INDEX(_xlfn.ANCHORARRAY(B86),3,2)</f>
         <v/>
       </c>
-      <c r="F17" s="34">
+      <c r="F17" s="36">
         <f>IF(N(E39)=0,"",IF(N(F39)=0,Span/E39,MIN(Span/E39,F39)))</f>
         <v/>
       </c>
-      <c r="G17" s="35" t="inlineStr">
+      <c r="G17" s="37" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="H17" s="36">
+      <c r="H17" s="38">
         <f>IF(N(E17)=0,"",Span/E17)</f>
         <v/>
       </c>
-      <c r="I17" s="37">
+      <c r="I17" s="39">
         <f>IF(OR(E17="",N(F17)=0),"",ABS(E17)/F17)</f>
         <v/>
       </c>
-      <c r="J17" s="38">
+      <c r="J17" s="40">
         <f>IF(I17="","–",IF(I17&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
@@ -2271,40 +2447,58 @@
           <t>1000WB258</t>
         </is>
       </c>
+      <c r="AP17" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AQ17" s="5" t="inlineStr">
+        <is>
+          <t>RC slab – per 100 mm (25 kN/m³)</t>
+        </is>
+      </c>
+      <c r="AR17" s="30" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AS17" s="31" t="inlineStr">
+        <is>
+          <t>scale by thickness / 100</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="14" customHeight="1">
-      <c r="B18" s="32" t="inlineStr">
+      <c r="B18" s="34" t="inlineStr">
         <is>
           <t>Δq</t>
         </is>
       </c>
-      <c r="D18" s="33" t="inlineStr">
+      <c r="D18" s="35" t="inlineStr">
         <is>
           <t>Live load only</t>
         </is>
       </c>
-      <c r="E18" s="34" cm="1">
+      <c r="E18" s="36" cm="1">
         <f t="array" ref="E18">INDEX(_xlfn.ANCHORARRAY(B86),4,2)</f>
         <v/>
       </c>
-      <c r="F18" s="34">
+      <c r="F18" s="36">
         <f>IF(N(E40)=0,"",IF(N(F40)=0,Span/E40,MIN(Span/E40,F40)))</f>
         <v/>
       </c>
-      <c r="G18" s="35" t="inlineStr">
+      <c r="G18" s="37" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="H18" s="36">
+      <c r="H18" s="38">
         <f>IF(N(E18)=0,"",Span/E18)</f>
         <v/>
       </c>
-      <c r="I18" s="37">
+      <c r="I18" s="39">
         <f>IF(OR(E18="",N(F18)=0),"",ABS(E18)/F18)</f>
         <v/>
       </c>
-      <c r="J18" s="38">
+      <c r="J18" s="40">
         <f>IF(I18="","–",IF(I18&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
@@ -2321,40 +2515,58 @@
           <t>1000WB215</t>
         </is>
       </c>
+      <c r="AP18" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="AQ18" s="5" t="inlineStr">
+        <is>
+          <t>Partitions allowance</t>
+        </is>
+      </c>
+      <c r="AR18" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS18" s="31" t="inlineStr">
+        <is>
+          <t>allowance – check AS/NZS 1170.1</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="14" customHeight="1">
-      <c r="B19" s="32" t="inlineStr">
+      <c r="B19" s="34" t="inlineStr">
         <is>
           <t>Δ1kN</t>
         </is>
       </c>
-      <c r="D19" s="33" t="inlineStr">
+      <c r="D19" s="35" t="inlineStr">
         <is>
           <t>1 kN at midspan</t>
         </is>
       </c>
-      <c r="E19" s="34" cm="1">
+      <c r="E19" s="36" cm="1">
         <f t="array" ref="E19">INDEX(_xlfn.ANCHORARRAY(B86),5,2)</f>
         <v/>
       </c>
-      <c r="F19" s="34">
+      <c r="F19" s="36">
         <f>IF(N(E41)=0,"",IF(N(F41)=0,Span/E41,MIN(Span/E41,F41)))</f>
         <v/>
       </c>
-      <c r="G19" s="35" t="inlineStr">
+      <c r="G19" s="37" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="H19" s="36">
+      <c r="H19" s="38">
         <f>IF(N(E19)=0,"",Span/E19)</f>
         <v/>
       </c>
-      <c r="I19" s="37">
+      <c r="I19" s="39">
         <f>IF(OR(E19="",N(F19)=0),"",ABS(E19)/F19)</f>
         <v/>
       </c>
-      <c r="J19" s="38">
+      <c r="J19" s="40">
         <f>IF(I19="","–",IF(I19&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
@@ -2371,21 +2583,39 @@
           <t>900WB282</t>
         </is>
       </c>
+      <c r="AP19" s="2" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AQ19" s="5" t="inlineStr">
+        <is>
+          <t>Roof – non-trafficable</t>
+        </is>
+      </c>
+      <c r="AR19" s="30" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AS19" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.1 Cl. 3.5.1: 0.12 + 1.2/A ≥ 0.25 kPa</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="14" customHeight="1">
-      <c r="B20" s="30" t="inlineStr">
+      <c r="B20" s="32" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
-      <c r="C20" s="31" t="n"/>
-      <c r="D20" s="31" t="n"/>
-      <c r="E20" s="31" t="n"/>
-      <c r="F20" s="31" t="n"/>
-      <c r="G20" s="31" t="n"/>
-      <c r="H20" s="31" t="n"/>
-      <c r="I20" s="31" t="n"/>
-      <c r="J20" s="31" t="n"/>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="33" t="n"/>
+      <c r="E20" s="33" t="n"/>
+      <c r="F20" s="33" t="n"/>
+      <c r="G20" s="33" t="n"/>
+      <c r="H20" s="33" t="n"/>
+      <c r="I20" s="33" t="n"/>
+      <c r="J20" s="33" t="n"/>
       <c r="M20" s="22" t="n"/>
       <c r="N20" s="23" t="n"/>
       <c r="O20" s="23" t="n"/>
@@ -2399,37 +2629,55 @@
           <t>900WB257</t>
         </is>
       </c>
+      <c r="AP20" s="2" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AQ20" s="5" t="inlineStr">
+        <is>
+          <t>Residential – habitable areas</t>
+        </is>
+      </c>
+      <c r="AR20" s="30" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AS20" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.1 Table 3.1 – verify category</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="14" customHeight="1">
-      <c r="B21" s="32" t="inlineStr">
+      <c r="B21" s="34" t="inlineStr">
         <is>
           <t>M* / φMbx</t>
         </is>
       </c>
-      <c r="D21" s="33" t="inlineStr">
+      <c r="D21" s="35" t="inlineStr">
         <is>
           <t>Bending – gravity (top flange critical)</t>
         </is>
       </c>
-      <c r="E21" s="39" cm="1">
+      <c r="E21" s="41" cm="1">
         <f t="array" ref="E21">INDEX(_xlfn.ANCHORARRAY(Z8),1,2)</f>
         <v/>
       </c>
-      <c r="F21" s="39" cm="1">
+      <c r="F21" s="41" cm="1">
         <f t="array" ref="F21">INDEX(_xlfn.ANCHORARRAY(Z8),1,3)</f>
         <v/>
       </c>
-      <c r="G21" s="35" t="inlineStr">
+      <c r="G21" s="37" t="inlineStr">
         <is>
           <t>kN·m</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr"/>
-      <c r="I21" s="37">
+      <c r="I21" s="39">
         <f>IF(OR(E21="",N(F21)=0),"",ABS(E21)/F21)</f>
         <v/>
       </c>
-      <c r="J21" s="38">
+      <c r="J21" s="40">
         <f>IF(I21="","–",IF(I21&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
@@ -2446,36 +2694,54 @@
           <t>900WB218</t>
         </is>
       </c>
+      <c r="AP21" s="2" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AQ21" s="5" t="inlineStr">
+        <is>
+          <t>Residential – balconies</t>
+        </is>
+      </c>
+      <c r="AR21" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS21" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.1 Table 3.1 – verify category</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="14" customHeight="1">
-      <c r="B22" s="32" t="inlineStr">
+      <c r="B22" s="34" t="inlineStr">
         <is>
           <t>M* / φMbx</t>
         </is>
       </c>
-      <c r="D22" s="33">
+      <c r="D22" s="35">
         <f>IF(NumUpliftCombos=0,"Bending – uplift (no uplift combinations)","Bending – uplift (bottom flange critical)")</f>
         <v/>
       </c>
-      <c r="E22" s="39" cm="1">
+      <c r="E22" s="41" cm="1">
         <f t="array" ref="E22">INDEX(_xlfn.ANCHORARRAY(Z8),2,2)</f>
         <v/>
       </c>
-      <c r="F22" s="39" cm="1">
+      <c r="F22" s="41" cm="1">
         <f t="array" ref="F22">INDEX(_xlfn.ANCHORARRAY(Z8),2,3)</f>
         <v/>
       </c>
-      <c r="G22" s="35" t="inlineStr">
+      <c r="G22" s="37" t="inlineStr">
         <is>
           <t>kN·m</t>
         </is>
       </c>
       <c r="H22" s="19" t="inlineStr"/>
-      <c r="I22" s="37">
+      <c r="I22" s="39">
         <f>IF(OR(E22="",N(F22)=0),"",ABS(E22)/F22)</f>
         <v/>
       </c>
-      <c r="J22" s="38">
+      <c r="J22" s="40">
         <f>IF(I22="","–",IF(I22&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
@@ -2492,37 +2758,55 @@
           <t>900WB175</t>
         </is>
       </c>
+      <c r="AP22" s="2" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AQ22" s="5" t="inlineStr">
+        <is>
+          <t>Offices – general use</t>
+        </is>
+      </c>
+      <c r="AR22" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS22" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.1 Table 3.1 – verify category</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="14" customHeight="1">
-      <c r="B23" s="32" t="inlineStr">
+      <c r="B23" s="34" t="inlineStr">
         <is>
           <t>V* / φVv</t>
         </is>
       </c>
-      <c r="D23" s="33" t="inlineStr">
+      <c r="D23" s="35" t="inlineStr">
         <is>
           <t>Shear</t>
         </is>
       </c>
-      <c r="E23" s="39" cm="1">
+      <c r="E23" s="41" cm="1">
         <f t="array" ref="E23">INDEX(_xlfn.ANCHORARRAY(Z8),3,2)</f>
         <v/>
       </c>
-      <c r="F23" s="39" cm="1">
+      <c r="F23" s="41" cm="1">
         <f t="array" ref="F23">INDEX(_xlfn.ANCHORARRAY(Z8),3,3)</f>
         <v/>
       </c>
-      <c r="G23" s="35" t="inlineStr">
+      <c r="G23" s="37" t="inlineStr">
         <is>
           <t>kN</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr"/>
-      <c r="I23" s="37">
+      <c r="I23" s="39">
         <f>IF(OR(E23="",N(F23)=0),"",ABS(E23)/F23)</f>
         <v/>
       </c>
-      <c r="J23" s="38">
+      <c r="J23" s="40">
         <f>IF(I23="","–",IF(I23&lt;=1,"OK","NG"))</f>
         <v/>
       </c>
@@ -2537,6 +2821,24 @@
       <c r="AN23" s="20" t="inlineStr">
         <is>
           <t>800WB192</t>
+        </is>
+      </c>
+      <c r="AP23" s="2" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AQ23" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="AR23" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="AS23" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.1 Table 3.1 – verify category</t>
         </is>
       </c>
     </row>
@@ -2552,6 +2854,24 @@
       <c r="AN24" s="20" t="inlineStr">
         <is>
           <t>800WB168</t>
+        </is>
+      </c>
+      <c r="AP24" s="2" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AQ24" s="5" t="inlineStr">
+        <is>
+          <t>Assembly / crowds</t>
+        </is>
+      </c>
+      <c r="AR24" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS24" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.1 Table 3.1 – verify category</t>
         </is>
       </c>
     </row>
@@ -2582,9 +2902,27 @@
           <t>800WB146</t>
         </is>
       </c>
+      <c r="AP25" s="2" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AQ25" s="5" t="inlineStr">
+        <is>
+          <t>Car park – light vehicles</t>
+        </is>
+      </c>
+      <c r="AR25" s="30" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AS25" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.1 Table 3.1 – verify category</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="14" customHeight="1">
-      <c r="B26" s="40" t="inlineStr">
+      <c r="B26" s="42" t="inlineStr">
         <is>
           <t>Section type</t>
         </is>
@@ -2594,7 +2932,7 @@
           <t>UB</t>
         </is>
       </c>
-      <c r="G26" s="41" t="inlineStr">
+      <c r="G26" s="43" t="inlineStr">
         <is>
           <t>Section properties (add-in)</t>
         </is>
@@ -2612,9 +2950,27 @@
           <t>800WB122</t>
         </is>
       </c>
+      <c r="AP26" s="2" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AQ26" s="5" t="inlineStr">
+        <is>
+          <t>Plant room – light</t>
+        </is>
+      </c>
+      <c r="AR26" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS26" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.1 Table 3.1 – verify category</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="14" customHeight="1">
-      <c r="B27" s="40" t="inlineStr">
+      <c r="B27" s="42" t="inlineStr">
         <is>
           <t>Section size</t>
         </is>
@@ -2624,16 +2980,16 @@
           <t>310UB40.4</t>
         </is>
       </c>
-      <c r="G27" s="42" t="inlineStr">
+      <c r="G27" s="44" t="inlineStr">
         <is>
           <t>Mass</t>
         </is>
       </c>
-      <c r="H27" s="39" cm="1">
+      <c r="H27" s="41" cm="1">
         <f t="array" ref="H27">OAR.SECTION(SectionSize,"Mass",Grade)</f>
         <v/>
       </c>
-      <c r="I27" s="43" t="inlineStr">
+      <c r="I27" s="45" t="inlineStr">
         <is>
           <t>kg/m</t>
         </is>
@@ -2651,31 +3007,49 @@
           <t>700WB173</t>
         </is>
       </c>
+      <c r="AP27" s="2" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AQ27" s="5" t="inlineStr">
+        <is>
+          <t>Storage – per metre of height</t>
+        </is>
+      </c>
+      <c r="AR27" s="30" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="AS27" s="31" t="inlineStr">
+        <is>
+          <t>multiply by storage height</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="14" customHeight="1">
-      <c r="B28" s="40" t="inlineStr">
+      <c r="B28" s="42" t="inlineStr">
         <is>
           <t>Steel grade</t>
         </is>
       </c>
-      <c r="E28" s="44" t="n">
+      <c r="E28" s="46" t="n">
         <v>300</v>
       </c>
-      <c r="F28" s="43" t="inlineStr">
+      <c r="F28" s="45" t="inlineStr">
         <is>
           <t>MPa</t>
         </is>
       </c>
-      <c r="G28" s="42" t="inlineStr">
+      <c r="G28" s="44" t="inlineStr">
         <is>
           <t>Ix</t>
         </is>
       </c>
-      <c r="H28" s="39" cm="1">
+      <c r="H28" s="41" cm="1">
         <f t="array" ref="H28">OAR.SECTION(SectionSize,"Ix",Grade)</f>
         <v/>
       </c>
-      <c r="I28" s="43" t="inlineStr">
+      <c r="I28" s="45" t="inlineStr">
         <is>
           <t>×10⁶ mm⁴</t>
         </is>
@@ -2693,31 +3067,47 @@
           <t>700WB150</t>
         </is>
       </c>
+      <c r="AP28" s="2" t="inlineStr">
+        <is>
+          <t>Wd</t>
+        </is>
+      </c>
+      <c r="AQ28" s="5" t="inlineStr">
+        <is>
+          <t>External wind – downward</t>
+        </is>
+      </c>
+      <c r="AR28" s="30" t="n"/>
+      <c r="AS28" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.2 – enter pressure</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="14" customHeight="1">
-      <c r="B29" s="40" t="inlineStr">
+      <c r="B29" s="42" t="inlineStr">
         <is>
           <t>Span (centre to centre of supports)</t>
         </is>
       </c>
-      <c r="E29" s="45" t="n">
+      <c r="E29" s="47" t="n">
         <v>8300</v>
       </c>
-      <c r="F29" s="43" t="inlineStr">
+      <c r="F29" s="45" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="G29" s="42" t="inlineStr">
+      <c r="G29" s="44" t="inlineStr">
         <is>
           <t>Iy</t>
         </is>
       </c>
-      <c r="H29" s="34" cm="1">
+      <c r="H29" s="36" cm="1">
         <f t="array" ref="H29">OAR.SECTION(SectionSize,"Iy",Grade)</f>
         <v/>
       </c>
-      <c r="I29" s="43" t="inlineStr">
+      <c r="I29" s="45" t="inlineStr">
         <is>
           <t>×10⁶ mm⁴</t>
         </is>
@@ -2735,9 +3125,25 @@
           <t>700WB130</t>
         </is>
       </c>
+      <c r="AP29" s="2" t="inlineStr">
+        <is>
+          <t>Wu</t>
+        </is>
+      </c>
+      <c r="AQ29" s="5" t="inlineStr">
+        <is>
+          <t>External wind – net uplift</t>
+        </is>
+      </c>
+      <c r="AR29" s="30" t="n"/>
+      <c r="AS29" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.2 – enter pressure</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="14" customHeight="1">
-      <c r="B30" s="40" t="inlineStr">
+      <c r="B30" s="42" t="inlineStr">
         <is>
           <t>Support condition</t>
         </is>
@@ -2747,17 +3153,17 @@
           <t>Simply supported</t>
         </is>
       </c>
-      <c r="F30" s="46" t="n"/>
-      <c r="G30" s="42" t="inlineStr">
+      <c r="F30" s="48" t="n"/>
+      <c r="G30" s="44" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="H30" s="39" cm="1">
+      <c r="H30" s="41" cm="1">
         <f t="array" ref="H30">OAR.SECTION(SectionSize,"J",Grade)</f>
         <v/>
       </c>
-      <c r="I30" s="43" t="inlineStr">
+      <c r="I30" s="45" t="inlineStr">
         <is>
           <t>×10³ mm⁴</t>
         </is>
@@ -2775,31 +3181,47 @@
           <t>700WB115</t>
         </is>
       </c>
+      <c r="AP30" s="2" t="inlineStr">
+        <is>
+          <t>Wid</t>
+        </is>
+      </c>
+      <c r="AQ30" s="5" t="inlineStr">
+        <is>
+          <t>Internal suction (−cpi)</t>
+        </is>
+      </c>
+      <c r="AR30" s="30" t="n"/>
+      <c r="AS30" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.2 – enter pressure</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="14" customHeight="1">
-      <c r="B31" s="40" t="inlineStr">
+      <c r="B31" s="42" t="inlineStr">
         <is>
           <t>Elastic modulus</t>
         </is>
       </c>
-      <c r="E31" s="45" t="n">
+      <c r="E31" s="47" t="n">
         <v>200000</v>
       </c>
-      <c r="F31" s="43" t="inlineStr">
+      <c r="F31" s="45" t="inlineStr">
         <is>
           <t>MPa</t>
         </is>
       </c>
-      <c r="G31" s="42" t="inlineStr">
+      <c r="G31" s="44" t="inlineStr">
         <is>
           <t>Iw</t>
         </is>
       </c>
-      <c r="H31" s="39" cm="1">
+      <c r="H31" s="41" cm="1">
         <f t="array" ref="H31">OAR.SECTION(SectionSize,"Iw",Grade)</f>
         <v/>
       </c>
-      <c r="I31" s="43" t="inlineStr">
+      <c r="I31" s="45" t="inlineStr">
         <is>
           <t>×10⁹ mm⁶</t>
         </is>
@@ -2817,9 +3239,25 @@
           <t>760UB244</t>
         </is>
       </c>
+      <c r="AP31" s="2" t="inlineStr">
+        <is>
+          <t>Wiu</t>
+        </is>
+      </c>
+      <c r="AQ31" s="5" t="inlineStr">
+        <is>
+          <t>Internal pressure (+cpi)</t>
+        </is>
+      </c>
+      <c r="AR31" s="30" t="n"/>
+      <c r="AS31" s="31" t="inlineStr">
+        <is>
+          <t>AS/NZS 1170.2 – enter pressure</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="14" customHeight="1">
-      <c r="B32" s="40" t="inlineStr">
+      <c r="B32" s="42" t="inlineStr">
         <is>
           <t>Include self-weight</t>
         </is>
@@ -2829,16 +3267,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G32" s="42" t="inlineStr">
+      <c r="G32" s="44" t="inlineStr">
         <is>
           <t>Zex</t>
         </is>
       </c>
-      <c r="H32" s="47" cm="1">
+      <c r="H32" s="49" cm="1">
         <f t="array" ref="H32">OAR.SECTION(SectionSize,"Ze",Grade)</f>
         <v/>
       </c>
-      <c r="I32" s="43" t="inlineStr">
+      <c r="I32" s="45" t="inlineStr">
         <is>
           <t>×10³ mm³</t>
         </is>
@@ -2858,16 +3296,16 @@
       </c>
     </row>
     <row r="33" ht="14" customHeight="1">
-      <c r="G33" s="42" t="inlineStr">
+      <c r="G33" s="44" t="inlineStr">
         <is>
           <t>φMsx</t>
         </is>
       </c>
-      <c r="H33" s="39" cm="1">
+      <c r="H33" s="41" cm="1">
         <f t="array" ref="H33">OAR.SECTION(SectionSize,"phiMsx",Grade)</f>
         <v/>
       </c>
-      <c r="I33" s="43" t="inlineStr">
+      <c r="I33" s="45" t="inlineStr">
         <is>
           <t>kN·m</t>
         </is>
@@ -2930,28 +3368,28 @@
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
-      <c r="B36" s="48" t="inlineStr">
+      <c r="B36" s="50" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C36" s="46" t="n"/>
-      <c r="D36" s="48" t="inlineStr">
+      <c r="C36" s="48" t="n"/>
+      <c r="D36" s="50" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E36" s="48" t="inlineStr">
+      <c r="E36" s="50" t="inlineStr">
         <is>
           <t xml:space="preserve">Span / </t>
         </is>
       </c>
-      <c r="F36" s="48" t="inlineStr">
+      <c r="F36" s="50" t="inlineStr">
         <is>
           <t>Max (mm)</t>
         </is>
       </c>
-      <c r="G36" s="48" t="inlineStr">
+      <c r="G36" s="50" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
@@ -2971,24 +3409,24 @@
       </c>
     </row>
     <row r="37" ht="14" customHeight="1">
-      <c r="B37" s="49" t="inlineStr">
+      <c r="B37" s="51" t="inlineStr">
         <is>
           <t>Δg</t>
         </is>
       </c>
-      <c r="C37" s="50" t="n"/>
-      <c r="D37" s="51" t="inlineStr">
+      <c r="C37" s="52" t="n"/>
+      <c r="D37" s="53" t="inlineStr">
         <is>
           <t>Dead load</t>
         </is>
       </c>
-      <c r="E37" s="44" t="n">
+      <c r="E37" s="46" t="n">
         <v>500</v>
       </c>
-      <c r="F37" s="52" t="n">
+      <c r="F37" s="54" t="n">
         <v>20</v>
       </c>
-      <c r="G37" s="53" t="inlineStr">
+      <c r="G37" s="55" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3013,24 +3451,24 @@
       </c>
     </row>
     <row r="38" ht="14" customHeight="1">
-      <c r="B38" s="49" t="inlineStr">
+      <c r="B38" s="51" t="inlineStr">
         <is>
           <t>Δg+ψl·q</t>
         </is>
       </c>
-      <c r="C38" s="50" t="n"/>
-      <c r="D38" s="51" t="inlineStr">
+      <c r="C38" s="52" t="n"/>
+      <c r="D38" s="53" t="inlineStr">
         <is>
           <t>Long term (ψl)</t>
         </is>
       </c>
-      <c r="E38" s="44" t="n">
+      <c r="E38" s="46" t="n">
         <v>360</v>
       </c>
-      <c r="F38" s="52" t="n">
+      <c r="F38" s="54" t="n">
         <v>25</v>
       </c>
-      <c r="G38" s="52" t="n">
+      <c r="G38" s="54" t="n">
         <v>0.4</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
@@ -3053,24 +3491,24 @@
       </c>
     </row>
     <row r="39" ht="14" customHeight="1">
-      <c r="B39" s="49" t="inlineStr">
+      <c r="B39" s="51" t="inlineStr">
         <is>
           <t>Δg+ψs·q</t>
         </is>
       </c>
-      <c r="C39" s="50" t="n"/>
-      <c r="D39" s="51" t="inlineStr">
+      <c r="C39" s="52" t="n"/>
+      <c r="D39" s="53" t="inlineStr">
         <is>
           <t>Short term (ψs)</t>
         </is>
       </c>
-      <c r="E39" s="44" t="n">
+      <c r="E39" s="46" t="n">
         <v>300</v>
       </c>
-      <c r="F39" s="52" t="n">
+      <c r="F39" s="54" t="n">
         <v>30</v>
       </c>
-      <c r="G39" s="52" t="n">
+      <c r="G39" s="54" t="n">
         <v>0.7</v>
       </c>
       <c r="M39" s="22" t="n"/>
@@ -3088,36 +3526,36 @@
       </c>
     </row>
     <row r="40" ht="14" customHeight="1">
-      <c r="B40" s="49" t="inlineStr">
+      <c r="B40" s="51" t="inlineStr">
         <is>
           <t>Δq</t>
         </is>
       </c>
-      <c r="C40" s="50" t="n"/>
-      <c r="D40" s="51" t="inlineStr">
+      <c r="C40" s="52" t="n"/>
+      <c r="D40" s="53" t="inlineStr">
         <is>
           <t>Live load only</t>
         </is>
       </c>
-      <c r="E40" s="44" t="n">
+      <c r="E40" s="46" t="n">
         <v>250</v>
       </c>
-      <c r="F40" s="52" t="n">
+      <c r="F40" s="54" t="n">
         <v>30</v>
       </c>
-      <c r="G40" s="53" t="inlineStr">
+      <c r="G40" s="55" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="M40" s="54" t="n"/>
-      <c r="N40" s="55" t="n"/>
-      <c r="O40" s="55" t="n"/>
-      <c r="P40" s="55" t="n"/>
-      <c r="Q40" s="55" t="n"/>
-      <c r="R40" s="55" t="n"/>
-      <c r="S40" s="55" t="n"/>
-      <c r="T40" s="56" t="n"/>
+      <c r="M40" s="56" t="n"/>
+      <c r="N40" s="57" t="n"/>
+      <c r="O40" s="57" t="n"/>
+      <c r="P40" s="57" t="n"/>
+      <c r="Q40" s="57" t="n"/>
+      <c r="R40" s="57" t="n"/>
+      <c r="S40" s="57" t="n"/>
+      <c r="T40" s="58" t="n"/>
       <c r="AN40" s="20" t="inlineStr">
         <is>
           <t>610UB101</t>
@@ -3125,24 +3563,24 @@
       </c>
     </row>
     <row r="41" ht="14" customHeight="1">
-      <c r="B41" s="49" t="inlineStr">
+      <c r="B41" s="51" t="inlineStr">
         <is>
           <t>Δ1kN</t>
         </is>
       </c>
-      <c r="C41" s="50" t="n"/>
-      <c r="D41" s="51" t="inlineStr">
+      <c r="C41" s="52" t="n"/>
+      <c r="D41" s="53" t="inlineStr">
         <is>
           <t>1 kN point load at midspan</t>
         </is>
       </c>
-      <c r="E41" s="44" t="n">
+      <c r="E41" s="46" t="n">
         <v>1000</v>
       </c>
-      <c r="F41" s="52" t="n">
+      <c r="F41" s="54" t="n">
         <v>1.5</v>
       </c>
-      <c r="G41" s="53" t="inlineStr">
+      <c r="G41" s="55" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -3231,107 +3669,107 @@
       </c>
     </row>
     <row r="46" ht="26" customHeight="1">
-      <c r="B46" s="57" t="inlineStr">
+      <c r="B46" s="59" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C46" s="57" t="inlineStr">
+      <c r="C46" s="59" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D46" s="57" t="inlineStr">
+      <c r="D46" s="59" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E46" s="57" t="inlineStr">
+      <c r="E46" s="59" t="inlineStr">
         <is>
           <t>Trib (m | m²)</t>
         </is>
       </c>
-      <c r="F46" s="57" t="inlineStr">
+      <c r="F46" s="59" t="inlineStr">
         <is>
           <t>Press. (kPa)</t>
         </is>
       </c>
-      <c r="G46" s="57" t="inlineStr">
+      <c r="G46" s="59" t="inlineStr">
         <is>
           <t>+ Direct (kN/m | kN)</t>
         </is>
       </c>
-      <c r="H46" s="57" t="inlineStr">
+      <c r="H46" s="59" t="inlineStr">
         <is>
           <t>Start (mm)</t>
         </is>
       </c>
-      <c r="I46" s="57" t="inlineStr">
+      <c r="I46" s="59" t="inlineStr">
         <is>
           <t>End (mm)</t>
         </is>
       </c>
-      <c r="J46" s="57" t="inlineStr">
+      <c r="J46" s="59" t="inlineStr">
         <is>
           <t>Load</t>
         </is>
       </c>
-      <c r="M46" s="29" t="inlineStr">
+      <c r="M46" s="25" t="inlineStr">
         <is>
           <t>Include</t>
         </is>
       </c>
-      <c r="N46" s="29" t="inlineStr">
+      <c r="N46" s="25" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="O46" s="29" t="inlineStr">
+      <c r="O46" s="25" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="P46" s="29" t="inlineStr">
+      <c r="P46" s="25" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="Q46" s="29" t="inlineStr">
+      <c r="Q46" s="25" t="inlineStr">
         <is>
           <t>Crit. flange</t>
         </is>
       </c>
-      <c r="R46" s="29" t="inlineStr">
+      <c r="R46" s="25" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="S46" s="29" t="inlineStr">
+      <c r="S46" s="25" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="T46" s="29" t="inlineStr">
+      <c r="T46" s="25" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="U46" s="29" t="inlineStr">
+      <c r="U46" s="25" t="inlineStr">
         <is>
           <t>Wd</t>
         </is>
       </c>
-      <c r="V46" s="29" t="inlineStr">
+      <c r="V46" s="25" t="inlineStr">
         <is>
           <t>Wu</t>
         </is>
       </c>
-      <c r="W46" s="29" t="inlineStr">
+      <c r="W46" s="25" t="inlineStr">
         <is>
           <t>Wid</t>
         </is>
       </c>
-      <c r="X46" s="29" t="inlineStr">
+      <c r="X46" s="25" t="inlineStr">
         <is>
           <t>Wiu</t>
         </is>
@@ -3358,21 +3796,22 @@
           <t>Roof sheeting + purlins</t>
         </is>
       </c>
-      <c r="E47" s="58" t="n">
+      <c r="E47" s="60" t="n">
         <v>5.65</v>
       </c>
-      <c r="F47" s="59" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G47" s="59" t="n"/>
-      <c r="H47" s="45" t="n"/>
-      <c r="I47" s="45" t="n"/>
-      <c r="J47" s="60">
+      <c r="F47" s="30">
+        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(D47,LoadLib_B1[Description],0)),"")</f>
+        <v/>
+      </c>
+      <c r="G47" s="30" t="n"/>
+      <c r="H47" s="47" t="n"/>
+      <c r="I47" s="47" t="n"/>
+      <c r="J47" s="61">
         <f>IF(B47="","",N(E47)*N(F47)+N(G47))</f>
         <v/>
       </c>
       <c r="M47" s="2" t="n"/>
-      <c r="N47" s="61">
+      <c r="N47" s="62">
         <f>IF(M47="No",0,IF(P47="",0,IF(M47="Yes",1,IF(OR(CombSet="All",O47="Custom",AND(O47="Gravity",CombSet&lt;&gt;"Custom"),AND(O47="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3396,22 +3835,22 @@
           <t>1.35G</t>
         </is>
       </c>
-      <c r="S47" s="59" t="n">
+      <c r="S47" s="30" t="n">
         <v>1.35</v>
       </c>
-      <c r="T47" s="59" t="n">
+      <c r="T47" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="U47" s="59" t="n">
+      <c r="U47" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="V47" s="59" t="n">
+      <c r="V47" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="W47" s="59" t="n">
+      <c r="W47" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="X47" s="59" t="n">
+      <c r="X47" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AN47" s="20" t="inlineStr">
@@ -3436,21 +3875,22 @@
           <t>Ceiling + services</t>
         </is>
       </c>
-      <c r="E48" s="58" t="n">
+      <c r="E48" s="60" t="n">
         <v>5.65</v>
       </c>
-      <c r="F48" s="59" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G48" s="59" t="n"/>
-      <c r="H48" s="45" t="n"/>
-      <c r="I48" s="45" t="n"/>
-      <c r="J48" s="60">
+      <c r="F48" s="30">
+        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(D48,LoadLib_B1[Description],0)),"")</f>
+        <v/>
+      </c>
+      <c r="G48" s="30" t="n"/>
+      <c r="H48" s="47" t="n"/>
+      <c r="I48" s="47" t="n"/>
+      <c r="J48" s="61">
         <f>IF(B48="","",N(E48)*N(F48)+N(G48))</f>
         <v/>
       </c>
       <c r="M48" s="2" t="n"/>
-      <c r="N48" s="61">
+      <c r="N48" s="62">
         <f>IF(M48="No",0,IF(P48="",0,IF(M48="Yes",1,IF(OR(CombSet="All",O48="Custom",AND(O48="Gravity",CombSet&lt;&gt;"Custom"),AND(O48="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3474,22 +3914,22 @@
           <t>1.2G + 1.5Q</t>
         </is>
       </c>
-      <c r="S48" s="59" t="n">
+      <c r="S48" s="30" t="n">
         <v>1.2</v>
       </c>
-      <c r="T48" s="59" t="n">
+      <c r="T48" s="30" t="n">
         <v>1.5</v>
       </c>
-      <c r="U48" s="59" t="n">
+      <c r="U48" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="V48" s="59" t="n">
+      <c r="V48" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="W48" s="59" t="n">
+      <c r="W48" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="X48" s="59" t="n">
+      <c r="X48" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AN48" s="20" t="inlineStr">
@@ -3514,19 +3954,19 @@
           <t>Beam bracket / misc.</t>
         </is>
       </c>
-      <c r="E49" s="58" t="n"/>
-      <c r="F49" s="59" t="n"/>
-      <c r="G49" s="59" t="n">
+      <c r="E49" s="60" t="n"/>
+      <c r="F49" s="30" t="n"/>
+      <c r="G49" s="30" t="n">
         <v>0.05</v>
       </c>
-      <c r="H49" s="45" t="n"/>
-      <c r="I49" s="45" t="n"/>
-      <c r="J49" s="60">
+      <c r="H49" s="47" t="n"/>
+      <c r="I49" s="47" t="n"/>
+      <c r="J49" s="61">
         <f>IF(B49="","",N(E49)*N(F49)+N(G49))</f>
         <v/>
       </c>
       <c r="M49" s="2" t="n"/>
-      <c r="N49" s="61">
+      <c r="N49" s="62">
         <f>IF(M49="No",0,IF(P49="",0,IF(M49="Yes",1,IF(OR(CombSet="All",O49="Custom",AND(O49="Gravity",CombSet&lt;&gt;"Custom"),AND(O49="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3550,23 +3990,23 @@
           <t>1.2G + 1.5ψlQ</t>
         </is>
       </c>
-      <c r="S49" s="59" t="n">
+      <c r="S49" s="30" t="n">
         <v>1.2</v>
       </c>
-      <c r="T49" s="59">
+      <c r="T49" s="30">
         <f>1.5*PsiL</f>
         <v/>
       </c>
-      <c r="U49" s="59" t="n">
+      <c r="U49" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="V49" s="59" t="n">
+      <c r="V49" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="W49" s="59" t="n">
+      <c r="W49" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="X49" s="59" t="n">
+      <c r="X49" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AN49" s="20" t="inlineStr">
@@ -3588,24 +4028,25 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Roof live (non-trafficable)</t>
-        </is>
-      </c>
-      <c r="E50" s="58" t="n">
+          <t>Roof – non-trafficable</t>
+        </is>
+      </c>
+      <c r="E50" s="60" t="n">
         <v>5.65</v>
       </c>
-      <c r="F50" s="59" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G50" s="59" t="n"/>
-      <c r="H50" s="45" t="n"/>
-      <c r="I50" s="45" t="n"/>
-      <c r="J50" s="60">
+      <c r="F50" s="30">
+        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(D50,LoadLib_B1[Description],0)),"")</f>
+        <v/>
+      </c>
+      <c r="G50" s="30" t="n"/>
+      <c r="H50" s="47" t="n"/>
+      <c r="I50" s="47" t="n"/>
+      <c r="J50" s="61">
         <f>IF(B50="","",N(E50)*N(F50)+N(G50))</f>
         <v/>
       </c>
       <c r="M50" s="2" t="n"/>
-      <c r="N50" s="61">
+      <c r="N50" s="62">
         <f>IF(M50="No",0,IF(P50="",0,IF(M50="Yes",1,IF(OR(CombSet="All",O50="Custom",AND(O50="Gravity",CombSet&lt;&gt;"Custom"),AND(O50="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3629,23 +4070,23 @@
           <t>1.2G + ψcQ + Wd + Wi(−cpi)</t>
         </is>
       </c>
-      <c r="S50" s="59" t="n">
+      <c r="S50" s="30" t="n">
         <v>1.2</v>
       </c>
-      <c r="T50" s="59">
+      <c r="T50" s="30">
         <f>PsiC</f>
         <v/>
       </c>
-      <c r="U50" s="59" t="n">
+      <c r="U50" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="V50" s="59" t="n">
+      <c r="V50" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="W50" s="59" t="n">
+      <c r="W50" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="X50" s="59" t="n">
+      <c r="X50" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AN50" s="20" t="inlineStr">
@@ -3670,21 +4111,21 @@
           <t>External wind – net uplift</t>
         </is>
       </c>
-      <c r="E51" s="58" t="n">
+      <c r="E51" s="60" t="n">
         <v>5.65</v>
       </c>
-      <c r="F51" s="59" t="n">
+      <c r="F51" s="30" t="n">
         <v>1.72</v>
       </c>
-      <c r="G51" s="59" t="n"/>
-      <c r="H51" s="45" t="n"/>
-      <c r="I51" s="45" t="n"/>
-      <c r="J51" s="60">
+      <c r="G51" s="30" t="n"/>
+      <c r="H51" s="47" t="n"/>
+      <c r="I51" s="47" t="n"/>
+      <c r="J51" s="61">
         <f>IF(B51="","",N(E51)*N(F51)+N(G51))</f>
         <v/>
       </c>
       <c r="M51" s="2" t="n"/>
-      <c r="N51" s="61">
+      <c r="N51" s="62">
         <f>IF(M51="No",0,IF(P51="",0,IF(M51="Yes",1,IF(OR(CombSet="All",O51="Custom",AND(O51="Gravity",CombSet&lt;&gt;"Custom"),AND(O51="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3708,22 +4149,22 @@
           <t>0.9G + Wu + Wi(+cpi)</t>
         </is>
       </c>
-      <c r="S51" s="59" t="n">
+      <c r="S51" s="30" t="n">
         <v>0.9</v>
       </c>
-      <c r="T51" s="59" t="n">
+      <c r="T51" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="U51" s="59" t="n">
+      <c r="U51" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="V51" s="59" t="n">
+      <c r="V51" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="W51" s="59" t="n">
+      <c r="W51" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="X51" s="59" t="n">
+      <c r="X51" s="30" t="n">
         <v>1</v>
       </c>
       <c r="AN51" s="20" t="inlineStr">
@@ -3748,21 +4189,21 @@
           <t>External wind – downward</t>
         </is>
       </c>
-      <c r="E52" s="58" t="n">
+      <c r="E52" s="60" t="n">
         <v>5.65</v>
       </c>
-      <c r="F52" s="59" t="n">
+      <c r="F52" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="G52" s="59" t="n"/>
-      <c r="H52" s="45" t="n"/>
-      <c r="I52" s="45" t="n"/>
-      <c r="J52" s="60">
+      <c r="G52" s="30" t="n"/>
+      <c r="H52" s="47" t="n"/>
+      <c r="I52" s="47" t="n"/>
+      <c r="J52" s="61">
         <f>IF(B52="","",N(E52)*N(F52)+N(G52))</f>
         <v/>
       </c>
       <c r="M52" s="2" t="n"/>
-      <c r="N52" s="61">
+      <c r="N52" s="62">
         <f>IF(M52="No",0,IF(P52="",0,IF(M52="Yes",1,IF(OR(CombSet="All",O52="Custom",AND(O52="Gravity",CombSet&lt;&gt;"Custom"),AND(O52="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3774,12 +4215,12 @@
       <c r="P52" s="2" t="n"/>
       <c r="Q52" s="2" t="n"/>
       <c r="R52" s="5" t="n"/>
-      <c r="S52" s="59" t="n"/>
-      <c r="T52" s="59" t="n"/>
-      <c r="U52" s="59" t="n"/>
-      <c r="V52" s="59" t="n"/>
-      <c r="W52" s="59" t="n"/>
-      <c r="X52" s="59" t="n"/>
+      <c r="S52" s="30" t="n"/>
+      <c r="T52" s="30" t="n"/>
+      <c r="U52" s="30" t="n"/>
+      <c r="V52" s="30" t="n"/>
+      <c r="W52" s="30" t="n"/>
+      <c r="X52" s="30" t="n"/>
       <c r="AN52" s="20" t="inlineStr">
         <is>
           <t>310UB40.4</t>
@@ -3802,21 +4243,21 @@
           <t>Internal pressure (+cpi)</t>
         </is>
       </c>
-      <c r="E53" s="58" t="n">
+      <c r="E53" s="60" t="n">
         <v>5.65</v>
       </c>
-      <c r="F53" s="59" t="n">
+      <c r="F53" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="G53" s="59" t="n"/>
-      <c r="H53" s="45" t="n"/>
-      <c r="I53" s="45" t="n"/>
-      <c r="J53" s="60">
+      <c r="G53" s="30" t="n"/>
+      <c r="H53" s="47" t="n"/>
+      <c r="I53" s="47" t="n"/>
+      <c r="J53" s="61">
         <f>IF(B53="","",N(E53)*N(F53)+N(G53))</f>
         <v/>
       </c>
       <c r="M53" s="2" t="n"/>
-      <c r="N53" s="61">
+      <c r="N53" s="62">
         <f>IF(M53="No",0,IF(P53="",0,IF(M53="Yes",1,IF(OR(CombSet="All",O53="Custom",AND(O53="Gravity",CombSet&lt;&gt;"Custom"),AND(O53="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3828,12 +4269,12 @@
       <c r="P53" s="2" t="n"/>
       <c r="Q53" s="2" t="n"/>
       <c r="R53" s="5" t="n"/>
-      <c r="S53" s="59" t="n"/>
-      <c r="T53" s="59" t="n"/>
-      <c r="U53" s="59" t="n"/>
-      <c r="V53" s="59" t="n"/>
-      <c r="W53" s="59" t="n"/>
-      <c r="X53" s="59" t="n"/>
+      <c r="S53" s="30" t="n"/>
+      <c r="T53" s="30" t="n"/>
+      <c r="U53" s="30" t="n"/>
+      <c r="V53" s="30" t="n"/>
+      <c r="W53" s="30" t="n"/>
+      <c r="X53" s="30" t="n"/>
       <c r="AN53" s="20" t="inlineStr">
         <is>
           <t>310UB32</t>
@@ -3856,21 +4297,21 @@
           <t>Internal suction (−cpi)</t>
         </is>
       </c>
-      <c r="E54" s="58" t="n">
+      <c r="E54" s="60" t="n">
         <v>5.65</v>
       </c>
-      <c r="F54" s="59" t="n">
+      <c r="F54" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="G54" s="59" t="n"/>
-      <c r="H54" s="45" t="n"/>
-      <c r="I54" s="45" t="n"/>
-      <c r="J54" s="60">
+      <c r="G54" s="30" t="n"/>
+      <c r="H54" s="47" t="n"/>
+      <c r="I54" s="47" t="n"/>
+      <c r="J54" s="61">
         <f>IF(B54="","",N(E54)*N(F54)+N(G54))</f>
         <v/>
       </c>
       <c r="M54" s="2" t="n"/>
-      <c r="N54" s="61">
+      <c r="N54" s="62">
         <f>IF(M54="No",0,IF(P54="",0,IF(M54="Yes",1,IF(OR(CombSet="All",O54="Custom",AND(O54="Gravity",CombSet&lt;&gt;"Custom"),AND(O54="Wind",CombSet="Roof")),1,0))))</f>
         <v/>
       </c>
@@ -3882,12 +4323,12 @@
       <c r="P54" s="2" t="n"/>
       <c r="Q54" s="2" t="n"/>
       <c r="R54" s="5" t="n"/>
-      <c r="S54" s="59" t="n"/>
-      <c r="T54" s="59" t="n"/>
-      <c r="U54" s="59" t="n"/>
-      <c r="V54" s="59" t="n"/>
-      <c r="W54" s="59" t="n"/>
-      <c r="X54" s="59" t="n"/>
+      <c r="S54" s="30" t="n"/>
+      <c r="T54" s="30" t="n"/>
+      <c r="U54" s="30" t="n"/>
+      <c r="V54" s="30" t="n"/>
+      <c r="W54" s="30" t="n"/>
+      <c r="X54" s="30" t="n"/>
       <c r="AN54" s="20" t="inlineStr">
         <is>
           <t>250UB37.3</t>
@@ -3910,20 +4351,20 @@
           <t>Mech. unit on platform (example)</t>
         </is>
       </c>
-      <c r="E55" s="58" t="n">
+      <c r="E55" s="60" t="n">
         <v>1.5</v>
       </c>
-      <c r="F55" s="59" t="n">
+      <c r="F55" s="30" t="n">
         <v>0.5</v>
       </c>
-      <c r="G55" s="59" t="n">
+      <c r="G55" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="H55" s="45" t="n">
+      <c r="H55" s="47" t="n">
         <v>4150</v>
       </c>
-      <c r="I55" s="45" t="n"/>
-      <c r="J55" s="60">
+      <c r="I55" s="47" t="n"/>
+      <c r="J55" s="61">
         <f>IF(B55="","",N(E55)*N(F55)+N(G55))</f>
         <v/>
       </c>
@@ -3937,12 +4378,12 @@
       <c r="B56" s="2" t="n"/>
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="5" t="n"/>
-      <c r="E56" s="58" t="n"/>
-      <c r="F56" s="59" t="n"/>
-      <c r="G56" s="59" t="n"/>
-      <c r="H56" s="45" t="n"/>
-      <c r="I56" s="45" t="n"/>
-      <c r="J56" s="60">
+      <c r="E56" s="60" t="n"/>
+      <c r="F56" s="30" t="n"/>
+      <c r="G56" s="30" t="n"/>
+      <c r="H56" s="47" t="n"/>
+      <c r="I56" s="47" t="n"/>
+      <c r="J56" s="61">
         <f>IF(B56="","",N(E56)*N(F56)+N(G56))</f>
         <v/>
       </c>
@@ -3951,7 +4392,7 @@
           <t>Active uplift (bottom flange) combinations:</t>
         </is>
       </c>
-      <c r="S56" s="47">
+      <c r="S56" s="49">
         <f>COUNTIFS(CombLib_B1[Active],1,CombLib_B1[Crit. flange],"Bottom")</f>
         <v/>
       </c>
@@ -3965,12 +4406,12 @@
       <c r="B57" s="2" t="n"/>
       <c r="C57" s="2" t="n"/>
       <c r="D57" s="5" t="n"/>
-      <c r="E57" s="58" t="n"/>
-      <c r="F57" s="59" t="n"/>
-      <c r="G57" s="59" t="n"/>
-      <c r="H57" s="45" t="n"/>
-      <c r="I57" s="45" t="n"/>
-      <c r="J57" s="60">
+      <c r="E57" s="60" t="n"/>
+      <c r="F57" s="30" t="n"/>
+      <c r="G57" s="30" t="n"/>
+      <c r="H57" s="47" t="n"/>
+      <c r="I57" s="47" t="n"/>
+      <c r="J57" s="61">
         <f>IF(B57="","",N(E57)*N(F57)+N(G57))</f>
         <v/>
       </c>
@@ -3988,32 +4429,32 @@
       </c>
     </row>
     <row r="59" ht="14" customHeight="1">
-      <c r="E59" s="48" t="inlineStr">
+      <c r="E59" s="50" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="F59" s="48" t="inlineStr">
+      <c r="F59" s="50" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="G59" s="48" t="inlineStr">
+      <c r="G59" s="50" t="inlineStr">
         <is>
           <t>Wd</t>
         </is>
       </c>
-      <c r="H59" s="48" t="inlineStr">
+      <c r="H59" s="50" t="inlineStr">
         <is>
           <t>Wu</t>
         </is>
       </c>
-      <c r="I59" s="48" t="inlineStr">
+      <c r="I59" s="50" t="inlineStr">
         <is>
           <t>Wid</t>
         </is>
       </c>
-      <c r="J59" s="48" t="inlineStr">
+      <c r="J59" s="50" t="inlineStr">
         <is>
           <t>Wiu</t>
         </is>
@@ -4025,32 +4466,32 @@
       </c>
     </row>
     <row r="60" ht="14" customHeight="1">
-      <c r="B60" s="41" t="inlineStr">
+      <c r="B60" s="43" t="inlineStr">
         <is>
           <t>Full-span UDL totals (excl. self-weight):</t>
         </is>
       </c>
-      <c r="E60" s="60">
+      <c r="E60" s="61">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"G",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-      <c r="F60" s="60">
+      <c r="F60" s="61">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"Q",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-      <c r="G60" s="60">
+      <c r="G60" s="61">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"Wd",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-      <c r="H60" s="60">
+      <c r="H60" s="61">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"Wu",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-      <c r="I60" s="60">
+      <c r="I60" s="61">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"Wid",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
-      <c r="J60" s="60">
+      <c r="J60" s="61">
         <f>SUMIFS(Loads_B1[Load],Loads_B1[Case],"Wiu",Loads_B1[Type],"UDL")</f>
         <v/>
       </c>
@@ -4088,7 +4529,7 @@
       </c>
     </row>
     <row r="63" ht="14" customHeight="1">
-      <c r="B63" s="40" t="inlineStr">
+      <c r="B63" s="42" t="inlineStr">
         <is>
           <t>Combination set</t>
         </is>
@@ -4098,12 +4539,12 @@
           <t>Roof</t>
         </is>
       </c>
-      <c r="F63" s="42" t="inlineStr">
+      <c r="F63" s="44" t="inlineStr">
         <is>
           <t>ψc</t>
         </is>
       </c>
-      <c r="G63" s="52" t="n">
+      <c r="G63" s="54" t="n">
         <v>0.4</v>
       </c>
       <c r="H63" s="6" t="inlineStr">
@@ -4130,47 +4571,47 @@
       </c>
     </row>
     <row r="65" ht="14" customHeight="1">
-      <c r="B65" s="29" t="inlineStr">
+      <c r="B65" s="25" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C65" s="29" t="inlineStr">
+      <c r="C65" s="25" t="inlineStr">
         <is>
           <t>Crit. flange</t>
         </is>
       </c>
-      <c r="D65" s="29" t="inlineStr">
+      <c r="D65" s="25" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="E65" s="29" t="inlineStr">
+      <c r="E65" s="25" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="F65" s="29" t="inlineStr">
+      <c r="F65" s="25" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="G65" s="29" t="inlineStr">
+      <c r="G65" s="25" t="inlineStr">
         <is>
           <t>Wd</t>
         </is>
       </c>
-      <c r="H65" s="29" t="inlineStr">
+      <c r="H65" s="25" t="inlineStr">
         <is>
           <t>Wu</t>
         </is>
       </c>
-      <c r="I65" s="29" t="inlineStr">
+      <c r="I65" s="25" t="inlineStr">
         <is>
           <t>Wid</t>
         </is>
       </c>
-      <c r="J65" s="29" t="inlineStr">
+      <c r="J65" s="25" t="inlineStr">
         <is>
           <t>Wiu</t>
         </is>
@@ -4182,18 +4623,18 @@
       </c>
     </row>
     <row r="66" ht="14" customHeight="1">
-      <c r="B66" s="32" cm="1">
+      <c r="B66" s="34" cm="1">
         <f t="array" ref="B66">_xlfn._xlws.FILTER(CombLib_B1[[ID]:[Wiu]],CombLib_B1[Active]=1,"No combinations selected")</f>
         <v/>
       </c>
-      <c r="C66" s="32" t="n"/>
-      <c r="D66" s="40" t="n"/>
-      <c r="E66" s="62" t="n"/>
-      <c r="F66" s="62" t="n"/>
-      <c r="G66" s="62" t="n"/>
-      <c r="H66" s="62" t="n"/>
-      <c r="I66" s="62" t="n"/>
-      <c r="J66" s="62" t="n"/>
+      <c r="C66" s="34" t="n"/>
+      <c r="D66" s="42" t="n"/>
+      <c r="E66" s="63" t="n"/>
+      <c r="F66" s="63" t="n"/>
+      <c r="G66" s="63" t="n"/>
+      <c r="H66" s="63" t="n"/>
+      <c r="I66" s="63" t="n"/>
+      <c r="J66" s="63" t="n"/>
       <c r="AN66" s="20" t="inlineStr">
         <is>
           <t>380PFC</t>
@@ -4201,15 +4642,15 @@
       </c>
     </row>
     <row r="67" ht="14" customHeight="1">
-      <c r="B67" s="32" t="n"/>
-      <c r="C67" s="32" t="n"/>
-      <c r="D67" s="40" t="n"/>
-      <c r="E67" s="62" t="n"/>
-      <c r="F67" s="62" t="n"/>
-      <c r="G67" s="62" t="n"/>
-      <c r="H67" s="62" t="n"/>
-      <c r="I67" s="62" t="n"/>
-      <c r="J67" s="62" t="n"/>
+      <c r="B67" s="34" t="n"/>
+      <c r="C67" s="34" t="n"/>
+      <c r="D67" s="42" t="n"/>
+      <c r="E67" s="63" t="n"/>
+      <c r="F67" s="63" t="n"/>
+      <c r="G67" s="63" t="n"/>
+      <c r="H67" s="63" t="n"/>
+      <c r="I67" s="63" t="n"/>
+      <c r="J67" s="63" t="n"/>
       <c r="AN67" s="20" t="inlineStr">
         <is>
           <t>300PFC</t>
@@ -4217,15 +4658,15 @@
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
-      <c r="B68" s="32" t="n"/>
-      <c r="C68" s="32" t="n"/>
-      <c r="D68" s="40" t="n"/>
-      <c r="E68" s="62" t="n"/>
-      <c r="F68" s="62" t="n"/>
-      <c r="G68" s="62" t="n"/>
-      <c r="H68" s="62" t="n"/>
-      <c r="I68" s="62" t="n"/>
-      <c r="J68" s="62" t="n"/>
+      <c r="B68" s="34" t="n"/>
+      <c r="C68" s="34" t="n"/>
+      <c r="D68" s="42" t="n"/>
+      <c r="E68" s="63" t="n"/>
+      <c r="F68" s="63" t="n"/>
+      <c r="G68" s="63" t="n"/>
+      <c r="H68" s="63" t="n"/>
+      <c r="I68" s="63" t="n"/>
+      <c r="J68" s="63" t="n"/>
       <c r="AN68" s="20" t="inlineStr">
         <is>
           <t>250PFC</t>
@@ -4233,15 +4674,15 @@
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
-      <c r="B69" s="32" t="n"/>
-      <c r="C69" s="32" t="n"/>
-      <c r="D69" s="40" t="n"/>
-      <c r="E69" s="62" t="n"/>
-      <c r="F69" s="62" t="n"/>
-      <c r="G69" s="62" t="n"/>
-      <c r="H69" s="62" t="n"/>
-      <c r="I69" s="62" t="n"/>
-      <c r="J69" s="62" t="n"/>
+      <c r="B69" s="34" t="n"/>
+      <c r="C69" s="34" t="n"/>
+      <c r="D69" s="42" t="n"/>
+      <c r="E69" s="63" t="n"/>
+      <c r="F69" s="63" t="n"/>
+      <c r="G69" s="63" t="n"/>
+      <c r="H69" s="63" t="n"/>
+      <c r="I69" s="63" t="n"/>
+      <c r="J69" s="63" t="n"/>
       <c r="AN69" s="20" t="inlineStr">
         <is>
           <t>230PFC</t>
@@ -4249,15 +4690,15 @@
       </c>
     </row>
     <row r="70" ht="14" customHeight="1">
-      <c r="B70" s="32" t="n"/>
-      <c r="C70" s="32" t="n"/>
-      <c r="D70" s="40" t="n"/>
-      <c r="E70" s="62" t="n"/>
-      <c r="F70" s="62" t="n"/>
-      <c r="G70" s="62" t="n"/>
-      <c r="H70" s="62" t="n"/>
-      <c r="I70" s="62" t="n"/>
-      <c r="J70" s="62" t="n"/>
+      <c r="B70" s="34" t="n"/>
+      <c r="C70" s="34" t="n"/>
+      <c r="D70" s="42" t="n"/>
+      <c r="E70" s="63" t="n"/>
+      <c r="F70" s="63" t="n"/>
+      <c r="G70" s="63" t="n"/>
+      <c r="H70" s="63" t="n"/>
+      <c r="I70" s="63" t="n"/>
+      <c r="J70" s="63" t="n"/>
       <c r="AN70" s="20" t="inlineStr">
         <is>
           <t>200PFC</t>
@@ -4265,15 +4706,15 @@
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
-      <c r="B71" s="32" t="n"/>
-      <c r="C71" s="32" t="n"/>
-      <c r="D71" s="40" t="n"/>
-      <c r="E71" s="62" t="n"/>
-      <c r="F71" s="62" t="n"/>
-      <c r="G71" s="62" t="n"/>
-      <c r="H71" s="62" t="n"/>
-      <c r="I71" s="62" t="n"/>
-      <c r="J71" s="62" t="n"/>
+      <c r="B71" s="34" t="n"/>
+      <c r="C71" s="34" t="n"/>
+      <c r="D71" s="42" t="n"/>
+      <c r="E71" s="63" t="n"/>
+      <c r="F71" s="63" t="n"/>
+      <c r="G71" s="63" t="n"/>
+      <c r="H71" s="63" t="n"/>
+      <c r="I71" s="63" t="n"/>
+      <c r="J71" s="63" t="n"/>
       <c r="AN71" s="20" t="inlineStr">
         <is>
           <t>180PFC</t>
@@ -4281,15 +4722,15 @@
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
-      <c r="B72" s="32" t="n"/>
-      <c r="C72" s="32" t="n"/>
-      <c r="D72" s="40" t="n"/>
-      <c r="E72" s="62" t="n"/>
-      <c r="F72" s="62" t="n"/>
-      <c r="G72" s="62" t="n"/>
-      <c r="H72" s="62" t="n"/>
-      <c r="I72" s="62" t="n"/>
-      <c r="J72" s="62" t="n"/>
+      <c r="B72" s="34" t="n"/>
+      <c r="C72" s="34" t="n"/>
+      <c r="D72" s="42" t="n"/>
+      <c r="E72" s="63" t="n"/>
+      <c r="F72" s="63" t="n"/>
+      <c r="G72" s="63" t="n"/>
+      <c r="H72" s="63" t="n"/>
+      <c r="I72" s="63" t="n"/>
+      <c r="J72" s="63" t="n"/>
       <c r="AN72" s="20" t="inlineStr">
         <is>
           <t>150PFC</t>
@@ -4297,15 +4738,15 @@
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
-      <c r="B73" s="32" t="n"/>
-      <c r="C73" s="32" t="n"/>
-      <c r="D73" s="40" t="n"/>
-      <c r="E73" s="62" t="n"/>
-      <c r="F73" s="62" t="n"/>
-      <c r="G73" s="62" t="n"/>
-      <c r="H73" s="62" t="n"/>
-      <c r="I73" s="62" t="n"/>
-      <c r="J73" s="62" t="n"/>
+      <c r="B73" s="34" t="n"/>
+      <c r="C73" s="34" t="n"/>
+      <c r="D73" s="42" t="n"/>
+      <c r="E73" s="63" t="n"/>
+      <c r="F73" s="63" t="n"/>
+      <c r="G73" s="63" t="n"/>
+      <c r="H73" s="63" t="n"/>
+      <c r="I73" s="63" t="n"/>
+      <c r="J73" s="63" t="n"/>
       <c r="AN73" s="20" t="inlineStr">
         <is>
           <t>125PFC</t>
@@ -4345,47 +4786,47 @@
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
-      <c r="B76" s="29" t="inlineStr">
+      <c r="B76" s="25" t="inlineStr">
         <is>
           <t>x (mm)</t>
         </is>
       </c>
-      <c r="C76" s="29" t="inlineStr">
+      <c r="C76" s="25" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
       </c>
-      <c r="D76" s="29" t="inlineStr">
+      <c r="D76" s="25" t="inlineStr">
         <is>
           <t>Restraint provided by</t>
         </is>
       </c>
-      <c r="E76" s="29" t="inlineStr">
+      <c r="E76" s="25" t="inlineStr">
         <is>
           <t>Top flange</t>
         </is>
       </c>
-      <c r="F76" s="29" t="inlineStr">
+      <c r="F76" s="25" t="inlineStr">
         <is>
           <t>Bottom fl.</t>
         </is>
       </c>
-      <c r="G76" s="29" t="inlineStr">
+      <c r="G76" s="25" t="inlineStr">
         <is>
           <t>αm override</t>
         </is>
       </c>
-      <c r="H76" s="29" t="inlineStr">
+      <c r="H76" s="25" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="I76" s="29" t="inlineStr">
+      <c r="I76" s="25" t="inlineStr">
         <is>
           <t>Top</t>
         </is>
       </c>
-      <c r="J76" s="29" t="inlineStr">
+      <c r="J76" s="25" t="inlineStr">
         <is>
           <t>Bottom</t>
         </is>
@@ -4397,7 +4838,7 @@
       </c>
     </row>
     <row r="77" ht="14" customHeight="1">
-      <c r="B77" s="63">
+      <c r="B77" s="64">
         <f>0</f>
         <v/>
       </c>
@@ -4421,16 +4862,16 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G77" s="59" t="n"/>
-      <c r="H77" s="32" t="inlineStr">
+      <c r="G77" s="30" t="n"/>
+      <c r="H77" s="34" t="inlineStr">
         <is>
           <t>kl</t>
         </is>
       </c>
-      <c r="I77" s="59" t="n">
+      <c r="I77" s="30" t="n">
         <v>1.4</v>
       </c>
-      <c r="J77" s="59" t="n">
+      <c r="J77" s="30" t="n">
         <v>1</v>
       </c>
       <c r="AN77" s="20" t="inlineStr">
@@ -4440,7 +4881,7 @@
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
-      <c r="B78" s="45" t="n">
+      <c r="B78" s="47" t="n">
         <v>2767</v>
       </c>
       <c r="C78" s="2" t="inlineStr"/>
@@ -4459,16 +4900,16 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G78" s="59" t="n"/>
-      <c r="H78" s="32" t="inlineStr">
+      <c r="G78" s="30" t="n"/>
+      <c r="H78" s="34" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="I78" s="59" t="n">
+      <c r="I78" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="J78" s="59" t="n">
+      <c r="J78" s="30" t="n">
         <v>1</v>
       </c>
       <c r="AN78" s="20" t="inlineStr">
@@ -4478,7 +4919,7 @@
       </c>
     </row>
     <row r="79" ht="14" customHeight="1">
-      <c r="B79" s="45" t="n">
+      <c r="B79" s="47" t="n">
         <v>5533</v>
       </c>
       <c r="C79" s="2" t="inlineStr"/>
@@ -4497,7 +4938,7 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G79" s="59" t="n"/>
+      <c r="G79" s="30" t="n"/>
       <c r="H79" s="15" t="inlineStr">
         <is>
           <t>kt from restraint</t>
@@ -4510,7 +4951,7 @@
       </c>
     </row>
     <row r="80" ht="14" customHeight="1">
-      <c r="B80" s="63">
+      <c r="B80" s="64">
         <f>Span</f>
         <v/>
       </c>
@@ -4534,7 +4975,7 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G80" s="59" t="n"/>
+      <c r="G80" s="30" t="n"/>
       <c r="H80" s="15" t="inlineStr">
         <is>
           <t>types (add-in)</t>
@@ -4547,12 +4988,12 @@
       </c>
     </row>
     <row r="81" ht="14" customHeight="1">
-      <c r="B81" s="45" t="n"/>
+      <c r="B81" s="47" t="n"/>
       <c r="C81" s="2" t="n"/>
       <c r="D81" s="5" t="n"/>
       <c r="E81" s="2" t="n"/>
       <c r="F81" s="2" t="n"/>
-      <c r="G81" s="59" t="n"/>
+      <c r="G81" s="30" t="n"/>
       <c r="AN81" s="20" t="inlineStr">
         <is>
           <t>250UC73</t>
@@ -4599,32 +5040,32 @@
       </c>
     </row>
     <row r="85" ht="14" customHeight="1">
-      <c r="B85" s="57" t="inlineStr">
+      <c r="B85" s="59" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C85" s="57" t="inlineStr">
+      <c r="C85" s="59" t="inlineStr">
         <is>
           <t>Δ max (mm)</t>
         </is>
       </c>
-      <c r="D85" s="57" t="inlineStr">
+      <c r="D85" s="59" t="inlineStr">
         <is>
           <t>at x (mm)</t>
         </is>
       </c>
-      <c r="E85" s="57" t="inlineStr">
+      <c r="E85" s="59" t="inlineStr">
         <is>
           <t>Limit (mm)</t>
         </is>
       </c>
-      <c r="F85" s="57" t="inlineStr">
+      <c r="F85" s="59" t="inlineStr">
         <is>
           <t>L / Δ</t>
         </is>
       </c>
-      <c r="G85" s="57" t="inlineStr">
+      <c r="G85" s="59" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
@@ -4636,15 +5077,15 @@
       </c>
     </row>
     <row r="86" ht="14" customHeight="1">
-      <c r="B86" s="32" cm="1">
+      <c r="B86" s="34" cm="1">
         <f t="array" ref="B86">OAR.SLS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],$E$37:$F$41,PsiL,PsiS)</f>
         <v/>
       </c>
-      <c r="C86" s="62" t="n"/>
-      <c r="D86" s="64" t="n"/>
-      <c r="E86" s="62" t="n"/>
-      <c r="F86" s="65" t="n"/>
-      <c r="G86" s="66" t="n"/>
+      <c r="C86" s="63" t="n"/>
+      <c r="D86" s="65" t="n"/>
+      <c r="E86" s="63" t="n"/>
+      <c r="F86" s="66" t="n"/>
+      <c r="G86" s="67" t="n"/>
       <c r="H86" s="6" t="inlineStr">
         <is>
           <t>Δ1kN: 1 kN at midspan,</t>
@@ -4657,12 +5098,12 @@
       </c>
     </row>
     <row r="87" ht="14" customHeight="1">
-      <c r="B87" s="32" t="n"/>
-      <c r="C87" s="62" t="n"/>
-      <c r="D87" s="64" t="n"/>
-      <c r="E87" s="62" t="n"/>
-      <c r="F87" s="65" t="n"/>
-      <c r="G87" s="66" t="n"/>
+      <c r="B87" s="34" t="n"/>
+      <c r="C87" s="63" t="n"/>
+      <c r="D87" s="65" t="n"/>
+      <c r="E87" s="63" t="n"/>
+      <c r="F87" s="66" t="n"/>
+      <c r="G87" s="67" t="n"/>
       <c r="H87" s="6" t="inlineStr">
         <is>
           <t>beam alone</t>
@@ -4675,12 +5116,12 @@
       </c>
     </row>
     <row r="88" ht="14" customHeight="1">
-      <c r="B88" s="32" t="n"/>
-      <c r="C88" s="62" t="n"/>
-      <c r="D88" s="64" t="n"/>
-      <c r="E88" s="62" t="n"/>
-      <c r="F88" s="65" t="n"/>
-      <c r="G88" s="66" t="n"/>
+      <c r="B88" s="34" t="n"/>
+      <c r="C88" s="63" t="n"/>
+      <c r="D88" s="65" t="n"/>
+      <c r="E88" s="63" t="n"/>
+      <c r="F88" s="66" t="n"/>
+      <c r="G88" s="67" t="n"/>
       <c r="AN88" s="20" t="inlineStr">
         <is>
           <t>100UC15</t>
@@ -4688,24 +5129,24 @@
       </c>
     </row>
     <row r="89" ht="14" customHeight="1">
-      <c r="B89" s="32" t="n"/>
-      <c r="C89" s="62" t="n"/>
-      <c r="D89" s="64" t="n"/>
-      <c r="E89" s="62" t="n"/>
-      <c r="F89" s="65" t="n"/>
-      <c r="G89" s="66" t="n"/>
+      <c r="B89" s="34" t="n"/>
+      <c r="C89" s="63" t="n"/>
+      <c r="D89" s="65" t="n"/>
+      <c r="E89" s="63" t="n"/>
+      <c r="F89" s="66" t="n"/>
+      <c r="G89" s="67" t="n"/>
     </row>
     <row r="90" ht="14" customHeight="1">
-      <c r="B90" s="32" t="n"/>
-      <c r="C90" s="62" t="n"/>
-      <c r="D90" s="64" t="n"/>
-      <c r="E90" s="62" t="n"/>
-      <c r="F90" s="65" t="n"/>
-      <c r="G90" s="66" t="n"/>
+      <c r="B90" s="34" t="n"/>
+      <c r="C90" s="63" t="n"/>
+      <c r="D90" s="65" t="n"/>
+      <c r="E90" s="63" t="n"/>
+      <c r="F90" s="66" t="n"/>
+      <c r="G90" s="67" t="n"/>
     </row>
     <row r="91" ht="14" customHeight="1"/>
     <row r="92" ht="14" customHeight="1">
-      <c r="B92" s="67" t="inlineStr">
+      <c r="B92" s="68" t="inlineStr">
         <is>
           <t>Deflected shapes (mm, plotted downward;  x in m)</t>
         </is>
@@ -4739,12 +5180,12 @@
       <c r="J105" s="11" t="n"/>
     </row>
     <row r="106" ht="14" customHeight="1">
-      <c r="B106" s="67" t="inlineStr">
+      <c r="B106" s="68" t="inlineStr">
         <is>
           <t>Bending moment envelope (kN·m, sagging down;  x in m)</t>
         </is>
       </c>
-      <c r="F106" s="67" t="inlineStr">
+      <c r="F106" s="68" t="inlineStr">
         <is>
           <t>Shear force envelope (kN;  x in m)</t>
         </is>
@@ -4765,230 +5206,230 @@
     <row r="119" ht="14" customHeight="1"/>
     <row r="120" ht="14" customHeight="1"/>
     <row r="121" ht="16" customHeight="1">
-      <c r="B121" s="57" t="inlineStr">
+      <c r="B121" s="59" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="C121" s="57" t="inlineStr">
+      <c r="C121" s="59" t="inlineStr">
         <is>
           <t>Segment (m)</t>
         </is>
       </c>
-      <c r="D121" s="57" t="inlineStr">
+      <c r="D121" s="59" t="inlineStr">
         <is>
           <t>Ends</t>
         </is>
       </c>
-      <c r="E121" s="57" t="inlineStr">
+      <c r="E121" s="59" t="inlineStr">
         <is>
           <t>Le (m)</t>
         </is>
       </c>
-      <c r="F121" s="57" t="inlineStr">
+      <c r="F121" s="59" t="inlineStr">
         <is>
           <t>αm</t>
         </is>
       </c>
-      <c r="G121" s="57" t="inlineStr">
+      <c r="G121" s="59" t="inlineStr">
         <is>
           <t>αs</t>
         </is>
       </c>
-      <c r="H121" s="57" t="inlineStr">
+      <c r="H121" s="59" t="inlineStr">
         <is>
           <t>φMb (kN·m)</t>
         </is>
       </c>
-      <c r="I121" s="57" t="inlineStr">
+      <c r="I121" s="59" t="inlineStr">
         <is>
           <t>M* (kN·m)</t>
         </is>
       </c>
-      <c r="J121" s="57" t="inlineStr">
+      <c r="J121" s="59" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
     </row>
     <row r="122" ht="14" customHeight="1">
-      <c r="B122" s="32" cm="1">
+      <c r="B122" s="34" cm="1">
         <f t="array" ref="B122">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
         <v/>
       </c>
-      <c r="C122" s="32" t="n"/>
-      <c r="D122" s="32" t="n"/>
-      <c r="E122" s="62" t="n"/>
-      <c r="F122" s="68" t="n"/>
-      <c r="G122" s="68" t="n"/>
-      <c r="H122" s="69" t="n"/>
-      <c r="I122" s="69" t="n"/>
-      <c r="J122" s="66" t="n"/>
+      <c r="C122" s="34" t="n"/>
+      <c r="D122" s="34" t="n"/>
+      <c r="E122" s="63" t="n"/>
+      <c r="F122" s="69" t="n"/>
+      <c r="G122" s="69" t="n"/>
+      <c r="H122" s="70" t="n"/>
+      <c r="I122" s="70" t="n"/>
+      <c r="J122" s="67" t="n"/>
     </row>
     <row r="123" ht="14" customHeight="1">
-      <c r="B123" s="32" t="n"/>
-      <c r="C123" s="32" t="n"/>
-      <c r="D123" s="32" t="n"/>
-      <c r="E123" s="62" t="n"/>
-      <c r="F123" s="68" t="n"/>
-      <c r="G123" s="68" t="n"/>
-      <c r="H123" s="69" t="n"/>
-      <c r="I123" s="69" t="n"/>
-      <c r="J123" s="66" t="n"/>
+      <c r="B123" s="34" t="n"/>
+      <c r="C123" s="34" t="n"/>
+      <c r="D123" s="34" t="n"/>
+      <c r="E123" s="63" t="n"/>
+      <c r="F123" s="69" t="n"/>
+      <c r="G123" s="69" t="n"/>
+      <c r="H123" s="70" t="n"/>
+      <c r="I123" s="70" t="n"/>
+      <c r="J123" s="67" t="n"/>
     </row>
     <row r="124" ht="14" customHeight="1">
-      <c r="B124" s="32" t="n"/>
-      <c r="C124" s="32" t="n"/>
-      <c r="D124" s="32" t="n"/>
-      <c r="E124" s="62" t="n"/>
-      <c r="F124" s="68" t="n"/>
-      <c r="G124" s="68" t="n"/>
-      <c r="H124" s="69" t="n"/>
-      <c r="I124" s="69" t="n"/>
-      <c r="J124" s="66" t="n"/>
+      <c r="B124" s="34" t="n"/>
+      <c r="C124" s="34" t="n"/>
+      <c r="D124" s="34" t="n"/>
+      <c r="E124" s="63" t="n"/>
+      <c r="F124" s="69" t="n"/>
+      <c r="G124" s="69" t="n"/>
+      <c r="H124" s="70" t="n"/>
+      <c r="I124" s="70" t="n"/>
+      <c r="J124" s="67" t="n"/>
     </row>
     <row r="125" ht="14" customHeight="1">
-      <c r="B125" s="32" t="n"/>
-      <c r="C125" s="32" t="n"/>
-      <c r="D125" s="32" t="n"/>
-      <c r="E125" s="62" t="n"/>
-      <c r="F125" s="68" t="n"/>
-      <c r="G125" s="68" t="n"/>
-      <c r="H125" s="69" t="n"/>
-      <c r="I125" s="69" t="n"/>
-      <c r="J125" s="66" t="n"/>
+      <c r="B125" s="34" t="n"/>
+      <c r="C125" s="34" t="n"/>
+      <c r="D125" s="34" t="n"/>
+      <c r="E125" s="63" t="n"/>
+      <c r="F125" s="69" t="n"/>
+      <c r="G125" s="69" t="n"/>
+      <c r="H125" s="70" t="n"/>
+      <c r="I125" s="70" t="n"/>
+      <c r="J125" s="67" t="n"/>
     </row>
     <row r="126" ht="14" customHeight="1">
-      <c r="B126" s="32" t="n"/>
-      <c r="C126" s="32" t="n"/>
-      <c r="D126" s="32" t="n"/>
-      <c r="E126" s="62" t="n"/>
-      <c r="F126" s="68" t="n"/>
-      <c r="G126" s="68" t="n"/>
-      <c r="H126" s="69" t="n"/>
-      <c r="I126" s="69" t="n"/>
-      <c r="J126" s="66" t="n"/>
+      <c r="B126" s="34" t="n"/>
+      <c r="C126" s="34" t="n"/>
+      <c r="D126" s="34" t="n"/>
+      <c r="E126" s="63" t="n"/>
+      <c r="F126" s="69" t="n"/>
+      <c r="G126" s="69" t="n"/>
+      <c r="H126" s="70" t="n"/>
+      <c r="I126" s="70" t="n"/>
+      <c r="J126" s="67" t="n"/>
     </row>
     <row r="127" ht="14" customHeight="1">
-      <c r="B127" s="32" t="n"/>
-      <c r="C127" s="32" t="n"/>
-      <c r="D127" s="32" t="n"/>
-      <c r="E127" s="62" t="n"/>
-      <c r="F127" s="68" t="n"/>
-      <c r="G127" s="68" t="n"/>
-      <c r="H127" s="69" t="n"/>
-      <c r="I127" s="69" t="n"/>
-      <c r="J127" s="66" t="n"/>
+      <c r="B127" s="34" t="n"/>
+      <c r="C127" s="34" t="n"/>
+      <c r="D127" s="34" t="n"/>
+      <c r="E127" s="63" t="n"/>
+      <c r="F127" s="69" t="n"/>
+      <c r="G127" s="69" t="n"/>
+      <c r="H127" s="70" t="n"/>
+      <c r="I127" s="70" t="n"/>
+      <c r="J127" s="67" t="n"/>
     </row>
     <row r="128" ht="14" customHeight="1">
-      <c r="B128" s="32" t="n"/>
-      <c r="C128" s="32" t="n"/>
-      <c r="D128" s="32" t="n"/>
-      <c r="E128" s="62" t="n"/>
-      <c r="F128" s="68" t="n"/>
-      <c r="G128" s="68" t="n"/>
-      <c r="H128" s="69" t="n"/>
-      <c r="I128" s="69" t="n"/>
-      <c r="J128" s="66" t="n"/>
+      <c r="B128" s="34" t="n"/>
+      <c r="C128" s="34" t="n"/>
+      <c r="D128" s="34" t="n"/>
+      <c r="E128" s="63" t="n"/>
+      <c r="F128" s="69" t="n"/>
+      <c r="G128" s="69" t="n"/>
+      <c r="H128" s="70" t="n"/>
+      <c r="I128" s="70" t="n"/>
+      <c r="J128" s="67" t="n"/>
     </row>
     <row r="129" ht="14" customHeight="1">
-      <c r="B129" s="32" t="n"/>
-      <c r="C129" s="32" t="n"/>
-      <c r="D129" s="32" t="n"/>
-      <c r="E129" s="62" t="n"/>
-      <c r="F129" s="68" t="n"/>
-      <c r="G129" s="68" t="n"/>
-      <c r="H129" s="69" t="n"/>
-      <c r="I129" s="69" t="n"/>
-      <c r="J129" s="66" t="n"/>
+      <c r="B129" s="34" t="n"/>
+      <c r="C129" s="34" t="n"/>
+      <c r="D129" s="34" t="n"/>
+      <c r="E129" s="63" t="n"/>
+      <c r="F129" s="69" t="n"/>
+      <c r="G129" s="69" t="n"/>
+      <c r="H129" s="70" t="n"/>
+      <c r="I129" s="70" t="n"/>
+      <c r="J129" s="67" t="n"/>
     </row>
     <row r="130" ht="14" customHeight="1">
-      <c r="B130" s="32" t="n"/>
-      <c r="C130" s="32" t="n"/>
-      <c r="D130" s="32" t="n"/>
-      <c r="E130" s="62" t="n"/>
-      <c r="F130" s="68" t="n"/>
-      <c r="G130" s="68" t="n"/>
-      <c r="H130" s="69" t="n"/>
-      <c r="I130" s="69" t="n"/>
-      <c r="J130" s="66" t="n"/>
+      <c r="B130" s="34" t="n"/>
+      <c r="C130" s="34" t="n"/>
+      <c r="D130" s="34" t="n"/>
+      <c r="E130" s="63" t="n"/>
+      <c r="F130" s="69" t="n"/>
+      <c r="G130" s="69" t="n"/>
+      <c r="H130" s="70" t="n"/>
+      <c r="I130" s="70" t="n"/>
+      <c r="J130" s="67" t="n"/>
     </row>
     <row r="131" ht="14" customHeight="1">
-      <c r="B131" s="32" t="n"/>
-      <c r="C131" s="32" t="n"/>
-      <c r="D131" s="32" t="n"/>
-      <c r="E131" s="62" t="n"/>
-      <c r="F131" s="68" t="n"/>
-      <c r="G131" s="68" t="n"/>
-      <c r="H131" s="69" t="n"/>
-      <c r="I131" s="69" t="n"/>
-      <c r="J131" s="66" t="n"/>
+      <c r="B131" s="34" t="n"/>
+      <c r="C131" s="34" t="n"/>
+      <c r="D131" s="34" t="n"/>
+      <c r="E131" s="63" t="n"/>
+      <c r="F131" s="69" t="n"/>
+      <c r="G131" s="69" t="n"/>
+      <c r="H131" s="70" t="n"/>
+      <c r="I131" s="70" t="n"/>
+      <c r="J131" s="67" t="n"/>
     </row>
     <row r="132" ht="14" customHeight="1">
-      <c r="B132" s="32" t="n"/>
-      <c r="C132" s="32" t="n"/>
-      <c r="D132" s="32" t="n"/>
-      <c r="E132" s="62" t="n"/>
-      <c r="F132" s="68" t="n"/>
-      <c r="G132" s="68" t="n"/>
-      <c r="H132" s="69" t="n"/>
-      <c r="I132" s="69" t="n"/>
-      <c r="J132" s="66" t="n"/>
+      <c r="B132" s="34" t="n"/>
+      <c r="C132" s="34" t="n"/>
+      <c r="D132" s="34" t="n"/>
+      <c r="E132" s="63" t="n"/>
+      <c r="F132" s="69" t="n"/>
+      <c r="G132" s="69" t="n"/>
+      <c r="H132" s="70" t="n"/>
+      <c r="I132" s="70" t="n"/>
+      <c r="J132" s="67" t="n"/>
     </row>
     <row r="133" ht="14" customHeight="1">
-      <c r="B133" s="32" t="n"/>
-      <c r="C133" s="32" t="n"/>
-      <c r="D133" s="32" t="n"/>
-      <c r="E133" s="62" t="n"/>
-      <c r="F133" s="68" t="n"/>
-      <c r="G133" s="68" t="n"/>
-      <c r="H133" s="69" t="n"/>
-      <c r="I133" s="69" t="n"/>
-      <c r="J133" s="66" t="n"/>
+      <c r="B133" s="34" t="n"/>
+      <c r="C133" s="34" t="n"/>
+      <c r="D133" s="34" t="n"/>
+      <c r="E133" s="63" t="n"/>
+      <c r="F133" s="69" t="n"/>
+      <c r="G133" s="69" t="n"/>
+      <c r="H133" s="70" t="n"/>
+      <c r="I133" s="70" t="n"/>
+      <c r="J133" s="67" t="n"/>
     </row>
     <row r="134" ht="14" customHeight="1">
-      <c r="B134" s="32" t="n"/>
-      <c r="C134" s="32" t="n"/>
-      <c r="D134" s="32" t="n"/>
-      <c r="E134" s="62" t="n"/>
-      <c r="F134" s="68" t="n"/>
-      <c r="G134" s="68" t="n"/>
-      <c r="H134" s="69" t="n"/>
-      <c r="I134" s="69" t="n"/>
-      <c r="J134" s="66" t="n"/>
+      <c r="B134" s="34" t="n"/>
+      <c r="C134" s="34" t="n"/>
+      <c r="D134" s="34" t="n"/>
+      <c r="E134" s="63" t="n"/>
+      <c r="F134" s="69" t="n"/>
+      <c r="G134" s="69" t="n"/>
+      <c r="H134" s="70" t="n"/>
+      <c r="I134" s="70" t="n"/>
+      <c r="J134" s="67" t="n"/>
     </row>
     <row r="135" ht="14" customHeight="1">
-      <c r="B135" s="32" t="n"/>
-      <c r="C135" s="32" t="n"/>
-      <c r="D135" s="32" t="n"/>
-      <c r="E135" s="62" t="n"/>
-      <c r="F135" s="68" t="n"/>
-      <c r="G135" s="68" t="n"/>
-      <c r="H135" s="69" t="n"/>
-      <c r="I135" s="69" t="n"/>
-      <c r="J135" s="66" t="n"/>
+      <c r="B135" s="34" t="n"/>
+      <c r="C135" s="34" t="n"/>
+      <c r="D135" s="34" t="n"/>
+      <c r="E135" s="63" t="n"/>
+      <c r="F135" s="69" t="n"/>
+      <c r="G135" s="69" t="n"/>
+      <c r="H135" s="70" t="n"/>
+      <c r="I135" s="70" t="n"/>
+      <c r="J135" s="67" t="n"/>
     </row>
     <row r="136" ht="14" customHeight="1">
-      <c r="B136" s="32" t="n"/>
-      <c r="C136" s="32" t="n"/>
-      <c r="D136" s="32" t="n"/>
-      <c r="E136" s="62" t="n"/>
-      <c r="F136" s="68" t="n"/>
-      <c r="G136" s="68" t="n"/>
-      <c r="H136" s="69" t="n"/>
-      <c r="I136" s="69" t="n"/>
-      <c r="J136" s="66" t="n"/>
+      <c r="B136" s="34" t="n"/>
+      <c r="C136" s="34" t="n"/>
+      <c r="D136" s="34" t="n"/>
+      <c r="E136" s="63" t="n"/>
+      <c r="F136" s="69" t="n"/>
+      <c r="G136" s="69" t="n"/>
+      <c r="H136" s="70" t="n"/>
+      <c r="I136" s="70" t="n"/>
+      <c r="J136" s="67" t="n"/>
     </row>
     <row r="137" ht="14" customHeight="1">
-      <c r="B137" s="32" t="n"/>
-      <c r="C137" s="32" t="n"/>
-      <c r="D137" s="32" t="n"/>
-      <c r="E137" s="62" t="n"/>
-      <c r="F137" s="68" t="n"/>
-      <c r="G137" s="68" t="n"/>
-      <c r="H137" s="69" t="n"/>
-      <c r="I137" s="69" t="n"/>
-      <c r="J137" s="66" t="n"/>
+      <c r="B137" s="34" t="n"/>
+      <c r="C137" s="34" t="n"/>
+      <c r="D137" s="34" t="n"/>
+      <c r="E137" s="63" t="n"/>
+      <c r="F137" s="69" t="n"/>
+      <c r="G137" s="69" t="n"/>
+      <c r="H137" s="70" t="n"/>
+      <c r="I137" s="70" t="n"/>
+      <c r="J137" s="67" t="n"/>
     </row>
     <row r="138" ht="14" customHeight="1">
       <c r="B138" s="15" t="inlineStr">
@@ -5021,117 +5462,117 @@
       </c>
     </row>
     <row r="142">
-      <c r="D142" s="70" cm="1">
+      <c r="D142" s="71" cm="1">
         <f t="array" ref="D142">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
         <v/>
       </c>
-      <c r="E142" s="71" t="n"/>
-      <c r="F142" s="33" t="n"/>
+      <c r="E142" s="72" t="n"/>
+      <c r="F142" s="35" t="n"/>
     </row>
     <row r="143">
-      <c r="D143" s="70" t="n"/>
-      <c r="E143" s="71" t="n"/>
-      <c r="F143" s="33" t="n"/>
+      <c r="D143" s="71" t="n"/>
+      <c r="E143" s="72" t="n"/>
+      <c r="F143" s="35" t="n"/>
     </row>
     <row r="144">
-      <c r="D144" s="70" t="n"/>
-      <c r="E144" s="71" t="n"/>
-      <c r="F144" s="33" t="n"/>
+      <c r="D144" s="71" t="n"/>
+      <c r="E144" s="72" t="n"/>
+      <c r="F144" s="35" t="n"/>
     </row>
     <row r="145">
-      <c r="D145" s="70" t="n"/>
-      <c r="E145" s="71" t="n"/>
-      <c r="F145" s="33" t="n"/>
+      <c r="D145" s="71" t="n"/>
+      <c r="E145" s="72" t="n"/>
+      <c r="F145" s="35" t="n"/>
     </row>
     <row r="146">
-      <c r="D146" s="70" t="n"/>
-      <c r="E146" s="71" t="n"/>
-      <c r="F146" s="33" t="n"/>
+      <c r="D146" s="71" t="n"/>
+      <c r="E146" s="72" t="n"/>
+      <c r="F146" s="35" t="n"/>
     </row>
     <row r="147">
-      <c r="D147" s="70" t="n"/>
-      <c r="E147" s="71" t="n"/>
-      <c r="F147" s="33" t="n"/>
+      <c r="D147" s="71" t="n"/>
+      <c r="E147" s="72" t="n"/>
+      <c r="F147" s="35" t="n"/>
     </row>
     <row r="148">
-      <c r="D148" s="70" t="n"/>
-      <c r="E148" s="71" t="n"/>
-      <c r="F148" s="33" t="n"/>
+      <c r="D148" s="71" t="n"/>
+      <c r="E148" s="72" t="n"/>
+      <c r="F148" s="35" t="n"/>
     </row>
     <row r="149">
-      <c r="D149" s="70" t="n"/>
-      <c r="E149" s="71" t="n"/>
-      <c r="F149" s="33" t="n"/>
+      <c r="D149" s="71" t="n"/>
+      <c r="E149" s="72" t="n"/>
+      <c r="F149" s="35" t="n"/>
     </row>
     <row r="150">
-      <c r="D150" s="70" t="n"/>
-      <c r="E150" s="71" t="n"/>
-      <c r="F150" s="33" t="n"/>
+      <c r="D150" s="71" t="n"/>
+      <c r="E150" s="72" t="n"/>
+      <c r="F150" s="35" t="n"/>
     </row>
     <row r="151">
-      <c r="D151" s="70" t="n"/>
-      <c r="E151" s="71" t="n"/>
-      <c r="F151" s="33" t="n"/>
+      <c r="D151" s="71" t="n"/>
+      <c r="E151" s="72" t="n"/>
+      <c r="F151" s="35" t="n"/>
     </row>
     <row r="152">
-      <c r="D152" s="70" t="n"/>
-      <c r="E152" s="71" t="n"/>
-      <c r="F152" s="33" t="n"/>
+      <c r="D152" s="71" t="n"/>
+      <c r="E152" s="72" t="n"/>
+      <c r="F152" s="35" t="n"/>
     </row>
     <row r="153">
-      <c r="D153" s="70" t="n"/>
-      <c r="E153" s="71" t="n"/>
-      <c r="F153" s="33" t="n"/>
+      <c r="D153" s="71" t="n"/>
+      <c r="E153" s="72" t="n"/>
+      <c r="F153" s="35" t="n"/>
     </row>
     <row r="154">
-      <c r="D154" s="70" t="n"/>
-      <c r="E154" s="71" t="n"/>
-      <c r="F154" s="33" t="n"/>
+      <c r="D154" s="71" t="n"/>
+      <c r="E154" s="72" t="n"/>
+      <c r="F154" s="35" t="n"/>
     </row>
     <row r="155">
-      <c r="D155" s="70" t="n"/>
-      <c r="E155" s="71" t="n"/>
-      <c r="F155" s="33" t="n"/>
+      <c r="D155" s="71" t="n"/>
+      <c r="E155" s="72" t="n"/>
+      <c r="F155" s="35" t="n"/>
     </row>
     <row r="156">
-      <c r="D156" s="70" t="n"/>
-      <c r="E156" s="71" t="n"/>
-      <c r="F156" s="33" t="n"/>
+      <c r="D156" s="71" t="n"/>
+      <c r="E156" s="72" t="n"/>
+      <c r="F156" s="35" t="n"/>
     </row>
     <row r="157">
-      <c r="D157" s="70" t="n"/>
-      <c r="E157" s="71" t="n"/>
-      <c r="F157" s="33" t="n"/>
+      <c r="D157" s="71" t="n"/>
+      <c r="E157" s="72" t="n"/>
+      <c r="F157" s="35" t="n"/>
     </row>
     <row r="158">
-      <c r="D158" s="70" t="n"/>
-      <c r="E158" s="71" t="n"/>
-      <c r="F158" s="33" t="n"/>
+      <c r="D158" s="71" t="n"/>
+      <c r="E158" s="72" t="n"/>
+      <c r="F158" s="35" t="n"/>
     </row>
     <row r="159">
-      <c r="D159" s="70" t="n"/>
-      <c r="E159" s="71" t="n"/>
-      <c r="F159" s="33" t="n"/>
+      <c r="D159" s="71" t="n"/>
+      <c r="E159" s="72" t="n"/>
+      <c r="F159" s="35" t="n"/>
     </row>
     <row r="160">
-      <c r="D160" s="70" t="n"/>
-      <c r="E160" s="71" t="n"/>
-      <c r="F160" s="33" t="n"/>
+      <c r="D160" s="71" t="n"/>
+      <c r="E160" s="72" t="n"/>
+      <c r="F160" s="35" t="n"/>
     </row>
     <row r="161">
-      <c r="D161" s="70" t="n"/>
-      <c r="E161" s="71" t="n"/>
-      <c r="F161" s="33" t="n"/>
+      <c r="D161" s="71" t="n"/>
+      <c r="E161" s="72" t="n"/>
+      <c r="F161" s="35" t="n"/>
     </row>
     <row r="162">
-      <c r="D162" s="70" t="n"/>
-      <c r="E162" s="71" t="n"/>
-      <c r="F162" s="33" t="n"/>
+      <c r="D162" s="71" t="n"/>
+      <c r="E162" s="72" t="n"/>
+      <c r="F162" s="35" t="n"/>
     </row>
     <row r="163">
-      <c r="D163" s="70" t="n"/>
-      <c r="E163" s="71" t="n"/>
-      <c r="F163" s="33" t="n"/>
+      <c r="D163" s="71" t="n"/>
+      <c r="E163" s="72" t="n"/>
+      <c r="F163" s="35" t="n"/>
     </row>
     <row r="165" ht="20" customHeight="1">
       <c r="B165" s="10" t="inlineStr">
@@ -5149,103 +5590,103 @@
       <c r="J165" s="11" t="n"/>
     </row>
     <row r="166">
-      <c r="B166" s="57" t="inlineStr">
+      <c r="B166" s="59" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="C166" s="57" t="inlineStr">
+      <c r="C166" s="59" t="inlineStr">
         <is>
           <t>V* (kN)</t>
         </is>
       </c>
-      <c r="D166" s="57" t="inlineStr">
+      <c r="D166" s="59" t="inlineStr">
         <is>
           <t>at x (m)</t>
         </is>
       </c>
-      <c r="E166" s="57" t="inlineStr">
+      <c r="E166" s="59" t="inlineStr">
         <is>
           <t>φVv (kN)</t>
         </is>
       </c>
-      <c r="F166" s="57" t="inlineStr">
+      <c r="F166" s="59" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
-      <c r="G166" s="57" t="inlineStr">
+      <c r="G166" s="59" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="B167" s="32" cm="1">
+      <c r="B167" s="34" cm="1">
         <f t="array" ref="B167">OAR.SHEAR(SectionSize,Grade,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
         <v/>
       </c>
-      <c r="C167" s="69" t="n"/>
-      <c r="D167" s="62" t="n"/>
-      <c r="E167" s="69" t="n"/>
-      <c r="F167" s="66" t="n"/>
-      <c r="G167" s="72" t="n"/>
+      <c r="C167" s="70" t="n"/>
+      <c r="D167" s="63" t="n"/>
+      <c r="E167" s="70" t="n"/>
+      <c r="F167" s="67" t="n"/>
+      <c r="G167" s="73" t="n"/>
     </row>
     <row r="168">
-      <c r="B168" s="32" t="n"/>
-      <c r="C168" s="69" t="n"/>
-      <c r="D168" s="62" t="n"/>
-      <c r="E168" s="69" t="n"/>
-      <c r="F168" s="66" t="n"/>
-      <c r="G168" s="72" t="n"/>
+      <c r="B168" s="34" t="n"/>
+      <c r="C168" s="70" t="n"/>
+      <c r="D168" s="63" t="n"/>
+      <c r="E168" s="70" t="n"/>
+      <c r="F168" s="67" t="n"/>
+      <c r="G168" s="73" t="n"/>
     </row>
     <row r="169">
-      <c r="B169" s="32" t="n"/>
-      <c r="C169" s="69" t="n"/>
-      <c r="D169" s="62" t="n"/>
-      <c r="E169" s="69" t="n"/>
-      <c r="F169" s="66" t="n"/>
-      <c r="G169" s="72" t="n"/>
+      <c r="B169" s="34" t="n"/>
+      <c r="C169" s="70" t="n"/>
+      <c r="D169" s="63" t="n"/>
+      <c r="E169" s="70" t="n"/>
+      <c r="F169" s="67" t="n"/>
+      <c r="G169" s="73" t="n"/>
     </row>
     <row r="170">
-      <c r="B170" s="32" t="n"/>
-      <c r="C170" s="69" t="n"/>
-      <c r="D170" s="62" t="n"/>
-      <c r="E170" s="69" t="n"/>
-      <c r="F170" s="66" t="n"/>
-      <c r="G170" s="72" t="n"/>
+      <c r="B170" s="34" t="n"/>
+      <c r="C170" s="70" t="n"/>
+      <c r="D170" s="63" t="n"/>
+      <c r="E170" s="70" t="n"/>
+      <c r="F170" s="67" t="n"/>
+      <c r="G170" s="73" t="n"/>
     </row>
     <row r="171">
-      <c r="B171" s="32" t="n"/>
-      <c r="C171" s="69" t="n"/>
-      <c r="D171" s="62" t="n"/>
-      <c r="E171" s="69" t="n"/>
-      <c r="F171" s="66" t="n"/>
-      <c r="G171" s="72" t="n"/>
+      <c r="B171" s="34" t="n"/>
+      <c r="C171" s="70" t="n"/>
+      <c r="D171" s="63" t="n"/>
+      <c r="E171" s="70" t="n"/>
+      <c r="F171" s="67" t="n"/>
+      <c r="G171" s="73" t="n"/>
     </row>
     <row r="172">
-      <c r="B172" s="32" t="n"/>
-      <c r="C172" s="69" t="n"/>
-      <c r="D172" s="62" t="n"/>
-      <c r="E172" s="69" t="n"/>
-      <c r="F172" s="66" t="n"/>
-      <c r="G172" s="72" t="n"/>
+      <c r="B172" s="34" t="n"/>
+      <c r="C172" s="70" t="n"/>
+      <c r="D172" s="63" t="n"/>
+      <c r="E172" s="70" t="n"/>
+      <c r="F172" s="67" t="n"/>
+      <c r="G172" s="73" t="n"/>
     </row>
     <row r="173">
-      <c r="B173" s="32" t="n"/>
-      <c r="C173" s="69" t="n"/>
-      <c r="D173" s="62" t="n"/>
-      <c r="E173" s="69" t="n"/>
-      <c r="F173" s="66" t="n"/>
-      <c r="G173" s="72" t="n"/>
+      <c r="B173" s="34" t="n"/>
+      <c r="C173" s="70" t="n"/>
+      <c r="D173" s="63" t="n"/>
+      <c r="E173" s="70" t="n"/>
+      <c r="F173" s="67" t="n"/>
+      <c r="G173" s="73" t="n"/>
     </row>
     <row r="174">
-      <c r="B174" s="32" t="n"/>
-      <c r="C174" s="69" t="n"/>
-      <c r="D174" s="62" t="n"/>
-      <c r="E174" s="69" t="n"/>
-      <c r="F174" s="66" t="n"/>
-      <c r="G174" s="72" t="n"/>
+      <c r="B174" s="34" t="n"/>
+      <c r="C174" s="70" t="n"/>
+      <c r="D174" s="63" t="n"/>
+      <c r="E174" s="70" t="n"/>
+      <c r="F174" s="67" t="n"/>
+      <c r="G174" s="73" t="n"/>
     </row>
     <row r="176" ht="20" customHeight="1">
       <c r="B176" s="10" t="inlineStr">
@@ -5270,39 +5711,39 @@
       </c>
     </row>
     <row r="178">
-      <c r="B178" s="29" t="inlineStr">
+      <c r="B178" s="25" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="D178" s="29" t="inlineStr">
+      <c r="D178" s="25" t="inlineStr">
         <is>
           <t>Left (kN)</t>
         </is>
       </c>
-      <c r="E178" s="29" t="inlineStr">
+      <c r="E178" s="25" t="inlineStr">
         <is>
           <t>Right (kN)</t>
         </is>
       </c>
-      <c r="F178" s="29" t="inlineStr">
+      <c r="F178" s="25" t="inlineStr">
         <is>
           <t>Transfer names</t>
         </is>
       </c>
     </row>
     <row r="179">
-      <c r="B179" s="49" t="inlineStr">
+      <c r="B179" s="51" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="C179" s="50" t="n"/>
-      <c r="D179" s="34" cm="1">
+      <c r="C179" s="52" t="n"/>
+      <c r="D179" s="36" cm="1">
         <f t="array" ref="D179">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,2)</f>
         <v/>
       </c>
-      <c r="E179" s="34" cm="1">
+      <c r="E179" s="36" cm="1">
         <f t="array" ref="E179">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,3)</f>
         <v/>
       </c>
@@ -5313,17 +5754,17 @@
       </c>
     </row>
     <row r="180">
-      <c r="B180" s="49" t="inlineStr">
+      <c r="B180" s="51" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C180" s="50" t="n"/>
-      <c r="D180" s="34" cm="1">
+      <c r="C180" s="52" t="n"/>
+      <c r="D180" s="36" cm="1">
         <f t="array" ref="D180">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,2)</f>
         <v/>
       </c>
-      <c r="E180" s="34" cm="1">
+      <c r="E180" s="36" cm="1">
         <f t="array" ref="E180">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,3)</f>
         <v/>
       </c>
@@ -5334,17 +5775,17 @@
       </c>
     </row>
     <row r="181">
-      <c r="B181" s="49" t="inlineStr">
+      <c r="B181" s="51" t="inlineStr">
         <is>
           <t>Wd</t>
         </is>
       </c>
-      <c r="C181" s="50" t="n"/>
-      <c r="D181" s="34" cm="1">
+      <c r="C181" s="52" t="n"/>
+      <c r="D181" s="36" cm="1">
         <f t="array" ref="D181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,2)</f>
         <v/>
       </c>
-      <c r="E181" s="34" cm="1">
+      <c r="E181" s="36" cm="1">
         <f t="array" ref="E181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,3)</f>
         <v/>
       </c>
@@ -5355,17 +5796,17 @@
       </c>
     </row>
     <row r="182">
-      <c r="B182" s="49" t="inlineStr">
+      <c r="B182" s="51" t="inlineStr">
         <is>
           <t>Wu</t>
         </is>
       </c>
-      <c r="C182" s="50" t="n"/>
-      <c r="D182" s="34" cm="1">
+      <c r="C182" s="52" t="n"/>
+      <c r="D182" s="36" cm="1">
         <f t="array" ref="D182">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,2)</f>
         <v/>
       </c>
-      <c r="E182" s="34" cm="1">
+      <c r="E182" s="36" cm="1">
         <f t="array" ref="E182">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,3)</f>
         <v/>
       </c>
@@ -5376,17 +5817,17 @@
       </c>
     </row>
     <row r="183">
-      <c r="B183" s="49" t="inlineStr">
+      <c r="B183" s="51" t="inlineStr">
         <is>
           <t>Wid</t>
         </is>
       </c>
-      <c r="C183" s="50" t="n"/>
-      <c r="D183" s="34" cm="1">
+      <c r="C183" s="52" t="n"/>
+      <c r="D183" s="36" cm="1">
         <f t="array" ref="D183">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,2)</f>
         <v/>
       </c>
-      <c r="E183" s="34" cm="1">
+      <c r="E183" s="36" cm="1">
         <f t="array" ref="E183">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,3)</f>
         <v/>
       </c>
@@ -5397,17 +5838,17 @@
       </c>
     </row>
     <row r="184">
-      <c r="B184" s="49" t="inlineStr">
+      <c r="B184" s="51" t="inlineStr">
         <is>
           <t>Wiu</t>
         </is>
       </c>
-      <c r="C184" s="50" t="n"/>
-      <c r="D184" s="34" cm="1">
+      <c r="C184" s="52" t="n"/>
+      <c r="D184" s="36" cm="1">
         <f t="array" ref="D184">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,2)</f>
         <v/>
       </c>
-      <c r="E184" s="34" cm="1">
+      <c r="E184" s="36" cm="1">
         <f t="array" ref="E184">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,3)</f>
         <v/>
       </c>
@@ -5425,94 +5866,94 @@
       </c>
     </row>
     <row r="187">
-      <c r="B187" s="57" t="inlineStr">
+      <c r="B187" s="59" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C187" s="57" t="inlineStr">
+      <c r="C187" s="59" t="inlineStr">
         <is>
           <t>Left (kN)</t>
         </is>
       </c>
-      <c r="D187" s="57" t="inlineStr">
+      <c r="D187" s="59" t="inlineStr">
         <is>
           <t>Right (kN)</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="B188" s="32" cm="1">
+      <c r="B188" s="34" cm="1">
         <f t="array" ref="B188">OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
         <v/>
       </c>
-      <c r="C188" s="62" t="n"/>
-      <c r="D188" s="62" t="n"/>
+      <c r="C188" s="63" t="n"/>
+      <c r="D188" s="63" t="n"/>
     </row>
     <row r="189">
-      <c r="B189" s="32" t="n"/>
-      <c r="C189" s="62" t="n"/>
-      <c r="D189" s="62" t="n"/>
+      <c r="B189" s="34" t="n"/>
+      <c r="C189" s="63" t="n"/>
+      <c r="D189" s="63" t="n"/>
     </row>
     <row r="190">
-      <c r="B190" s="32" t="n"/>
-      <c r="C190" s="62" t="n"/>
-      <c r="D190" s="62" t="n"/>
+      <c r="B190" s="34" t="n"/>
+      <c r="C190" s="63" t="n"/>
+      <c r="D190" s="63" t="n"/>
     </row>
     <row r="191">
-      <c r="B191" s="32" t="n"/>
-      <c r="C191" s="62" t="n"/>
-      <c r="D191" s="62" t="n"/>
+      <c r="B191" s="34" t="n"/>
+      <c r="C191" s="63" t="n"/>
+      <c r="D191" s="63" t="n"/>
     </row>
     <row r="192">
-      <c r="B192" s="32" t="n"/>
-      <c r="C192" s="62" t="n"/>
-      <c r="D192" s="62" t="n"/>
+      <c r="B192" s="34" t="n"/>
+      <c r="C192" s="63" t="n"/>
+      <c r="D192" s="63" t="n"/>
     </row>
     <row r="193">
-      <c r="B193" s="32" t="n"/>
-      <c r="C193" s="62" t="n"/>
-      <c r="D193" s="62" t="n"/>
+      <c r="B193" s="34" t="n"/>
+      <c r="C193" s="63" t="n"/>
+      <c r="D193" s="63" t="n"/>
     </row>
     <row r="194">
-      <c r="B194" s="32" t="n"/>
-      <c r="C194" s="62" t="n"/>
-      <c r="D194" s="62" t="n"/>
+      <c r="B194" s="34" t="n"/>
+      <c r="C194" s="63" t="n"/>
+      <c r="D194" s="63" t="n"/>
     </row>
     <row r="195">
-      <c r="B195" s="32" t="n"/>
-      <c r="C195" s="62" t="n"/>
-      <c r="D195" s="62" t="n"/>
+      <c r="B195" s="34" t="n"/>
+      <c r="C195" s="63" t="n"/>
+      <c r="D195" s="63" t="n"/>
     </row>
     <row r="196">
-      <c r="B196" s="32" t="n"/>
-      <c r="C196" s="62" t="n"/>
-      <c r="D196" s="62" t="n"/>
+      <c r="B196" s="34" t="n"/>
+      <c r="C196" s="63" t="n"/>
+      <c r="D196" s="63" t="n"/>
     </row>
     <row r="197">
-      <c r="B197" s="32" t="n"/>
-      <c r="C197" s="62" t="n"/>
-      <c r="D197" s="62" t="n"/>
+      <c r="B197" s="34" t="n"/>
+      <c r="C197" s="63" t="n"/>
+      <c r="D197" s="63" t="n"/>
     </row>
     <row r="198">
-      <c r="B198" s="32" t="n"/>
-      <c r="C198" s="62" t="n"/>
-      <c r="D198" s="62" t="n"/>
+      <c r="B198" s="34" t="n"/>
+      <c r="C198" s="63" t="n"/>
+      <c r="D198" s="63" t="n"/>
     </row>
     <row r="199">
-      <c r="B199" s="32" t="n"/>
-      <c r="C199" s="62" t="n"/>
-      <c r="D199" s="62" t="n"/>
+      <c r="B199" s="34" t="n"/>
+      <c r="C199" s="63" t="n"/>
+      <c r="D199" s="63" t="n"/>
     </row>
     <row r="200">
-      <c r="B200" s="32" t="n"/>
-      <c r="C200" s="62" t="n"/>
-      <c r="D200" s="62" t="n"/>
+      <c r="B200" s="34" t="n"/>
+      <c r="C200" s="63" t="n"/>
+      <c r="D200" s="63" t="n"/>
     </row>
     <row r="201">
-      <c r="B201" s="32" t="n"/>
-      <c r="C201" s="62" t="n"/>
-      <c r="D201" s="62" t="n"/>
+      <c r="B201" s="34" t="n"/>
+      <c r="C201" s="63" t="n"/>
+      <c r="D201" s="63" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="40">
@@ -5650,7 +6091,7 @@
       <formula>$B188&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="12">
+  <dataValidations count="13">
     <dataValidation sqref="E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"UB,UC,WB,PFC"</formula1>
     </dataValidation>
@@ -5668,6 +6109,9 @@
     </dataValidation>
     <dataValidation sqref="C47:C57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"UDL,PUDL,Point"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D47:D57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>OFFSET($AQ$10,MATCH($B47,$AP$10:$AP$71,0)-1,0,COUNTIF($AP$10:$AP$71,$B47),1)</formula1>
     </dataValidation>
     <dataValidation sqref="M47:M84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
@@ -5704,10 +6148,11 @@
     <brk id="139" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  <tableParts count="3">
+  <tableParts count="4">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
v0.2.3: applied load diagram (OAR.LOADDIAGRAM); BMD full width, shear diagram removed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -52,26 +52,26 @@
     <definedName name="w_Wid" localSheetId="0">'B1'!$I$60</definedName>
     <definedName name="w_Wiu" localSheetId="0">'B1'!$J$60</definedName>
     <definedName name="NumUpliftCombos" localSheetId="0">'B1'!$S$56</definedName>
-    <definedName name="CombSet" localSheetId="0">'B1'!$E$63</definedName>
-    <definedName name="PsiC" localSheetId="0">'B1'!$G$63</definedName>
-    <definedName name="kl_Top" localSheetId="0">'B1'!$I$77</definedName>
-    <definedName name="kl_Bot" localSheetId="0">'B1'!$J$77</definedName>
-    <definedName name="kr_Top" localSheetId="0">'B1'!$I$78</definedName>
-    <definedName name="kr_Bot" localSheetId="0">'B1'!$J$78</definedName>
-    <definedName name="RxnL_G" localSheetId="0">'B1'!$D$179</definedName>
-    <definedName name="RxnR_G" localSheetId="0">'B1'!$E$179</definedName>
-    <definedName name="RxnL_Q" localSheetId="0">'B1'!$D$180</definedName>
-    <definedName name="RxnR_Q" localSheetId="0">'B1'!$E$180</definedName>
-    <definedName name="RxnL_Wd" localSheetId="0">'B1'!$D$181</definedName>
-    <definedName name="RxnR_Wd" localSheetId="0">'B1'!$E$181</definedName>
-    <definedName name="RxnL_Wu" localSheetId="0">'B1'!$D$182</definedName>
-    <definedName name="RxnR_Wu" localSheetId="0">'B1'!$E$182</definedName>
-    <definedName name="RxnL_Wid" localSheetId="0">'B1'!$D$183</definedName>
-    <definedName name="RxnR_Wid" localSheetId="0">'B1'!$E$183</definedName>
-    <definedName name="RxnL_Wiu" localSheetId="0">'B1'!$D$184</definedName>
-    <definedName name="RxnR_Wiu" localSheetId="0">'B1'!$E$184</definedName>
-    <definedName name="Out_Reactions" localSheetId="0">'B1'!$B$188</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'B1'!$A$1:$K$202</definedName>
+    <definedName name="CombSet" localSheetId="0">'B1'!$E$76</definedName>
+    <definedName name="PsiC" localSheetId="0">'B1'!$G$76</definedName>
+    <definedName name="kl_Top" localSheetId="0">'B1'!$I$90</definedName>
+    <definedName name="kl_Bot" localSheetId="0">'B1'!$J$90</definedName>
+    <definedName name="kr_Top" localSheetId="0">'B1'!$I$91</definedName>
+    <definedName name="kr_Bot" localSheetId="0">'B1'!$J$91</definedName>
+    <definedName name="RxnL_G" localSheetId="0">'B1'!$D$190</definedName>
+    <definedName name="RxnR_G" localSheetId="0">'B1'!$E$190</definedName>
+    <definedName name="RxnL_Q" localSheetId="0">'B1'!$D$191</definedName>
+    <definedName name="RxnR_Q" localSheetId="0">'B1'!$E$191</definedName>
+    <definedName name="RxnL_Wd" localSheetId="0">'B1'!$D$192</definedName>
+    <definedName name="RxnR_Wd" localSheetId="0">'B1'!$E$192</definedName>
+    <definedName name="RxnL_Wu" localSheetId="0">'B1'!$D$193</definedName>
+    <definedName name="RxnR_Wu" localSheetId="0">'B1'!$E$193</definedName>
+    <definedName name="RxnL_Wid" localSheetId="0">'B1'!$D$194</definedName>
+    <definedName name="RxnR_Wid" localSheetId="0">'B1'!$E$194</definedName>
+    <definedName name="RxnL_Wiu" localSheetId="0">'B1'!$D$195</definedName>
+    <definedName name="RxnR_Wiu" localSheetId="0">'B1'!$E$195</definedName>
+    <definedName name="Out_Reactions" localSheetId="0">'B1'!$B$199</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'B1'!$A$1:$K$213</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -559,6 +559,9 @@
     <xf numFmtId="170" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -573,9 +576,6 @@
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="171" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -754,6 +754,333 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'B1'!AA90</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="465A52"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'B1'!$Z$91:$Z$170</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'B1'!$AA$91:$AA$170</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'B1'!AB90</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="C07A2C"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'B1'!$Z$91:$Z$170</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'B1'!$AB$91:$AB$170</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'B1'!AC90</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="6E8FB5"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'B1'!$Z$91:$Z$170</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'B1'!$AC$91:$AC$170</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'B1'!AD90</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="9C5DA6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'B1'!$Z$91:$Z$170</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'B1'!$AD$91:$AD$170</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'B1'!AE90</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="8FA89C"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'B1'!$Z$91:$Z$170</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'B1'!$AE$91:$AE$170</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'B1'!AF90</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="B8ADA5"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'B1'!$Z$91:$Z$170</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'B1'!$AF$91:$AF$170</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <v>Point loads (kN)</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="triangle"/>
+            <size val="7"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="262626"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <errBars>
+            <errDir val="y"/>
+            <errBarType val="minus"/>
+            <errValType val="percentage"/>
+            <noEndCap val="1"/>
+            <val val="100"/>
+          </errBars>
+          <xVal>
+            <numRef>
+              <f>'B1'!$AH$91:$AH$110</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'B1'!$AI$90:$AI$110</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
+              <a:solidFill>
+                <a:srgbClr val="E3E3E3"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>kN/m · kN</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="t"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -966,7 +1293,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -1107,157 +1434,16 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
-  <chart>
-    <plotArea>
-      <scatterChart>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'B1'!AC13</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-              <a:solidFill>
-                <a:srgbClr val="465A52"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'B1'!$Z$14:$Z$74</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'B1'!$AC$14:$AC$74</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'B1'!AD13</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-              <a:solidFill>
-                <a:srgbClr val="B8ADA5"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'B1'!$Z$14:$Z$74</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'B1'!$AD$14:$AD$74</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <axId val="10"/>
-        <axId val="20"/>
-      </scatterChart>
-      <valAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-          <min val="0"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="low"/>
-        <crossAx val="20"/>
-      </valAx>
-      <valAx>
-        <axId val="20"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
-              <a:solidFill>
-                <a:srgbClr val="E3E3E3"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>V* (kN)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="low"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="t"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>92</row>
+      <row>62</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6336000" cy="1944000"/>
+    <ext cx="6336000" cy="1800000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1276,10 +1462,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>106</row>
+      <row>105</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3131999" cy="2232000"/>
+    <ext cx="6336000" cy="1944000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1296,12 +1482,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>1</col>
       <colOff>0</colOff>
-      <row>106</row>
+      <row>119</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3131999" cy="2232000"/>
+    <ext cx="6336000" cy="1944000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -1397,8 +1583,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Restraints_B1" displayName="Restraints_B1" ref="B76:G81" headerRowCount="1">
-  <autoFilter ref="B76:G81"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Restraints_B1" displayName="Restraints_B1" ref="B89:G94" headerRowCount="1">
+  <autoFilter ref="B89:G94"/>
   <tableColumns count="6">
     <tableColumn id="2" name="x (mm)"/>
     <tableColumn id="3" name="Ref"/>
@@ -1701,7 +1887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AS201"/>
+  <dimension ref="B1:AS212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.5" customWidth="1" min="1" max="1"/>
@@ -1942,7 +2128,7 @@
       <c r="S8" s="17" t="n"/>
       <c r="T8" s="18" t="n"/>
       <c r="Z8" s="19" cm="1">
-        <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
+        <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79),Restraints_B1[#Data],$I$90:$J$91)</f>
         <v/>
       </c>
       <c r="AL8" s="19" cm="1">
@@ -2185,7 +2371,7 @@
       <c r="S13" s="23" t="n"/>
       <c r="T13" s="24" t="n"/>
       <c r="Z13" s="19" cm="1">
-        <f t="array" ref="Z13">OAR.ENVELOPE(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),60)</f>
+        <f t="array" ref="Z13">OAR.ENVELOPE(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79),60)</f>
         <v/>
       </c>
       <c r="AF13" s="19" cm="1">
@@ -2274,7 +2460,7 @@
         </is>
       </c>
       <c r="E15" s="36" cm="1">
-        <f t="array" ref="E15">INDEX(_xlfn.ANCHORARRAY(B86),1,2)</f>
+        <f t="array" ref="E15">INDEX(_xlfn.ANCHORARRAY(B99),1,2)</f>
         <v/>
       </c>
       <c r="F15" s="36">
@@ -2342,7 +2528,7 @@
         </is>
       </c>
       <c r="E16" s="36" cm="1">
-        <f t="array" ref="E16">INDEX(_xlfn.ANCHORARRAY(B86),2,2)</f>
+        <f t="array" ref="E16">INDEX(_xlfn.ANCHORARRAY(B99),2,2)</f>
         <v/>
       </c>
       <c r="F16" s="36">
@@ -2410,7 +2596,7 @@
         </is>
       </c>
       <c r="E17" s="36" cm="1">
-        <f t="array" ref="E17">INDEX(_xlfn.ANCHORARRAY(B86),3,2)</f>
+        <f t="array" ref="E17">INDEX(_xlfn.ANCHORARRAY(B99),3,2)</f>
         <v/>
       </c>
       <c r="F17" s="36">
@@ -2478,7 +2664,7 @@
         </is>
       </c>
       <c r="E18" s="36" cm="1">
-        <f t="array" ref="E18">INDEX(_xlfn.ANCHORARRAY(B86),4,2)</f>
+        <f t="array" ref="E18">INDEX(_xlfn.ANCHORARRAY(B99),4,2)</f>
         <v/>
       </c>
       <c r="F18" s="36">
@@ -2546,7 +2732,7 @@
         </is>
       </c>
       <c r="E19" s="36" cm="1">
-        <f t="array" ref="E19">INDEX(_xlfn.ANCHORARRAY(B86),5,2)</f>
+        <f t="array" ref="E19">INDEX(_xlfn.ANCHORARRAY(B99),5,2)</f>
         <v/>
       </c>
       <c r="F19" s="36">
@@ -4508,689 +4694,699 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="B62" s="10" t="inlineStr">
+    <row r="62" ht="14" customHeight="1">
+      <c r="B62" s="63" t="inlineStr">
+        <is>
+          <t>Applied loads (unfactored; line loads kN/m, point loads kN with stems; + = downward;  x in m)</t>
+        </is>
+      </c>
+      <c r="AN62" s="20" t="inlineStr">
+        <is>
+          <t>180UB18.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="14" customHeight="1">
+      <c r="AN63" s="20" t="inlineStr">
+        <is>
+          <t>180UB16.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="14" customHeight="1">
+      <c r="AN64" s="20" t="inlineStr">
+        <is>
+          <t>150UB18</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="14" customHeight="1">
+      <c r="AN65" s="20" t="inlineStr">
+        <is>
+          <t>150UB14</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="14" customHeight="1">
+      <c r="AN66" s="20" t="inlineStr">
+        <is>
+          <t>380PFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="14" customHeight="1">
+      <c r="AN67" s="20" t="inlineStr">
+        <is>
+          <t>300PFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="14" customHeight="1">
+      <c r="AN68" s="20" t="inlineStr">
+        <is>
+          <t>250PFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="14" customHeight="1">
+      <c r="AN69" s="20" t="inlineStr">
+        <is>
+          <t>230PFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="14" customHeight="1">
+      <c r="AN70" s="20" t="inlineStr">
+        <is>
+          <t>200PFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="14" customHeight="1">
+      <c r="AN71" s="20" t="inlineStr">
+        <is>
+          <t>180PFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="14" customHeight="1">
+      <c r="AN72" s="20" t="inlineStr">
+        <is>
+          <t>150PFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="14" customHeight="1">
+      <c r="AN73" s="20" t="inlineStr">
+        <is>
+          <t>125PFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="14" customHeight="1">
+      <c r="AN74" s="20" t="inlineStr">
+        <is>
+          <t>100PFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="B75" s="10" t="inlineStr">
         <is>
           <t>Load Combinations (AS/NZS 1170.0)</t>
         </is>
       </c>
-      <c r="C62" s="11" t="n"/>
-      <c r="D62" s="11" t="n"/>
-      <c r="E62" s="11" t="n"/>
-      <c r="F62" s="11" t="n"/>
-      <c r="G62" s="11" t="n"/>
-      <c r="H62" s="11" t="n"/>
-      <c r="I62" s="11" t="n"/>
-      <c r="J62" s="11" t="n"/>
-      <c r="AN62" s="20" t="inlineStr">
-        <is>
-          <t>180UB18.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="14" customHeight="1">
-      <c r="B63" s="42" t="inlineStr">
+      <c r="C75" s="11" t="n"/>
+      <c r="D75" s="11" t="n"/>
+      <c r="E75" s="11" t="n"/>
+      <c r="F75" s="11" t="n"/>
+      <c r="G75" s="11" t="n"/>
+      <c r="H75" s="11" t="n"/>
+      <c r="I75" s="11" t="n"/>
+      <c r="J75" s="11" t="n"/>
+      <c r="AN75" s="20" t="inlineStr">
+        <is>
+          <t>75PFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="14" customHeight="1">
+      <c r="B76" s="42" t="inlineStr">
         <is>
           <t>Combination set</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E76" s="2" t="inlineStr">
         <is>
           <t>Roof</t>
         </is>
       </c>
-      <c r="F63" s="44" t="inlineStr">
+      <c r="F76" s="44" t="inlineStr">
         <is>
           <t>ψc</t>
         </is>
       </c>
-      <c r="G63" s="54" t="n">
+      <c r="G76" s="54" t="n">
         <v>0.4</v>
       </c>
-      <c r="H63" s="6" t="inlineStr">
+      <c r="H76" s="6" t="inlineStr">
         <is>
           <t>Table 4.1 (roofs 0.0)</t>
         </is>
       </c>
-      <c r="AN63" s="20" t="inlineStr">
-        <is>
-          <t>180UB16.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="14" customHeight="1">
-      <c r="B64" s="15" t="inlineStr">
+      <c r="AN76" s="20" t="inlineStr">
+        <is>
+          <t>310UC158</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="14" customHeight="1">
+      <c r="B77" s="15" t="inlineStr">
         <is>
           <t>Floor = gravity only.  Roof = gravity + wind.  All = every library row.  Custom = only rows set to Yes / Custom.  Edit in the library to the right →</t>
         </is>
       </c>
-      <c r="AN64" s="20" t="inlineStr">
-        <is>
-          <t>150UB18</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="14" customHeight="1">
-      <c r="B65" s="25" t="inlineStr">
+      <c r="AN77" s="20" t="inlineStr">
+        <is>
+          <t>310UC137</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="14" customHeight="1">
+      <c r="B78" s="25" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C65" s="25" t="inlineStr">
+      <c r="C78" s="25" t="inlineStr">
         <is>
           <t>Crit. flange</t>
         </is>
       </c>
-      <c r="D65" s="25" t="inlineStr">
+      <c r="D78" s="25" t="inlineStr">
         <is>
           <t>Combination</t>
         </is>
       </c>
-      <c r="E65" s="25" t="inlineStr">
+      <c r="E78" s="25" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="F65" s="25" t="inlineStr">
+      <c r="F78" s="25" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="G65" s="25" t="inlineStr">
+      <c r="G78" s="25" t="inlineStr">
         <is>
           <t>Wd</t>
         </is>
       </c>
-      <c r="H65" s="25" t="inlineStr">
+      <c r="H78" s="25" t="inlineStr">
         <is>
           <t>Wu</t>
         </is>
       </c>
-      <c r="I65" s="25" t="inlineStr">
+      <c r="I78" s="25" t="inlineStr">
         <is>
           <t>Wid</t>
         </is>
       </c>
-      <c r="J65" s="25" t="inlineStr">
+      <c r="J78" s="25" t="inlineStr">
         <is>
           <t>Wiu</t>
         </is>
       </c>
-      <c r="AN65" s="20" t="inlineStr">
-        <is>
-          <t>150UB14</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="14" customHeight="1">
-      <c r="B66" s="34" cm="1">
-        <f t="array" ref="B66">_xlfn._xlws.FILTER(CombLib_B1[[ID]:[Wiu]],CombLib_B1[Active]=1,"No combinations selected")</f>
-        <v/>
-      </c>
-      <c r="C66" s="34" t="n"/>
-      <c r="D66" s="42" t="n"/>
-      <c r="E66" s="63" t="n"/>
-      <c r="F66" s="63" t="n"/>
-      <c r="G66" s="63" t="n"/>
-      <c r="H66" s="63" t="n"/>
-      <c r="I66" s="63" t="n"/>
-      <c r="J66" s="63" t="n"/>
-      <c r="AN66" s="20" t="inlineStr">
-        <is>
-          <t>380PFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="14" customHeight="1">
-      <c r="B67" s="34" t="n"/>
-      <c r="C67" s="34" t="n"/>
-      <c r="D67" s="42" t="n"/>
-      <c r="E67" s="63" t="n"/>
-      <c r="F67" s="63" t="n"/>
-      <c r="G67" s="63" t="n"/>
-      <c r="H67" s="63" t="n"/>
-      <c r="I67" s="63" t="n"/>
-      <c r="J67" s="63" t="n"/>
-      <c r="AN67" s="20" t="inlineStr">
-        <is>
-          <t>300PFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="14" customHeight="1">
-      <c r="B68" s="34" t="n"/>
-      <c r="C68" s="34" t="n"/>
-      <c r="D68" s="42" t="n"/>
-      <c r="E68" s="63" t="n"/>
-      <c r="F68" s="63" t="n"/>
-      <c r="G68" s="63" t="n"/>
-      <c r="H68" s="63" t="n"/>
-      <c r="I68" s="63" t="n"/>
-      <c r="J68" s="63" t="n"/>
-      <c r="AN68" s="20" t="inlineStr">
-        <is>
-          <t>250PFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="14" customHeight="1">
-      <c r="B69" s="34" t="n"/>
-      <c r="C69" s="34" t="n"/>
-      <c r="D69" s="42" t="n"/>
-      <c r="E69" s="63" t="n"/>
-      <c r="F69" s="63" t="n"/>
-      <c r="G69" s="63" t="n"/>
-      <c r="H69" s="63" t="n"/>
-      <c r="I69" s="63" t="n"/>
-      <c r="J69" s="63" t="n"/>
-      <c r="AN69" s="20" t="inlineStr">
-        <is>
-          <t>230PFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="14" customHeight="1">
-      <c r="B70" s="34" t="n"/>
-      <c r="C70" s="34" t="n"/>
-      <c r="D70" s="42" t="n"/>
-      <c r="E70" s="63" t="n"/>
-      <c r="F70" s="63" t="n"/>
-      <c r="G70" s="63" t="n"/>
-      <c r="H70" s="63" t="n"/>
-      <c r="I70" s="63" t="n"/>
-      <c r="J70" s="63" t="n"/>
-      <c r="AN70" s="20" t="inlineStr">
-        <is>
-          <t>200PFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="14" customHeight="1">
-      <c r="B71" s="34" t="n"/>
-      <c r="C71" s="34" t="n"/>
-      <c r="D71" s="42" t="n"/>
-      <c r="E71" s="63" t="n"/>
-      <c r="F71" s="63" t="n"/>
-      <c r="G71" s="63" t="n"/>
-      <c r="H71" s="63" t="n"/>
-      <c r="I71" s="63" t="n"/>
-      <c r="J71" s="63" t="n"/>
-      <c r="AN71" s="20" t="inlineStr">
-        <is>
-          <t>180PFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="14" customHeight="1">
-      <c r="B72" s="34" t="n"/>
-      <c r="C72" s="34" t="n"/>
-      <c r="D72" s="42" t="n"/>
-      <c r="E72" s="63" t="n"/>
-      <c r="F72" s="63" t="n"/>
-      <c r="G72" s="63" t="n"/>
-      <c r="H72" s="63" t="n"/>
-      <c r="I72" s="63" t="n"/>
-      <c r="J72" s="63" t="n"/>
-      <c r="AN72" s="20" t="inlineStr">
-        <is>
-          <t>150PFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="14" customHeight="1">
-      <c r="B73" s="34" t="n"/>
-      <c r="C73" s="34" t="n"/>
-      <c r="D73" s="42" t="n"/>
-      <c r="E73" s="63" t="n"/>
-      <c r="F73" s="63" t="n"/>
-      <c r="G73" s="63" t="n"/>
-      <c r="H73" s="63" t="n"/>
-      <c r="I73" s="63" t="n"/>
-      <c r="J73" s="63" t="n"/>
-      <c r="AN73" s="20" t="inlineStr">
-        <is>
-          <t>125PFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="B74" s="10" t="inlineStr">
+      <c r="AN78" s="20" t="inlineStr">
+        <is>
+          <t>310UC118</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="14" customHeight="1">
+      <c r="B79" s="34" cm="1">
+        <f t="array" ref="B79">_xlfn._xlws.FILTER(CombLib_B1[[ID]:[Wiu]],CombLib_B1[Active]=1,"No combinations selected")</f>
+        <v/>
+      </c>
+      <c r="C79" s="34" t="n"/>
+      <c r="D79" s="42" t="n"/>
+      <c r="E79" s="64" t="n"/>
+      <c r="F79" s="64" t="n"/>
+      <c r="G79" s="64" t="n"/>
+      <c r="H79" s="64" t="n"/>
+      <c r="I79" s="64" t="n"/>
+      <c r="J79" s="64" t="n"/>
+      <c r="AN79" s="20" t="inlineStr">
+        <is>
+          <t>310UC97</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="14" customHeight="1">
+      <c r="B80" s="34" t="n"/>
+      <c r="C80" s="34" t="n"/>
+      <c r="D80" s="42" t="n"/>
+      <c r="E80" s="64" t="n"/>
+      <c r="F80" s="64" t="n"/>
+      <c r="G80" s="64" t="n"/>
+      <c r="H80" s="64" t="n"/>
+      <c r="I80" s="64" t="n"/>
+      <c r="J80" s="64" t="n"/>
+      <c r="AN80" s="20" t="inlineStr">
+        <is>
+          <t>250UC89.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="14" customHeight="1">
+      <c r="B81" s="34" t="n"/>
+      <c r="C81" s="34" t="n"/>
+      <c r="D81" s="42" t="n"/>
+      <c r="E81" s="64" t="n"/>
+      <c r="F81" s="64" t="n"/>
+      <c r="G81" s="64" t="n"/>
+      <c r="H81" s="64" t="n"/>
+      <c r="I81" s="64" t="n"/>
+      <c r="J81" s="64" t="n"/>
+      <c r="AN81" s="20" t="inlineStr">
+        <is>
+          <t>250UC73</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="14" customHeight="1">
+      <c r="B82" s="34" t="n"/>
+      <c r="C82" s="34" t="n"/>
+      <c r="D82" s="42" t="n"/>
+      <c r="E82" s="64" t="n"/>
+      <c r="F82" s="64" t="n"/>
+      <c r="G82" s="64" t="n"/>
+      <c r="H82" s="64" t="n"/>
+      <c r="I82" s="64" t="n"/>
+      <c r="J82" s="64" t="n"/>
+      <c r="AN82" s="20" t="inlineStr">
+        <is>
+          <t>200UC59.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="14" customHeight="1">
+      <c r="B83" s="34" t="n"/>
+      <c r="C83" s="34" t="n"/>
+      <c r="D83" s="42" t="n"/>
+      <c r="E83" s="64" t="n"/>
+      <c r="F83" s="64" t="n"/>
+      <c r="G83" s="64" t="n"/>
+      <c r="H83" s="64" t="n"/>
+      <c r="I83" s="64" t="n"/>
+      <c r="J83" s="64" t="n"/>
+      <c r="AN83" s="20" t="inlineStr">
+        <is>
+          <t>200UC52</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="14" customHeight="1">
+      <c r="B84" s="34" t="n"/>
+      <c r="C84" s="34" t="n"/>
+      <c r="D84" s="42" t="n"/>
+      <c r="E84" s="64" t="n"/>
+      <c r="F84" s="64" t="n"/>
+      <c r="G84" s="64" t="n"/>
+      <c r="H84" s="64" t="n"/>
+      <c r="I84" s="64" t="n"/>
+      <c r="J84" s="64" t="n"/>
+      <c r="AN84" s="20" t="inlineStr">
+        <is>
+          <t>200UC46</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="14" customHeight="1">
+      <c r="B85" s="34" t="n"/>
+      <c r="C85" s="34" t="n"/>
+      <c r="D85" s="42" t="n"/>
+      <c r="E85" s="64" t="n"/>
+      <c r="F85" s="64" t="n"/>
+      <c r="G85" s="64" t="n"/>
+      <c r="H85" s="64" t="n"/>
+      <c r="I85" s="64" t="n"/>
+      <c r="J85" s="64" t="n"/>
+      <c r="AN85" s="20" t="inlineStr">
+        <is>
+          <t>150UC37</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="14" customHeight="1">
+      <c r="B86" s="34" t="n"/>
+      <c r="C86" s="34" t="n"/>
+      <c r="D86" s="42" t="n"/>
+      <c r="E86" s="64" t="n"/>
+      <c r="F86" s="64" t="n"/>
+      <c r="G86" s="64" t="n"/>
+      <c r="H86" s="64" t="n"/>
+      <c r="I86" s="64" t="n"/>
+      <c r="J86" s="64" t="n"/>
+      <c r="AN86" s="20" t="inlineStr">
+        <is>
+          <t>150UC30</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="B87" s="10" t="inlineStr">
         <is>
           <t>Lateral Restraints (AS 4100 Cl. 5.4)</t>
         </is>
       </c>
-      <c r="C74" s="11" t="n"/>
-      <c r="D74" s="11" t="n"/>
-      <c r="E74" s="11" t="n"/>
-      <c r="F74" s="11" t="n"/>
-      <c r="G74" s="11" t="n"/>
-      <c r="H74" s="11" t="n"/>
-      <c r="I74" s="11" t="n"/>
-      <c r="J74" s="11" t="n"/>
-      <c r="AN74" s="20" t="inlineStr">
-        <is>
-          <t>100PFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="14" customHeight="1">
-      <c r="B75" s="15" t="inlineStr">
+      <c r="C87" s="11" t="n"/>
+      <c r="D87" s="11" t="n"/>
+      <c r="E87" s="11" t="n"/>
+      <c r="F87" s="11" t="n"/>
+      <c r="G87" s="11" t="n"/>
+      <c r="H87" s="11" t="n"/>
+      <c r="I87" s="11" t="n"/>
+      <c r="J87" s="11" t="n"/>
+      <c r="AN87" s="20" t="inlineStr">
+        <is>
+          <t>150UC23</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="14" customHeight="1">
+      <c r="B88" s="15" t="inlineStr">
         <is>
           <t>Restraint type at each cross-section for the critical flange: F, P, L or U (– = none). Supports must be F or P.</t>
         </is>
       </c>
-      <c r="AN75" s="20" t="inlineStr">
-        <is>
-          <t>75PFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="14" customHeight="1">
-      <c r="B76" s="25" t="inlineStr">
+      <c r="AN88" s="20" t="inlineStr">
+        <is>
+          <t>100UC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="14" customHeight="1">
+      <c r="B89" s="25" t="inlineStr">
         <is>
           <t>x (mm)</t>
         </is>
       </c>
-      <c r="C76" s="25" t="inlineStr">
+      <c r="C89" s="25" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
       </c>
-      <c r="D76" s="25" t="inlineStr">
+      <c r="D89" s="25" t="inlineStr">
         <is>
           <t>Restraint provided by</t>
         </is>
       </c>
-      <c r="E76" s="25" t="inlineStr">
+      <c r="E89" s="25" t="inlineStr">
         <is>
           <t>Top flange</t>
         </is>
       </c>
-      <c r="F76" s="25" t="inlineStr">
+      <c r="F89" s="25" t="inlineStr">
         <is>
           <t>Bottom fl.</t>
         </is>
       </c>
-      <c r="G76" s="25" t="inlineStr">
+      <c r="G89" s="25" t="inlineStr">
         <is>
           <t>αm override</t>
         </is>
       </c>
-      <c r="H76" s="25" t="inlineStr">
+      <c r="H89" s="25" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="I76" s="25" t="inlineStr">
+      <c r="I89" s="25" t="inlineStr">
         <is>
           <t>Top</t>
         </is>
       </c>
-      <c r="J76" s="25" t="inlineStr">
+      <c r="J89" s="25" t="inlineStr">
         <is>
           <t>Bottom</t>
         </is>
       </c>
-      <c r="AN76" s="20" t="inlineStr">
-        <is>
-          <t>310UC158</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="14" customHeight="1">
-      <c r="B77" s="64">
+      <c r="Z89" s="15" t="inlineStr">
+        <is>
+          <t>Applied line loads (OAR.LOADDIAGRAM)</t>
+        </is>
+      </c>
+      <c r="AH89" s="15" t="inlineStr">
+        <is>
+          <t>Point loads</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="14" customHeight="1">
+      <c r="B90" s="65">
         <f>0</f>
         <v/>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D77" s="5" t="inlineStr">
+      <c r="D90" s="5" t="inlineStr">
         <is>
           <t>Left support – cleat</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E90" s="2" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="F90" s="2" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G77" s="30" t="n"/>
-      <c r="H77" s="34" t="inlineStr">
+      <c r="G90" s="30" t="n"/>
+      <c r="H90" s="34" t="inlineStr">
         <is>
           <t>kl</t>
         </is>
       </c>
-      <c r="I77" s="30" t="n">
+      <c r="I90" s="30" t="n">
         <v>1.4</v>
       </c>
-      <c r="J77" s="30" t="n">
+      <c r="J90" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="AN77" s="20" t="inlineStr">
-        <is>
-          <t>310UC137</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="14" customHeight="1">
-      <c r="B78" s="47" t="n">
+      <c r="Z90" s="19" cm="1">
+        <f t="array" ref="Z90">OAR.LOADDIAGRAM(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],"line")</f>
+        <v/>
+      </c>
+      <c r="AH90" s="19" cm="1">
+        <f t="array" ref="AH90">OAR.LOADDIAGRAM(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],"point")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91" ht="14" customHeight="1">
+      <c r="B91" s="47" t="n">
         <v>2767</v>
       </c>
-      <c r="C78" s="2" t="inlineStr"/>
-      <c r="D78" s="5" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr"/>
+      <c r="D91" s="5" t="inlineStr">
         <is>
           <t>Purlin + fly brace</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
+      <c r="E91" s="2" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G78" s="30" t="n"/>
-      <c r="H78" s="34" t="inlineStr">
+      <c r="G91" s="30" t="n"/>
+      <c r="H91" s="34" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="I78" s="30" t="n">
+      <c r="I91" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="J78" s="30" t="n">
+      <c r="J91" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="AN78" s="20" t="inlineStr">
-        <is>
-          <t>310UC118</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="14" customHeight="1">
-      <c r="B79" s="47" t="n">
+    </row>
+    <row r="92" ht="14" customHeight="1">
+      <c r="B92" s="47" t="n">
         <v>5533</v>
       </c>
-      <c r="C79" s="2" t="inlineStr"/>
-      <c r="D79" s="5" t="inlineStr">
+      <c r="C92" s="2" t="inlineStr"/>
+      <c r="D92" s="5" t="inlineStr">
         <is>
           <t>Purlin + fly brace</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr">
+      <c r="E92" s="2" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr">
+      <c r="F92" s="2" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G79" s="30" t="n"/>
-      <c r="H79" s="15" t="inlineStr">
+      <c r="G92" s="30" t="n"/>
+      <c r="H92" s="15" t="inlineStr">
         <is>
           <t>kt from restraint</t>
         </is>
       </c>
-      <c r="AN79" s="20" t="inlineStr">
-        <is>
-          <t>310UC97</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="14" customHeight="1">
-      <c r="B80" s="64">
+    </row>
+    <row r="93" ht="14" customHeight="1">
+      <c r="B93" s="65">
         <f>Span</f>
         <v/>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="D80" s="5" t="inlineStr">
+      <c r="D93" s="5" t="inlineStr">
         <is>
           <t>Right support – cleat</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E93" s="2" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr">
+      <c r="F93" s="2" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="G80" s="30" t="n"/>
-      <c r="H80" s="15" t="inlineStr">
+      <c r="G93" s="30" t="n"/>
+      <c r="H93" s="15" t="inlineStr">
         <is>
           <t>types (add-in)</t>
         </is>
       </c>
-      <c r="AN80" s="20" t="inlineStr">
-        <is>
-          <t>250UC89.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="14" customHeight="1">
-      <c r="B81" s="47" t="n"/>
-      <c r="C81" s="2" t="n"/>
-      <c r="D81" s="5" t="n"/>
-      <c r="E81" s="2" t="n"/>
-      <c r="F81" s="2" t="n"/>
-      <c r="G81" s="30" t="n"/>
-      <c r="AN81" s="20" t="inlineStr">
-        <is>
-          <t>250UC73</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="14" customHeight="1">
-      <c r="B82" s="15" t="inlineStr">
+    </row>
+    <row r="94" ht="14" customHeight="1">
+      <c r="B94" s="47" t="n"/>
+      <c r="C94" s="2" t="n"/>
+      <c r="D94" s="5" t="n"/>
+      <c r="E94" s="2" t="n"/>
+      <c r="F94" s="2" t="n"/>
+      <c r="G94" s="30" t="n"/>
+    </row>
+    <row r="95" ht="14" customHeight="1">
+      <c r="B95" s="15" t="inlineStr">
         <is>
           <t>αm override applies to the segment starting at that row (blank = Cl. 5.6.1.1(a)(iii)); flagged * in the output.</t>
         </is>
       </c>
-      <c r="AN82" s="20" t="inlineStr">
-        <is>
-          <t>200UC59.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="14" customHeight="1">
-      <c r="AN83" s="20" t="inlineStr">
-        <is>
-          <t>200UC52</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="20" customHeight="1">
-      <c r="B84" s="10" t="inlineStr">
+    </row>
+    <row r="96" ht="14" customHeight="1"/>
+    <row r="97" ht="20" customHeight="1">
+      <c r="B97" s="10" t="inlineStr">
         <is>
           <t>Serviceability Checks</t>
         </is>
       </c>
-      <c r="C84" s="11" t="n"/>
-      <c r="D84" s="11" t="n"/>
-      <c r="E84" s="11" t="n"/>
-      <c r="F84" s="11" t="n"/>
-      <c r="G84" s="11" t="n"/>
-      <c r="H84" s="11" t="n"/>
-      <c r="I84" s="11" t="n"/>
-      <c r="J84" s="11" t="n"/>
-      <c r="AN84" s="20" t="inlineStr">
-        <is>
-          <t>200UC46</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="14" customHeight="1">
-      <c r="B85" s="59" t="inlineStr">
+      <c r="C97" s="11" t="n"/>
+      <c r="D97" s="11" t="n"/>
+      <c r="E97" s="11" t="n"/>
+      <c r="F97" s="11" t="n"/>
+      <c r="G97" s="11" t="n"/>
+      <c r="H97" s="11" t="n"/>
+      <c r="I97" s="11" t="n"/>
+      <c r="J97" s="11" t="n"/>
+    </row>
+    <row r="98" ht="14" customHeight="1">
+      <c r="B98" s="59" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C85" s="59" t="inlineStr">
+      <c r="C98" s="59" t="inlineStr">
         <is>
           <t>Δ max (mm)</t>
         </is>
       </c>
-      <c r="D85" s="59" t="inlineStr">
+      <c r="D98" s="59" t="inlineStr">
         <is>
           <t>at x (mm)</t>
         </is>
       </c>
-      <c r="E85" s="59" t="inlineStr">
+      <c r="E98" s="59" t="inlineStr">
         <is>
           <t>Limit (mm)</t>
         </is>
       </c>
-      <c r="F85" s="59" t="inlineStr">
+      <c r="F98" s="59" t="inlineStr">
         <is>
           <t>L / Δ</t>
         </is>
       </c>
-      <c r="G85" s="59" t="inlineStr">
+      <c r="G98" s="59" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
-      <c r="AN85" s="20" t="inlineStr">
-        <is>
-          <t>150UC37</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="14" customHeight="1">
-      <c r="B86" s="34" cm="1">
-        <f t="array" ref="B86">OAR.SLS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],$E$37:$F$41,PsiL,PsiS)</f>
-        <v/>
-      </c>
-      <c r="C86" s="63" t="n"/>
-      <c r="D86" s="65" t="n"/>
-      <c r="E86" s="63" t="n"/>
-      <c r="F86" s="66" t="n"/>
-      <c r="G86" s="67" t="n"/>
-      <c r="H86" s="6" t="inlineStr">
+    </row>
+    <row r="99" ht="14" customHeight="1">
+      <c r="B99" s="34" cm="1">
+        <f t="array" ref="B99">OAR.SLS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],$E$37:$F$41,PsiL,PsiS)</f>
+        <v/>
+      </c>
+      <c r="C99" s="64" t="n"/>
+      <c r="D99" s="66" t="n"/>
+      <c r="E99" s="64" t="n"/>
+      <c r="F99" s="67" t="n"/>
+      <c r="G99" s="68" t="n"/>
+      <c r="H99" s="6" t="inlineStr">
         <is>
           <t>Δ1kN: 1 kN at midspan,</t>
         </is>
       </c>
-      <c r="AN86" s="20" t="inlineStr">
-        <is>
-          <t>150UC30</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="14" customHeight="1">
-      <c r="B87" s="34" t="n"/>
-      <c r="C87" s="63" t="n"/>
-      <c r="D87" s="65" t="n"/>
-      <c r="E87" s="63" t="n"/>
-      <c r="F87" s="66" t="n"/>
-      <c r="G87" s="67" t="n"/>
-      <c r="H87" s="6" t="inlineStr">
+    </row>
+    <row r="100" ht="14" customHeight="1">
+      <c r="B100" s="34" t="n"/>
+      <c r="C100" s="64" t="n"/>
+      <c r="D100" s="66" t="n"/>
+      <c r="E100" s="64" t="n"/>
+      <c r="F100" s="67" t="n"/>
+      <c r="G100" s="68" t="n"/>
+      <c r="H100" s="6" t="inlineStr">
         <is>
           <t>beam alone</t>
         </is>
       </c>
-      <c r="AN87" s="20" t="inlineStr">
-        <is>
-          <t>150UC23</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="14" customHeight="1">
-      <c r="B88" s="34" t="n"/>
-      <c r="C88" s="63" t="n"/>
-      <c r="D88" s="65" t="n"/>
-      <c r="E88" s="63" t="n"/>
-      <c r="F88" s="66" t="n"/>
-      <c r="G88" s="67" t="n"/>
-      <c r="AN88" s="20" t="inlineStr">
-        <is>
-          <t>100UC15</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="14" customHeight="1">
-      <c r="B89" s="34" t="n"/>
-      <c r="C89" s="63" t="n"/>
-      <c r="D89" s="65" t="n"/>
-      <c r="E89" s="63" t="n"/>
-      <c r="F89" s="66" t="n"/>
-      <c r="G89" s="67" t="n"/>
-    </row>
-    <row r="90" ht="14" customHeight="1">
-      <c r="B90" s="34" t="n"/>
-      <c r="C90" s="63" t="n"/>
-      <c r="D90" s="65" t="n"/>
-      <c r="E90" s="63" t="n"/>
-      <c r="F90" s="66" t="n"/>
-      <c r="G90" s="67" t="n"/>
-    </row>
-    <row r="91" ht="14" customHeight="1"/>
-    <row r="92" ht="14" customHeight="1">
-      <c r="B92" s="68" t="inlineStr">
+    </row>
+    <row r="101" ht="14" customHeight="1">
+      <c r="B101" s="34" t="n"/>
+      <c r="C101" s="64" t="n"/>
+      <c r="D101" s="66" t="n"/>
+      <c r="E101" s="64" t="n"/>
+      <c r="F101" s="67" t="n"/>
+      <c r="G101" s="68" t="n"/>
+    </row>
+    <row r="102" ht="14" customHeight="1">
+      <c r="B102" s="34" t="n"/>
+      <c r="C102" s="64" t="n"/>
+      <c r="D102" s="66" t="n"/>
+      <c r="E102" s="64" t="n"/>
+      <c r="F102" s="67" t="n"/>
+      <c r="G102" s="68" t="n"/>
+    </row>
+    <row r="103" ht="14" customHeight="1">
+      <c r="B103" s="34" t="n"/>
+      <c r="C103" s="64" t="n"/>
+      <c r="D103" s="66" t="n"/>
+      <c r="E103" s="64" t="n"/>
+      <c r="F103" s="67" t="n"/>
+      <c r="G103" s="68" t="n"/>
+    </row>
+    <row r="104" ht="14" customHeight="1"/>
+    <row r="105" ht="14" customHeight="1">
+      <c r="B105" s="63" t="inlineStr">
         <is>
           <t>Deflected shapes (mm, plotted downward;  x in m)</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="14" customHeight="1"/>
-    <row r="94" ht="14" customHeight="1"/>
-    <row r="95" ht="14" customHeight="1"/>
-    <row r="96" ht="14" customHeight="1"/>
-    <row r="97" ht="14" customHeight="1"/>
-    <row r="98" ht="14" customHeight="1"/>
-    <row r="99" ht="14" customHeight="1"/>
-    <row r="100" ht="14" customHeight="1"/>
-    <row r="101" ht="14" customHeight="1"/>
-    <row r="102" ht="14" customHeight="1"/>
-    <row r="103" ht="14" customHeight="1"/>
-    <row r="104" ht="14" customHeight="1"/>
-    <row r="105" ht="20" customHeight="1">
-      <c r="B105" s="10" t="inlineStr">
-        <is>
-          <t>ULS Strength Checks – Bending (AS 4100 Cl. 5.6)</t>
-        </is>
-      </c>
-      <c r="C105" s="11" t="n"/>
-      <c r="D105" s="11" t="n"/>
-      <c r="E105" s="11" t="n"/>
-      <c r="F105" s="11" t="n"/>
-      <c r="G105" s="11" t="n"/>
-      <c r="H105" s="11" t="n"/>
-      <c r="I105" s="11" t="n"/>
-      <c r="J105" s="11" t="n"/>
-    </row>
-    <row r="106" ht="14" customHeight="1">
-      <c r="B106" s="68" t="inlineStr">
-        <is>
-          <t>Bending moment envelope (kN·m, sagging down;  x in m)</t>
-        </is>
-      </c>
-      <c r="F106" s="68" t="inlineStr">
-        <is>
-          <t>Shear force envelope (kN;  x in m)</t>
-        </is>
-      </c>
-    </row>
+    <row r="106" ht="14" customHeight="1"/>
     <row r="107" ht="14" customHeight="1"/>
     <row r="108" ht="14" customHeight="1"/>
     <row r="109" ht="14" customHeight="1"/>
@@ -5202,325 +5398,300 @@
     <row r="115" ht="14" customHeight="1"/>
     <row r="116" ht="14" customHeight="1"/>
     <row r="117" ht="14" customHeight="1"/>
-    <row r="118" ht="14" customHeight="1"/>
-    <row r="119" ht="14" customHeight="1"/>
+    <row r="118" ht="20" customHeight="1">
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>ULS Strength Checks – Bending (AS 4100 Cl. 5.6)</t>
+        </is>
+      </c>
+      <c r="C118" s="11" t="n"/>
+      <c r="D118" s="11" t="n"/>
+      <c r="E118" s="11" t="n"/>
+      <c r="F118" s="11" t="n"/>
+      <c r="G118" s="11" t="n"/>
+      <c r="H118" s="11" t="n"/>
+      <c r="I118" s="11" t="n"/>
+      <c r="J118" s="11" t="n"/>
+    </row>
+    <row r="119" ht="14" customHeight="1">
+      <c r="B119" s="63" t="inlineStr">
+        <is>
+          <t>Bending moment envelope, all active combinations (kN·m, sagging plotted down;  x in m)</t>
+        </is>
+      </c>
+    </row>
     <row r="120" ht="14" customHeight="1"/>
-    <row r="121" ht="16" customHeight="1">
-      <c r="B121" s="59" t="inlineStr">
+    <row r="121" ht="14" customHeight="1"/>
+    <row r="122" ht="14" customHeight="1"/>
+    <row r="123" ht="14" customHeight="1"/>
+    <row r="124" ht="14" customHeight="1"/>
+    <row r="125" ht="14" customHeight="1"/>
+    <row r="126" ht="14" customHeight="1"/>
+    <row r="127" ht="14" customHeight="1"/>
+    <row r="128" ht="14" customHeight="1"/>
+    <row r="129" ht="14" customHeight="1"/>
+    <row r="130" ht="14" customHeight="1"/>
+    <row r="131" ht="14" customHeight="1"/>
+    <row r="132" ht="16" customHeight="1">
+      <c r="B132" s="59" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="C121" s="59" t="inlineStr">
+      <c r="C132" s="59" t="inlineStr">
         <is>
           <t>Segment (m)</t>
         </is>
       </c>
-      <c r="D121" s="59" t="inlineStr">
+      <c r="D132" s="59" t="inlineStr">
         <is>
           <t>Ends</t>
         </is>
       </c>
-      <c r="E121" s="59" t="inlineStr">
+      <c r="E132" s="59" t="inlineStr">
         <is>
           <t>Le (m)</t>
         </is>
       </c>
-      <c r="F121" s="59" t="inlineStr">
+      <c r="F132" s="59" t="inlineStr">
         <is>
           <t>αm</t>
         </is>
       </c>
-      <c r="G121" s="59" t="inlineStr">
+      <c r="G132" s="59" t="inlineStr">
         <is>
           <t>αs</t>
         </is>
       </c>
-      <c r="H121" s="59" t="inlineStr">
+      <c r="H132" s="59" t="inlineStr">
         <is>
           <t>φMb (kN·m)</t>
         </is>
       </c>
-      <c r="I121" s="59" t="inlineStr">
+      <c r="I132" s="59" t="inlineStr">
         <is>
           <t>M* (kN·m)</t>
         </is>
       </c>
-      <c r="J121" s="59" t="inlineStr">
+      <c r="J132" s="59" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
     </row>
-    <row r="122" ht="14" customHeight="1">
-      <c r="B122" s="34" cm="1">
-        <f t="array" ref="B122">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
-        <v/>
-      </c>
-      <c r="C122" s="34" t="n"/>
-      <c r="D122" s="34" t="n"/>
-      <c r="E122" s="63" t="n"/>
-      <c r="F122" s="69" t="n"/>
-      <c r="G122" s="69" t="n"/>
-      <c r="H122" s="70" t="n"/>
-      <c r="I122" s="70" t="n"/>
-      <c r="J122" s="67" t="n"/>
-    </row>
-    <row r="123" ht="14" customHeight="1">
-      <c r="B123" s="34" t="n"/>
-      <c r="C123" s="34" t="n"/>
-      <c r="D123" s="34" t="n"/>
-      <c r="E123" s="63" t="n"/>
-      <c r="F123" s="69" t="n"/>
-      <c r="G123" s="69" t="n"/>
-      <c r="H123" s="70" t="n"/>
-      <c r="I123" s="70" t="n"/>
-      <c r="J123" s="67" t="n"/>
-    </row>
-    <row r="124" ht="14" customHeight="1">
-      <c r="B124" s="34" t="n"/>
-      <c r="C124" s="34" t="n"/>
-      <c r="D124" s="34" t="n"/>
-      <c r="E124" s="63" t="n"/>
-      <c r="F124" s="69" t="n"/>
-      <c r="G124" s="69" t="n"/>
-      <c r="H124" s="70" t="n"/>
-      <c r="I124" s="70" t="n"/>
-      <c r="J124" s="67" t="n"/>
-    </row>
-    <row r="125" ht="14" customHeight="1">
-      <c r="B125" s="34" t="n"/>
-      <c r="C125" s="34" t="n"/>
-      <c r="D125" s="34" t="n"/>
-      <c r="E125" s="63" t="n"/>
-      <c r="F125" s="69" t="n"/>
-      <c r="G125" s="69" t="n"/>
-      <c r="H125" s="70" t="n"/>
-      <c r="I125" s="70" t="n"/>
-      <c r="J125" s="67" t="n"/>
-    </row>
-    <row r="126" ht="14" customHeight="1">
-      <c r="B126" s="34" t="n"/>
-      <c r="C126" s="34" t="n"/>
-      <c r="D126" s="34" t="n"/>
-      <c r="E126" s="63" t="n"/>
-      <c r="F126" s="69" t="n"/>
-      <c r="G126" s="69" t="n"/>
-      <c r="H126" s="70" t="n"/>
-      <c r="I126" s="70" t="n"/>
-      <c r="J126" s="67" t="n"/>
-    </row>
-    <row r="127" ht="14" customHeight="1">
-      <c r="B127" s="34" t="n"/>
-      <c r="C127" s="34" t="n"/>
-      <c r="D127" s="34" t="n"/>
-      <c r="E127" s="63" t="n"/>
-      <c r="F127" s="69" t="n"/>
-      <c r="G127" s="69" t="n"/>
-      <c r="H127" s="70" t="n"/>
-      <c r="I127" s="70" t="n"/>
-      <c r="J127" s="67" t="n"/>
-    </row>
-    <row r="128" ht="14" customHeight="1">
-      <c r="B128" s="34" t="n"/>
-      <c r="C128" s="34" t="n"/>
-      <c r="D128" s="34" t="n"/>
-      <c r="E128" s="63" t="n"/>
-      <c r="F128" s="69" t="n"/>
-      <c r="G128" s="69" t="n"/>
-      <c r="H128" s="70" t="n"/>
-      <c r="I128" s="70" t="n"/>
-      <c r="J128" s="67" t="n"/>
-    </row>
-    <row r="129" ht="14" customHeight="1">
-      <c r="B129" s="34" t="n"/>
-      <c r="C129" s="34" t="n"/>
-      <c r="D129" s="34" t="n"/>
-      <c r="E129" s="63" t="n"/>
-      <c r="F129" s="69" t="n"/>
-      <c r="G129" s="69" t="n"/>
-      <c r="H129" s="70" t="n"/>
-      <c r="I129" s="70" t="n"/>
-      <c r="J129" s="67" t="n"/>
-    </row>
-    <row r="130" ht="14" customHeight="1">
-      <c r="B130" s="34" t="n"/>
-      <c r="C130" s="34" t="n"/>
-      <c r="D130" s="34" t="n"/>
-      <c r="E130" s="63" t="n"/>
-      <c r="F130" s="69" t="n"/>
-      <c r="G130" s="69" t="n"/>
-      <c r="H130" s="70" t="n"/>
-      <c r="I130" s="70" t="n"/>
-      <c r="J130" s="67" t="n"/>
-    </row>
-    <row r="131" ht="14" customHeight="1">
-      <c r="B131" s="34" t="n"/>
-      <c r="C131" s="34" t="n"/>
-      <c r="D131" s="34" t="n"/>
-      <c r="E131" s="63" t="n"/>
-      <c r="F131" s="69" t="n"/>
-      <c r="G131" s="69" t="n"/>
-      <c r="H131" s="70" t="n"/>
-      <c r="I131" s="70" t="n"/>
-      <c r="J131" s="67" t="n"/>
-    </row>
-    <row r="132" ht="14" customHeight="1">
-      <c r="B132" s="34" t="n"/>
-      <c r="C132" s="34" t="n"/>
-      <c r="D132" s="34" t="n"/>
-      <c r="E132" s="63" t="n"/>
-      <c r="F132" s="69" t="n"/>
-      <c r="G132" s="69" t="n"/>
-      <c r="H132" s="70" t="n"/>
-      <c r="I132" s="70" t="n"/>
-      <c r="J132" s="67" t="n"/>
-    </row>
     <row r="133" ht="14" customHeight="1">
-      <c r="B133" s="34" t="n"/>
+      <c r="B133" s="34" cm="1">
+        <f t="array" ref="B133">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79),Restraints_B1[#Data],$I$90:$J$91)</f>
+        <v/>
+      </c>
       <c r="C133" s="34" t="n"/>
       <c r="D133" s="34" t="n"/>
-      <c r="E133" s="63" t="n"/>
+      <c r="E133" s="64" t="n"/>
       <c r="F133" s="69" t="n"/>
       <c r="G133" s="69" t="n"/>
       <c r="H133" s="70" t="n"/>
       <c r="I133" s="70" t="n"/>
-      <c r="J133" s="67" t="n"/>
+      <c r="J133" s="68" t="n"/>
     </row>
     <row r="134" ht="14" customHeight="1">
       <c r="B134" s="34" t="n"/>
       <c r="C134" s="34" t="n"/>
       <c r="D134" s="34" t="n"/>
-      <c r="E134" s="63" t="n"/>
+      <c r="E134" s="64" t="n"/>
       <c r="F134" s="69" t="n"/>
       <c r="G134" s="69" t="n"/>
       <c r="H134" s="70" t="n"/>
       <c r="I134" s="70" t="n"/>
-      <c r="J134" s="67" t="n"/>
+      <c r="J134" s="68" t="n"/>
     </row>
     <row r="135" ht="14" customHeight="1">
       <c r="B135" s="34" t="n"/>
       <c r="C135" s="34" t="n"/>
       <c r="D135" s="34" t="n"/>
-      <c r="E135" s="63" t="n"/>
+      <c r="E135" s="64" t="n"/>
       <c r="F135" s="69" t="n"/>
       <c r="G135" s="69" t="n"/>
       <c r="H135" s="70" t="n"/>
       <c r="I135" s="70" t="n"/>
-      <c r="J135" s="67" t="n"/>
+      <c r="J135" s="68" t="n"/>
     </row>
     <row r="136" ht="14" customHeight="1">
       <c r="B136" s="34" t="n"/>
       <c r="C136" s="34" t="n"/>
       <c r="D136" s="34" t="n"/>
-      <c r="E136" s="63" t="n"/>
+      <c r="E136" s="64" t="n"/>
       <c r="F136" s="69" t="n"/>
       <c r="G136" s="69" t="n"/>
       <c r="H136" s="70" t="n"/>
       <c r="I136" s="70" t="n"/>
-      <c r="J136" s="67" t="n"/>
+      <c r="J136" s="68" t="n"/>
     </row>
     <row r="137" ht="14" customHeight="1">
       <c r="B137" s="34" t="n"/>
       <c r="C137" s="34" t="n"/>
       <c r="D137" s="34" t="n"/>
-      <c r="E137" s="63" t="n"/>
+      <c r="E137" s="64" t="n"/>
       <c r="F137" s="69" t="n"/>
       <c r="G137" s="69" t="n"/>
       <c r="H137" s="70" t="n"/>
       <c r="I137" s="70" t="n"/>
-      <c r="J137" s="67" t="n"/>
+      <c r="J137" s="68" t="n"/>
     </row>
     <row r="138" ht="14" customHeight="1">
-      <c r="B138" s="15" t="inlineStr">
+      <c r="B138" s="34" t="n"/>
+      <c r="C138" s="34" t="n"/>
+      <c r="D138" s="34" t="n"/>
+      <c r="E138" s="64" t="n"/>
+      <c r="F138" s="69" t="n"/>
+      <c r="G138" s="69" t="n"/>
+      <c r="H138" s="70" t="n"/>
+      <c r="I138" s="70" t="n"/>
+      <c r="J138" s="68" t="n"/>
+    </row>
+    <row r="139" ht="14" customHeight="1">
+      <c r="B139" s="34" t="n"/>
+      <c r="C139" s="34" t="n"/>
+      <c r="D139" s="34" t="n"/>
+      <c r="E139" s="64" t="n"/>
+      <c r="F139" s="69" t="n"/>
+      <c r="G139" s="69" t="n"/>
+      <c r="H139" s="70" t="n"/>
+      <c r="I139" s="70" t="n"/>
+      <c r="J139" s="68" t="n"/>
+    </row>
+    <row r="140">
+      <c r="B140" s="34" t="n"/>
+      <c r="C140" s="34" t="n"/>
+      <c r="D140" s="34" t="n"/>
+      <c r="E140" s="64" t="n"/>
+      <c r="F140" s="69" t="n"/>
+      <c r="G140" s="69" t="n"/>
+      <c r="H140" s="70" t="n"/>
+      <c r="I140" s="70" t="n"/>
+      <c r="J140" s="68" t="n"/>
+    </row>
+    <row r="141">
+      <c r="B141" s="34" t="n"/>
+      <c r="C141" s="34" t="n"/>
+      <c r="D141" s="34" t="n"/>
+      <c r="E141" s="64" t="n"/>
+      <c r="F141" s="69" t="n"/>
+      <c r="G141" s="69" t="n"/>
+      <c r="H141" s="70" t="n"/>
+      <c r="I141" s="70" t="n"/>
+      <c r="J141" s="68" t="n"/>
+    </row>
+    <row r="142">
+      <c r="B142" s="34" t="n"/>
+      <c r="C142" s="34" t="n"/>
+      <c r="D142" s="34" t="n"/>
+      <c r="E142" s="64" t="n"/>
+      <c r="F142" s="69" t="n"/>
+      <c r="G142" s="69" t="n"/>
+      <c r="H142" s="70" t="n"/>
+      <c r="I142" s="70" t="n"/>
+      <c r="J142" s="68" t="n"/>
+    </row>
+    <row r="143">
+      <c r="B143" s="34" t="n"/>
+      <c r="C143" s="34" t="n"/>
+      <c r="D143" s="34" t="n"/>
+      <c r="E143" s="64" t="n"/>
+      <c r="F143" s="69" t="n"/>
+      <c r="G143" s="69" t="n"/>
+      <c r="H143" s="70" t="n"/>
+      <c r="I143" s="70" t="n"/>
+      <c r="J143" s="68" t="n"/>
+    </row>
+    <row r="144">
+      <c r="B144" s="34" t="n"/>
+      <c r="C144" s="34" t="n"/>
+      <c r="D144" s="34" t="n"/>
+      <c r="E144" s="64" t="n"/>
+      <c r="F144" s="69" t="n"/>
+      <c r="G144" s="69" t="n"/>
+      <c r="H144" s="70" t="n"/>
+      <c r="I144" s="70" t="n"/>
+      <c r="J144" s="68" t="n"/>
+    </row>
+    <row r="145">
+      <c r="B145" s="34" t="n"/>
+      <c r="C145" s="34" t="n"/>
+      <c r="D145" s="34" t="n"/>
+      <c r="E145" s="64" t="n"/>
+      <c r="F145" s="69" t="n"/>
+      <c r="G145" s="69" t="n"/>
+      <c r="H145" s="70" t="n"/>
+      <c r="I145" s="70" t="n"/>
+      <c r="J145" s="68" t="n"/>
+    </row>
+    <row r="146">
+      <c r="B146" s="34" t="n"/>
+      <c r="C146" s="34" t="n"/>
+      <c r="D146" s="34" t="n"/>
+      <c r="E146" s="64" t="n"/>
+      <c r="F146" s="69" t="n"/>
+      <c r="G146" s="69" t="n"/>
+      <c r="H146" s="70" t="n"/>
+      <c r="I146" s="70" t="n"/>
+      <c r="J146" s="68" t="n"/>
+    </row>
+    <row r="147">
+      <c r="B147" s="34" t="n"/>
+      <c r="C147" s="34" t="n"/>
+      <c r="D147" s="34" t="n"/>
+      <c r="E147" s="64" t="n"/>
+      <c r="F147" s="69" t="n"/>
+      <c r="G147" s="69" t="n"/>
+      <c r="H147" s="70" t="n"/>
+      <c r="I147" s="70" t="n"/>
+      <c r="J147" s="68" t="n"/>
+    </row>
+    <row r="148">
+      <c r="B148" s="34" t="n"/>
+      <c r="C148" s="34" t="n"/>
+      <c r="D148" s="34" t="n"/>
+      <c r="E148" s="64" t="n"/>
+      <c r="F148" s="69" t="n"/>
+      <c r="G148" s="69" t="n"/>
+      <c r="H148" s="70" t="n"/>
+      <c r="I148" s="70" t="n"/>
+      <c r="J148" s="68" t="n"/>
+    </row>
+    <row r="149">
+      <c r="B149" s="15" t="inlineStr">
         <is>
           <t>* αm overridden in the restraints table.  Full working for the governing segment follows.</t>
         </is>
       </c>
     </row>
-    <row r="139" ht="14" customHeight="1"/>
-    <row r="140" ht="20" customHeight="1">
-      <c r="B140" s="10" t="inlineStr">
+    <row r="151" ht="20" customHeight="1">
+      <c r="B151" s="10" t="inlineStr">
         <is>
           <t>Governing Segment – Working</t>
         </is>
       </c>
-      <c r="C140" s="11" t="n"/>
-      <c r="D140" s="11" t="n"/>
-      <c r="E140" s="11" t="n"/>
-      <c r="F140" s="11" t="n"/>
-      <c r="G140" s="11" t="n"/>
-      <c r="H140" s="11" t="n"/>
-      <c r="I140" s="11" t="n"/>
-      <c r="J140" s="11" t="n"/>
-    </row>
-    <row r="141">
-      <c r="B141" s="15" t="inlineStr">
+      <c r="C151" s="11" t="n"/>
+      <c r="D151" s="11" t="n"/>
+      <c r="E151" s="11" t="n"/>
+      <c r="F151" s="11" t="n"/>
+      <c r="G151" s="11" t="n"/>
+      <c r="H151" s="11" t="n"/>
+      <c r="I151" s="11" t="n"/>
+      <c r="J151" s="11" t="n"/>
+    </row>
+    <row r="152">
+      <c r="B152" s="15" t="inlineStr">
         <is>
           <t>OAR.ULSDETAIL: change the comboId / segment arguments to show any other segment.</t>
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="D142" s="71" cm="1">
-        <f t="array" ref="D142">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
-        <v/>
-      </c>
-      <c r="E142" s="72" t="n"/>
-      <c r="F142" s="35" t="n"/>
-    </row>
-    <row r="143">
-      <c r="D143" s="71" t="n"/>
-      <c r="E143" s="72" t="n"/>
-      <c r="F143" s="35" t="n"/>
-    </row>
-    <row r="144">
-      <c r="D144" s="71" t="n"/>
-      <c r="E144" s="72" t="n"/>
-      <c r="F144" s="35" t="n"/>
-    </row>
-    <row r="145">
-      <c r="D145" s="71" t="n"/>
-      <c r="E145" s="72" t="n"/>
-      <c r="F145" s="35" t="n"/>
-    </row>
-    <row r="146">
-      <c r="D146" s="71" t="n"/>
-      <c r="E146" s="72" t="n"/>
-      <c r="F146" s="35" t="n"/>
-    </row>
-    <row r="147">
-      <c r="D147" s="71" t="n"/>
-      <c r="E147" s="72" t="n"/>
-      <c r="F147" s="35" t="n"/>
-    </row>
-    <row r="148">
-      <c r="D148" s="71" t="n"/>
-      <c r="E148" s="72" t="n"/>
-      <c r="F148" s="35" t="n"/>
-    </row>
-    <row r="149">
-      <c r="D149" s="71" t="n"/>
-      <c r="E149" s="72" t="n"/>
-      <c r="F149" s="35" t="n"/>
-    </row>
-    <row r="150">
-      <c r="D150" s="71" t="n"/>
-      <c r="E150" s="72" t="n"/>
-      <c r="F150" s="35" t="n"/>
-    </row>
-    <row r="151">
-      <c r="D151" s="71" t="n"/>
-      <c r="E151" s="72" t="n"/>
-      <c r="F151" s="35" t="n"/>
-    </row>
-    <row r="152">
-      <c r="D152" s="71" t="n"/>
-      <c r="E152" s="72" t="n"/>
-      <c r="F152" s="35" t="n"/>
-    </row>
     <row r="153">
-      <c r="D153" s="71" t="n"/>
+      <c r="D153" s="71" cm="1">
+        <f t="array" ref="D153">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79),Restraints_B1[#Data],$I$90:$J$91)</f>
+        <v/>
+      </c>
       <c r="E153" s="72" t="n"/>
       <c r="F153" s="35" t="n"/>
     </row>
@@ -5574,124 +5745,65 @@
       <c r="E163" s="72" t="n"/>
       <c r="F163" s="35" t="n"/>
     </row>
-    <row r="165" ht="20" customHeight="1">
-      <c r="B165" s="10" t="inlineStr">
-        <is>
-          <t>Shear (AS 4100 Cl. 5.11)</t>
-        </is>
-      </c>
-      <c r="C165" s="11" t="n"/>
-      <c r="D165" s="11" t="n"/>
-      <c r="E165" s="11" t="n"/>
-      <c r="F165" s="11" t="n"/>
-      <c r="G165" s="11" t="n"/>
-      <c r="H165" s="11" t="n"/>
-      <c r="I165" s="11" t="n"/>
-      <c r="J165" s="11" t="n"/>
+    <row r="164">
+      <c r="D164" s="71" t="n"/>
+      <c r="E164" s="72" t="n"/>
+      <c r="F164" s="35" t="n"/>
+    </row>
+    <row r="165">
+      <c r="D165" s="71" t="n"/>
+      <c r="E165" s="72" t="n"/>
+      <c r="F165" s="35" t="n"/>
     </row>
     <row r="166">
-      <c r="B166" s="59" t="inlineStr">
-        <is>
-          <t>Combo</t>
-        </is>
-      </c>
-      <c r="C166" s="59" t="inlineStr">
-        <is>
-          <t>V* (kN)</t>
-        </is>
-      </c>
-      <c r="D166" s="59" t="inlineStr">
-        <is>
-          <t>at x (m)</t>
-        </is>
-      </c>
-      <c r="E166" s="59" t="inlineStr">
-        <is>
-          <t>φVv (kN)</t>
-        </is>
-      </c>
-      <c r="F166" s="59" t="inlineStr">
-        <is>
-          <t>Utilisation</t>
-        </is>
-      </c>
-      <c r="G166" s="59" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
+      <c r="D166" s="71" t="n"/>
+      <c r="E166" s="72" t="n"/>
+      <c r="F166" s="35" t="n"/>
     </row>
     <row r="167">
-      <c r="B167" s="34" cm="1">
-        <f t="array" ref="B167">OAR.SHEAR(SectionSize,Grade,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
-        <v/>
-      </c>
-      <c r="C167" s="70" t="n"/>
-      <c r="D167" s="63" t="n"/>
-      <c r="E167" s="70" t="n"/>
-      <c r="F167" s="67" t="n"/>
-      <c r="G167" s="73" t="n"/>
+      <c r="D167" s="71" t="n"/>
+      <c r="E167" s="72" t="n"/>
+      <c r="F167" s="35" t="n"/>
     </row>
     <row r="168">
-      <c r="B168" s="34" t="n"/>
-      <c r="C168" s="70" t="n"/>
-      <c r="D168" s="63" t="n"/>
-      <c r="E168" s="70" t="n"/>
-      <c r="F168" s="67" t="n"/>
-      <c r="G168" s="73" t="n"/>
+      <c r="D168" s="71" t="n"/>
+      <c r="E168" s="72" t="n"/>
+      <c r="F168" s="35" t="n"/>
     </row>
     <row r="169">
-      <c r="B169" s="34" t="n"/>
-      <c r="C169" s="70" t="n"/>
-      <c r="D169" s="63" t="n"/>
-      <c r="E169" s="70" t="n"/>
-      <c r="F169" s="67" t="n"/>
-      <c r="G169" s="73" t="n"/>
+      <c r="D169" s="71" t="n"/>
+      <c r="E169" s="72" t="n"/>
+      <c r="F169" s="35" t="n"/>
     </row>
     <row r="170">
-      <c r="B170" s="34" t="n"/>
-      <c r="C170" s="70" t="n"/>
-      <c r="D170" s="63" t="n"/>
-      <c r="E170" s="70" t="n"/>
-      <c r="F170" s="67" t="n"/>
-      <c r="G170" s="73" t="n"/>
+      <c r="D170" s="71" t="n"/>
+      <c r="E170" s="72" t="n"/>
+      <c r="F170" s="35" t="n"/>
     </row>
     <row r="171">
-      <c r="B171" s="34" t="n"/>
-      <c r="C171" s="70" t="n"/>
-      <c r="D171" s="63" t="n"/>
-      <c r="E171" s="70" t="n"/>
-      <c r="F171" s="67" t="n"/>
-      <c r="G171" s="73" t="n"/>
+      <c r="D171" s="71" t="n"/>
+      <c r="E171" s="72" t="n"/>
+      <c r="F171" s="35" t="n"/>
     </row>
     <row r="172">
-      <c r="B172" s="34" t="n"/>
-      <c r="C172" s="70" t="n"/>
-      <c r="D172" s="63" t="n"/>
-      <c r="E172" s="70" t="n"/>
-      <c r="F172" s="67" t="n"/>
-      <c r="G172" s="73" t="n"/>
+      <c r="D172" s="71" t="n"/>
+      <c r="E172" s="72" t="n"/>
+      <c r="F172" s="35" t="n"/>
     </row>
     <row r="173">
-      <c r="B173" s="34" t="n"/>
-      <c r="C173" s="70" t="n"/>
-      <c r="D173" s="63" t="n"/>
-      <c r="E173" s="70" t="n"/>
-      <c r="F173" s="67" t="n"/>
-      <c r="G173" s="73" t="n"/>
+      <c r="D173" s="71" t="n"/>
+      <c r="E173" s="72" t="n"/>
+      <c r="F173" s="35" t="n"/>
     </row>
     <row r="174">
-      <c r="B174" s="34" t="n"/>
-      <c r="C174" s="70" t="n"/>
-      <c r="D174" s="63" t="n"/>
-      <c r="E174" s="70" t="n"/>
-      <c r="F174" s="67" t="n"/>
-      <c r="G174" s="73" t="n"/>
+      <c r="D174" s="71" t="n"/>
+      <c r="E174" s="72" t="n"/>
+      <c r="F174" s="35" t="n"/>
     </row>
     <row r="176" ht="20" customHeight="1">
       <c r="B176" s="10" t="inlineStr">
         <is>
-          <t>Support Reactions</t>
+          <t>Shear (AS 4100 Cl. 5.11)</t>
         </is>
       </c>
       <c r="C176" s="11" t="n"/>
@@ -5704,296 +5816,410 @@
       <c r="J176" s="11" t="n"/>
     </row>
     <row r="177">
-      <c r="B177" s="15" t="inlineStr">
+      <c r="B177" s="59" t="inlineStr">
+        <is>
+          <t>Combo</t>
+        </is>
+      </c>
+      <c r="C177" s="59" t="inlineStr">
+        <is>
+          <t>V* (kN)</t>
+        </is>
+      </c>
+      <c r="D177" s="59" t="inlineStr">
+        <is>
+          <t>at x (m)</t>
+        </is>
+      </c>
+      <c r="E177" s="59" t="inlineStr">
+        <is>
+          <t>φVv (kN)</t>
+        </is>
+      </c>
+      <c r="F177" s="59" t="inlineStr">
+        <is>
+          <t>Utilisation</t>
+        </is>
+      </c>
+      <c r="G177" s="59" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="B178" s="34" cm="1">
+        <f t="array" ref="B178">OAR.SHEAR(SectionSize,Grade,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79))</f>
+        <v/>
+      </c>
+      <c r="C178" s="70" t="n"/>
+      <c r="D178" s="64" t="n"/>
+      <c r="E178" s="70" t="n"/>
+      <c r="F178" s="68" t="n"/>
+      <c r="G178" s="73" t="n"/>
+    </row>
+    <row r="179">
+      <c r="B179" s="34" t="n"/>
+      <c r="C179" s="70" t="n"/>
+      <c r="D179" s="64" t="n"/>
+      <c r="E179" s="70" t="n"/>
+      <c r="F179" s="68" t="n"/>
+      <c r="G179" s="73" t="n"/>
+    </row>
+    <row r="180">
+      <c r="B180" s="34" t="n"/>
+      <c r="C180" s="70" t="n"/>
+      <c r="D180" s="64" t="n"/>
+      <c r="E180" s="70" t="n"/>
+      <c r="F180" s="68" t="n"/>
+      <c r="G180" s="73" t="n"/>
+    </row>
+    <row r="181">
+      <c r="B181" s="34" t="n"/>
+      <c r="C181" s="70" t="n"/>
+      <c r="D181" s="64" t="n"/>
+      <c r="E181" s="70" t="n"/>
+      <c r="F181" s="68" t="n"/>
+      <c r="G181" s="73" t="n"/>
+    </row>
+    <row r="182">
+      <c r="B182" s="34" t="n"/>
+      <c r="C182" s="70" t="n"/>
+      <c r="D182" s="64" t="n"/>
+      <c r="E182" s="70" t="n"/>
+      <c r="F182" s="68" t="n"/>
+      <c r="G182" s="73" t="n"/>
+    </row>
+    <row r="183">
+      <c r="B183" s="34" t="n"/>
+      <c r="C183" s="70" t="n"/>
+      <c r="D183" s="64" t="n"/>
+      <c r="E183" s="70" t="n"/>
+      <c r="F183" s="68" t="n"/>
+      <c r="G183" s="73" t="n"/>
+    </row>
+    <row r="184">
+      <c r="B184" s="34" t="n"/>
+      <c r="C184" s="70" t="n"/>
+      <c r="D184" s="64" t="n"/>
+      <c r="E184" s="70" t="n"/>
+      <c r="F184" s="68" t="n"/>
+      <c r="G184" s="73" t="n"/>
+    </row>
+    <row r="185">
+      <c r="B185" s="34" t="n"/>
+      <c r="C185" s="70" t="n"/>
+      <c r="D185" s="64" t="n"/>
+      <c r="E185" s="70" t="n"/>
+      <c r="F185" s="68" t="n"/>
+      <c r="G185" s="73" t="n"/>
+    </row>
+    <row r="187" ht="20" customHeight="1">
+      <c r="B187" s="10" t="inlineStr">
+        <is>
+          <t>Support Reactions</t>
+        </is>
+      </c>
+      <c r="C187" s="11" t="n"/>
+      <c r="D187" s="11" t="n"/>
+      <c r="E187" s="11" t="n"/>
+      <c r="F187" s="11" t="n"/>
+      <c r="G187" s="11" t="n"/>
+      <c r="H187" s="11" t="n"/>
+      <c r="I187" s="11" t="n"/>
+      <c r="J187" s="11" t="n"/>
+    </row>
+    <row r="188">
+      <c r="B188" s="15" t="inlineStr">
         <is>
           <t>Unfactored, per case, positive in the case direction (Wu/Wiu = uplift). Self-weight is in G.  To load another beam: add a Point row with the same case and set Direct to e.g. ='B1'!RxnR_G</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="B178" s="25" t="inlineStr">
+    <row r="189">
+      <c r="B189" s="25" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="D178" s="25" t="inlineStr">
+      <c r="D189" s="25" t="inlineStr">
         <is>
           <t>Left (kN)</t>
         </is>
       </c>
-      <c r="E178" s="25" t="inlineStr">
+      <c r="E189" s="25" t="inlineStr">
         <is>
           <t>Right (kN)</t>
         </is>
       </c>
-      <c r="F178" s="25" t="inlineStr">
+      <c r="F189" s="25" t="inlineStr">
         <is>
           <t>Transfer names</t>
         </is>
       </c>
     </row>
-    <row r="179">
-      <c r="B179" s="51" t="inlineStr">
+    <row r="190">
+      <c r="B190" s="51" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="C179" s="52" t="n"/>
-      <c r="D179" s="36" cm="1">
-        <f t="array" ref="D179">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,2)</f>
-        <v/>
-      </c>
-      <c r="E179" s="36" cm="1">
-        <f t="array" ref="E179">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,3)</f>
-        <v/>
-      </c>
-      <c r="F179" s="21" t="inlineStr">
+      <c r="C190" s="52" t="n"/>
+      <c r="D190" s="36" cm="1">
+        <f t="array" ref="D190">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),1,2)</f>
+        <v/>
+      </c>
+      <c r="E190" s="36" cm="1">
+        <f t="array" ref="E190">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),1,3)</f>
+        <v/>
+      </c>
+      <c r="F190" s="21" t="inlineStr">
         <is>
           <t>RxnL_G  ·  RxnR_G</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="B180" s="51" t="inlineStr">
+    <row r="191">
+      <c r="B191" s="51" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="C180" s="52" t="n"/>
-      <c r="D180" s="36" cm="1">
-        <f t="array" ref="D180">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,2)</f>
-        <v/>
-      </c>
-      <c r="E180" s="36" cm="1">
-        <f t="array" ref="E180">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,3)</f>
-        <v/>
-      </c>
-      <c r="F180" s="21" t="inlineStr">
+      <c r="C191" s="52" t="n"/>
+      <c r="D191" s="36" cm="1">
+        <f t="array" ref="D191">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),2,2)</f>
+        <v/>
+      </c>
+      <c r="E191" s="36" cm="1">
+        <f t="array" ref="E191">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),2,3)</f>
+        <v/>
+      </c>
+      <c r="F191" s="21" t="inlineStr">
         <is>
           <t>RxnL_Q  ·  RxnR_Q</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="B181" s="51" t="inlineStr">
+    <row r="192">
+      <c r="B192" s="51" t="inlineStr">
         <is>
           <t>Wd</t>
         </is>
       </c>
-      <c r="C181" s="52" t="n"/>
-      <c r="D181" s="36" cm="1">
-        <f t="array" ref="D181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,2)</f>
-        <v/>
-      </c>
-      <c r="E181" s="36" cm="1">
-        <f t="array" ref="E181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,3)</f>
-        <v/>
-      </c>
-      <c r="F181" s="21" t="inlineStr">
+      <c r="C192" s="52" t="n"/>
+      <c r="D192" s="36" cm="1">
+        <f t="array" ref="D192">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),3,2)</f>
+        <v/>
+      </c>
+      <c r="E192" s="36" cm="1">
+        <f t="array" ref="E192">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),3,3)</f>
+        <v/>
+      </c>
+      <c r="F192" s="21" t="inlineStr">
         <is>
           <t>RxnL_Wd  ·  RxnR_Wd</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="B182" s="51" t="inlineStr">
+    <row r="193">
+      <c r="B193" s="51" t="inlineStr">
         <is>
           <t>Wu</t>
         </is>
       </c>
-      <c r="C182" s="52" t="n"/>
-      <c r="D182" s="36" cm="1">
-        <f t="array" ref="D182">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,2)</f>
-        <v/>
-      </c>
-      <c r="E182" s="36" cm="1">
-        <f t="array" ref="E182">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,3)</f>
-        <v/>
-      </c>
-      <c r="F182" s="21" t="inlineStr">
+      <c r="C193" s="52" t="n"/>
+      <c r="D193" s="36" cm="1">
+        <f t="array" ref="D193">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),4,2)</f>
+        <v/>
+      </c>
+      <c r="E193" s="36" cm="1">
+        <f t="array" ref="E193">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),4,3)</f>
+        <v/>
+      </c>
+      <c r="F193" s="21" t="inlineStr">
         <is>
           <t>RxnL_Wu  ·  RxnR_Wu</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="B183" s="51" t="inlineStr">
+    <row r="194">
+      <c r="B194" s="51" t="inlineStr">
         <is>
           <t>Wid</t>
         </is>
       </c>
-      <c r="C183" s="52" t="n"/>
-      <c r="D183" s="36" cm="1">
-        <f t="array" ref="D183">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,2)</f>
-        <v/>
-      </c>
-      <c r="E183" s="36" cm="1">
-        <f t="array" ref="E183">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,3)</f>
-        <v/>
-      </c>
-      <c r="F183" s="21" t="inlineStr">
+      <c r="C194" s="52" t="n"/>
+      <c r="D194" s="36" cm="1">
+        <f t="array" ref="D194">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),5,2)</f>
+        <v/>
+      </c>
+      <c r="E194" s="36" cm="1">
+        <f t="array" ref="E194">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),5,3)</f>
+        <v/>
+      </c>
+      <c r="F194" s="21" t="inlineStr">
         <is>
           <t>RxnL_Wid  ·  RxnR_Wid</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="B184" s="51" t="inlineStr">
+    <row r="195">
+      <c r="B195" s="51" t="inlineStr">
         <is>
           <t>Wiu</t>
         </is>
       </c>
-      <c r="C184" s="52" t="n"/>
-      <c r="D184" s="36" cm="1">
-        <f t="array" ref="D184">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,2)</f>
-        <v/>
-      </c>
-      <c r="E184" s="36" cm="1">
-        <f t="array" ref="E184">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,3)</f>
-        <v/>
-      </c>
-      <c r="F184" s="21" t="inlineStr">
+      <c r="C195" s="52" t="n"/>
+      <c r="D195" s="36" cm="1">
+        <f t="array" ref="D195">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),6,2)</f>
+        <v/>
+      </c>
+      <c r="E195" s="36" cm="1">
+        <f t="array" ref="E195">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),6,3)</f>
+        <v/>
+      </c>
+      <c r="F195" s="21" t="inlineStr">
         <is>
           <t>RxnL_Wiu  ·  RxnR_Wiu</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="B186" s="15" t="inlineStr">
+    <row r="197">
+      <c r="B197" s="15" t="inlineStr">
         <is>
           <t>All cases and active combinations (kN, + = upward reaction; uplift cases show negative)</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="B187" s="59" t="inlineStr">
+    <row r="198">
+      <c r="B198" s="59" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C187" s="59" t="inlineStr">
+      <c r="C198" s="59" t="inlineStr">
         <is>
           <t>Left (kN)</t>
         </is>
       </c>
-      <c r="D187" s="59" t="inlineStr">
+      <c r="D198" s="59" t="inlineStr">
         <is>
           <t>Right (kN)</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="B188" s="34" cm="1">
-        <f t="array" ref="B188">OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
-        <v/>
-      </c>
-      <c r="C188" s="63" t="n"/>
-      <c r="D188" s="63" t="n"/>
-    </row>
-    <row r="189">
-      <c r="B189" s="34" t="n"/>
-      <c r="C189" s="63" t="n"/>
-      <c r="D189" s="63" t="n"/>
-    </row>
-    <row r="190">
-      <c r="B190" s="34" t="n"/>
-      <c r="C190" s="63" t="n"/>
-      <c r="D190" s="63" t="n"/>
-    </row>
-    <row r="191">
-      <c r="B191" s="34" t="n"/>
-      <c r="C191" s="63" t="n"/>
-      <c r="D191" s="63" t="n"/>
-    </row>
-    <row r="192">
-      <c r="B192" s="34" t="n"/>
-      <c r="C192" s="63" t="n"/>
-      <c r="D192" s="63" t="n"/>
-    </row>
-    <row r="193">
-      <c r="B193" s="34" t="n"/>
-      <c r="C193" s="63" t="n"/>
-      <c r="D193" s="63" t="n"/>
-    </row>
-    <row r="194">
-      <c r="B194" s="34" t="n"/>
-      <c r="C194" s="63" t="n"/>
-      <c r="D194" s="63" t="n"/>
-    </row>
-    <row r="195">
-      <c r="B195" s="34" t="n"/>
-      <c r="C195" s="63" t="n"/>
-      <c r="D195" s="63" t="n"/>
-    </row>
-    <row r="196">
-      <c r="B196" s="34" t="n"/>
-      <c r="C196" s="63" t="n"/>
-      <c r="D196" s="63" t="n"/>
-    </row>
-    <row r="197">
-      <c r="B197" s="34" t="n"/>
-      <c r="C197" s="63" t="n"/>
-      <c r="D197" s="63" t="n"/>
-    </row>
-    <row r="198">
-      <c r="B198" s="34" t="n"/>
-      <c r="C198" s="63" t="n"/>
-      <c r="D198" s="63" t="n"/>
-    </row>
     <row r="199">
-      <c r="B199" s="34" t="n"/>
-      <c r="C199" s="63" t="n"/>
-      <c r="D199" s="63" t="n"/>
+      <c r="B199" s="34" cm="1">
+        <f t="array" ref="B199">OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79))</f>
+        <v/>
+      </c>
+      <c r="C199" s="64" t="n"/>
+      <c r="D199" s="64" t="n"/>
     </row>
     <row r="200">
       <c r="B200" s="34" t="n"/>
-      <c r="C200" s="63" t="n"/>
-      <c r="D200" s="63" t="n"/>
+      <c r="C200" s="64" t="n"/>
+      <c r="D200" s="64" t="n"/>
     </row>
     <row r="201">
       <c r="B201" s="34" t="n"/>
-      <c r="C201" s="63" t="n"/>
-      <c r="D201" s="63" t="n"/>
+      <c r="C201" s="64" t="n"/>
+      <c r="D201" s="64" t="n"/>
+    </row>
+    <row r="202">
+      <c r="B202" s="34" t="n"/>
+      <c r="C202" s="64" t="n"/>
+      <c r="D202" s="64" t="n"/>
+    </row>
+    <row r="203">
+      <c r="B203" s="34" t="n"/>
+      <c r="C203" s="64" t="n"/>
+      <c r="D203" s="64" t="n"/>
+    </row>
+    <row r="204">
+      <c r="B204" s="34" t="n"/>
+      <c r="C204" s="64" t="n"/>
+      <c r="D204" s="64" t="n"/>
+    </row>
+    <row r="205">
+      <c r="B205" s="34" t="n"/>
+      <c r="C205" s="64" t="n"/>
+      <c r="D205" s="64" t="n"/>
+    </row>
+    <row r="206">
+      <c r="B206" s="34" t="n"/>
+      <c r="C206" s="64" t="n"/>
+      <c r="D206" s="64" t="n"/>
+    </row>
+    <row r="207">
+      <c r="B207" s="34" t="n"/>
+      <c r="C207" s="64" t="n"/>
+      <c r="D207" s="64" t="n"/>
+    </row>
+    <row r="208">
+      <c r="B208" s="34" t="n"/>
+      <c r="C208" s="64" t="n"/>
+      <c r="D208" s="64" t="n"/>
+    </row>
+    <row r="209">
+      <c r="B209" s="34" t="n"/>
+      <c r="C209" s="64" t="n"/>
+      <c r="D209" s="64" t="n"/>
+    </row>
+    <row r="210">
+      <c r="B210" s="34" t="n"/>
+      <c r="C210" s="64" t="n"/>
+      <c r="D210" s="64" t="n"/>
+    </row>
+    <row r="211">
+      <c r="B211" s="34" t="n"/>
+      <c r="C211" s="64" t="n"/>
+      <c r="D211" s="64" t="n"/>
+    </row>
+    <row r="212">
+      <c r="B212" s="34" t="n"/>
+      <c r="C212" s="64" t="n"/>
+      <c r="D212" s="64" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="F182:G182"/>
     <mergeCell ref="B16:C16"/>
-    <mergeCell ref="F178:G178"/>
+    <mergeCell ref="F191:G191"/>
     <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F183:G183"/>
+    <mergeCell ref="B194:C194"/>
+    <mergeCell ref="B190:C190"/>
     <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B193:C193"/>
+    <mergeCell ref="F193:G193"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B184:C184"/>
-    <mergeCell ref="B180:C180"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B39:C39"/>
+    <mergeCell ref="F192:G192"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="M8:T40"/>
+    <mergeCell ref="B195:C195"/>
+    <mergeCell ref="F189:G189"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="G2:J2"/>
-    <mergeCell ref="B179:C179"/>
+    <mergeCell ref="F194:G194"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B181:C181"/>
-    <mergeCell ref="F181:G181"/>
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B182:C182"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="E30:F30"/>
+    <mergeCell ref="B191:C191"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B178:C178"/>
-    <mergeCell ref="F180:G180"/>
-    <mergeCell ref="F184:G184"/>
+    <mergeCell ref="F190:G190"/>
     <mergeCell ref="B40:C40"/>
-    <mergeCell ref="F179:G179"/>
     <mergeCell ref="I1:J1"/>
-    <mergeCell ref="B183:C183"/>
+    <mergeCell ref="B192:C192"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="B15:C15"/>
+    <mergeCell ref="F195:G195"/>
     <mergeCell ref="I10:J10"/>
+    <mergeCell ref="B189:C189"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="I9:J9"/>
@@ -6041,9 +6267,9 @@
       <formula>$C47="Point"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B66:J73">
+  <conditionalFormatting sqref="B79:J86">
     <cfRule type="expression" priority="10" dxfId="7">
-      <formula>$B66&lt;&gt;""</formula>
+      <formula>$B79&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:J22">
@@ -6051,44 +6277,44 @@
       <formula>NumUpliftCombos=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B86:G90">
+  <conditionalFormatting sqref="B99:G103">
     <cfRule type="expression" priority="12" dxfId="7">
-      <formula>$B86&lt;&gt;""</formula>
+      <formula>$B99&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G86:G90">
+  <conditionalFormatting sqref="G99:G103">
     <cfRule type="expression" priority="13" dxfId="0">
-      <formula>AND(ISNUMBER(G86),G86&gt;1)</formula>
+      <formula>AND(ISNUMBER(G99),G99&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B122:J137">
+  <conditionalFormatting sqref="B133:J148">
     <cfRule type="expression" priority="14" dxfId="7">
-      <formula>$B122&lt;&gt;""</formula>
+      <formula>$B133&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J122:J137">
+  <conditionalFormatting sqref="J133:J148">
     <cfRule type="expression" priority="15" dxfId="0">
-      <formula>AND(ISNUMBER(J122),J122&gt;1)</formula>
+      <formula>AND(ISNUMBER(J133),J133&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C122:C137">
+  <conditionalFormatting sqref="C133:C148">
     <cfRule type="expression" priority="16" dxfId="9">
-      <formula>RIGHT(C122,1)="*"</formula>
+      <formula>RIGHT(C133,1)="*"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B167:F174">
+  <conditionalFormatting sqref="B178:F185">
     <cfRule type="expression" priority="17" dxfId="7">
-      <formula>$B167&lt;&gt;""</formula>
+      <formula>$B178&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F167:F174">
+  <conditionalFormatting sqref="F178:F185">
     <cfRule type="expression" priority="18" dxfId="0">
-      <formula>AND(ISNUMBER(F167),F167&gt;1)</formula>
+      <formula>AND(ISNUMBER(F178),F178&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B188:D201">
+  <conditionalFormatting sqref="B199:D212">
     <cfRule type="expression" priority="19" dxfId="7">
-      <formula>$B188&lt;&gt;""</formula>
+      <formula>$B199&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="13">
@@ -6122,10 +6348,10 @@
     <dataValidation sqref="Q47:Q84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Top,Bottom"</formula1>
     </dataValidation>
-    <dataValidation sqref="E63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Floor,Roof,All,Custom"</formula1>
     </dataValidation>
-    <dataValidation sqref="E77:F81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E90:F94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"F,P,L,U,–"</formula1>
     </dataValidation>
     <dataValidation sqref="E27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Section size" error="Pick a section from the list for the selected Section type." type="list">
@@ -6144,8 +6370,8 @@
   </headerFooter>
   <rowBreaks count="3" manualBreakCount="3">
     <brk id="42" min="0" max="16383" man="1"/>
-    <brk id="83" min="0" max="16383" man="1"/>
-    <brk id="139" min="0" max="16383" man="1"/>
+    <brk id="96" min="0" max="16383" man="1"/>
+    <brk id="150" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <tableParts count="4">

</xml_diff>

<commit_message>
Sheet: remove applied load diagram (OAR.LOADDIAGRAM kept in the add-in)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -52,26 +52,26 @@
     <definedName name="w_Wid" localSheetId="0">'B1'!$I$60</definedName>
     <definedName name="w_Wiu" localSheetId="0">'B1'!$J$60</definedName>
     <definedName name="NumUpliftCombos" localSheetId="0">'B1'!$S$56</definedName>
-    <definedName name="CombSet" localSheetId="0">'B1'!$E$76</definedName>
-    <definedName name="PsiC" localSheetId="0">'B1'!$G$76</definedName>
-    <definedName name="kl_Top" localSheetId="0">'B1'!$I$90</definedName>
-    <definedName name="kl_Bot" localSheetId="0">'B1'!$J$90</definedName>
-    <definedName name="kr_Top" localSheetId="0">'B1'!$I$91</definedName>
-    <definedName name="kr_Bot" localSheetId="0">'B1'!$J$91</definedName>
-    <definedName name="RxnL_G" localSheetId="0">'B1'!$D$190</definedName>
-    <definedName name="RxnR_G" localSheetId="0">'B1'!$E$190</definedName>
-    <definedName name="RxnL_Q" localSheetId="0">'B1'!$D$191</definedName>
-    <definedName name="RxnR_Q" localSheetId="0">'B1'!$E$191</definedName>
-    <definedName name="RxnL_Wd" localSheetId="0">'B1'!$D$192</definedName>
-    <definedName name="RxnR_Wd" localSheetId="0">'B1'!$E$192</definedName>
-    <definedName name="RxnL_Wu" localSheetId="0">'B1'!$D$193</definedName>
-    <definedName name="RxnR_Wu" localSheetId="0">'B1'!$E$193</definedName>
-    <definedName name="RxnL_Wid" localSheetId="0">'B1'!$D$194</definedName>
-    <definedName name="RxnR_Wid" localSheetId="0">'B1'!$E$194</definedName>
-    <definedName name="RxnL_Wiu" localSheetId="0">'B1'!$D$195</definedName>
-    <definedName name="RxnR_Wiu" localSheetId="0">'B1'!$E$195</definedName>
-    <definedName name="Out_Reactions" localSheetId="0">'B1'!$B$199</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'B1'!$A$1:$K$213</definedName>
+    <definedName name="CombSet" localSheetId="0">'B1'!$E$63</definedName>
+    <definedName name="PsiC" localSheetId="0">'B1'!$G$63</definedName>
+    <definedName name="kl_Top" localSheetId="0">'B1'!$I$77</definedName>
+    <definedName name="kl_Bot" localSheetId="0">'B1'!$J$77</definedName>
+    <definedName name="kr_Top" localSheetId="0">'B1'!$I$78</definedName>
+    <definedName name="kr_Bot" localSheetId="0">'B1'!$J$78</definedName>
+    <definedName name="RxnL_G" localSheetId="0">'B1'!$D$177</definedName>
+    <definedName name="RxnR_G" localSheetId="0">'B1'!$E$177</definedName>
+    <definedName name="RxnL_Q" localSheetId="0">'B1'!$D$178</definedName>
+    <definedName name="RxnR_Q" localSheetId="0">'B1'!$E$178</definedName>
+    <definedName name="RxnL_Wd" localSheetId="0">'B1'!$D$179</definedName>
+    <definedName name="RxnR_Wd" localSheetId="0">'B1'!$E$179</definedName>
+    <definedName name="RxnL_Wu" localSheetId="0">'B1'!$D$180</definedName>
+    <definedName name="RxnR_Wu" localSheetId="0">'B1'!$E$180</definedName>
+    <definedName name="RxnL_Wid" localSheetId="0">'B1'!$D$181</definedName>
+    <definedName name="RxnR_Wid" localSheetId="0">'B1'!$E$181</definedName>
+    <definedName name="RxnL_Wiu" localSheetId="0">'B1'!$D$182</definedName>
+    <definedName name="RxnR_Wiu" localSheetId="0">'B1'!$E$182</definedName>
+    <definedName name="Out_Reactions" localSheetId="0">'B1'!$B$186</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'B1'!$A$1:$K$200</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -559,9 +559,6 @@
     <xf numFmtId="170" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -576,6 +573,9 @@
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="171" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -754,333 +754,6 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
-  <chart>
-    <plotArea>
-      <scatterChart>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'B1'!AA90</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-              <a:solidFill>
-                <a:srgbClr val="465A52"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'B1'!$Z$91:$Z$170</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'B1'!$AA$91:$AA$170</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'B1'!AB90</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-              <a:solidFill>
-                <a:srgbClr val="C07A2C"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'B1'!$Z$91:$Z$170</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'B1'!$AB$91:$AB$170</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'B1'!AC90</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-              <a:solidFill>
-                <a:srgbClr val="6E8FB5"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'B1'!$Z$91:$Z$170</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'B1'!$AC$91:$AC$170</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <strRef>
-              <f>'B1'!AD90</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-              <a:solidFill>
-                <a:srgbClr val="9C5DA6"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'B1'!$Z$91:$Z$170</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'B1'!$AD$91:$AD$170</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <tx>
-            <strRef>
-              <f>'B1'!AE90</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-              <a:solidFill>
-                <a:srgbClr val="8FA89C"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'B1'!$Z$91:$Z$170</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'B1'!$AE$91:$AE$170</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="5"/>
-          <order val="5"/>
-          <tx>
-            <strRef>
-              <f>'B1'!AF90</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
-              <a:solidFill>
-                <a:srgbClr val="B8ADA5"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'B1'!$Z$91:$Z$170</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'B1'!$AF$91:$AF$170</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="6"/>
-          <order val="6"/>
-          <tx>
-            <v>Point loads (kN)</v>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="triangle"/>
-            <size val="7"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="262626"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <errBars>
-            <errDir val="y"/>
-            <errBarType val="minus"/>
-            <errValType val="percentage"/>
-            <noEndCap val="1"/>
-            <val val="100"/>
-          </errBars>
-          <xVal>
-            <numRef>
-              <f>'B1'!$AH$91:$AH$110</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'B1'!$AI$90:$AI$110</f>
-            </numRef>
-          </yVal>
-        </ser>
-        <axId val="10"/>
-        <axId val="20"/>
-      </scatterChart>
-      <valAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-          <min val="0"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="low"/>
-        <crossAx val="20"/>
-      </valAx>
-      <valAx>
-        <axId val="20"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350">
-              <a:solidFill>
-                <a:srgbClr val="E3E3E3"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>kN/m · kN</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="low"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="t"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -1293,7 +966,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -1440,10 +1113,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>62</row>
+      <row>92</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6336000" cy="1800000"/>
+    <ext cx="6336000" cy="1944000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1462,7 +1135,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>105</row>
+      <row>106</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6336000" cy="1944000"/>
@@ -1484,39 +1157,17 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>119</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6336000" cy="1944000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="3" name="Chart 3"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2686050" cy="381000"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1583,8 +1234,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Restraints_B1" displayName="Restraints_B1" ref="B89:G94" headerRowCount="1">
-  <autoFilter ref="B89:G94"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Restraints_B1" displayName="Restraints_B1" ref="B76:G81" headerRowCount="1">
+  <autoFilter ref="B76:G81"/>
   <tableColumns count="6">
     <tableColumn id="2" name="x (mm)"/>
     <tableColumn id="3" name="Ref"/>
@@ -1887,7 +1538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:AS212"/>
+  <dimension ref="B1:AS199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.5" customWidth="1" min="1" max="1"/>
@@ -2128,7 +1779,7 @@
       <c r="S8" s="17" t="n"/>
       <c r="T8" s="18" t="n"/>
       <c r="Z8" s="19" cm="1">
-        <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79),Restraints_B1[#Data],$I$90:$J$91)</f>
+        <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
         <v/>
       </c>
       <c r="AL8" s="19" cm="1">
@@ -2371,7 +2022,7 @@
       <c r="S13" s="23" t="n"/>
       <c r="T13" s="24" t="n"/>
       <c r="Z13" s="19" cm="1">
-        <f t="array" ref="Z13">OAR.ENVELOPE(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79),60)</f>
+        <f t="array" ref="Z13">OAR.ENVELOPE(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),60)</f>
         <v/>
       </c>
       <c r="AF13" s="19" cm="1">
@@ -2460,7 +2111,7 @@
         </is>
       </c>
       <c r="E15" s="36" cm="1">
-        <f t="array" ref="E15">INDEX(_xlfn.ANCHORARRAY(B99),1,2)</f>
+        <f t="array" ref="E15">INDEX(_xlfn.ANCHORARRAY(B86),1,2)</f>
         <v/>
       </c>
       <c r="F15" s="36">
@@ -2528,7 +2179,7 @@
         </is>
       </c>
       <c r="E16" s="36" cm="1">
-        <f t="array" ref="E16">INDEX(_xlfn.ANCHORARRAY(B99),2,2)</f>
+        <f t="array" ref="E16">INDEX(_xlfn.ANCHORARRAY(B86),2,2)</f>
         <v/>
       </c>
       <c r="F16" s="36">
@@ -2596,7 +2247,7 @@
         </is>
       </c>
       <c r="E17" s="36" cm="1">
-        <f t="array" ref="E17">INDEX(_xlfn.ANCHORARRAY(B99),3,2)</f>
+        <f t="array" ref="E17">INDEX(_xlfn.ANCHORARRAY(B86),3,2)</f>
         <v/>
       </c>
       <c r="F17" s="36">
@@ -2664,7 +2315,7 @@
         </is>
       </c>
       <c r="E18" s="36" cm="1">
-        <f t="array" ref="E18">INDEX(_xlfn.ANCHORARRAY(B99),4,2)</f>
+        <f t="array" ref="E18">INDEX(_xlfn.ANCHORARRAY(B86),4,2)</f>
         <v/>
       </c>
       <c r="F18" s="36">
@@ -2732,7 +2383,7 @@
         </is>
       </c>
       <c r="E19" s="36" cm="1">
-        <f t="array" ref="E19">INDEX(_xlfn.ANCHORARRAY(B99),5,2)</f>
+        <f t="array" ref="E19">INDEX(_xlfn.ANCHORARRAY(B86),5,2)</f>
         <v/>
       </c>
       <c r="F19" s="36">
@@ -4694,12 +4345,20 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="14" customHeight="1">
-      <c r="B62" s="63" t="inlineStr">
-        <is>
-          <t>Applied loads (unfactored; line loads kN/m, point loads kN with stems; + = downward;  x in m)</t>
-        </is>
-      </c>
+    <row r="62" ht="20" customHeight="1">
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>Load Combinations (AS/NZS 1170.0)</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="n"/>
+      <c r="D62" s="11" t="n"/>
+      <c r="E62" s="11" t="n"/>
+      <c r="F62" s="11" t="n"/>
+      <c r="G62" s="11" t="n"/>
+      <c r="H62" s="11" t="n"/>
+      <c r="I62" s="11" t="n"/>
+      <c r="J62" s="11" t="n"/>
       <c r="AN62" s="20" t="inlineStr">
         <is>
           <t>180UB18.1</t>
@@ -4707,6 +4366,29 @@
       </c>
     </row>
     <row r="63" ht="14" customHeight="1">
+      <c r="B63" s="42" t="inlineStr">
+        <is>
+          <t>Combination set</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Roof</t>
+        </is>
+      </c>
+      <c r="F63" s="44" t="inlineStr">
+        <is>
+          <t>ψc</t>
+        </is>
+      </c>
+      <c r="G63" s="54" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>Table 4.1 (roofs 0.0)</t>
+        </is>
+      </c>
       <c r="AN63" s="20" t="inlineStr">
         <is>
           <t>180UB16.1</t>
@@ -4714,6 +4396,11 @@
       </c>
     </row>
     <row r="64" ht="14" customHeight="1">
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>Floor = gravity only.  Roof = gravity + wind.  All = every library row.  Custom = only rows set to Yes / Custom.  Edit in the library to the right →</t>
+        </is>
+      </c>
       <c r="AN64" s="20" t="inlineStr">
         <is>
           <t>150UB18</t>
@@ -4721,6 +4408,51 @@
       </c>
     </row>
     <row r="65" ht="14" customHeight="1">
+      <c r="B65" s="25" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C65" s="25" t="inlineStr">
+        <is>
+          <t>Crit. flange</t>
+        </is>
+      </c>
+      <c r="D65" s="25" t="inlineStr">
+        <is>
+          <t>Combination</t>
+        </is>
+      </c>
+      <c r="E65" s="25" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F65" s="25" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G65" s="25" t="inlineStr">
+        <is>
+          <t>Wd</t>
+        </is>
+      </c>
+      <c r="H65" s="25" t="inlineStr">
+        <is>
+          <t>Wu</t>
+        </is>
+      </c>
+      <c r="I65" s="25" t="inlineStr">
+        <is>
+          <t>Wid</t>
+        </is>
+      </c>
+      <c r="J65" s="25" t="inlineStr">
+        <is>
+          <t>Wiu</t>
+        </is>
+      </c>
       <c r="AN65" s="20" t="inlineStr">
         <is>
           <t>150UB14</t>
@@ -4728,6 +4460,18 @@
       </c>
     </row>
     <row r="66" ht="14" customHeight="1">
+      <c r="B66" s="34" cm="1">
+        <f t="array" ref="B66">_xlfn._xlws.FILTER(CombLib_B1[[ID]:[Wiu]],CombLib_B1[Active]=1,"No combinations selected")</f>
+        <v/>
+      </c>
+      <c r="C66" s="34" t="n"/>
+      <c r="D66" s="42" t="n"/>
+      <c r="E66" s="63" t="n"/>
+      <c r="F66" s="63" t="n"/>
+      <c r="G66" s="63" t="n"/>
+      <c r="H66" s="63" t="n"/>
+      <c r="I66" s="63" t="n"/>
+      <c r="J66" s="63" t="n"/>
       <c r="AN66" s="20" t="inlineStr">
         <is>
           <t>380PFC</t>
@@ -4735,6 +4479,15 @@
       </c>
     </row>
     <row r="67" ht="14" customHeight="1">
+      <c r="B67" s="34" t="n"/>
+      <c r="C67" s="34" t="n"/>
+      <c r="D67" s="42" t="n"/>
+      <c r="E67" s="63" t="n"/>
+      <c r="F67" s="63" t="n"/>
+      <c r="G67" s="63" t="n"/>
+      <c r="H67" s="63" t="n"/>
+      <c r="I67" s="63" t="n"/>
+      <c r="J67" s="63" t="n"/>
       <c r="AN67" s="20" t="inlineStr">
         <is>
           <t>300PFC</t>
@@ -4742,6 +4495,15 @@
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
+      <c r="B68" s="34" t="n"/>
+      <c r="C68" s="34" t="n"/>
+      <c r="D68" s="42" t="n"/>
+      <c r="E68" s="63" t="n"/>
+      <c r="F68" s="63" t="n"/>
+      <c r="G68" s="63" t="n"/>
+      <c r="H68" s="63" t="n"/>
+      <c r="I68" s="63" t="n"/>
+      <c r="J68" s="63" t="n"/>
       <c r="AN68" s="20" t="inlineStr">
         <is>
           <t>250PFC</t>
@@ -4749,6 +4511,15 @@
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
+      <c r="B69" s="34" t="n"/>
+      <c r="C69" s="34" t="n"/>
+      <c r="D69" s="42" t="n"/>
+      <c r="E69" s="63" t="n"/>
+      <c r="F69" s="63" t="n"/>
+      <c r="G69" s="63" t="n"/>
+      <c r="H69" s="63" t="n"/>
+      <c r="I69" s="63" t="n"/>
+      <c r="J69" s="63" t="n"/>
       <c r="AN69" s="20" t="inlineStr">
         <is>
           <t>230PFC</t>
@@ -4756,6 +4527,15 @@
       </c>
     </row>
     <row r="70" ht="14" customHeight="1">
+      <c r="B70" s="34" t="n"/>
+      <c r="C70" s="34" t="n"/>
+      <c r="D70" s="42" t="n"/>
+      <c r="E70" s="63" t="n"/>
+      <c r="F70" s="63" t="n"/>
+      <c r="G70" s="63" t="n"/>
+      <c r="H70" s="63" t="n"/>
+      <c r="I70" s="63" t="n"/>
+      <c r="J70" s="63" t="n"/>
       <c r="AN70" s="20" t="inlineStr">
         <is>
           <t>200PFC</t>
@@ -4763,6 +4543,15 @@
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
+      <c r="B71" s="34" t="n"/>
+      <c r="C71" s="34" t="n"/>
+      <c r="D71" s="42" t="n"/>
+      <c r="E71" s="63" t="n"/>
+      <c r="F71" s="63" t="n"/>
+      <c r="G71" s="63" t="n"/>
+      <c r="H71" s="63" t="n"/>
+      <c r="I71" s="63" t="n"/>
+      <c r="J71" s="63" t="n"/>
       <c r="AN71" s="20" t="inlineStr">
         <is>
           <t>180PFC</t>
@@ -4770,6 +4559,15 @@
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
+      <c r="B72" s="34" t="n"/>
+      <c r="C72" s="34" t="n"/>
+      <c r="D72" s="42" t="n"/>
+      <c r="E72" s="63" t="n"/>
+      <c r="F72" s="63" t="n"/>
+      <c r="G72" s="63" t="n"/>
+      <c r="H72" s="63" t="n"/>
+      <c r="I72" s="63" t="n"/>
+      <c r="J72" s="63" t="n"/>
       <c r="AN72" s="20" t="inlineStr">
         <is>
           <t>150PFC</t>
@@ -4777,33 +4575,47 @@
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
+      <c r="B73" s="34" t="n"/>
+      <c r="C73" s="34" t="n"/>
+      <c r="D73" s="42" t="n"/>
+      <c r="E73" s="63" t="n"/>
+      <c r="F73" s="63" t="n"/>
+      <c r="G73" s="63" t="n"/>
+      <c r="H73" s="63" t="n"/>
+      <c r="I73" s="63" t="n"/>
+      <c r="J73" s="63" t="n"/>
       <c r="AN73" s="20" t="inlineStr">
         <is>
           <t>125PFC</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="14" customHeight="1">
+    <row r="74" ht="20" customHeight="1">
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>Lateral Restraints (AS 4100 Cl. 5.4)</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="n"/>
+      <c r="D74" s="11" t="n"/>
+      <c r="E74" s="11" t="n"/>
+      <c r="F74" s="11" t="n"/>
+      <c r="G74" s="11" t="n"/>
+      <c r="H74" s="11" t="n"/>
+      <c r="I74" s="11" t="n"/>
+      <c r="J74" s="11" t="n"/>
       <c r="AN74" s="20" t="inlineStr">
         <is>
           <t>100PFC</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="B75" s="10" t="inlineStr">
-        <is>
-          <t>Load Combinations (AS/NZS 1170.0)</t>
-        </is>
-      </c>
-      <c r="C75" s="11" t="n"/>
-      <c r="D75" s="11" t="n"/>
-      <c r="E75" s="11" t="n"/>
-      <c r="F75" s="11" t="n"/>
-      <c r="G75" s="11" t="n"/>
-      <c r="H75" s="11" t="n"/>
-      <c r="I75" s="11" t="n"/>
-      <c r="J75" s="11" t="n"/>
+    <row r="75" ht="14" customHeight="1">
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>Restraint type at each cross-section for the critical flange: F, P, L or U (– = none). Supports must be F or P.</t>
+        </is>
+      </c>
       <c r="AN75" s="20" t="inlineStr">
         <is>
           <t>75PFC</t>
@@ -4811,27 +4623,49 @@
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
-      <c r="B76" s="42" t="inlineStr">
-        <is>
-          <t>Combination set</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>Roof</t>
-        </is>
-      </c>
-      <c r="F76" s="44" t="inlineStr">
-        <is>
-          <t>ψc</t>
-        </is>
-      </c>
-      <c r="G76" s="54" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H76" s="6" t="inlineStr">
-        <is>
-          <t>Table 4.1 (roofs 0.0)</t>
+      <c r="B76" s="25" t="inlineStr">
+        <is>
+          <t>x (mm)</t>
+        </is>
+      </c>
+      <c r="C76" s="25" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="D76" s="25" t="inlineStr">
+        <is>
+          <t>Restraint provided by</t>
+        </is>
+      </c>
+      <c r="E76" s="25" t="inlineStr">
+        <is>
+          <t>Top flange</t>
+        </is>
+      </c>
+      <c r="F76" s="25" t="inlineStr">
+        <is>
+          <t>Bottom fl.</t>
+        </is>
+      </c>
+      <c r="G76" s="25" t="inlineStr">
+        <is>
+          <t>αm override</t>
+        </is>
+      </c>
+      <c r="H76" s="25" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="I76" s="25" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="J76" s="25" t="inlineStr">
+        <is>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="AN76" s="20" t="inlineStr">
@@ -4841,10 +4675,41 @@
       </c>
     </row>
     <row r="77" ht="14" customHeight="1">
-      <c r="B77" s="15" t="inlineStr">
-        <is>
-          <t>Floor = gravity only.  Roof = gravity + wind.  All = every library row.  Custom = only rows set to Yes / Custom.  Edit in the library to the right →</t>
-        </is>
+      <c r="B77" s="64">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Left support – cleat</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G77" s="30" t="n"/>
+      <c r="H77" s="34" t="inlineStr">
+        <is>
+          <t>kl</t>
+        </is>
+      </c>
+      <c r="I77" s="30" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J77" s="30" t="n">
+        <v>1</v>
       </c>
       <c r="AN77" s="20" t="inlineStr">
         <is>
@@ -4853,50 +4718,36 @@
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
-      <c r="B78" s="25" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="C78" s="25" t="inlineStr">
-        <is>
-          <t>Crit. flange</t>
-        </is>
-      </c>
-      <c r="D78" s="25" t="inlineStr">
-        <is>
-          <t>Combination</t>
-        </is>
-      </c>
-      <c r="E78" s="25" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="F78" s="25" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="G78" s="25" t="inlineStr">
-        <is>
-          <t>Wd</t>
-        </is>
-      </c>
-      <c r="H78" s="25" t="inlineStr">
-        <is>
-          <t>Wu</t>
-        </is>
-      </c>
-      <c r="I78" s="25" t="inlineStr">
-        <is>
-          <t>Wid</t>
-        </is>
-      </c>
-      <c r="J78" s="25" t="inlineStr">
-        <is>
-          <t>Wiu</t>
-        </is>
+      <c r="B78" s="47" t="n">
+        <v>2767</v>
+      </c>
+      <c r="C78" s="2" t="inlineStr"/>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Purlin + fly brace</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G78" s="30" t="n"/>
+      <c r="H78" s="34" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="I78" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J78" s="30" t="n">
+        <v>1</v>
       </c>
       <c r="AN78" s="20" t="inlineStr">
         <is>
@@ -4905,18 +4756,31 @@
       </c>
     </row>
     <row r="79" ht="14" customHeight="1">
-      <c r="B79" s="34" cm="1">
-        <f t="array" ref="B79">_xlfn._xlws.FILTER(CombLib_B1[[ID]:[Wiu]],CombLib_B1[Active]=1,"No combinations selected")</f>
-        <v/>
-      </c>
-      <c r="C79" s="34" t="n"/>
-      <c r="D79" s="42" t="n"/>
-      <c r="E79" s="64" t="n"/>
-      <c r="F79" s="64" t="n"/>
-      <c r="G79" s="64" t="n"/>
-      <c r="H79" s="64" t="n"/>
-      <c r="I79" s="64" t="n"/>
-      <c r="J79" s="64" t="n"/>
+      <c r="B79" s="47" t="n">
+        <v>5533</v>
+      </c>
+      <c r="C79" s="2" t="inlineStr"/>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>Purlin + fly brace</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G79" s="30" t="n"/>
+      <c r="H79" s="15" t="inlineStr">
+        <is>
+          <t>kt from restraint</t>
+        </is>
+      </c>
       <c r="AN79" s="20" t="inlineStr">
         <is>
           <t>310UC97</t>
@@ -4924,15 +4788,36 @@
       </c>
     </row>
     <row r="80" ht="14" customHeight="1">
-      <c r="B80" s="34" t="n"/>
-      <c r="C80" s="34" t="n"/>
-      <c r="D80" s="42" t="n"/>
-      <c r="E80" s="64" t="n"/>
-      <c r="F80" s="64" t="n"/>
-      <c r="G80" s="64" t="n"/>
-      <c r="H80" s="64" t="n"/>
-      <c r="I80" s="64" t="n"/>
-      <c r="J80" s="64" t="n"/>
+      <c r="B80" s="64">
+        <f>Span</f>
+        <v/>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Right support – cleat</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G80" s="30" t="n"/>
+      <c r="H80" s="15" t="inlineStr">
+        <is>
+          <t>types (add-in)</t>
+        </is>
+      </c>
       <c r="AN80" s="20" t="inlineStr">
         <is>
           <t>250UC89.5</t>
@@ -4940,15 +4825,12 @@
       </c>
     </row>
     <row r="81" ht="14" customHeight="1">
-      <c r="B81" s="34" t="n"/>
-      <c r="C81" s="34" t="n"/>
-      <c r="D81" s="42" t="n"/>
-      <c r="E81" s="64" t="n"/>
-      <c r="F81" s="64" t="n"/>
-      <c r="G81" s="64" t="n"/>
-      <c r="H81" s="64" t="n"/>
-      <c r="I81" s="64" t="n"/>
-      <c r="J81" s="64" t="n"/>
+      <c r="B81" s="47" t="n"/>
+      <c r="C81" s="2" t="n"/>
+      <c r="D81" s="5" t="n"/>
+      <c r="E81" s="2" t="n"/>
+      <c r="F81" s="2" t="n"/>
+      <c r="G81" s="30" t="n"/>
       <c r="AN81" s="20" t="inlineStr">
         <is>
           <t>250UC73</t>
@@ -4956,15 +4838,11 @@
       </c>
     </row>
     <row r="82" ht="14" customHeight="1">
-      <c r="B82" s="34" t="n"/>
-      <c r="C82" s="34" t="n"/>
-      <c r="D82" s="42" t="n"/>
-      <c r="E82" s="64" t="n"/>
-      <c r="F82" s="64" t="n"/>
-      <c r="G82" s="64" t="n"/>
-      <c r="H82" s="64" t="n"/>
-      <c r="I82" s="64" t="n"/>
-      <c r="J82" s="64" t="n"/>
+      <c r="B82" s="15" t="inlineStr">
+        <is>
+          <t>αm override applies to the segment starting at that row (blank = Cl. 5.6.1.1(a)(iii)); flagged * in the output.</t>
+        </is>
+      </c>
       <c r="AN82" s="20" t="inlineStr">
         <is>
           <t>200UC59.5</t>
@@ -4972,31 +4850,26 @@
       </c>
     </row>
     <row r="83" ht="14" customHeight="1">
-      <c r="B83" s="34" t="n"/>
-      <c r="C83" s="34" t="n"/>
-      <c r="D83" s="42" t="n"/>
-      <c r="E83" s="64" t="n"/>
-      <c r="F83" s="64" t="n"/>
-      <c r="G83" s="64" t="n"/>
-      <c r="H83" s="64" t="n"/>
-      <c r="I83" s="64" t="n"/>
-      <c r="J83" s="64" t="n"/>
       <c r="AN83" s="20" t="inlineStr">
         <is>
           <t>200UC52</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="14" customHeight="1">
-      <c r="B84" s="34" t="n"/>
-      <c r="C84" s="34" t="n"/>
-      <c r="D84" s="42" t="n"/>
-      <c r="E84" s="64" t="n"/>
-      <c r="F84" s="64" t="n"/>
-      <c r="G84" s="64" t="n"/>
-      <c r="H84" s="64" t="n"/>
-      <c r="I84" s="64" t="n"/>
-      <c r="J84" s="64" t="n"/>
+    <row r="84" ht="20" customHeight="1">
+      <c r="B84" s="10" t="inlineStr">
+        <is>
+          <t>Serviceability Checks</t>
+        </is>
+      </c>
+      <c r="C84" s="11" t="n"/>
+      <c r="D84" s="11" t="n"/>
+      <c r="E84" s="11" t="n"/>
+      <c r="F84" s="11" t="n"/>
+      <c r="G84" s="11" t="n"/>
+      <c r="H84" s="11" t="n"/>
+      <c r="I84" s="11" t="n"/>
+      <c r="J84" s="11" t="n"/>
       <c r="AN84" s="20" t="inlineStr">
         <is>
           <t>200UC46</t>
@@ -5004,15 +4877,36 @@
       </c>
     </row>
     <row r="85" ht="14" customHeight="1">
-      <c r="B85" s="34" t="n"/>
-      <c r="C85" s="34" t="n"/>
-      <c r="D85" s="42" t="n"/>
-      <c r="E85" s="64" t="n"/>
-      <c r="F85" s="64" t="n"/>
-      <c r="G85" s="64" t="n"/>
-      <c r="H85" s="64" t="n"/>
-      <c r="I85" s="64" t="n"/>
-      <c r="J85" s="64" t="n"/>
+      <c r="B85" s="59" t="inlineStr">
+        <is>
+          <t>Case</t>
+        </is>
+      </c>
+      <c r="C85" s="59" t="inlineStr">
+        <is>
+          <t>Δ max (mm)</t>
+        </is>
+      </c>
+      <c r="D85" s="59" t="inlineStr">
+        <is>
+          <t>at x (mm)</t>
+        </is>
+      </c>
+      <c r="E85" s="59" t="inlineStr">
+        <is>
+          <t>Limit (mm)</t>
+        </is>
+      </c>
+      <c r="F85" s="59" t="inlineStr">
+        <is>
+          <t>L / Δ</t>
+        </is>
+      </c>
+      <c r="G85" s="59" t="inlineStr">
+        <is>
+          <t>Utilisation</t>
+        </is>
+      </c>
       <c r="AN85" s="20" t="inlineStr">
         <is>
           <t>150UC37</t>
@@ -5020,35 +4914,38 @@
       </c>
     </row>
     <row r="86" ht="14" customHeight="1">
-      <c r="B86" s="34" t="n"/>
-      <c r="C86" s="34" t="n"/>
-      <c r="D86" s="42" t="n"/>
-      <c r="E86" s="64" t="n"/>
-      <c r="F86" s="64" t="n"/>
-      <c r="G86" s="64" t="n"/>
-      <c r="H86" s="64" t="n"/>
-      <c r="I86" s="64" t="n"/>
-      <c r="J86" s="64" t="n"/>
+      <c r="B86" s="34" cm="1">
+        <f t="array" ref="B86">OAR.SLS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],$E$37:$F$41,PsiL,PsiS)</f>
+        <v/>
+      </c>
+      <c r="C86" s="63" t="n"/>
+      <c r="D86" s="65" t="n"/>
+      <c r="E86" s="63" t="n"/>
+      <c r="F86" s="66" t="n"/>
+      <c r="G86" s="67" t="n"/>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>Δ1kN: 1 kN at midspan,</t>
+        </is>
+      </c>
       <c r="AN86" s="20" t="inlineStr">
         <is>
           <t>150UC30</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="20" customHeight="1">
-      <c r="B87" s="10" t="inlineStr">
-        <is>
-          <t>Lateral Restraints (AS 4100 Cl. 5.4)</t>
-        </is>
-      </c>
-      <c r="C87" s="11" t="n"/>
-      <c r="D87" s="11" t="n"/>
-      <c r="E87" s="11" t="n"/>
-      <c r="F87" s="11" t="n"/>
-      <c r="G87" s="11" t="n"/>
-      <c r="H87" s="11" t="n"/>
-      <c r="I87" s="11" t="n"/>
-      <c r="J87" s="11" t="n"/>
+    <row r="87" ht="14" customHeight="1">
+      <c r="B87" s="34" t="n"/>
+      <c r="C87" s="63" t="n"/>
+      <c r="D87" s="65" t="n"/>
+      <c r="E87" s="63" t="n"/>
+      <c r="F87" s="66" t="n"/>
+      <c r="G87" s="67" t="n"/>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>beam alone</t>
+        </is>
+      </c>
       <c r="AN87" s="20" t="inlineStr">
         <is>
           <t>150UC23</t>
@@ -5056,11 +4953,12 @@
       </c>
     </row>
     <row r="88" ht="14" customHeight="1">
-      <c r="B88" s="15" t="inlineStr">
-        <is>
-          <t>Restraint type at each cross-section for the critical flange: F, P, L or U (– = none). Supports must be F or P.</t>
-        </is>
-      </c>
+      <c r="B88" s="34" t="n"/>
+      <c r="C88" s="63" t="n"/>
+      <c r="D88" s="65" t="n"/>
+      <c r="E88" s="63" t="n"/>
+      <c r="F88" s="66" t="n"/>
+      <c r="G88" s="67" t="n"/>
       <c r="AN88" s="20" t="inlineStr">
         <is>
           <t>100UC15</t>
@@ -5068,325 +4966,63 @@
       </c>
     </row>
     <row r="89" ht="14" customHeight="1">
-      <c r="B89" s="25" t="inlineStr">
-        <is>
-          <t>x (mm)</t>
-        </is>
-      </c>
-      <c r="C89" s="25" t="inlineStr">
-        <is>
-          <t>Ref</t>
-        </is>
-      </c>
-      <c r="D89" s="25" t="inlineStr">
-        <is>
-          <t>Restraint provided by</t>
-        </is>
-      </c>
-      <c r="E89" s="25" t="inlineStr">
-        <is>
-          <t>Top flange</t>
-        </is>
-      </c>
-      <c r="F89" s="25" t="inlineStr">
-        <is>
-          <t>Bottom fl.</t>
-        </is>
-      </c>
-      <c r="G89" s="25" t="inlineStr">
-        <is>
-          <t>αm override</t>
-        </is>
-      </c>
-      <c r="H89" s="25" t="inlineStr">
-        <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="I89" s="25" t="inlineStr">
-        <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="J89" s="25" t="inlineStr">
-        <is>
-          <t>Bottom</t>
-        </is>
-      </c>
-      <c r="Z89" s="15" t="inlineStr">
-        <is>
-          <t>Applied line loads (OAR.LOADDIAGRAM)</t>
-        </is>
-      </c>
-      <c r="AH89" s="15" t="inlineStr">
-        <is>
-          <t>Point loads</t>
-        </is>
-      </c>
+      <c r="B89" s="34" t="n"/>
+      <c r="C89" s="63" t="n"/>
+      <c r="D89" s="65" t="n"/>
+      <c r="E89" s="63" t="n"/>
+      <c r="F89" s="66" t="n"/>
+      <c r="G89" s="67" t="n"/>
     </row>
     <row r="90" ht="14" customHeight="1">
-      <c r="B90" s="65">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D90" s="5" t="inlineStr">
-        <is>
-          <t>Left support – cleat</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G90" s="30" t="n"/>
-      <c r="H90" s="34" t="inlineStr">
-        <is>
-          <t>kl</t>
-        </is>
-      </c>
-      <c r="I90" s="30" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="J90" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z90" s="19" cm="1">
-        <f t="array" ref="Z90">OAR.LOADDIAGRAM(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],"line")</f>
-        <v/>
-      </c>
-      <c r="AH90" s="19" cm="1">
-        <f t="array" ref="AH90">OAR.LOADDIAGRAM(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],"point")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91" ht="14" customHeight="1">
-      <c r="B91" s="47" t="n">
-        <v>2767</v>
-      </c>
-      <c r="C91" s="2" t="inlineStr"/>
-      <c r="D91" s="5" t="inlineStr">
-        <is>
-          <t>Purlin + fly brace</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G91" s="30" t="n"/>
-      <c r="H91" s="34" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="I91" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="J91" s="30" t="n">
-        <v>1</v>
-      </c>
-    </row>
+      <c r="B90" s="34" t="n"/>
+      <c r="C90" s="63" t="n"/>
+      <c r="D90" s="65" t="n"/>
+      <c r="E90" s="63" t="n"/>
+      <c r="F90" s="66" t="n"/>
+      <c r="G90" s="67" t="n"/>
+    </row>
+    <row r="91" ht="14" customHeight="1"/>
     <row r="92" ht="14" customHeight="1">
-      <c r="B92" s="47" t="n">
-        <v>5533</v>
-      </c>
-      <c r="C92" s="2" t="inlineStr"/>
-      <c r="D92" s="5" t="inlineStr">
-        <is>
-          <t>Purlin + fly brace</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G92" s="30" t="n"/>
-      <c r="H92" s="15" t="inlineStr">
-        <is>
-          <t>kt from restraint</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="14" customHeight="1">
-      <c r="B93" s="65">
-        <f>Span</f>
-        <v/>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D93" s="5" t="inlineStr">
-        <is>
-          <t>Right support – cleat</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="F93" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="G93" s="30" t="n"/>
-      <c r="H93" s="15" t="inlineStr">
-        <is>
-          <t>types (add-in)</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="14" customHeight="1">
-      <c r="B94" s="47" t="n"/>
-      <c r="C94" s="2" t="n"/>
-      <c r="D94" s="5" t="n"/>
-      <c r="E94" s="2" t="n"/>
-      <c r="F94" s="2" t="n"/>
-      <c r="G94" s="30" t="n"/>
-    </row>
-    <row r="95" ht="14" customHeight="1">
-      <c r="B95" s="15" t="inlineStr">
-        <is>
-          <t>αm override applies to the segment starting at that row (blank = Cl. 5.6.1.1(a)(iii)); flagged * in the output.</t>
-        </is>
-      </c>
-    </row>
+      <c r="B92" s="68" t="inlineStr">
+        <is>
+          <t>Deflected shapes (mm, plotted downward;  x in m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="14" customHeight="1"/>
+    <row r="94" ht="14" customHeight="1"/>
+    <row r="95" ht="14" customHeight="1"/>
     <row r="96" ht="14" customHeight="1"/>
-    <row r="97" ht="20" customHeight="1">
-      <c r="B97" s="10" t="inlineStr">
-        <is>
-          <t>Serviceability Checks</t>
-        </is>
-      </c>
-      <c r="C97" s="11" t="n"/>
-      <c r="D97" s="11" t="n"/>
-      <c r="E97" s="11" t="n"/>
-      <c r="F97" s="11" t="n"/>
-      <c r="G97" s="11" t="n"/>
-      <c r="H97" s="11" t="n"/>
-      <c r="I97" s="11" t="n"/>
-      <c r="J97" s="11" t="n"/>
-    </row>
-    <row r="98" ht="14" customHeight="1">
-      <c r="B98" s="59" t="inlineStr">
-        <is>
-          <t>Case</t>
-        </is>
-      </c>
-      <c r="C98" s="59" t="inlineStr">
-        <is>
-          <t>Δ max (mm)</t>
-        </is>
-      </c>
-      <c r="D98" s="59" t="inlineStr">
-        <is>
-          <t>at x (mm)</t>
-        </is>
-      </c>
-      <c r="E98" s="59" t="inlineStr">
-        <is>
-          <t>Limit (mm)</t>
-        </is>
-      </c>
-      <c r="F98" s="59" t="inlineStr">
-        <is>
-          <t>L / Δ</t>
-        </is>
-      </c>
-      <c r="G98" s="59" t="inlineStr">
-        <is>
-          <t>Utilisation</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="14" customHeight="1">
-      <c r="B99" s="34" cm="1">
-        <f t="array" ref="B99">OAR.SLS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],$E$37:$F$41,PsiL,PsiS)</f>
-        <v/>
-      </c>
-      <c r="C99" s="64" t="n"/>
-      <c r="D99" s="66" t="n"/>
-      <c r="E99" s="64" t="n"/>
-      <c r="F99" s="67" t="n"/>
-      <c r="G99" s="68" t="n"/>
-      <c r="H99" s="6" t="inlineStr">
-        <is>
-          <t>Δ1kN: 1 kN at midspan,</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="14" customHeight="1">
-      <c r="B100" s="34" t="n"/>
-      <c r="C100" s="64" t="n"/>
-      <c r="D100" s="66" t="n"/>
-      <c r="E100" s="64" t="n"/>
-      <c r="F100" s="67" t="n"/>
-      <c r="G100" s="68" t="n"/>
-      <c r="H100" s="6" t="inlineStr">
-        <is>
-          <t>beam alone</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="14" customHeight="1">
-      <c r="B101" s="34" t="n"/>
-      <c r="C101" s="64" t="n"/>
-      <c r="D101" s="66" t="n"/>
-      <c r="E101" s="64" t="n"/>
-      <c r="F101" s="67" t="n"/>
-      <c r="G101" s="68" t="n"/>
-    </row>
-    <row r="102" ht="14" customHeight="1">
-      <c r="B102" s="34" t="n"/>
-      <c r="C102" s="64" t="n"/>
-      <c r="D102" s="66" t="n"/>
-      <c r="E102" s="64" t="n"/>
-      <c r="F102" s="67" t="n"/>
-      <c r="G102" s="68" t="n"/>
-    </row>
-    <row r="103" ht="14" customHeight="1">
-      <c r="B103" s="34" t="n"/>
-      <c r="C103" s="64" t="n"/>
-      <c r="D103" s="66" t="n"/>
-      <c r="E103" s="64" t="n"/>
-      <c r="F103" s="67" t="n"/>
-      <c r="G103" s="68" t="n"/>
-    </row>
+    <row r="97" ht="14" customHeight="1"/>
+    <row r="98" ht="14" customHeight="1"/>
+    <row r="99" ht="14" customHeight="1"/>
+    <row r="100" ht="14" customHeight="1"/>
+    <row r="101" ht="14" customHeight="1"/>
+    <row r="102" ht="14" customHeight="1"/>
+    <row r="103" ht="14" customHeight="1"/>
     <row r="104" ht="14" customHeight="1"/>
-    <row r="105" ht="14" customHeight="1">
-      <c r="B105" s="63" t="inlineStr">
-        <is>
-          <t>Deflected shapes (mm, plotted downward;  x in m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="14" customHeight="1"/>
+    <row r="105" ht="20" customHeight="1">
+      <c r="B105" s="10" t="inlineStr">
+        <is>
+          <t>ULS Strength Checks – Bending (AS 4100 Cl. 5.6)</t>
+        </is>
+      </c>
+      <c r="C105" s="11" t="n"/>
+      <c r="D105" s="11" t="n"/>
+      <c r="E105" s="11" t="n"/>
+      <c r="F105" s="11" t="n"/>
+      <c r="G105" s="11" t="n"/>
+      <c r="H105" s="11" t="n"/>
+      <c r="I105" s="11" t="n"/>
+      <c r="J105" s="11" t="n"/>
+    </row>
+    <row r="106" ht="14" customHeight="1">
+      <c r="B106" s="68" t="inlineStr">
+        <is>
+          <t>Bending moment envelope, all active combinations (kN·m, sagging plotted down;  x in m)</t>
+        </is>
+      </c>
+    </row>
     <row r="107" ht="14" customHeight="1"/>
     <row r="108" ht="14" customHeight="1"/>
     <row r="109" ht="14" customHeight="1"/>
@@ -5398,300 +5034,333 @@
     <row r="115" ht="14" customHeight="1"/>
     <row r="116" ht="14" customHeight="1"/>
     <row r="117" ht="14" customHeight="1"/>
-    <row r="118" ht="20" customHeight="1">
-      <c r="B118" s="10" t="inlineStr">
-        <is>
-          <t>ULS Strength Checks – Bending (AS 4100 Cl. 5.6)</t>
-        </is>
-      </c>
-      <c r="C118" s="11" t="n"/>
-      <c r="D118" s="11" t="n"/>
-      <c r="E118" s="11" t="n"/>
-      <c r="F118" s="11" t="n"/>
-      <c r="G118" s="11" t="n"/>
-      <c r="H118" s="11" t="n"/>
-      <c r="I118" s="11" t="n"/>
-      <c r="J118" s="11" t="n"/>
-    </row>
-    <row r="119" ht="14" customHeight="1">
-      <c r="B119" s="63" t="inlineStr">
-        <is>
-          <t>Bending moment envelope, all active combinations (kN·m, sagging plotted down;  x in m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="14" customHeight="1"/>
-    <row r="121" ht="14" customHeight="1"/>
-    <row r="122" ht="14" customHeight="1"/>
-    <row r="123" ht="14" customHeight="1"/>
-    <row r="124" ht="14" customHeight="1"/>
-    <row r="125" ht="14" customHeight="1"/>
-    <row r="126" ht="14" customHeight="1"/>
-    <row r="127" ht="14" customHeight="1"/>
-    <row r="128" ht="14" customHeight="1"/>
-    <row r="129" ht="14" customHeight="1"/>
-    <row r="130" ht="14" customHeight="1"/>
-    <row r="131" ht="14" customHeight="1"/>
-    <row r="132" ht="16" customHeight="1">
-      <c r="B132" s="59" t="inlineStr">
+    <row r="118" ht="14" customHeight="1"/>
+    <row r="119" ht="16" customHeight="1">
+      <c r="B119" s="59" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="C132" s="59" t="inlineStr">
+      <c r="C119" s="59" t="inlineStr">
         <is>
           <t>Segment (m)</t>
         </is>
       </c>
-      <c r="D132" s="59" t="inlineStr">
+      <c r="D119" s="59" t="inlineStr">
         <is>
           <t>Ends</t>
         </is>
       </c>
-      <c r="E132" s="59" t="inlineStr">
+      <c r="E119" s="59" t="inlineStr">
         <is>
           <t>Le (m)</t>
         </is>
       </c>
-      <c r="F132" s="59" t="inlineStr">
+      <c r="F119" s="59" t="inlineStr">
         <is>
           <t>αm</t>
         </is>
       </c>
-      <c r="G132" s="59" t="inlineStr">
+      <c r="G119" s="59" t="inlineStr">
         <is>
           <t>αs</t>
         </is>
       </c>
-      <c r="H132" s="59" t="inlineStr">
+      <c r="H119" s="59" t="inlineStr">
         <is>
           <t>φMb (kN·m)</t>
         </is>
       </c>
-      <c r="I132" s="59" t="inlineStr">
+      <c r="I119" s="59" t="inlineStr">
         <is>
           <t>M* (kN·m)</t>
         </is>
       </c>
-      <c r="J132" s="59" t="inlineStr">
+      <c r="J119" s="59" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
     </row>
+    <row r="120" ht="14" customHeight="1">
+      <c r="B120" s="34" cm="1">
+        <f t="array" ref="B120">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
+        <v/>
+      </c>
+      <c r="C120" s="34" t="n"/>
+      <c r="D120" s="34" t="n"/>
+      <c r="E120" s="63" t="n"/>
+      <c r="F120" s="69" t="n"/>
+      <c r="G120" s="69" t="n"/>
+      <c r="H120" s="70" t="n"/>
+      <c r="I120" s="70" t="n"/>
+      <c r="J120" s="67" t="n"/>
+    </row>
+    <row r="121" ht="14" customHeight="1">
+      <c r="B121" s="34" t="n"/>
+      <c r="C121" s="34" t="n"/>
+      <c r="D121" s="34" t="n"/>
+      <c r="E121" s="63" t="n"/>
+      <c r="F121" s="69" t="n"/>
+      <c r="G121" s="69" t="n"/>
+      <c r="H121" s="70" t="n"/>
+      <c r="I121" s="70" t="n"/>
+      <c r="J121" s="67" t="n"/>
+    </row>
+    <row r="122" ht="14" customHeight="1">
+      <c r="B122" s="34" t="n"/>
+      <c r="C122" s="34" t="n"/>
+      <c r="D122" s="34" t="n"/>
+      <c r="E122" s="63" t="n"/>
+      <c r="F122" s="69" t="n"/>
+      <c r="G122" s="69" t="n"/>
+      <c r="H122" s="70" t="n"/>
+      <c r="I122" s="70" t="n"/>
+      <c r="J122" s="67" t="n"/>
+    </row>
+    <row r="123" ht="14" customHeight="1">
+      <c r="B123" s="34" t="n"/>
+      <c r="C123" s="34" t="n"/>
+      <c r="D123" s="34" t="n"/>
+      <c r="E123" s="63" t="n"/>
+      <c r="F123" s="69" t="n"/>
+      <c r="G123" s="69" t="n"/>
+      <c r="H123" s="70" t="n"/>
+      <c r="I123" s="70" t="n"/>
+      <c r="J123" s="67" t="n"/>
+    </row>
+    <row r="124" ht="14" customHeight="1">
+      <c r="B124" s="34" t="n"/>
+      <c r="C124" s="34" t="n"/>
+      <c r="D124" s="34" t="n"/>
+      <c r="E124" s="63" t="n"/>
+      <c r="F124" s="69" t="n"/>
+      <c r="G124" s="69" t="n"/>
+      <c r="H124" s="70" t="n"/>
+      <c r="I124" s="70" t="n"/>
+      <c r="J124" s="67" t="n"/>
+    </row>
+    <row r="125" ht="14" customHeight="1">
+      <c r="B125" s="34" t="n"/>
+      <c r="C125" s="34" t="n"/>
+      <c r="D125" s="34" t="n"/>
+      <c r="E125" s="63" t="n"/>
+      <c r="F125" s="69" t="n"/>
+      <c r="G125" s="69" t="n"/>
+      <c r="H125" s="70" t="n"/>
+      <c r="I125" s="70" t="n"/>
+      <c r="J125" s="67" t="n"/>
+    </row>
+    <row r="126" ht="14" customHeight="1">
+      <c r="B126" s="34" t="n"/>
+      <c r="C126" s="34" t="n"/>
+      <c r="D126" s="34" t="n"/>
+      <c r="E126" s="63" t="n"/>
+      <c r="F126" s="69" t="n"/>
+      <c r="G126" s="69" t="n"/>
+      <c r="H126" s="70" t="n"/>
+      <c r="I126" s="70" t="n"/>
+      <c r="J126" s="67" t="n"/>
+    </row>
+    <row r="127" ht="14" customHeight="1">
+      <c r="B127" s="34" t="n"/>
+      <c r="C127" s="34" t="n"/>
+      <c r="D127" s="34" t="n"/>
+      <c r="E127" s="63" t="n"/>
+      <c r="F127" s="69" t="n"/>
+      <c r="G127" s="69" t="n"/>
+      <c r="H127" s="70" t="n"/>
+      <c r="I127" s="70" t="n"/>
+      <c r="J127" s="67" t="n"/>
+    </row>
+    <row r="128" ht="14" customHeight="1">
+      <c r="B128" s="34" t="n"/>
+      <c r="C128" s="34" t="n"/>
+      <c r="D128" s="34" t="n"/>
+      <c r="E128" s="63" t="n"/>
+      <c r="F128" s="69" t="n"/>
+      <c r="G128" s="69" t="n"/>
+      <c r="H128" s="70" t="n"/>
+      <c r="I128" s="70" t="n"/>
+      <c r="J128" s="67" t="n"/>
+    </row>
+    <row r="129" ht="14" customHeight="1">
+      <c r="B129" s="34" t="n"/>
+      <c r="C129" s="34" t="n"/>
+      <c r="D129" s="34" t="n"/>
+      <c r="E129" s="63" t="n"/>
+      <c r="F129" s="69" t="n"/>
+      <c r="G129" s="69" t="n"/>
+      <c r="H129" s="70" t="n"/>
+      <c r="I129" s="70" t="n"/>
+      <c r="J129" s="67" t="n"/>
+    </row>
+    <row r="130" ht="14" customHeight="1">
+      <c r="B130" s="34" t="n"/>
+      <c r="C130" s="34" t="n"/>
+      <c r="D130" s="34" t="n"/>
+      <c r="E130" s="63" t="n"/>
+      <c r="F130" s="69" t="n"/>
+      <c r="G130" s="69" t="n"/>
+      <c r="H130" s="70" t="n"/>
+      <c r="I130" s="70" t="n"/>
+      <c r="J130" s="67" t="n"/>
+    </row>
+    <row r="131" ht="14" customHeight="1">
+      <c r="B131" s="34" t="n"/>
+      <c r="C131" s="34" t="n"/>
+      <c r="D131" s="34" t="n"/>
+      <c r="E131" s="63" t="n"/>
+      <c r="F131" s="69" t="n"/>
+      <c r="G131" s="69" t="n"/>
+      <c r="H131" s="70" t="n"/>
+      <c r="I131" s="70" t="n"/>
+      <c r="J131" s="67" t="n"/>
+    </row>
+    <row r="132" ht="14" customHeight="1">
+      <c r="B132" s="34" t="n"/>
+      <c r="C132" s="34" t="n"/>
+      <c r="D132" s="34" t="n"/>
+      <c r="E132" s="63" t="n"/>
+      <c r="F132" s="69" t="n"/>
+      <c r="G132" s="69" t="n"/>
+      <c r="H132" s="70" t="n"/>
+      <c r="I132" s="70" t="n"/>
+      <c r="J132" s="67" t="n"/>
+    </row>
     <row r="133" ht="14" customHeight="1">
-      <c r="B133" s="34" cm="1">
-        <f t="array" ref="B133">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79),Restraints_B1[#Data],$I$90:$J$91)</f>
-        <v/>
-      </c>
+      <c r="B133" s="34" t="n"/>
       <c r="C133" s="34" t="n"/>
       <c r="D133" s="34" t="n"/>
-      <c r="E133" s="64" t="n"/>
+      <c r="E133" s="63" t="n"/>
       <c r="F133" s="69" t="n"/>
       <c r="G133" s="69" t="n"/>
       <c r="H133" s="70" t="n"/>
       <c r="I133" s="70" t="n"/>
-      <c r="J133" s="68" t="n"/>
+      <c r="J133" s="67" t="n"/>
     </row>
     <row r="134" ht="14" customHeight="1">
       <c r="B134" s="34" t="n"/>
       <c r="C134" s="34" t="n"/>
       <c r="D134" s="34" t="n"/>
-      <c r="E134" s="64" t="n"/>
+      <c r="E134" s="63" t="n"/>
       <c r="F134" s="69" t="n"/>
       <c r="G134" s="69" t="n"/>
       <c r="H134" s="70" t="n"/>
       <c r="I134" s="70" t="n"/>
-      <c r="J134" s="68" t="n"/>
+      <c r="J134" s="67" t="n"/>
     </row>
     <row r="135" ht="14" customHeight="1">
       <c r="B135" s="34" t="n"/>
       <c r="C135" s="34" t="n"/>
       <c r="D135" s="34" t="n"/>
-      <c r="E135" s="64" t="n"/>
+      <c r="E135" s="63" t="n"/>
       <c r="F135" s="69" t="n"/>
       <c r="G135" s="69" t="n"/>
       <c r="H135" s="70" t="n"/>
       <c r="I135" s="70" t="n"/>
-      <c r="J135" s="68" t="n"/>
+      <c r="J135" s="67" t="n"/>
     </row>
     <row r="136" ht="14" customHeight="1">
-      <c r="B136" s="34" t="n"/>
-      <c r="C136" s="34" t="n"/>
-      <c r="D136" s="34" t="n"/>
-      <c r="E136" s="64" t="n"/>
-      <c r="F136" s="69" t="n"/>
-      <c r="G136" s="69" t="n"/>
-      <c r="H136" s="70" t="n"/>
-      <c r="I136" s="70" t="n"/>
-      <c r="J136" s="68" t="n"/>
-    </row>
-    <row r="137" ht="14" customHeight="1">
-      <c r="B137" s="34" t="n"/>
-      <c r="C137" s="34" t="n"/>
-      <c r="D137" s="34" t="n"/>
-      <c r="E137" s="64" t="n"/>
-      <c r="F137" s="69" t="n"/>
-      <c r="G137" s="69" t="n"/>
-      <c r="H137" s="70" t="n"/>
-      <c r="I137" s="70" t="n"/>
-      <c r="J137" s="68" t="n"/>
-    </row>
-    <row r="138" ht="14" customHeight="1">
-      <c r="B138" s="34" t="n"/>
-      <c r="C138" s="34" t="n"/>
-      <c r="D138" s="34" t="n"/>
-      <c r="E138" s="64" t="n"/>
-      <c r="F138" s="69" t="n"/>
-      <c r="G138" s="69" t="n"/>
-      <c r="H138" s="70" t="n"/>
-      <c r="I138" s="70" t="n"/>
-      <c r="J138" s="68" t="n"/>
+      <c r="B136" s="15" t="inlineStr">
+        <is>
+          <t>* αm overridden in the restraints table.  Full working for the governing segment follows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="14" customHeight="1"/>
+    <row r="138" ht="20" customHeight="1">
+      <c r="B138" s="10" t="inlineStr">
+        <is>
+          <t>Governing Segment – Working</t>
+        </is>
+      </c>
+      <c r="C138" s="11" t="n"/>
+      <c r="D138" s="11" t="n"/>
+      <c r="E138" s="11" t="n"/>
+      <c r="F138" s="11" t="n"/>
+      <c r="G138" s="11" t="n"/>
+      <c r="H138" s="11" t="n"/>
+      <c r="I138" s="11" t="n"/>
+      <c r="J138" s="11" t="n"/>
     </row>
     <row r="139" ht="14" customHeight="1">
-      <c r="B139" s="34" t="n"/>
-      <c r="C139" s="34" t="n"/>
-      <c r="D139" s="34" t="n"/>
-      <c r="E139" s="64" t="n"/>
-      <c r="F139" s="69" t="n"/>
-      <c r="G139" s="69" t="n"/>
-      <c r="H139" s="70" t="n"/>
-      <c r="I139" s="70" t="n"/>
-      <c r="J139" s="68" t="n"/>
+      <c r="B139" s="15" t="inlineStr">
+        <is>
+          <t>OAR.ULSDETAIL: change the comboId / segment arguments to show any other segment.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
-      <c r="B140" s="34" t="n"/>
-      <c r="C140" s="34" t="n"/>
-      <c r="D140" s="34" t="n"/>
-      <c r="E140" s="64" t="n"/>
-      <c r="F140" s="69" t="n"/>
-      <c r="G140" s="69" t="n"/>
-      <c r="H140" s="70" t="n"/>
-      <c r="I140" s="70" t="n"/>
-      <c r="J140" s="68" t="n"/>
+      <c r="D140" s="71" cm="1">
+        <f t="array" ref="D140">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
+        <v/>
+      </c>
+      <c r="E140" s="72" t="n"/>
+      <c r="F140" s="35" t="n"/>
     </row>
     <row r="141">
-      <c r="B141" s="34" t="n"/>
-      <c r="C141" s="34" t="n"/>
-      <c r="D141" s="34" t="n"/>
-      <c r="E141" s="64" t="n"/>
-      <c r="F141" s="69" t="n"/>
-      <c r="G141" s="69" t="n"/>
-      <c r="H141" s="70" t="n"/>
-      <c r="I141" s="70" t="n"/>
-      <c r="J141" s="68" t="n"/>
+      <c r="D141" s="71" t="n"/>
+      <c r="E141" s="72" t="n"/>
+      <c r="F141" s="35" t="n"/>
     </row>
     <row r="142">
-      <c r="B142" s="34" t="n"/>
-      <c r="C142" s="34" t="n"/>
-      <c r="D142" s="34" t="n"/>
-      <c r="E142" s="64" t="n"/>
-      <c r="F142" s="69" t="n"/>
-      <c r="G142" s="69" t="n"/>
-      <c r="H142" s="70" t="n"/>
-      <c r="I142" s="70" t="n"/>
-      <c r="J142" s="68" t="n"/>
+      <c r="D142" s="71" t="n"/>
+      <c r="E142" s="72" t="n"/>
+      <c r="F142" s="35" t="n"/>
     </row>
     <row r="143">
-      <c r="B143" s="34" t="n"/>
-      <c r="C143" s="34" t="n"/>
-      <c r="D143" s="34" t="n"/>
-      <c r="E143" s="64" t="n"/>
-      <c r="F143" s="69" t="n"/>
-      <c r="G143" s="69" t="n"/>
-      <c r="H143" s="70" t="n"/>
-      <c r="I143" s="70" t="n"/>
-      <c r="J143" s="68" t="n"/>
+      <c r="D143" s="71" t="n"/>
+      <c r="E143" s="72" t="n"/>
+      <c r="F143" s="35" t="n"/>
     </row>
     <row r="144">
-      <c r="B144" s="34" t="n"/>
-      <c r="C144" s="34" t="n"/>
-      <c r="D144" s="34" t="n"/>
-      <c r="E144" s="64" t="n"/>
-      <c r="F144" s="69" t="n"/>
-      <c r="G144" s="69" t="n"/>
-      <c r="H144" s="70" t="n"/>
-      <c r="I144" s="70" t="n"/>
-      <c r="J144" s="68" t="n"/>
+      <c r="D144" s="71" t="n"/>
+      <c r="E144" s="72" t="n"/>
+      <c r="F144" s="35" t="n"/>
     </row>
     <row r="145">
-      <c r="B145" s="34" t="n"/>
-      <c r="C145" s="34" t="n"/>
-      <c r="D145" s="34" t="n"/>
-      <c r="E145" s="64" t="n"/>
-      <c r="F145" s="69" t="n"/>
-      <c r="G145" s="69" t="n"/>
-      <c r="H145" s="70" t="n"/>
-      <c r="I145" s="70" t="n"/>
-      <c r="J145" s="68" t="n"/>
+      <c r="D145" s="71" t="n"/>
+      <c r="E145" s="72" t="n"/>
+      <c r="F145" s="35" t="n"/>
     </row>
     <row r="146">
-      <c r="B146" s="34" t="n"/>
-      <c r="C146" s="34" t="n"/>
-      <c r="D146" s="34" t="n"/>
-      <c r="E146" s="64" t="n"/>
-      <c r="F146" s="69" t="n"/>
-      <c r="G146" s="69" t="n"/>
-      <c r="H146" s="70" t="n"/>
-      <c r="I146" s="70" t="n"/>
-      <c r="J146" s="68" t="n"/>
+      <c r="D146" s="71" t="n"/>
+      <c r="E146" s="72" t="n"/>
+      <c r="F146" s="35" t="n"/>
     </row>
     <row r="147">
-      <c r="B147" s="34" t="n"/>
-      <c r="C147" s="34" t="n"/>
-      <c r="D147" s="34" t="n"/>
-      <c r="E147" s="64" t="n"/>
-      <c r="F147" s="69" t="n"/>
-      <c r="G147" s="69" t="n"/>
-      <c r="H147" s="70" t="n"/>
-      <c r="I147" s="70" t="n"/>
-      <c r="J147" s="68" t="n"/>
+      <c r="D147" s="71" t="n"/>
+      <c r="E147" s="72" t="n"/>
+      <c r="F147" s="35" t="n"/>
     </row>
     <row r="148">
-      <c r="B148" s="34" t="n"/>
-      <c r="C148" s="34" t="n"/>
-      <c r="D148" s="34" t="n"/>
-      <c r="E148" s="64" t="n"/>
-      <c r="F148" s="69" t="n"/>
-      <c r="G148" s="69" t="n"/>
-      <c r="H148" s="70" t="n"/>
-      <c r="I148" s="70" t="n"/>
-      <c r="J148" s="68" t="n"/>
+      <c r="D148" s="71" t="n"/>
+      <c r="E148" s="72" t="n"/>
+      <c r="F148" s="35" t="n"/>
     </row>
     <row r="149">
-      <c r="B149" s="15" t="inlineStr">
-        <is>
-          <t>* αm overridden in the restraints table.  Full working for the governing segment follows.</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="20" customHeight="1">
-      <c r="B151" s="10" t="inlineStr">
-        <is>
-          <t>Governing Segment – Working</t>
-        </is>
-      </c>
-      <c r="C151" s="11" t="n"/>
-      <c r="D151" s="11" t="n"/>
-      <c r="E151" s="11" t="n"/>
-      <c r="F151" s="11" t="n"/>
-      <c r="G151" s="11" t="n"/>
-      <c r="H151" s="11" t="n"/>
-      <c r="I151" s="11" t="n"/>
-      <c r="J151" s="11" t="n"/>
+      <c r="D149" s="71" t="n"/>
+      <c r="E149" s="72" t="n"/>
+      <c r="F149" s="35" t="n"/>
+    </row>
+    <row r="150">
+      <c r="D150" s="71" t="n"/>
+      <c r="E150" s="72" t="n"/>
+      <c r="F150" s="35" t="n"/>
+    </row>
+    <row r="151">
+      <c r="D151" s="71" t="n"/>
+      <c r="E151" s="72" t="n"/>
+      <c r="F151" s="35" t="n"/>
     </row>
     <row r="152">
-      <c r="B152" s="15" t="inlineStr">
-        <is>
-          <t>OAR.ULSDETAIL: change the comboId / segment arguments to show any other segment.</t>
-        </is>
-      </c>
+      <c r="D152" s="71" t="n"/>
+      <c r="E152" s="72" t="n"/>
+      <c r="F152" s="35" t="n"/>
     </row>
     <row r="153">
-      <c r="D153" s="71" cm="1">
-        <f t="array" ref="D153">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79),Restraints_B1[#Data],$I$90:$J$91)</f>
-        <v/>
-      </c>
+      <c r="D153" s="71" t="n"/>
       <c r="E153" s="72" t="n"/>
       <c r="F153" s="35" t="n"/>
     </row>
@@ -5735,491 +5404,426 @@
       <c r="E161" s="72" t="n"/>
       <c r="F161" s="35" t="n"/>
     </row>
-    <row r="162">
-      <c r="D162" s="71" t="n"/>
-      <c r="E162" s="72" t="n"/>
-      <c r="F162" s="35" t="n"/>
-    </row>
-    <row r="163">
-      <c r="D163" s="71" t="n"/>
-      <c r="E163" s="72" t="n"/>
-      <c r="F163" s="35" t="n"/>
+    <row r="163" ht="20" customHeight="1">
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>Shear (AS 4100 Cl. 5.11)</t>
+        </is>
+      </c>
+      <c r="C163" s="11" t="n"/>
+      <c r="D163" s="11" t="n"/>
+      <c r="E163" s="11" t="n"/>
+      <c r="F163" s="11" t="n"/>
+      <c r="G163" s="11" t="n"/>
+      <c r="H163" s="11" t="n"/>
+      <c r="I163" s="11" t="n"/>
+      <c r="J163" s="11" t="n"/>
     </row>
     <row r="164">
-      <c r="D164" s="71" t="n"/>
-      <c r="E164" s="72" t="n"/>
-      <c r="F164" s="35" t="n"/>
+      <c r="B164" s="59" t="inlineStr">
+        <is>
+          <t>Combo</t>
+        </is>
+      </c>
+      <c r="C164" s="59" t="inlineStr">
+        <is>
+          <t>V* (kN)</t>
+        </is>
+      </c>
+      <c r="D164" s="59" t="inlineStr">
+        <is>
+          <t>at x (m)</t>
+        </is>
+      </c>
+      <c r="E164" s="59" t="inlineStr">
+        <is>
+          <t>φVv (kN)</t>
+        </is>
+      </c>
+      <c r="F164" s="59" t="inlineStr">
+        <is>
+          <t>Utilisation</t>
+        </is>
+      </c>
+      <c r="G164" s="59" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
     </row>
     <row r="165">
-      <c r="D165" s="71" t="n"/>
-      <c r="E165" s="72" t="n"/>
-      <c r="F165" s="35" t="n"/>
+      <c r="B165" s="34" cm="1">
+        <f t="array" ref="B165">OAR.SHEAR(SectionSize,Grade,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
+        <v/>
+      </c>
+      <c r="C165" s="70" t="n"/>
+      <c r="D165" s="63" t="n"/>
+      <c r="E165" s="70" t="n"/>
+      <c r="F165" s="67" t="n"/>
+      <c r="G165" s="73" t="n"/>
     </row>
     <row r="166">
-      <c r="D166" s="71" t="n"/>
-      <c r="E166" s="72" t="n"/>
-      <c r="F166" s="35" t="n"/>
+      <c r="B166" s="34" t="n"/>
+      <c r="C166" s="70" t="n"/>
+      <c r="D166" s="63" t="n"/>
+      <c r="E166" s="70" t="n"/>
+      <c r="F166" s="67" t="n"/>
+      <c r="G166" s="73" t="n"/>
     </row>
     <row r="167">
-      <c r="D167" s="71" t="n"/>
-      <c r="E167" s="72" t="n"/>
-      <c r="F167" s="35" t="n"/>
+      <c r="B167" s="34" t="n"/>
+      <c r="C167" s="70" t="n"/>
+      <c r="D167" s="63" t="n"/>
+      <c r="E167" s="70" t="n"/>
+      <c r="F167" s="67" t="n"/>
+      <c r="G167" s="73" t="n"/>
     </row>
     <row r="168">
-      <c r="D168" s="71" t="n"/>
-      <c r="E168" s="72" t="n"/>
-      <c r="F168" s="35" t="n"/>
+      <c r="B168" s="34" t="n"/>
+      <c r="C168" s="70" t="n"/>
+      <c r="D168" s="63" t="n"/>
+      <c r="E168" s="70" t="n"/>
+      <c r="F168" s="67" t="n"/>
+      <c r="G168" s="73" t="n"/>
     </row>
     <row r="169">
-      <c r="D169" s="71" t="n"/>
-      <c r="E169" s="72" t="n"/>
-      <c r="F169" s="35" t="n"/>
+      <c r="B169" s="34" t="n"/>
+      <c r="C169" s="70" t="n"/>
+      <c r="D169" s="63" t="n"/>
+      <c r="E169" s="70" t="n"/>
+      <c r="F169" s="67" t="n"/>
+      <c r="G169" s="73" t="n"/>
     </row>
     <row r="170">
-      <c r="D170" s="71" t="n"/>
-      <c r="E170" s="72" t="n"/>
-      <c r="F170" s="35" t="n"/>
+      <c r="B170" s="34" t="n"/>
+      <c r="C170" s="70" t="n"/>
+      <c r="D170" s="63" t="n"/>
+      <c r="E170" s="70" t="n"/>
+      <c r="F170" s="67" t="n"/>
+      <c r="G170" s="73" t="n"/>
     </row>
     <row r="171">
-      <c r="D171" s="71" t="n"/>
-      <c r="E171" s="72" t="n"/>
-      <c r="F171" s="35" t="n"/>
+      <c r="B171" s="34" t="n"/>
+      <c r="C171" s="70" t="n"/>
+      <c r="D171" s="63" t="n"/>
+      <c r="E171" s="70" t="n"/>
+      <c r="F171" s="67" t="n"/>
+      <c r="G171" s="73" t="n"/>
     </row>
     <row r="172">
-      <c r="D172" s="71" t="n"/>
-      <c r="E172" s="72" t="n"/>
-      <c r="F172" s="35" t="n"/>
-    </row>
-    <row r="173">
-      <c r="D173" s="71" t="n"/>
-      <c r="E173" s="72" t="n"/>
-      <c r="F173" s="35" t="n"/>
-    </row>
-    <row r="174">
-      <c r="D174" s="71" t="n"/>
-      <c r="E174" s="72" t="n"/>
-      <c r="F174" s="35" t="n"/>
-    </row>
-    <row r="176" ht="20" customHeight="1">
-      <c r="B176" s="10" t="inlineStr">
-        <is>
-          <t>Shear (AS 4100 Cl. 5.11)</t>
-        </is>
-      </c>
-      <c r="C176" s="11" t="n"/>
-      <c r="D176" s="11" t="n"/>
-      <c r="E176" s="11" t="n"/>
-      <c r="F176" s="11" t="n"/>
-      <c r="G176" s="11" t="n"/>
-      <c r="H176" s="11" t="n"/>
-      <c r="I176" s="11" t="n"/>
-      <c r="J176" s="11" t="n"/>
+      <c r="B172" s="34" t="n"/>
+      <c r="C172" s="70" t="n"/>
+      <c r="D172" s="63" t="n"/>
+      <c r="E172" s="70" t="n"/>
+      <c r="F172" s="67" t="n"/>
+      <c r="G172" s="73" t="n"/>
+    </row>
+    <row r="174" ht="20" customHeight="1">
+      <c r="B174" s="10" t="inlineStr">
+        <is>
+          <t>Support Reactions</t>
+        </is>
+      </c>
+      <c r="C174" s="11" t="n"/>
+      <c r="D174" s="11" t="n"/>
+      <c r="E174" s="11" t="n"/>
+      <c r="F174" s="11" t="n"/>
+      <c r="G174" s="11" t="n"/>
+      <c r="H174" s="11" t="n"/>
+      <c r="I174" s="11" t="n"/>
+      <c r="J174" s="11" t="n"/>
+    </row>
+    <row r="175">
+      <c r="B175" s="15" t="inlineStr">
+        <is>
+          <t>Unfactored, per case, positive in the case direction (Wu/Wiu = uplift). Self-weight is in G.  To load another beam: add a Point row with the same case and set Direct to e.g. ='B1'!RxnR_G</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="B176" s="25" t="inlineStr">
+        <is>
+          <t>Case</t>
+        </is>
+      </c>
+      <c r="D176" s="25" t="inlineStr">
+        <is>
+          <t>Left (kN)</t>
+        </is>
+      </c>
+      <c r="E176" s="25" t="inlineStr">
+        <is>
+          <t>Right (kN)</t>
+        </is>
+      </c>
+      <c r="F176" s="25" t="inlineStr">
+        <is>
+          <t>Transfer names</t>
+        </is>
+      </c>
     </row>
     <row r="177">
-      <c r="B177" s="59" t="inlineStr">
-        <is>
-          <t>Combo</t>
-        </is>
-      </c>
-      <c r="C177" s="59" t="inlineStr">
-        <is>
-          <t>V* (kN)</t>
-        </is>
-      </c>
-      <c r="D177" s="59" t="inlineStr">
-        <is>
-          <t>at x (m)</t>
-        </is>
-      </c>
-      <c r="E177" s="59" t="inlineStr">
-        <is>
-          <t>φVv (kN)</t>
-        </is>
-      </c>
-      <c r="F177" s="59" t="inlineStr">
-        <is>
-          <t>Utilisation</t>
-        </is>
-      </c>
-      <c r="G177" s="59" t="inlineStr">
-        <is>
-          <t>Note</t>
+      <c r="B177" s="51" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C177" s="52" t="n"/>
+      <c r="D177" s="36" cm="1">
+        <f t="array" ref="D177">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,2)</f>
+        <v/>
+      </c>
+      <c r="E177" s="36" cm="1">
+        <f t="array" ref="E177">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,3)</f>
+        <v/>
+      </c>
+      <c r="F177" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_G  ·  RxnR_G</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="B178" s="34" cm="1">
-        <f t="array" ref="B178">OAR.SHEAR(SectionSize,Grade,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79))</f>
-        <v/>
-      </c>
-      <c r="C178" s="70" t="n"/>
-      <c r="D178" s="64" t="n"/>
-      <c r="E178" s="70" t="n"/>
-      <c r="F178" s="68" t="n"/>
-      <c r="G178" s="73" t="n"/>
+      <c r="B178" s="51" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="C178" s="52" t="n"/>
+      <c r="D178" s="36" cm="1">
+        <f t="array" ref="D178">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,2)</f>
+        <v/>
+      </c>
+      <c r="E178" s="36" cm="1">
+        <f t="array" ref="E178">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,3)</f>
+        <v/>
+      </c>
+      <c r="F178" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_Q  ·  RxnR_Q</t>
+        </is>
+      </c>
     </row>
     <row r="179">
-      <c r="B179" s="34" t="n"/>
-      <c r="C179" s="70" t="n"/>
-      <c r="D179" s="64" t="n"/>
-      <c r="E179" s="70" t="n"/>
-      <c r="F179" s="68" t="n"/>
-      <c r="G179" s="73" t="n"/>
+      <c r="B179" s="51" t="inlineStr">
+        <is>
+          <t>Wd</t>
+        </is>
+      </c>
+      <c r="C179" s="52" t="n"/>
+      <c r="D179" s="36" cm="1">
+        <f t="array" ref="D179">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,2)</f>
+        <v/>
+      </c>
+      <c r="E179" s="36" cm="1">
+        <f t="array" ref="E179">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,3)</f>
+        <v/>
+      </c>
+      <c r="F179" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_Wd  ·  RxnR_Wd</t>
+        </is>
+      </c>
     </row>
     <row r="180">
-      <c r="B180" s="34" t="n"/>
-      <c r="C180" s="70" t="n"/>
-      <c r="D180" s="64" t="n"/>
-      <c r="E180" s="70" t="n"/>
-      <c r="F180" s="68" t="n"/>
-      <c r="G180" s="73" t="n"/>
+      <c r="B180" s="51" t="inlineStr">
+        <is>
+          <t>Wu</t>
+        </is>
+      </c>
+      <c r="C180" s="52" t="n"/>
+      <c r="D180" s="36" cm="1">
+        <f t="array" ref="D180">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,2)</f>
+        <v/>
+      </c>
+      <c r="E180" s="36" cm="1">
+        <f t="array" ref="E180">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,3)</f>
+        <v/>
+      </c>
+      <c r="F180" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_Wu  ·  RxnR_Wu</t>
+        </is>
+      </c>
     </row>
     <row r="181">
-      <c r="B181" s="34" t="n"/>
-      <c r="C181" s="70" t="n"/>
-      <c r="D181" s="64" t="n"/>
-      <c r="E181" s="70" t="n"/>
-      <c r="F181" s="68" t="n"/>
-      <c r="G181" s="73" t="n"/>
+      <c r="B181" s="51" t="inlineStr">
+        <is>
+          <t>Wid</t>
+        </is>
+      </c>
+      <c r="C181" s="52" t="n"/>
+      <c r="D181" s="36" cm="1">
+        <f t="array" ref="D181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,2)</f>
+        <v/>
+      </c>
+      <c r="E181" s="36" cm="1">
+        <f t="array" ref="E181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,3)</f>
+        <v/>
+      </c>
+      <c r="F181" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_Wid  ·  RxnR_Wid</t>
+        </is>
+      </c>
     </row>
     <row r="182">
-      <c r="B182" s="34" t="n"/>
-      <c r="C182" s="70" t="n"/>
-      <c r="D182" s="64" t="n"/>
-      <c r="E182" s="70" t="n"/>
-      <c r="F182" s="68" t="n"/>
-      <c r="G182" s="73" t="n"/>
-    </row>
-    <row r="183">
-      <c r="B183" s="34" t="n"/>
-      <c r="C183" s="70" t="n"/>
-      <c r="D183" s="64" t="n"/>
-      <c r="E183" s="70" t="n"/>
-      <c r="F183" s="68" t="n"/>
-      <c r="G183" s="73" t="n"/>
+      <c r="B182" s="51" t="inlineStr">
+        <is>
+          <t>Wiu</t>
+        </is>
+      </c>
+      <c r="C182" s="52" t="n"/>
+      <c r="D182" s="36" cm="1">
+        <f t="array" ref="D182">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,2)</f>
+        <v/>
+      </c>
+      <c r="E182" s="36" cm="1">
+        <f t="array" ref="E182">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,3)</f>
+        <v/>
+      </c>
+      <c r="F182" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_Wiu  ·  RxnR_Wiu</t>
+        </is>
+      </c>
     </row>
     <row r="184">
-      <c r="B184" s="34" t="n"/>
-      <c r="C184" s="70" t="n"/>
-      <c r="D184" s="64" t="n"/>
-      <c r="E184" s="70" t="n"/>
-      <c r="F184" s="68" t="n"/>
-      <c r="G184" s="73" t="n"/>
+      <c r="B184" s="15" t="inlineStr">
+        <is>
+          <t>All cases and active combinations (kN, + = upward reaction; uplift cases show negative)</t>
+        </is>
+      </c>
     </row>
     <row r="185">
-      <c r="B185" s="34" t="n"/>
-      <c r="C185" s="70" t="n"/>
-      <c r="D185" s="64" t="n"/>
-      <c r="E185" s="70" t="n"/>
-      <c r="F185" s="68" t="n"/>
-      <c r="G185" s="73" t="n"/>
-    </row>
-    <row r="187" ht="20" customHeight="1">
-      <c r="B187" s="10" t="inlineStr">
-        <is>
-          <t>Support Reactions</t>
-        </is>
-      </c>
-      <c r="C187" s="11" t="n"/>
-      <c r="D187" s="11" t="n"/>
-      <c r="E187" s="11" t="n"/>
-      <c r="F187" s="11" t="n"/>
-      <c r="G187" s="11" t="n"/>
-      <c r="H187" s="11" t="n"/>
-      <c r="I187" s="11" t="n"/>
-      <c r="J187" s="11" t="n"/>
+      <c r="B185" s="59" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C185" s="59" t="inlineStr">
+        <is>
+          <t>Left (kN)</t>
+        </is>
+      </c>
+      <c r="D185" s="59" t="inlineStr">
+        <is>
+          <t>Right (kN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="B186" s="34" cm="1">
+        <f t="array" ref="B186">OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
+        <v/>
+      </c>
+      <c r="C186" s="63" t="n"/>
+      <c r="D186" s="63" t="n"/>
+    </row>
+    <row r="187">
+      <c r="B187" s="34" t="n"/>
+      <c r="C187" s="63" t="n"/>
+      <c r="D187" s="63" t="n"/>
     </row>
     <row r="188">
-      <c r="B188" s="15" t="inlineStr">
-        <is>
-          <t>Unfactored, per case, positive in the case direction (Wu/Wiu = uplift). Self-weight is in G.  To load another beam: add a Point row with the same case and set Direct to e.g. ='B1'!RxnR_G</t>
-        </is>
-      </c>
+      <c r="B188" s="34" t="n"/>
+      <c r="C188" s="63" t="n"/>
+      <c r="D188" s="63" t="n"/>
     </row>
     <row r="189">
-      <c r="B189" s="25" t="inlineStr">
-        <is>
-          <t>Case</t>
-        </is>
-      </c>
-      <c r="D189" s="25" t="inlineStr">
-        <is>
-          <t>Left (kN)</t>
-        </is>
-      </c>
-      <c r="E189" s="25" t="inlineStr">
-        <is>
-          <t>Right (kN)</t>
-        </is>
-      </c>
-      <c r="F189" s="25" t="inlineStr">
-        <is>
-          <t>Transfer names</t>
-        </is>
-      </c>
+      <c r="B189" s="34" t="n"/>
+      <c r="C189" s="63" t="n"/>
+      <c r="D189" s="63" t="n"/>
     </row>
     <row r="190">
-      <c r="B190" s="51" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="C190" s="52" t="n"/>
-      <c r="D190" s="36" cm="1">
-        <f t="array" ref="D190">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),1,2)</f>
-        <v/>
-      </c>
-      <c r="E190" s="36" cm="1">
-        <f t="array" ref="E190">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),1,3)</f>
-        <v/>
-      </c>
-      <c r="F190" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_G  ·  RxnR_G</t>
-        </is>
-      </c>
+      <c r="B190" s="34" t="n"/>
+      <c r="C190" s="63" t="n"/>
+      <c r="D190" s="63" t="n"/>
     </row>
     <row r="191">
-      <c r="B191" s="51" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="C191" s="52" t="n"/>
-      <c r="D191" s="36" cm="1">
-        <f t="array" ref="D191">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),2,2)</f>
-        <v/>
-      </c>
-      <c r="E191" s="36" cm="1">
-        <f t="array" ref="E191">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),2,3)</f>
-        <v/>
-      </c>
-      <c r="F191" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_Q  ·  RxnR_Q</t>
-        </is>
-      </c>
+      <c r="B191" s="34" t="n"/>
+      <c r="C191" s="63" t="n"/>
+      <c r="D191" s="63" t="n"/>
     </row>
     <row r="192">
-      <c r="B192" s="51" t="inlineStr">
-        <is>
-          <t>Wd</t>
-        </is>
-      </c>
-      <c r="C192" s="52" t="n"/>
-      <c r="D192" s="36" cm="1">
-        <f t="array" ref="D192">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),3,2)</f>
-        <v/>
-      </c>
-      <c r="E192" s="36" cm="1">
-        <f t="array" ref="E192">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),3,3)</f>
-        <v/>
-      </c>
-      <c r="F192" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_Wd  ·  RxnR_Wd</t>
-        </is>
-      </c>
+      <c r="B192" s="34" t="n"/>
+      <c r="C192" s="63" t="n"/>
+      <c r="D192" s="63" t="n"/>
     </row>
     <row r="193">
-      <c r="B193" s="51" t="inlineStr">
-        <is>
-          <t>Wu</t>
-        </is>
-      </c>
-      <c r="C193" s="52" t="n"/>
-      <c r="D193" s="36" cm="1">
-        <f t="array" ref="D193">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),4,2)</f>
-        <v/>
-      </c>
-      <c r="E193" s="36" cm="1">
-        <f t="array" ref="E193">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),4,3)</f>
-        <v/>
-      </c>
-      <c r="F193" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_Wu  ·  RxnR_Wu</t>
-        </is>
-      </c>
+      <c r="B193" s="34" t="n"/>
+      <c r="C193" s="63" t="n"/>
+      <c r="D193" s="63" t="n"/>
     </row>
     <row r="194">
-      <c r="B194" s="51" t="inlineStr">
-        <is>
-          <t>Wid</t>
-        </is>
-      </c>
-      <c r="C194" s="52" t="n"/>
-      <c r="D194" s="36" cm="1">
-        <f t="array" ref="D194">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),5,2)</f>
-        <v/>
-      </c>
-      <c r="E194" s="36" cm="1">
-        <f t="array" ref="E194">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),5,3)</f>
-        <v/>
-      </c>
-      <c r="F194" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_Wid  ·  RxnR_Wid</t>
-        </is>
-      </c>
+      <c r="B194" s="34" t="n"/>
+      <c r="C194" s="63" t="n"/>
+      <c r="D194" s="63" t="n"/>
     </row>
     <row r="195">
-      <c r="B195" s="51" t="inlineStr">
-        <is>
-          <t>Wiu</t>
-        </is>
-      </c>
-      <c r="C195" s="52" t="n"/>
-      <c r="D195" s="36" cm="1">
-        <f t="array" ref="D195">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),6,2)</f>
-        <v/>
-      </c>
-      <c r="E195" s="36" cm="1">
-        <f t="array" ref="E195">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79)),6,3)</f>
-        <v/>
-      </c>
-      <c r="F195" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_Wiu  ·  RxnR_Wiu</t>
-        </is>
-      </c>
+      <c r="B195" s="34" t="n"/>
+      <c r="C195" s="63" t="n"/>
+      <c r="D195" s="63" t="n"/>
+    </row>
+    <row r="196">
+      <c r="B196" s="34" t="n"/>
+      <c r="C196" s="63" t="n"/>
+      <c r="D196" s="63" t="n"/>
     </row>
     <row r="197">
-      <c r="B197" s="15" t="inlineStr">
-        <is>
-          <t>All cases and active combinations (kN, + = upward reaction; uplift cases show negative)</t>
-        </is>
-      </c>
+      <c r="B197" s="34" t="n"/>
+      <c r="C197" s="63" t="n"/>
+      <c r="D197" s="63" t="n"/>
     </row>
     <row r="198">
-      <c r="B198" s="59" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="C198" s="59" t="inlineStr">
-        <is>
-          <t>Left (kN)</t>
-        </is>
-      </c>
-      <c r="D198" s="59" t="inlineStr">
-        <is>
-          <t>Right (kN)</t>
-        </is>
-      </c>
+      <c r="B198" s="34" t="n"/>
+      <c r="C198" s="63" t="n"/>
+      <c r="D198" s="63" t="n"/>
     </row>
     <row r="199">
-      <c r="B199" s="34" cm="1">
-        <f t="array" ref="B199">OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B79))</f>
-        <v/>
-      </c>
-      <c r="C199" s="64" t="n"/>
-      <c r="D199" s="64" t="n"/>
-    </row>
-    <row r="200">
-      <c r="B200" s="34" t="n"/>
-      <c r="C200" s="64" t="n"/>
-      <c r="D200" s="64" t="n"/>
-    </row>
-    <row r="201">
-      <c r="B201" s="34" t="n"/>
-      <c r="C201" s="64" t="n"/>
-      <c r="D201" s="64" t="n"/>
-    </row>
-    <row r="202">
-      <c r="B202" s="34" t="n"/>
-      <c r="C202" s="64" t="n"/>
-      <c r="D202" s="64" t="n"/>
-    </row>
-    <row r="203">
-      <c r="B203" s="34" t="n"/>
-      <c r="C203" s="64" t="n"/>
-      <c r="D203" s="64" t="n"/>
-    </row>
-    <row r="204">
-      <c r="B204" s="34" t="n"/>
-      <c r="C204" s="64" t="n"/>
-      <c r="D204" s="64" t="n"/>
-    </row>
-    <row r="205">
-      <c r="B205" s="34" t="n"/>
-      <c r="C205" s="64" t="n"/>
-      <c r="D205" s="64" t="n"/>
-    </row>
-    <row r="206">
-      <c r="B206" s="34" t="n"/>
-      <c r="C206" s="64" t="n"/>
-      <c r="D206" s="64" t="n"/>
-    </row>
-    <row r="207">
-      <c r="B207" s="34" t="n"/>
-      <c r="C207" s="64" t="n"/>
-      <c r="D207" s="64" t="n"/>
-    </row>
-    <row r="208">
-      <c r="B208" s="34" t="n"/>
-      <c r="C208" s="64" t="n"/>
-      <c r="D208" s="64" t="n"/>
-    </row>
-    <row r="209">
-      <c r="B209" s="34" t="n"/>
-      <c r="C209" s="64" t="n"/>
-      <c r="D209" s="64" t="n"/>
-    </row>
-    <row r="210">
-      <c r="B210" s="34" t="n"/>
-      <c r="C210" s="64" t="n"/>
-      <c r="D210" s="64" t="n"/>
-    </row>
-    <row r="211">
-      <c r="B211" s="34" t="n"/>
-      <c r="C211" s="64" t="n"/>
-      <c r="D211" s="64" t="n"/>
-    </row>
-    <row r="212">
-      <c r="B212" s="34" t="n"/>
-      <c r="C212" s="64" t="n"/>
-      <c r="D212" s="64" t="n"/>
+      <c r="B199" s="34" t="n"/>
+      <c r="C199" s="63" t="n"/>
+      <c r="D199" s="63" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="F182:G182"/>
     <mergeCell ref="B16:C16"/>
-    <mergeCell ref="F191:G191"/>
+    <mergeCell ref="F178:G178"/>
     <mergeCell ref="F10:G10"/>
-    <mergeCell ref="B194:C194"/>
-    <mergeCell ref="B190:C190"/>
     <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B193:C193"/>
-    <mergeCell ref="F193:G193"/>
     <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B180:C180"/>
+    <mergeCell ref="B176:C176"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B39:C39"/>
-    <mergeCell ref="F192:G192"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="M8:T40"/>
-    <mergeCell ref="B195:C195"/>
-    <mergeCell ref="F189:G189"/>
+    <mergeCell ref="F177:G177"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="G2:J2"/>
-    <mergeCell ref="F194:G194"/>
+    <mergeCell ref="B179:C179"/>
     <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B181:C181"/>
+    <mergeCell ref="F181:G181"/>
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B182:C182"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="E30:F30"/>
-    <mergeCell ref="B191:C191"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="F190:G190"/>
+    <mergeCell ref="B178:C178"/>
+    <mergeCell ref="F180:G180"/>
     <mergeCell ref="B40:C40"/>
+    <mergeCell ref="F179:G179"/>
     <mergeCell ref="I1:J1"/>
-    <mergeCell ref="B192:C192"/>
+    <mergeCell ref="F176:G176"/>
     <mergeCell ref="I4:J4"/>
+    <mergeCell ref="B177:C177"/>
     <mergeCell ref="B15:C15"/>
-    <mergeCell ref="F195:G195"/>
     <mergeCell ref="I10:J10"/>
-    <mergeCell ref="B189:C189"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="I9:J9"/>
@@ -6267,9 +5871,9 @@
       <formula>$C47="Point"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B79:J86">
+  <conditionalFormatting sqref="B66:J73">
     <cfRule type="expression" priority="10" dxfId="7">
-      <formula>$B79&lt;&gt;""</formula>
+      <formula>$B66&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:J22">
@@ -6277,44 +5881,44 @@
       <formula>NumUpliftCombos=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B99:G103">
+  <conditionalFormatting sqref="B86:G90">
     <cfRule type="expression" priority="12" dxfId="7">
-      <formula>$B99&lt;&gt;""</formula>
+      <formula>$B86&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G99:G103">
+  <conditionalFormatting sqref="G86:G90">
     <cfRule type="expression" priority="13" dxfId="0">
-      <formula>AND(ISNUMBER(G99),G99&gt;1)</formula>
+      <formula>AND(ISNUMBER(G86),G86&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B133:J148">
+  <conditionalFormatting sqref="B120:J135">
     <cfRule type="expression" priority="14" dxfId="7">
-      <formula>$B133&lt;&gt;""</formula>
+      <formula>$B120&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J133:J148">
+  <conditionalFormatting sqref="J120:J135">
     <cfRule type="expression" priority="15" dxfId="0">
-      <formula>AND(ISNUMBER(J133),J133&gt;1)</formula>
+      <formula>AND(ISNUMBER(J120),J120&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C133:C148">
+  <conditionalFormatting sqref="C120:C135">
     <cfRule type="expression" priority="16" dxfId="9">
-      <formula>RIGHT(C133,1)="*"</formula>
+      <formula>RIGHT(C120,1)="*"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B178:F185">
+  <conditionalFormatting sqref="B165:F172">
     <cfRule type="expression" priority="17" dxfId="7">
-      <formula>$B178&lt;&gt;""</formula>
+      <formula>$B165&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F178:F185">
+  <conditionalFormatting sqref="F165:F172">
     <cfRule type="expression" priority="18" dxfId="0">
-      <formula>AND(ISNUMBER(F178),F178&gt;1)</formula>
+      <formula>AND(ISNUMBER(F165),F165&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B199:D212">
+  <conditionalFormatting sqref="B186:D199">
     <cfRule type="expression" priority="19" dxfId="7">
-      <formula>$B199&lt;&gt;""</formula>
+      <formula>$B186&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="13">
@@ -6348,10 +5952,10 @@
     <dataValidation sqref="Q47:Q84" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Top,Bottom"</formula1>
     </dataValidation>
-    <dataValidation sqref="E76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Floor,Roof,All,Custom"</formula1>
     </dataValidation>
-    <dataValidation sqref="E90:F94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E77:F81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"F,P,L,U,–"</formula1>
     </dataValidation>
     <dataValidation sqref="E27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Section size" error="Pick a section from the list for the selected Section type." type="list">
@@ -6370,8 +5974,8 @@
   </headerFooter>
   <rowBreaks count="3" manualBreakCount="3">
     <brk id="42" min="0" max="16383" man="1"/>
-    <brk id="96" min="0" max="16383" man="1"/>
-    <brk id="150" min="0" max="16383" man="1"/>
+    <brk id="83" min="0" max="16383" man="1"/>
+    <brk id="137" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <tableParts count="4">

</xml_diff>

<commit_message>
Sheet: Load and pressure lookup as table calculated columns (auto-fill on new/cleared rows)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -1183,17 +1183,20 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Loads_B1" displayName="Loads_B1" ref="B46:J57" headerRowCount="1">
-  <autoFilter ref="B46:J57"/>
   <tableColumns count="9">
-    <tableColumn id="2" name="Case"/>
-    <tableColumn id="3" name="Type"/>
-    <tableColumn id="4" name="Description"/>
-    <tableColumn id="5" name="Trib (m | m²)"/>
-    <tableColumn id="6" name="Press. (kPa)"/>
-    <tableColumn id="7" name="+ Direct (kN/m | kN)"/>
-    <tableColumn id="8" name="Start (mm)"/>
-    <tableColumn id="9" name="End (mm)"/>
-    <tableColumn id="10" name="Load"/>
+    <tableColumn id="1" name="Case"/>
+    <tableColumn id="2" name="Type"/>
+    <tableColumn id="3" name="Description"/>
+    <tableColumn id="4" name="Trib (m | m²)"/>
+    <tableColumn id="5" name="Press. (kPa)">
+      <calculatedColumnFormula>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(Loads_B1[[#This Row],[Description]],LoadLib_B1[Description],0)),"")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" name="+ Direct (kN/m | kN)"/>
+    <tableColumn id="7" name="Start (mm)"/>
+    <tableColumn id="8" name="End (mm)"/>
+    <tableColumn id="9" name="Load">
+      <calculatedColumnFormula>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showRowStripes="0"/>
 </table>
@@ -3637,14 +3640,14 @@
         <v>5.65</v>
       </c>
       <c r="F47" s="30">
-        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(D47,LoadLib_B1[Description],0)),"")</f>
+        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(Loads_B1[[#This Row],[Description]],LoadLib_B1[Description],0)),"")</f>
         <v/>
       </c>
       <c r="G47" s="30" t="n"/>
       <c r="H47" s="47" t="n"/>
       <c r="I47" s="47" t="n"/>
       <c r="J47" s="61">
-        <f>IF(B47="","",N(E47)*N(F47)+N(G47))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="M47" s="2" t="n"/>
@@ -3716,14 +3719,14 @@
         <v>5.65</v>
       </c>
       <c r="F48" s="30">
-        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(D48,LoadLib_B1[Description],0)),"")</f>
+        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(Loads_B1[[#This Row],[Description]],LoadLib_B1[Description],0)),"")</f>
         <v/>
       </c>
       <c r="G48" s="30" t="n"/>
       <c r="H48" s="47" t="n"/>
       <c r="I48" s="47" t="n"/>
       <c r="J48" s="61">
-        <f>IF(B48="","",N(E48)*N(F48)+N(G48))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="M48" s="2" t="n"/>
@@ -3792,14 +3795,17 @@
         </is>
       </c>
       <c r="E49" s="60" t="n"/>
-      <c r="F49" s="30" t="n"/>
+      <c r="F49" s="30">
+        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(Loads_B1[[#This Row],[Description]],LoadLib_B1[Description],0)),"")</f>
+        <v/>
+      </c>
       <c r="G49" s="30" t="n">
         <v>0.05</v>
       </c>
       <c r="H49" s="47" t="n"/>
       <c r="I49" s="47" t="n"/>
       <c r="J49" s="61">
-        <f>IF(B49="","",N(E49)*N(F49)+N(G49))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="M49" s="2" t="n"/>
@@ -3872,14 +3878,14 @@
         <v>5.65</v>
       </c>
       <c r="F50" s="30">
-        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(D50,LoadLib_B1[Description],0)),"")</f>
+        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(Loads_B1[[#This Row],[Description]],LoadLib_B1[Description],0)),"")</f>
         <v/>
       </c>
       <c r="G50" s="30" t="n"/>
       <c r="H50" s="47" t="n"/>
       <c r="I50" s="47" t="n"/>
       <c r="J50" s="61">
-        <f>IF(B50="","",N(E50)*N(F50)+N(G50))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="M50" s="2" t="n"/>
@@ -3958,7 +3964,7 @@
       <c r="H51" s="47" t="n"/>
       <c r="I51" s="47" t="n"/>
       <c r="J51" s="61">
-        <f>IF(B51="","",N(E51)*N(F51)+N(G51))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="M51" s="2" t="n"/>
@@ -4036,7 +4042,7 @@
       <c r="H52" s="47" t="n"/>
       <c r="I52" s="47" t="n"/>
       <c r="J52" s="61">
-        <f>IF(B52="","",N(E52)*N(F52)+N(G52))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="M52" s="2" t="n"/>
@@ -4090,7 +4096,7 @@
       <c r="H53" s="47" t="n"/>
       <c r="I53" s="47" t="n"/>
       <c r="J53" s="61">
-        <f>IF(B53="","",N(E53)*N(F53)+N(G53))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="M53" s="2" t="n"/>
@@ -4144,7 +4150,7 @@
       <c r="H54" s="47" t="n"/>
       <c r="I54" s="47" t="n"/>
       <c r="J54" s="61">
-        <f>IF(B54="","",N(E54)*N(F54)+N(G54))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="M54" s="2" t="n"/>
@@ -4202,7 +4208,7 @@
       </c>
       <c r="I55" s="47" t="n"/>
       <c r="J55" s="61">
-        <f>IF(B55="","",N(E55)*N(F55)+N(G55))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="AN55" s="20" t="inlineStr">
@@ -4216,12 +4222,15 @@
       <c r="C56" s="2" t="n"/>
       <c r="D56" s="5" t="n"/>
       <c r="E56" s="60" t="n"/>
-      <c r="F56" s="30" t="n"/>
+      <c r="F56" s="30">
+        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(Loads_B1[[#This Row],[Description]],LoadLib_B1[Description],0)),"")</f>
+        <v/>
+      </c>
       <c r="G56" s="30" t="n"/>
       <c r="H56" s="47" t="n"/>
       <c r="I56" s="47" t="n"/>
       <c r="J56" s="61">
-        <f>IF(B56="","",N(E56)*N(F56)+N(G56))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="R56" s="1" t="inlineStr">
@@ -4244,12 +4253,15 @@
       <c r="C57" s="2" t="n"/>
       <c r="D57" s="5" t="n"/>
       <c r="E57" s="60" t="n"/>
-      <c r="F57" s="30" t="n"/>
+      <c r="F57" s="30">
+        <f>IFERROR(INDEX(LoadLib_B1[kPa],MATCH(Loads_B1[[#This Row],[Description]],LoadLib_B1[Description],0)),"")</f>
+        <v/>
+      </c>
       <c r="G57" s="30" t="n"/>
       <c r="H57" s="47" t="n"/>
       <c r="I57" s="47" t="n"/>
       <c r="J57" s="61">
-        <f>IF(B57="","",N(E57)*N(F57)+N(G57))</f>
+        <f>IF(Loads_B1[[#This Row],[Case]]="","",N(Loads_B1[[#This Row],[Trib (m | m²)]])*N(Loads_B1[[#This Row],[Press. (kPa)]])+N(Loads_B1[[#This Row],[+ Direct (kN/m | kN)]]))</f>
         <v/>
       </c>
       <c r="AN57" s="20" t="inlineStr">

</xml_diff>

<commit_message>
v0.2.4: αm override split into top/bottom columns; overrides that would be ignored now raise an error
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -54,24 +54,24 @@
     <definedName name="NumUpliftCombos" localSheetId="0">'B1'!$S$56</definedName>
     <definedName name="CombSet" localSheetId="0">'B1'!$E$63</definedName>
     <definedName name="PsiC" localSheetId="0">'B1'!$G$63</definedName>
-    <definedName name="kl_Top" localSheetId="0">'B1'!$I$77</definedName>
-    <definedName name="kl_Bot" localSheetId="0">'B1'!$J$77</definedName>
-    <definedName name="kr_Top" localSheetId="0">'B1'!$I$78</definedName>
-    <definedName name="kr_Bot" localSheetId="0">'B1'!$J$78</definedName>
-    <definedName name="RxnL_G" localSheetId="0">'B1'!$D$177</definedName>
-    <definedName name="RxnR_G" localSheetId="0">'B1'!$E$177</definedName>
-    <definedName name="RxnL_Q" localSheetId="0">'B1'!$D$178</definedName>
-    <definedName name="RxnR_Q" localSheetId="0">'B1'!$E$178</definedName>
-    <definedName name="RxnL_Wd" localSheetId="0">'B1'!$D$179</definedName>
-    <definedName name="RxnR_Wd" localSheetId="0">'B1'!$E$179</definedName>
-    <definedName name="RxnL_Wu" localSheetId="0">'B1'!$D$180</definedName>
-    <definedName name="RxnR_Wu" localSheetId="0">'B1'!$E$180</definedName>
-    <definedName name="RxnL_Wid" localSheetId="0">'B1'!$D$181</definedName>
-    <definedName name="RxnR_Wid" localSheetId="0">'B1'!$E$181</definedName>
-    <definedName name="RxnL_Wiu" localSheetId="0">'B1'!$D$182</definedName>
-    <definedName name="RxnR_Wiu" localSheetId="0">'B1'!$E$182</definedName>
-    <definedName name="Out_Reactions" localSheetId="0">'B1'!$B$186</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'B1'!$A$1:$K$200</definedName>
+    <definedName name="kl_Top" localSheetId="0">'B1'!$F$85</definedName>
+    <definedName name="kl_Bot" localSheetId="0">'B1'!$G$85</definedName>
+    <definedName name="kr_Top" localSheetId="0">'B1'!$F$86</definedName>
+    <definedName name="kr_Bot" localSheetId="0">'B1'!$G$86</definedName>
+    <definedName name="RxnL_G" localSheetId="0">'B1'!$D$181</definedName>
+    <definedName name="RxnR_G" localSheetId="0">'B1'!$E$181</definedName>
+    <definedName name="RxnL_Q" localSheetId="0">'B1'!$D$182</definedName>
+    <definedName name="RxnR_Q" localSheetId="0">'B1'!$E$182</definedName>
+    <definedName name="RxnL_Wd" localSheetId="0">'B1'!$D$183</definedName>
+    <definedName name="RxnR_Wd" localSheetId="0">'B1'!$E$183</definedName>
+    <definedName name="RxnL_Wu" localSheetId="0">'B1'!$D$184</definedName>
+    <definedName name="RxnR_Wu" localSheetId="0">'B1'!$E$184</definedName>
+    <definedName name="RxnL_Wid" localSheetId="0">'B1'!$D$185</definedName>
+    <definedName name="RxnR_Wid" localSheetId="0">'B1'!$E$185</definedName>
+    <definedName name="RxnL_Wiu" localSheetId="0">'B1'!$D$186</definedName>
+    <definedName name="RxnR_Wiu" localSheetId="0">'B1'!$E$186</definedName>
+    <definedName name="Out_Reactions" localSheetId="0">'B1'!$B$190</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'B1'!$A$1:$K$204</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1102,7 +1102,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>92</row>
+      <row>96</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6336000" cy="1944000"/>
@@ -1124,7 +1124,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>106</row>
+      <row>110</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6336000" cy="1944000"/>
@@ -1226,15 +1226,16 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Restraints_B1" displayName="Restraints_B1" ref="B76:G81" headerRowCount="1">
-  <autoFilter ref="B76:G81"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Restraints_B1" displayName="Restraints_B1" ref="B76:H81" headerRowCount="1">
+  <autoFilter ref="B76:H81"/>
+  <tableColumns count="7">
     <tableColumn id="2" name="x (mm)"/>
     <tableColumn id="3" name="Ref"/>
     <tableColumn id="4" name="Restraint provided by"/>
     <tableColumn id="5" name="Top flange"/>
     <tableColumn id="6" name="Bottom fl."/>
-    <tableColumn id="7" name="αm override"/>
+    <tableColumn id="7" name="αm top →"/>
+    <tableColumn id="8" name="αm bot. →"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showRowStripes="0"/>
 </table>
@@ -1530,7 +1531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:BB199"/>
+  <dimension ref="B1:BB203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.5" customWidth="1" min="1" max="1"/>
@@ -1780,7 +1781,7 @@
       <c r="S8" s="17" t="n"/>
       <c r="T8" s="18" t="n"/>
       <c r="Z8" s="19" cm="1">
-        <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
+        <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$F$85:$G$86)</f>
         <v/>
       </c>
       <c r="AL8" s="19" cm="1">
@@ -2181,7 +2182,7 @@
         </is>
       </c>
       <c r="E15" s="37" cm="1">
-        <f t="array" ref="E15">INDEX(_xlfn.ANCHORARRAY(B86),1,2)</f>
+        <f t="array" ref="E15">INDEX(_xlfn.ANCHORARRAY(B90),1,2)</f>
         <v/>
       </c>
       <c r="F15" s="37">
@@ -2281,7 +2282,7 @@
         </is>
       </c>
       <c r="E16" s="37" cm="1">
-        <f t="array" ref="E16">INDEX(_xlfn.ANCHORARRAY(B86),2,2)</f>
+        <f t="array" ref="E16">INDEX(_xlfn.ANCHORARRAY(B90),2,2)</f>
         <v/>
       </c>
       <c r="F16" s="37">
@@ -2381,7 +2382,7 @@
         </is>
       </c>
       <c r="E17" s="37" cm="1">
-        <f t="array" ref="E17">INDEX(_xlfn.ANCHORARRAY(B86),3,2)</f>
+        <f t="array" ref="E17">INDEX(_xlfn.ANCHORARRAY(B90),3,2)</f>
         <v/>
       </c>
       <c r="F17" s="37">
@@ -2481,7 +2482,7 @@
         </is>
       </c>
       <c r="E18" s="37" cm="1">
-        <f t="array" ref="E18">INDEX(_xlfn.ANCHORARRAY(B86),4,2)</f>
+        <f t="array" ref="E18">INDEX(_xlfn.ANCHORARRAY(B90),4,2)</f>
         <v/>
       </c>
       <c r="F18" s="37">
@@ -2581,7 +2582,7 @@
         </is>
       </c>
       <c r="E19" s="37" cm="1">
-        <f t="array" ref="E19">INDEX(_xlfn.ANCHORARRAY(B86),5,2)</f>
+        <f t="array" ref="E19">INDEX(_xlfn.ANCHORARRAY(B90),5,2)</f>
         <v/>
       </c>
       <c r="F19" s="37">
@@ -6617,22 +6618,12 @@
       </c>
       <c r="G76" s="25" t="inlineStr">
         <is>
-          <t>αm override</t>
+          <t>αm top →</t>
         </is>
       </c>
       <c r="H76" s="25" t="inlineStr">
         <is>
-          <t>Factor</t>
-        </is>
-      </c>
-      <c r="I76" s="25" t="inlineStr">
-        <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="J76" s="25" t="inlineStr">
-        <is>
-          <t>Bottom</t>
+          <t>αm bot. →</t>
         </is>
       </c>
       <c r="AN76" s="20" t="inlineStr">
@@ -6667,17 +6658,7 @@
         </is>
       </c>
       <c r="G77" s="30" t="n"/>
-      <c r="H77" s="35" t="inlineStr">
-        <is>
-          <t>kl</t>
-        </is>
-      </c>
-      <c r="I77" s="30" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="J77" s="30" t="n">
-        <v>1</v>
-      </c>
+      <c r="H77" s="30" t="n"/>
       <c r="AN77" s="20" t="inlineStr">
         <is>
           <t>310UC137</t>
@@ -6705,17 +6686,7 @@
         </is>
       </c>
       <c r="G78" s="30" t="n"/>
-      <c r="H78" s="35" t="inlineStr">
-        <is>
-          <t>kr</t>
-        </is>
-      </c>
-      <c r="I78" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="J78" s="30" t="n">
-        <v>1</v>
-      </c>
+      <c r="H78" s="30" t="n"/>
       <c r="AN78" s="20" t="inlineStr">
         <is>
           <t>310UC118</t>
@@ -6743,11 +6714,7 @@
         </is>
       </c>
       <c r="G79" s="30" t="n"/>
-      <c r="H79" s="15" t="inlineStr">
-        <is>
-          <t>kt from restraint</t>
-        </is>
-      </c>
+      <c r="H79" s="30" t="n"/>
       <c r="AN79" s="20" t="inlineStr">
         <is>
           <t>310UC97</t>
@@ -6780,11 +6747,7 @@
         </is>
       </c>
       <c r="G80" s="30" t="n"/>
-      <c r="H80" s="15" t="inlineStr">
-        <is>
-          <t>types (add-in)</t>
-        </is>
-      </c>
+      <c r="H80" s="30" t="n"/>
       <c r="AN80" s="20" t="inlineStr">
         <is>
           <t>250UC89.5</t>
@@ -6798,6 +6761,7 @@
       <c r="E81" s="2" t="n"/>
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="30" t="n"/>
+      <c r="H81" s="30" t="n"/>
       <c r="AN81" s="20" t="inlineStr">
         <is>
           <t>250UC73</t>
@@ -6807,7 +6771,7 @@
     <row r="82" ht="14" customHeight="1">
       <c r="B82" s="15" t="inlineStr">
         <is>
-          <t>αm override applies to the segment starting at that row (blank = Cl. 5.6.1.1(a)(iii)); flagged * in the output.</t>
+          <t>αm top / αm bot. → override αm for that flange's segment from this row to the next restraint on that flange (blank = Cl. 5.6.1.1(a)(iii)). Flagged * in the output.</t>
         </is>
       </c>
       <c r="AN82" s="20" t="inlineStr">
@@ -6823,143 +6787,194 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="20" customHeight="1">
-      <c r="B84" s="10" t="inlineStr">
+    <row r="84" ht="14" customHeight="1">
+      <c r="E84" s="25" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="F84" s="25" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="G84" s="25" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="AN84" s="20" t="inlineStr">
+        <is>
+          <t>200UC46</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="14" customHeight="1">
+      <c r="E85" s="35" t="inlineStr">
+        <is>
+          <t>kl</t>
+        </is>
+      </c>
+      <c r="F85" s="30" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G85" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" s="15" t="inlineStr">
+        <is>
+          <t>kl: load height, Table 5.6.3(2)</t>
+        </is>
+      </c>
+      <c r="AN85" s="20" t="inlineStr">
+        <is>
+          <t>150UC37</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="14" customHeight="1">
+      <c r="E86" s="35" t="inlineStr">
+        <is>
+          <t>kr</t>
+        </is>
+      </c>
+      <c r="F86" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H86" s="15" t="inlineStr">
+        <is>
+          <t>kr: rotation, Table 5.6.3(3); kt from restraints</t>
+        </is>
+      </c>
+      <c r="AN86" s="20" t="inlineStr">
+        <is>
+          <t>150UC30</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="14" customHeight="1">
+      <c r="AN87" s="20" t="inlineStr">
+        <is>
+          <t>150UC23</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="B88" s="10" t="inlineStr">
         <is>
           <t>Serviceability Checks</t>
         </is>
       </c>
-      <c r="C84" s="11" t="n"/>
-      <c r="D84" s="11" t="n"/>
-      <c r="E84" s="11" t="n"/>
-      <c r="F84" s="11" t="n"/>
-      <c r="G84" s="11" t="n"/>
-      <c r="H84" s="11" t="n"/>
-      <c r="I84" s="11" t="n"/>
-      <c r="J84" s="11" t="n"/>
-      <c r="AN84" s="20" t="inlineStr">
-        <is>
-          <t>200UC46</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="14" customHeight="1">
-      <c r="B85" s="60" t="inlineStr">
+      <c r="C88" s="11" t="n"/>
+      <c r="D88" s="11" t="n"/>
+      <c r="E88" s="11" t="n"/>
+      <c r="F88" s="11" t="n"/>
+      <c r="G88" s="11" t="n"/>
+      <c r="H88" s="11" t="n"/>
+      <c r="I88" s="11" t="n"/>
+      <c r="J88" s="11" t="n"/>
+      <c r="AN88" s="20" t="inlineStr">
+        <is>
+          <t>100UC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="14" customHeight="1">
+      <c r="B89" s="60" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C85" s="60" t="inlineStr">
+      <c r="C89" s="60" t="inlineStr">
         <is>
           <t>Δ max (mm)</t>
         </is>
       </c>
-      <c r="D85" s="60" t="inlineStr">
+      <c r="D89" s="60" t="inlineStr">
         <is>
           <t>at x (mm)</t>
         </is>
       </c>
-      <c r="E85" s="60" t="inlineStr">
+      <c r="E89" s="60" t="inlineStr">
         <is>
           <t>Limit (mm)</t>
         </is>
       </c>
-      <c r="F85" s="60" t="inlineStr">
+      <c r="F89" s="60" t="inlineStr">
         <is>
           <t>L / Δ</t>
         </is>
       </c>
-      <c r="G85" s="60" t="inlineStr">
+      <c r="G89" s="60" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
-      <c r="AN85" s="20" t="inlineStr">
-        <is>
-          <t>150UC37</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="14" customHeight="1">
-      <c r="B86" s="35" cm="1">
-        <f t="array" ref="B86">OAR.SLS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],$E$37:$F$41,PsiL,PsiS)</f>
-        <v/>
-      </c>
-      <c r="C86" s="64" t="n"/>
-      <c r="D86" s="66" t="n"/>
-      <c r="E86" s="64" t="n"/>
-      <c r="F86" s="67" t="n"/>
-      <c r="G86" s="68" t="n"/>
-      <c r="H86" s="6" t="inlineStr">
-        <is>
-          <t>Δ1kN: 1 kN at midspan,</t>
-        </is>
-      </c>
-      <c r="AN86" s="20" t="inlineStr">
-        <is>
-          <t>150UC30</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="14" customHeight="1">
-      <c r="B87" s="35" t="n"/>
-      <c r="C87" s="64" t="n"/>
-      <c r="D87" s="66" t="n"/>
-      <c r="E87" s="64" t="n"/>
-      <c r="F87" s="67" t="n"/>
-      <c r="G87" s="68" t="n"/>
-      <c r="H87" s="6" t="inlineStr">
-        <is>
-          <t>beam alone</t>
-        </is>
-      </c>
-      <c r="AN87" s="20" t="inlineStr">
-        <is>
-          <t>150UC23</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="14" customHeight="1">
-      <c r="B88" s="35" t="n"/>
-      <c r="C88" s="64" t="n"/>
-      <c r="D88" s="66" t="n"/>
-      <c r="E88" s="64" t="n"/>
-      <c r="F88" s="67" t="n"/>
-      <c r="G88" s="68" t="n"/>
-      <c r="AN88" s="20" t="inlineStr">
-        <is>
-          <t>100UC15</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="14" customHeight="1">
-      <c r="B89" s="35" t="n"/>
-      <c r="C89" s="64" t="n"/>
-      <c r="D89" s="66" t="n"/>
-      <c r="E89" s="64" t="n"/>
-      <c r="F89" s="67" t="n"/>
-      <c r="G89" s="68" t="n"/>
     </row>
     <row r="90" ht="14" customHeight="1">
-      <c r="B90" s="35" t="n"/>
+      <c r="B90" s="35" cm="1">
+        <f t="array" ref="B90">OAR.SLS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],$E$37:$F$41,PsiL,PsiS)</f>
+        <v/>
+      </c>
       <c r="C90" s="64" t="n"/>
       <c r="D90" s="66" t="n"/>
       <c r="E90" s="64" t="n"/>
       <c r="F90" s="67" t="n"/>
       <c r="G90" s="68" t="n"/>
-    </row>
-    <row r="91" ht="14" customHeight="1"/>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>Δ1kN: 1 kN at midspan,</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="14" customHeight="1">
+      <c r="B91" s="35" t="n"/>
+      <c r="C91" s="64" t="n"/>
+      <c r="D91" s="66" t="n"/>
+      <c r="E91" s="64" t="n"/>
+      <c r="F91" s="67" t="n"/>
+      <c r="G91" s="68" t="n"/>
+      <c r="H91" s="6" t="inlineStr">
+        <is>
+          <t>beam alone</t>
+        </is>
+      </c>
+    </row>
     <row r="92" ht="14" customHeight="1">
-      <c r="B92" s="69" t="inlineStr">
+      <c r="B92" s="35" t="n"/>
+      <c r="C92" s="64" t="n"/>
+      <c r="D92" s="66" t="n"/>
+      <c r="E92" s="64" t="n"/>
+      <c r="F92" s="67" t="n"/>
+      <c r="G92" s="68" t="n"/>
+    </row>
+    <row r="93" ht="14" customHeight="1">
+      <c r="B93" s="35" t="n"/>
+      <c r="C93" s="64" t="n"/>
+      <c r="D93" s="66" t="n"/>
+      <c r="E93" s="64" t="n"/>
+      <c r="F93" s="67" t="n"/>
+      <c r="G93" s="68" t="n"/>
+    </row>
+    <row r="94" ht="14" customHeight="1">
+      <c r="B94" s="35" t="n"/>
+      <c r="C94" s="64" t="n"/>
+      <c r="D94" s="66" t="n"/>
+      <c r="E94" s="64" t="n"/>
+      <c r="F94" s="67" t="n"/>
+      <c r="G94" s="68" t="n"/>
+    </row>
+    <row r="95" ht="14" customHeight="1"/>
+    <row r="96" ht="14" customHeight="1">
+      <c r="B96" s="69" t="inlineStr">
         <is>
           <t>Deflected shapes (mm, plotted downward;  x in m)</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="14" customHeight="1"/>
-    <row r="94" ht="14" customHeight="1"/>
-    <row r="95" ht="14" customHeight="1"/>
-    <row r="96" ht="14" customHeight="1"/>
     <row r="97" ht="14" customHeight="1"/>
     <row r="98" ht="14" customHeight="1"/>
     <row r="99" ht="14" customHeight="1"/>
@@ -6968,32 +6983,32 @@
     <row r="102" ht="14" customHeight="1"/>
     <row r="103" ht="14" customHeight="1"/>
     <row r="104" ht="14" customHeight="1"/>
-    <row r="105" ht="20" customHeight="1">
-      <c r="B105" s="10" t="inlineStr">
-        <is>
-          <t>ULS Strength Checks – Bending (AS 4100 Cl. 5.6)</t>
-        </is>
-      </c>
-      <c r="C105" s="11" t="n"/>
-      <c r="D105" s="11" t="n"/>
-      <c r="E105" s="11" t="n"/>
-      <c r="F105" s="11" t="n"/>
-      <c r="G105" s="11" t="n"/>
-      <c r="H105" s="11" t="n"/>
-      <c r="I105" s="11" t="n"/>
-      <c r="J105" s="11" t="n"/>
-    </row>
-    <row r="106" ht="14" customHeight="1">
-      <c r="B106" s="69" t="inlineStr">
-        <is>
-          <t>Bending moment envelope, all active combinations (kN·m, sagging plotted down;  x in m)</t>
-        </is>
-      </c>
-    </row>
+    <row r="105" ht="14" customHeight="1"/>
+    <row r="106" ht="14" customHeight="1"/>
     <row r="107" ht="14" customHeight="1"/>
     <row r="108" ht="14" customHeight="1"/>
-    <row r="109" ht="14" customHeight="1"/>
-    <row r="110" ht="14" customHeight="1"/>
+    <row r="109" ht="20" customHeight="1">
+      <c r="B109" s="10" t="inlineStr">
+        <is>
+          <t>ULS Strength Checks – Bending (AS 4100 Cl. 5.6)</t>
+        </is>
+      </c>
+      <c r="C109" s="11" t="n"/>
+      <c r="D109" s="11" t="n"/>
+      <c r="E109" s="11" t="n"/>
+      <c r="F109" s="11" t="n"/>
+      <c r="G109" s="11" t="n"/>
+      <c r="H109" s="11" t="n"/>
+      <c r="I109" s="11" t="n"/>
+      <c r="J109" s="11" t="n"/>
+    </row>
+    <row r="110" ht="14" customHeight="1">
+      <c r="B110" s="69" t="inlineStr">
+        <is>
+          <t>Bending moment envelope, all active combinations (kN·m, sagging plotted down;  x in m)</t>
+        </is>
+      </c>
+    </row>
     <row r="111" ht="14" customHeight="1"/>
     <row r="112" ht="14" customHeight="1"/>
     <row r="113" ht="14" customHeight="1"/>
@@ -7002,102 +7017,62 @@
     <row r="116" ht="14" customHeight="1"/>
     <row r="117" ht="14" customHeight="1"/>
     <row r="118" ht="14" customHeight="1"/>
-    <row r="119" ht="16" customHeight="1">
-      <c r="B119" s="60" t="inlineStr">
+    <row r="119" ht="14" customHeight="1"/>
+    <row r="120" ht="14" customHeight="1"/>
+    <row r="121" ht="14" customHeight="1"/>
+    <row r="122" ht="14" customHeight="1"/>
+    <row r="123" ht="16" customHeight="1">
+      <c r="B123" s="60" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="C119" s="60" t="inlineStr">
+      <c r="C123" s="60" t="inlineStr">
         <is>
           <t>Segment (m)</t>
         </is>
       </c>
-      <c r="D119" s="60" t="inlineStr">
+      <c r="D123" s="60" t="inlineStr">
         <is>
           <t>Ends</t>
         </is>
       </c>
-      <c r="E119" s="60" t="inlineStr">
+      <c r="E123" s="60" t="inlineStr">
         <is>
           <t>Le (m)</t>
         </is>
       </c>
-      <c r="F119" s="60" t="inlineStr">
+      <c r="F123" s="60" t="inlineStr">
         <is>
           <t>αm</t>
         </is>
       </c>
-      <c r="G119" s="60" t="inlineStr">
+      <c r="G123" s="60" t="inlineStr">
         <is>
           <t>αs</t>
         </is>
       </c>
-      <c r="H119" s="60" t="inlineStr">
+      <c r="H123" s="60" t="inlineStr">
         <is>
           <t>φMb (kN·m)</t>
         </is>
       </c>
-      <c r="I119" s="60" t="inlineStr">
+      <c r="I123" s="60" t="inlineStr">
         <is>
           <t>M* (kN·m)</t>
         </is>
       </c>
-      <c r="J119" s="60" t="inlineStr">
+      <c r="J123" s="60" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
     </row>
-    <row r="120" ht="14" customHeight="1">
-      <c r="B120" s="35" cm="1">
-        <f t="array" ref="B120">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
-        <v/>
-      </c>
-      <c r="C120" s="35" t="n"/>
-      <c r="D120" s="35" t="n"/>
-      <c r="E120" s="64" t="n"/>
-      <c r="F120" s="70" t="n"/>
-      <c r="G120" s="70" t="n"/>
-      <c r="H120" s="71" t="n"/>
-      <c r="I120" s="71" t="n"/>
-      <c r="J120" s="68" t="n"/>
-    </row>
-    <row r="121" ht="14" customHeight="1">
-      <c r="B121" s="35" t="n"/>
-      <c r="C121" s="35" t="n"/>
-      <c r="D121" s="35" t="n"/>
-      <c r="E121" s="64" t="n"/>
-      <c r="F121" s="70" t="n"/>
-      <c r="G121" s="70" t="n"/>
-      <c r="H121" s="71" t="n"/>
-      <c r="I121" s="71" t="n"/>
-      <c r="J121" s="68" t="n"/>
-    </row>
-    <row r="122" ht="14" customHeight="1">
-      <c r="B122" s="35" t="n"/>
-      <c r="C122" s="35" t="n"/>
-      <c r="D122" s="35" t="n"/>
-      <c r="E122" s="64" t="n"/>
-      <c r="F122" s="70" t="n"/>
-      <c r="G122" s="70" t="n"/>
-      <c r="H122" s="71" t="n"/>
-      <c r="I122" s="71" t="n"/>
-      <c r="J122" s="68" t="n"/>
-    </row>
-    <row r="123" ht="14" customHeight="1">
-      <c r="B123" s="35" t="n"/>
-      <c r="C123" s="35" t="n"/>
-      <c r="D123" s="35" t="n"/>
-      <c r="E123" s="64" t="n"/>
-      <c r="F123" s="70" t="n"/>
-      <c r="G123" s="70" t="n"/>
-      <c r="H123" s="71" t="n"/>
-      <c r="I123" s="71" t="n"/>
-      <c r="J123" s="68" t="n"/>
-    </row>
     <row r="124" ht="14" customHeight="1">
-      <c r="B124" s="35" t="n"/>
+      <c r="B124" s="35" cm="1">
+        <f t="array" ref="B124">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$F$85:$G$86)</f>
+        <v/>
+      </c>
       <c r="C124" s="35" t="n"/>
       <c r="D124" s="35" t="n"/>
       <c r="E124" s="64" t="n"/>
@@ -7229,60 +7204,83 @@
       <c r="J135" s="68" t="n"/>
     </row>
     <row r="136" ht="14" customHeight="1">
-      <c r="B136" s="15" t="inlineStr">
+      <c r="B136" s="35" t="n"/>
+      <c r="C136" s="35" t="n"/>
+      <c r="D136" s="35" t="n"/>
+      <c r="E136" s="64" t="n"/>
+      <c r="F136" s="70" t="n"/>
+      <c r="G136" s="70" t="n"/>
+      <c r="H136" s="71" t="n"/>
+      <c r="I136" s="71" t="n"/>
+      <c r="J136" s="68" t="n"/>
+    </row>
+    <row r="137" ht="14" customHeight="1">
+      <c r="B137" s="35" t="n"/>
+      <c r="C137" s="35" t="n"/>
+      <c r="D137" s="35" t="n"/>
+      <c r="E137" s="64" t="n"/>
+      <c r="F137" s="70" t="n"/>
+      <c r="G137" s="70" t="n"/>
+      <c r="H137" s="71" t="n"/>
+      <c r="I137" s="71" t="n"/>
+      <c r="J137" s="68" t="n"/>
+    </row>
+    <row r="138" ht="14" customHeight="1">
+      <c r="B138" s="35" t="n"/>
+      <c r="C138" s="35" t="n"/>
+      <c r="D138" s="35" t="n"/>
+      <c r="E138" s="64" t="n"/>
+      <c r="F138" s="70" t="n"/>
+      <c r="G138" s="70" t="n"/>
+      <c r="H138" s="71" t="n"/>
+      <c r="I138" s="71" t="n"/>
+      <c r="J138" s="68" t="n"/>
+    </row>
+    <row r="139" ht="14" customHeight="1">
+      <c r="B139" s="35" t="n"/>
+      <c r="C139" s="35" t="n"/>
+      <c r="D139" s="35" t="n"/>
+      <c r="E139" s="64" t="n"/>
+      <c r="F139" s="70" t="n"/>
+      <c r="G139" s="70" t="n"/>
+      <c r="H139" s="71" t="n"/>
+      <c r="I139" s="71" t="n"/>
+      <c r="J139" s="68" t="n"/>
+    </row>
+    <row r="140">
+      <c r="B140" s="15" t="inlineStr">
         <is>
           <t>* αm overridden in the restraints table.  Full working for the governing segment follows.</t>
         </is>
       </c>
     </row>
-    <row r="137" ht="14" customHeight="1"/>
-    <row r="138" ht="20" customHeight="1">
-      <c r="B138" s="10" t="inlineStr">
+    <row r="142" ht="20" customHeight="1">
+      <c r="B142" s="10" t="inlineStr">
         <is>
           <t>Governing Segment – Working</t>
         </is>
       </c>
-      <c r="C138" s="11" t="n"/>
-      <c r="D138" s="11" t="n"/>
-      <c r="E138" s="11" t="n"/>
-      <c r="F138" s="11" t="n"/>
-      <c r="G138" s="11" t="n"/>
-      <c r="H138" s="11" t="n"/>
-      <c r="I138" s="11" t="n"/>
-      <c r="J138" s="11" t="n"/>
-    </row>
-    <row r="139" ht="14" customHeight="1">
-      <c r="B139" s="15" t="inlineStr">
+      <c r="C142" s="11" t="n"/>
+      <c r="D142" s="11" t="n"/>
+      <c r="E142" s="11" t="n"/>
+      <c r="F142" s="11" t="n"/>
+      <c r="G142" s="11" t="n"/>
+      <c r="H142" s="11" t="n"/>
+      <c r="I142" s="11" t="n"/>
+      <c r="J142" s="11" t="n"/>
+    </row>
+    <row r="143">
+      <c r="B143" s="15" t="inlineStr">
         <is>
           <t>OAR.ULSDETAIL: change the comboId / segment arguments to show any other segment.</t>
         </is>
       </c>
     </row>
-    <row r="140">
-      <c r="D140" s="72" cm="1">
-        <f t="array" ref="D140">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$I$77:$J$78)</f>
-        <v/>
-      </c>
-      <c r="E140" s="73" t="n"/>
-      <c r="F140" s="36" t="n"/>
-    </row>
-    <row r="141">
-      <c r="D141" s="72" t="n"/>
-      <c r="E141" s="73" t="n"/>
-      <c r="F141" s="36" t="n"/>
-    </row>
-    <row r="142">
-      <c r="D142" s="72" t="n"/>
-      <c r="E142" s="73" t="n"/>
-      <c r="F142" s="36" t="n"/>
-    </row>
-    <row r="143">
-      <c r="D143" s="72" t="n"/>
-      <c r="E143" s="73" t="n"/>
-      <c r="F143" s="36" t="n"/>
-    </row>
     <row r="144">
-      <c r="D144" s="72" t="n"/>
+      <c r="D144" s="72" cm="1">
+        <f t="array" ref="D144">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$F$85:$G$86)</f>
+        <v/>
+      </c>
       <c r="E144" s="73" t="n"/>
       <c r="F144" s="36" t="n"/>
     </row>
@@ -7371,90 +7369,78 @@
       <c r="E161" s="73" t="n"/>
       <c r="F161" s="36" t="n"/>
     </row>
-    <row r="163" ht="20" customHeight="1">
-      <c r="B163" s="10" t="inlineStr">
+    <row r="162">
+      <c r="D162" s="72" t="n"/>
+      <c r="E162" s="73" t="n"/>
+      <c r="F162" s="36" t="n"/>
+    </row>
+    <row r="163">
+      <c r="D163" s="72" t="n"/>
+      <c r="E163" s="73" t="n"/>
+      <c r="F163" s="36" t="n"/>
+    </row>
+    <row r="164">
+      <c r="D164" s="72" t="n"/>
+      <c r="E164" s="73" t="n"/>
+      <c r="F164" s="36" t="n"/>
+    </row>
+    <row r="165">
+      <c r="D165" s="72" t="n"/>
+      <c r="E165" s="73" t="n"/>
+      <c r="F165" s="36" t="n"/>
+    </row>
+    <row r="167" ht="20" customHeight="1">
+      <c r="B167" s="10" t="inlineStr">
         <is>
           <t>Shear (AS 4100 Cl. 5.11)</t>
         </is>
       </c>
-      <c r="C163" s="11" t="n"/>
-      <c r="D163" s="11" t="n"/>
-      <c r="E163" s="11" t="n"/>
-      <c r="F163" s="11" t="n"/>
-      <c r="G163" s="11" t="n"/>
-      <c r="H163" s="11" t="n"/>
-      <c r="I163" s="11" t="n"/>
-      <c r="J163" s="11" t="n"/>
-    </row>
-    <row r="164">
-      <c r="B164" s="60" t="inlineStr">
+      <c r="C167" s="11" t="n"/>
+      <c r="D167" s="11" t="n"/>
+      <c r="E167" s="11" t="n"/>
+      <c r="F167" s="11" t="n"/>
+      <c r="G167" s="11" t="n"/>
+      <c r="H167" s="11" t="n"/>
+      <c r="I167" s="11" t="n"/>
+      <c r="J167" s="11" t="n"/>
+    </row>
+    <row r="168">
+      <c r="B168" s="60" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="C164" s="60" t="inlineStr">
+      <c r="C168" s="60" t="inlineStr">
         <is>
           <t>V* (kN)</t>
         </is>
       </c>
-      <c r="D164" s="60" t="inlineStr">
+      <c r="D168" s="60" t="inlineStr">
         <is>
           <t>at x (m)</t>
         </is>
       </c>
-      <c r="E164" s="60" t="inlineStr">
+      <c r="E168" s="60" t="inlineStr">
         <is>
           <t>φVv (kN)</t>
         </is>
       </c>
-      <c r="F164" s="60" t="inlineStr">
+      <c r="F168" s="60" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
-      <c r="G164" s="60" t="inlineStr">
+      <c r="G168" s="60" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="165">
-      <c r="B165" s="35" cm="1">
-        <f t="array" ref="B165">OAR.SHEAR(SectionSize,Grade,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
-        <v/>
-      </c>
-      <c r="C165" s="71" t="n"/>
-      <c r="D165" s="64" t="n"/>
-      <c r="E165" s="71" t="n"/>
-      <c r="F165" s="68" t="n"/>
-      <c r="G165" s="74" t="n"/>
-    </row>
-    <row r="166">
-      <c r="B166" s="35" t="n"/>
-      <c r="C166" s="71" t="n"/>
-      <c r="D166" s="64" t="n"/>
-      <c r="E166" s="71" t="n"/>
-      <c r="F166" s="68" t="n"/>
-      <c r="G166" s="74" t="n"/>
-    </row>
-    <row r="167">
-      <c r="B167" s="35" t="n"/>
-      <c r="C167" s="71" t="n"/>
-      <c r="D167" s="64" t="n"/>
-      <c r="E167" s="71" t="n"/>
-      <c r="F167" s="68" t="n"/>
-      <c r="G167" s="74" t="n"/>
-    </row>
-    <row r="168">
-      <c r="B168" s="35" t="n"/>
-      <c r="C168" s="71" t="n"/>
-      <c r="D168" s="64" t="n"/>
-      <c r="E168" s="71" t="n"/>
-      <c r="F168" s="68" t="n"/>
-      <c r="G168" s="74" t="n"/>
-    </row>
     <row r="169">
-      <c r="B169" s="35" t="n"/>
+      <c r="B169" s="35" cm="1">
+        <f t="array" ref="B169">OAR.SHEAR(SectionSize,Grade,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
+        <v/>
+      </c>
       <c r="C169" s="71" t="n"/>
       <c r="D169" s="64" t="n"/>
       <c r="E169" s="71" t="n"/>
@@ -7485,225 +7471,237 @@
       <c r="F172" s="68" t="n"/>
       <c r="G172" s="74" t="n"/>
     </row>
-    <row r="174" ht="20" customHeight="1">
-      <c r="B174" s="10" t="inlineStr">
+    <row r="173">
+      <c r="B173" s="35" t="n"/>
+      <c r="C173" s="71" t="n"/>
+      <c r="D173" s="64" t="n"/>
+      <c r="E173" s="71" t="n"/>
+      <c r="F173" s="68" t="n"/>
+      <c r="G173" s="74" t="n"/>
+    </row>
+    <row r="174">
+      <c r="B174" s="35" t="n"/>
+      <c r="C174" s="71" t="n"/>
+      <c r="D174" s="64" t="n"/>
+      <c r="E174" s="71" t="n"/>
+      <c r="F174" s="68" t="n"/>
+      <c r="G174" s="74" t="n"/>
+    </row>
+    <row r="175">
+      <c r="B175" s="35" t="n"/>
+      <c r="C175" s="71" t="n"/>
+      <c r="D175" s="64" t="n"/>
+      <c r="E175" s="71" t="n"/>
+      <c r="F175" s="68" t="n"/>
+      <c r="G175" s="74" t="n"/>
+    </row>
+    <row r="176">
+      <c r="B176" s="35" t="n"/>
+      <c r="C176" s="71" t="n"/>
+      <c r="D176" s="64" t="n"/>
+      <c r="E176" s="71" t="n"/>
+      <c r="F176" s="68" t="n"/>
+      <c r="G176" s="74" t="n"/>
+    </row>
+    <row r="178" ht="20" customHeight="1">
+      <c r="B178" s="10" t="inlineStr">
         <is>
           <t>Support Reactions</t>
         </is>
       </c>
-      <c r="C174" s="11" t="n"/>
-      <c r="D174" s="11" t="n"/>
-      <c r="E174" s="11" t="n"/>
-      <c r="F174" s="11" t="n"/>
-      <c r="G174" s="11" t="n"/>
-      <c r="H174" s="11" t="n"/>
-      <c r="I174" s="11" t="n"/>
-      <c r="J174" s="11" t="n"/>
-    </row>
-    <row r="175">
-      <c r="B175" s="15" t="inlineStr">
+      <c r="C178" s="11" t="n"/>
+      <c r="D178" s="11" t="n"/>
+      <c r="E178" s="11" t="n"/>
+      <c r="F178" s="11" t="n"/>
+      <c r="G178" s="11" t="n"/>
+      <c r="H178" s="11" t="n"/>
+      <c r="I178" s="11" t="n"/>
+      <c r="J178" s="11" t="n"/>
+    </row>
+    <row r="179">
+      <c r="B179" s="15" t="inlineStr">
         <is>
           <t>Unfactored, per case, positive in the case direction (Wu/Wiu = uplift). Self-weight is in G.  To load another beam: add a Point row with the same case and set Direct to e.g. ='B1'!RxnR_G</t>
         </is>
       </c>
     </row>
-    <row r="176">
-      <c r="B176" s="25" t="inlineStr">
+    <row r="180">
+      <c r="B180" s="25" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="D176" s="25" t="inlineStr">
+      <c r="D180" s="25" t="inlineStr">
         <is>
           <t>Left (kN)</t>
         </is>
       </c>
-      <c r="E176" s="25" t="inlineStr">
+      <c r="E180" s="25" t="inlineStr">
         <is>
           <t>Right (kN)</t>
         </is>
       </c>
-      <c r="F176" s="25" t="inlineStr">
+      <c r="F180" s="25" t="inlineStr">
         <is>
           <t>Transfer names</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="B177" s="52" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="C177" s="53" t="n"/>
-      <c r="D177" s="37" cm="1">
-        <f t="array" ref="D177">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,2)</f>
-        <v/>
-      </c>
-      <c r="E177" s="37" cm="1">
-        <f t="array" ref="E177">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,3)</f>
-        <v/>
-      </c>
-      <c r="F177" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_G  ·  RxnR_G</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="B178" s="52" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="C178" s="53" t="n"/>
-      <c r="D178" s="37" cm="1">
-        <f t="array" ref="D178">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,2)</f>
-        <v/>
-      </c>
-      <c r="E178" s="37" cm="1">
-        <f t="array" ref="E178">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,3)</f>
-        <v/>
-      </c>
-      <c r="F178" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_Q  ·  RxnR_Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="B179" s="52" t="inlineStr">
-        <is>
-          <t>Wd</t>
-        </is>
-      </c>
-      <c r="C179" s="53" t="n"/>
-      <c r="D179" s="37" cm="1">
-        <f t="array" ref="D179">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,2)</f>
-        <v/>
-      </c>
-      <c r="E179" s="37" cm="1">
-        <f t="array" ref="E179">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,3)</f>
-        <v/>
-      </c>
-      <c r="F179" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_Wd  ·  RxnR_Wd</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="B180" s="52" t="inlineStr">
-        <is>
-          <t>Wu</t>
-        </is>
-      </c>
-      <c r="C180" s="53" t="n"/>
-      <c r="D180" s="37" cm="1">
-        <f t="array" ref="D180">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,2)</f>
-        <v/>
-      </c>
-      <c r="E180" s="37" cm="1">
-        <f t="array" ref="E180">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,3)</f>
-        <v/>
-      </c>
-      <c r="F180" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_Wu  ·  RxnR_Wu</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="B181" s="52" t="inlineStr">
         <is>
-          <t>Wid</t>
+          <t>G</t>
         </is>
       </c>
       <c r="C181" s="53" t="n"/>
       <c r="D181" s="37" cm="1">
-        <f t="array" ref="D181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,2)</f>
+        <f t="array" ref="D181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,2)</f>
         <v/>
       </c>
       <c r="E181" s="37" cm="1">
-        <f t="array" ref="E181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,3)</f>
+        <f t="array" ref="E181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,3)</f>
         <v/>
       </c>
       <c r="F181" s="21" t="inlineStr">
         <is>
-          <t>RxnL_Wid  ·  RxnR_Wid</t>
+          <t>RxnL_G  ·  RxnR_G</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="B182" s="52" t="inlineStr">
         <is>
-          <t>Wiu</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="C182" s="53" t="n"/>
       <c r="D182" s="37" cm="1">
-        <f t="array" ref="D182">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,2)</f>
+        <f t="array" ref="D182">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,2)</f>
         <v/>
       </c>
       <c r="E182" s="37" cm="1">
-        <f t="array" ref="E182">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,3)</f>
+        <f t="array" ref="E182">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,3)</f>
         <v/>
       </c>
       <c r="F182" s="21" t="inlineStr">
         <is>
+          <t>RxnL_Q  ·  RxnR_Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="B183" s="52" t="inlineStr">
+        <is>
+          <t>Wd</t>
+        </is>
+      </c>
+      <c r="C183" s="53" t="n"/>
+      <c r="D183" s="37" cm="1">
+        <f t="array" ref="D183">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,2)</f>
+        <v/>
+      </c>
+      <c r="E183" s="37" cm="1">
+        <f t="array" ref="E183">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,3)</f>
+        <v/>
+      </c>
+      <c r="F183" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_Wd  ·  RxnR_Wd</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="B184" s="52" t="inlineStr">
+        <is>
+          <t>Wu</t>
+        </is>
+      </c>
+      <c r="C184" s="53" t="n"/>
+      <c r="D184" s="37" cm="1">
+        <f t="array" ref="D184">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,2)</f>
+        <v/>
+      </c>
+      <c r="E184" s="37" cm="1">
+        <f t="array" ref="E184">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,3)</f>
+        <v/>
+      </c>
+      <c r="F184" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_Wu  ·  RxnR_Wu</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="B185" s="52" t="inlineStr">
+        <is>
+          <t>Wid</t>
+        </is>
+      </c>
+      <c r="C185" s="53" t="n"/>
+      <c r="D185" s="37" cm="1">
+        <f t="array" ref="D185">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,2)</f>
+        <v/>
+      </c>
+      <c r="E185" s="37" cm="1">
+        <f t="array" ref="E185">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,3)</f>
+        <v/>
+      </c>
+      <c r="F185" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_Wid  ·  RxnR_Wid</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="B186" s="52" t="inlineStr">
+        <is>
+          <t>Wiu</t>
+        </is>
+      </c>
+      <c r="C186" s="53" t="n"/>
+      <c r="D186" s="37" cm="1">
+        <f t="array" ref="D186">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,2)</f>
+        <v/>
+      </c>
+      <c r="E186" s="37" cm="1">
+        <f t="array" ref="E186">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,3)</f>
+        <v/>
+      </c>
+      <c r="F186" s="21" t="inlineStr">
+        <is>
           <t>RxnL_Wiu  ·  RxnR_Wiu</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="B184" s="15" t="inlineStr">
+    <row r="188">
+      <c r="B188" s="15" t="inlineStr">
         <is>
           <t>All cases and active combinations (kN, + = upward reaction; uplift cases show negative)</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="B185" s="60" t="inlineStr">
+    <row r="189">
+      <c r="B189" s="60" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C185" s="60" t="inlineStr">
+      <c r="C189" s="60" t="inlineStr">
         <is>
           <t>Left (kN)</t>
         </is>
       </c>
-      <c r="D185" s="60" t="inlineStr">
+      <c r="D189" s="60" t="inlineStr">
         <is>
           <t>Right (kN)</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="B186" s="35" cm="1">
-        <f t="array" ref="B186">OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
-        <v/>
-      </c>
-      <c r="C186" s="64" t="n"/>
-      <c r="D186" s="64" t="n"/>
-    </row>
-    <row r="187">
-      <c r="B187" s="35" t="n"/>
-      <c r="C187" s="64" t="n"/>
-      <c r="D187" s="64" t="n"/>
-    </row>
-    <row r="188">
-      <c r="B188" s="35" t="n"/>
-      <c r="C188" s="64" t="n"/>
-      <c r="D188" s="64" t="n"/>
-    </row>
-    <row r="189">
-      <c r="B189" s="35" t="n"/>
-      <c r="C189" s="64" t="n"/>
-      <c r="D189" s="64" t="n"/>
-    </row>
     <row r="190">
-      <c r="B190" s="35" t="n"/>
+      <c r="B190" s="35" cm="1">
+        <f t="array" ref="B190">OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
+        <v/>
+      </c>
       <c r="C190" s="64" t="n"/>
       <c r="D190" s="64" t="n"/>
     </row>
@@ -7752,26 +7750,45 @@
       <c r="C199" s="64" t="n"/>
       <c r="D199" s="64" t="n"/>
     </row>
+    <row r="200">
+      <c r="B200" s="35" t="n"/>
+      <c r="C200" s="64" t="n"/>
+      <c r="D200" s="64" t="n"/>
+    </row>
+    <row r="201">
+      <c r="B201" s="35" t="n"/>
+      <c r="C201" s="64" t="n"/>
+      <c r="D201" s="64" t="n"/>
+    </row>
+    <row r="202">
+      <c r="B202" s="35" t="n"/>
+      <c r="C202" s="64" t="n"/>
+      <c r="D202" s="64" t="n"/>
+    </row>
+    <row r="203">
+      <c r="B203" s="35" t="n"/>
+      <c r="C203" s="64" t="n"/>
+      <c r="D203" s="64" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="40">
     <mergeCell ref="F182:G182"/>
     <mergeCell ref="B16:C16"/>
-    <mergeCell ref="F178:G178"/>
+    <mergeCell ref="B185:C185"/>
     <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F183:G183"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B184:C184"/>
     <mergeCell ref="B180:C180"/>
-    <mergeCell ref="B176:C176"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="M8:T40"/>
-    <mergeCell ref="F177:G177"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="G2:J2"/>
-    <mergeCell ref="B179:C179"/>
+    <mergeCell ref="B181:C181"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B181:C181"/>
     <mergeCell ref="F181:G181"/>
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="I3:J3"/>
@@ -7779,16 +7796,17 @@
     <mergeCell ref="B182:C182"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="E30:F30"/>
+    <mergeCell ref="F185:G185"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B178:C178"/>
     <mergeCell ref="F180:G180"/>
+    <mergeCell ref="B186:C186"/>
+    <mergeCell ref="F184:G184"/>
     <mergeCell ref="B40:C40"/>
-    <mergeCell ref="F179:G179"/>
     <mergeCell ref="I1:J1"/>
-    <mergeCell ref="F176:G176"/>
+    <mergeCell ref="B183:C183"/>
     <mergeCell ref="I4:J4"/>
-    <mergeCell ref="B177:C177"/>
+    <mergeCell ref="F186:G186"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="B36:C36"/>
@@ -7848,44 +7866,44 @@
       <formula>NumUpliftCombos=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B86:G90">
+  <conditionalFormatting sqref="B90:G94">
     <cfRule type="expression" priority="12" dxfId="7">
-      <formula>$B86&lt;&gt;""</formula>
+      <formula>$B90&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G86:G90">
+  <conditionalFormatting sqref="G90:G94">
     <cfRule type="expression" priority="13" dxfId="0">
-      <formula>AND(ISNUMBER(G86),G86&gt;1)</formula>
+      <formula>AND(ISNUMBER(G90),G90&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B120:J135">
+  <conditionalFormatting sqref="B124:J139">
     <cfRule type="expression" priority="14" dxfId="7">
-      <formula>$B120&lt;&gt;""</formula>
+      <formula>$B124&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J120:J135">
+  <conditionalFormatting sqref="J124:J139">
     <cfRule type="expression" priority="15" dxfId="0">
-      <formula>AND(ISNUMBER(J120),J120&gt;1)</formula>
+      <formula>AND(ISNUMBER(J124),J124&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C120:C135">
+  <conditionalFormatting sqref="C124:C139">
     <cfRule type="expression" priority="16" dxfId="9">
-      <formula>RIGHT(C120,1)="*"</formula>
+      <formula>RIGHT(C124,1)="*"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B165:F172">
+  <conditionalFormatting sqref="B169:F176">
     <cfRule type="expression" priority="17" dxfId="7">
-      <formula>$B165&lt;&gt;""</formula>
+      <formula>$B169&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F165:F172">
+  <conditionalFormatting sqref="F169:F176">
     <cfRule type="expression" priority="18" dxfId="0">
-      <formula>AND(ISNUMBER(F165),F165&gt;1)</formula>
+      <formula>AND(ISNUMBER(F169),F169&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B186:D199">
+  <conditionalFormatting sqref="B190:D203">
     <cfRule type="expression" priority="19" dxfId="7">
-      <formula>$B186&lt;&gt;""</formula>
+      <formula>$B190&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="13">
@@ -7941,8 +7959,8 @@
   </headerFooter>
   <rowBreaks count="3" manualBreakCount="3">
     <brk id="42" min="0" max="16383" man="1"/>
-    <brk id="83" min="0" max="16383" man="1"/>
-    <brk id="137" min="0" max="16383" man="1"/>
+    <brk id="87" min="0" max="16383" man="1"/>
+    <brk id="141" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <tableParts count="4">

</xml_diff>

<commit_message>
v0.2.5: continuous flange restraint option (φMb = φMsx); restraints table with supports plus five blank internal rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -54,24 +54,26 @@
     <definedName name="NumUpliftCombos" localSheetId="0">'B1'!$S$56</definedName>
     <definedName name="CombSet" localSheetId="0">'B1'!$E$63</definedName>
     <definedName name="PsiC" localSheetId="0">'B1'!$G$63</definedName>
-    <definedName name="kl_Top" localSheetId="0">'B1'!$F$85</definedName>
-    <definedName name="kl_Bot" localSheetId="0">'B1'!$G$85</definedName>
-    <definedName name="kr_Top" localSheetId="0">'B1'!$F$86</definedName>
-    <definedName name="kr_Bot" localSheetId="0">'B1'!$G$86</definedName>
-    <definedName name="RxnL_G" localSheetId="0">'B1'!$D$181</definedName>
-    <definedName name="RxnR_G" localSheetId="0">'B1'!$E$181</definedName>
-    <definedName name="RxnL_Q" localSheetId="0">'B1'!$D$182</definedName>
-    <definedName name="RxnR_Q" localSheetId="0">'B1'!$E$182</definedName>
-    <definedName name="RxnL_Wd" localSheetId="0">'B1'!$D$183</definedName>
-    <definedName name="RxnR_Wd" localSheetId="0">'B1'!$E$183</definedName>
-    <definedName name="RxnL_Wu" localSheetId="0">'B1'!$D$184</definedName>
-    <definedName name="RxnR_Wu" localSheetId="0">'B1'!$E$184</definedName>
-    <definedName name="RxnL_Wid" localSheetId="0">'B1'!$D$185</definedName>
-    <definedName name="RxnR_Wid" localSheetId="0">'B1'!$E$185</definedName>
-    <definedName name="RxnL_Wiu" localSheetId="0">'B1'!$D$186</definedName>
-    <definedName name="RxnR_Wiu" localSheetId="0">'B1'!$E$186</definedName>
-    <definedName name="Out_Reactions" localSheetId="0">'B1'!$B$190</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'B1'!$A$1:$K$204</definedName>
+    <definedName name="kl_Top" localSheetId="0">'B1'!$F$87</definedName>
+    <definedName name="kl_Bot" localSheetId="0">'B1'!$G$87</definedName>
+    <definedName name="kr_Top" localSheetId="0">'B1'!$F$88</definedName>
+    <definedName name="kr_Bot" localSheetId="0">'B1'!$G$88</definedName>
+    <definedName name="Cont_Top" localSheetId="0">'B1'!$F$89</definedName>
+    <definedName name="Cont_Bot" localSheetId="0">'B1'!$G$89</definedName>
+    <definedName name="RxnL_G" localSheetId="0">'B1'!$D$184</definedName>
+    <definedName name="RxnR_G" localSheetId="0">'B1'!$E$184</definedName>
+    <definedName name="RxnL_Q" localSheetId="0">'B1'!$D$185</definedName>
+    <definedName name="RxnR_Q" localSheetId="0">'B1'!$E$185</definedName>
+    <definedName name="RxnL_Wd" localSheetId="0">'B1'!$D$186</definedName>
+    <definedName name="RxnR_Wd" localSheetId="0">'B1'!$E$186</definedName>
+    <definedName name="RxnL_Wu" localSheetId="0">'B1'!$D$187</definedName>
+    <definedName name="RxnR_Wu" localSheetId="0">'B1'!$E$187</definedName>
+    <definedName name="RxnL_Wid" localSheetId="0">'B1'!$D$188</definedName>
+    <definedName name="RxnR_Wid" localSheetId="0">'B1'!$E$188</definedName>
+    <definedName name="RxnL_Wiu" localSheetId="0">'B1'!$D$189</definedName>
+    <definedName name="RxnR_Wiu" localSheetId="0">'B1'!$E$189</definedName>
+    <definedName name="Out_Reactions" localSheetId="0">'B1'!$B$193</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'B1'!$A$1:$K$207</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1102,7 +1104,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>96</row>
+      <row>99</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6336000" cy="1944000"/>
@@ -1124,7 +1126,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>110</row>
+      <row>113</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6336000" cy="1944000"/>
@@ -1226,8 +1228,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Restraints_B1" displayName="Restraints_B1" ref="B76:H81" headerRowCount="1">
-  <autoFilter ref="B76:H81"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Restraints_B1" displayName="Restraints_B1" ref="B76:H83" headerRowCount="1">
+  <autoFilter ref="B76:H83"/>
   <tableColumns count="7">
     <tableColumn id="2" name="x (mm)"/>
     <tableColumn id="3" name="Ref"/>
@@ -1531,7 +1533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:BB203"/>
+  <dimension ref="B1:BB206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="1.5" customWidth="1" min="1" max="1"/>
@@ -1781,7 +1783,7 @@
       <c r="S8" s="17" t="n"/>
       <c r="T8" s="18" t="n"/>
       <c r="Z8" s="19" cm="1">
-        <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$F$85:$G$86)</f>
+        <f t="array" ref="Z8">OAR.GOVERNING(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$F$87:$G$89)</f>
         <v/>
       </c>
       <c r="AL8" s="19" cm="1">
@@ -2182,7 +2184,7 @@
         </is>
       </c>
       <c r="E15" s="37" cm="1">
-        <f t="array" ref="E15">INDEX(_xlfn.ANCHORARRAY(B90),1,2)</f>
+        <f t="array" ref="E15">INDEX(_xlfn.ANCHORARRAY(B93),1,2)</f>
         <v/>
       </c>
       <c r="F15" s="37">
@@ -2282,7 +2284,7 @@
         </is>
       </c>
       <c r="E16" s="37" cm="1">
-        <f t="array" ref="E16">INDEX(_xlfn.ANCHORARRAY(B90),2,2)</f>
+        <f t="array" ref="E16">INDEX(_xlfn.ANCHORARRAY(B93),2,2)</f>
         <v/>
       </c>
       <c r="F16" s="37">
@@ -2382,7 +2384,7 @@
         </is>
       </c>
       <c r="E17" s="37" cm="1">
-        <f t="array" ref="E17">INDEX(_xlfn.ANCHORARRAY(B90),3,2)</f>
+        <f t="array" ref="E17">INDEX(_xlfn.ANCHORARRAY(B93),3,2)</f>
         <v/>
       </c>
       <c r="F17" s="37">
@@ -2482,7 +2484,7 @@
         </is>
       </c>
       <c r="E18" s="37" cm="1">
-        <f t="array" ref="E18">INDEX(_xlfn.ANCHORARRAY(B90),4,2)</f>
+        <f t="array" ref="E18">INDEX(_xlfn.ANCHORARRAY(B93),4,2)</f>
         <v/>
       </c>
       <c r="F18" s="37">
@@ -2582,7 +2584,7 @@
         </is>
       </c>
       <c r="E19" s="37" cm="1">
-        <f t="array" ref="E19">INDEX(_xlfn.ANCHORARRAY(B90),5,2)</f>
+        <f t="array" ref="E19">INDEX(_xlfn.ANCHORARRAY(B93),5,2)</f>
         <v/>
       </c>
       <c r="F19" s="37">
@@ -6666,25 +6668,11 @@
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
-      <c r="B78" s="48" t="n">
-        <v>2767</v>
-      </c>
-      <c r="C78" s="2" t="inlineStr"/>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>Purlin + fly brace</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
+      <c r="B78" s="48" t="n"/>
+      <c r="C78" s="2" t="n"/>
+      <c r="D78" s="5" t="n"/>
+      <c r="E78" s="2" t="n"/>
+      <c r="F78" s="2" t="n"/>
       <c r="G78" s="30" t="n"/>
       <c r="H78" s="30" t="n"/>
       <c r="AN78" s="20" t="inlineStr">
@@ -6694,25 +6682,11 @@
       </c>
     </row>
     <row r="79" ht="14" customHeight="1">
-      <c r="B79" s="48" t="n">
-        <v>5533</v>
-      </c>
-      <c r="C79" s="2" t="inlineStr"/>
-      <c r="D79" s="5" t="inlineStr">
-        <is>
-          <t>Purlin + fly brace</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
+      <c r="B79" s="48" t="n"/>
+      <c r="C79" s="2" t="n"/>
+      <c r="D79" s="5" t="n"/>
+      <c r="E79" s="2" t="n"/>
+      <c r="F79" s="2" t="n"/>
       <c r="G79" s="30" t="n"/>
       <c r="H79" s="30" t="n"/>
       <c r="AN79" s="20" t="inlineStr">
@@ -6722,30 +6696,11 @@
       </c>
     </row>
     <row r="80" ht="14" customHeight="1">
-      <c r="B80" s="65">
-        <f>Span</f>
-        <v/>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t>Right support – cleat</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
+      <c r="B80" s="48" t="n"/>
+      <c r="C80" s="2" t="n"/>
+      <c r="D80" s="5" t="n"/>
+      <c r="E80" s="2" t="n"/>
+      <c r="F80" s="2" t="n"/>
       <c r="G80" s="30" t="n"/>
       <c r="H80" s="30" t="n"/>
       <c r="AN80" s="20" t="inlineStr">
@@ -6769,195 +6724,224 @@
       </c>
     </row>
     <row r="82" ht="14" customHeight="1">
-      <c r="B82" s="15" t="inlineStr">
+      <c r="B82" s="48" t="n"/>
+      <c r="C82" s="2" t="n"/>
+      <c r="D82" s="5" t="n"/>
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="2" t="n"/>
+      <c r="G82" s="30" t="n"/>
+      <c r="H82" s="30" t="n"/>
+      <c r="AN82" s="20" t="inlineStr">
+        <is>
+          <t>200UC59.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="14" customHeight="1">
+      <c r="B83" s="65">
+        <f>Span</f>
+        <v/>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>Right support – cleat</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="G83" s="30" t="n"/>
+      <c r="H83" s="30" t="n"/>
+      <c r="AN83" s="20" t="inlineStr">
+        <is>
+          <t>200UC52</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="14" customHeight="1">
+      <c r="B84" s="15" t="inlineStr">
         <is>
           <t>αm top / αm bot. → override αm for that flange's segment from this row to the next restraint on that flange (blank = Cl. 5.6.1.1(a)(iii)). Flagged * in the output.</t>
         </is>
       </c>
-      <c r="AN82" s="20" t="inlineStr">
-        <is>
-          <t>200UC59.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="14" customHeight="1">
-      <c r="AN83" s="20" t="inlineStr">
-        <is>
-          <t>200UC52</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="14" customHeight="1">
-      <c r="E84" s="25" t="inlineStr">
+      <c r="AN84" s="20" t="inlineStr">
+        <is>
+          <t>200UC46</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="14" customHeight="1">
+      <c r="AN85" s="20" t="inlineStr">
+        <is>
+          <t>150UC37</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="14" customHeight="1">
+      <c r="E86" s="25" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="F84" s="25" t="inlineStr">
+      <c r="F86" s="25" t="inlineStr">
         <is>
           <t>Top</t>
         </is>
       </c>
-      <c r="G84" s="25" t="inlineStr">
+      <c r="G86" s="25" t="inlineStr">
         <is>
           <t>Bottom</t>
         </is>
       </c>
-      <c r="AN84" s="20" t="inlineStr">
-        <is>
-          <t>200UC46</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="14" customHeight="1">
-      <c r="E85" s="35" t="inlineStr">
+      <c r="AN86" s="20" t="inlineStr">
+        <is>
+          <t>150UC30</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="14" customHeight="1">
+      <c r="E87" s="35" t="inlineStr">
         <is>
           <t>kl</t>
         </is>
       </c>
-      <c r="F85" s="30" t="n">
+      <c r="F87" s="30" t="n">
         <v>1.4</v>
       </c>
-      <c r="G85" s="30" t="n">
+      <c r="G87" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="H85" s="15" t="inlineStr">
+      <c r="H87" s="15" t="inlineStr">
         <is>
           <t>kl: load height, Table 5.6.3(2)</t>
         </is>
       </c>
-      <c r="AN85" s="20" t="inlineStr">
-        <is>
-          <t>150UC37</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="14" customHeight="1">
-      <c r="E86" s="35" t="inlineStr">
+      <c r="AN87" s="20" t="inlineStr">
+        <is>
+          <t>150UC23</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="14" customHeight="1">
+      <c r="E88" s="35" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="F86" s="30" t="n">
+      <c r="F88" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="G86" s="30" t="n">
+      <c r="G88" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="H86" s="15" t="inlineStr">
+      <c r="H88" s="15" t="inlineStr">
         <is>
           <t>kr: rotation, Table 5.6.3(3); kt from restraints</t>
         </is>
       </c>
-      <c r="AN86" s="20" t="inlineStr">
-        <is>
-          <t>150UC30</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="14" customHeight="1">
-      <c r="AN87" s="20" t="inlineStr">
-        <is>
-          <t>150UC23</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="20" customHeight="1">
-      <c r="B88" s="10" t="inlineStr">
+      <c r="AN88" s="20" t="inlineStr">
+        <is>
+          <t>100UC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="14" customHeight="1">
+      <c r="E89" s="35" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H89" s="15" t="inlineStr">
+        <is>
+          <t>Yes = flange continuously restrained: φMb = φMsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="14" customHeight="1"/>
+    <row r="91" ht="20" customHeight="1">
+      <c r="B91" s="10" t="inlineStr">
         <is>
           <t>Serviceability Checks</t>
         </is>
       </c>
-      <c r="C88" s="11" t="n"/>
-      <c r="D88" s="11" t="n"/>
-      <c r="E88" s="11" t="n"/>
-      <c r="F88" s="11" t="n"/>
-      <c r="G88" s="11" t="n"/>
-      <c r="H88" s="11" t="n"/>
-      <c r="I88" s="11" t="n"/>
-      <c r="J88" s="11" t="n"/>
-      <c r="AN88" s="20" t="inlineStr">
-        <is>
-          <t>100UC15</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="14" customHeight="1">
-      <c r="B89" s="60" t="inlineStr">
+      <c r="C91" s="11" t="n"/>
+      <c r="D91" s="11" t="n"/>
+      <c r="E91" s="11" t="n"/>
+      <c r="F91" s="11" t="n"/>
+      <c r="G91" s="11" t="n"/>
+      <c r="H91" s="11" t="n"/>
+      <c r="I91" s="11" t="n"/>
+      <c r="J91" s="11" t="n"/>
+    </row>
+    <row r="92" ht="14" customHeight="1">
+      <c r="B92" s="60" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C89" s="60" t="inlineStr">
+      <c r="C92" s="60" t="inlineStr">
         <is>
           <t>Δ max (mm)</t>
         </is>
       </c>
-      <c r="D89" s="60" t="inlineStr">
+      <c r="D92" s="60" t="inlineStr">
         <is>
           <t>at x (mm)</t>
         </is>
       </c>
-      <c r="E89" s="60" t="inlineStr">
+      <c r="E92" s="60" t="inlineStr">
         <is>
           <t>Limit (mm)</t>
         </is>
       </c>
-      <c r="F89" s="60" t="inlineStr">
+      <c r="F92" s="60" t="inlineStr">
         <is>
           <t>L / Δ</t>
         </is>
       </c>
-      <c r="G89" s="60" t="inlineStr">
+      <c r="G92" s="60" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="14" customHeight="1">
-      <c r="B90" s="35" cm="1">
-        <f t="array" ref="B90">OAR.SLS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],$E$37:$F$41,PsiL,PsiS)</f>
-        <v/>
-      </c>
-      <c r="C90" s="64" t="n"/>
-      <c r="D90" s="66" t="n"/>
-      <c r="E90" s="64" t="n"/>
-      <c r="F90" s="67" t="n"/>
-      <c r="G90" s="68" t="n"/>
-      <c r="H90" s="6" t="inlineStr">
-        <is>
-          <t>Δ1kN: 1 kN at midspan,</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="14" customHeight="1">
-      <c r="B91" s="35" t="n"/>
-      <c r="C91" s="64" t="n"/>
-      <c r="D91" s="66" t="n"/>
-      <c r="E91" s="64" t="n"/>
-      <c r="F91" s="67" t="n"/>
-      <c r="G91" s="68" t="n"/>
-      <c r="H91" s="6" t="inlineStr">
-        <is>
-          <t>beam alone</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="14" customHeight="1">
-      <c r="B92" s="35" t="n"/>
-      <c r="C92" s="64" t="n"/>
-      <c r="D92" s="66" t="n"/>
-      <c r="E92" s="64" t="n"/>
-      <c r="F92" s="67" t="n"/>
-      <c r="G92" s="68" t="n"/>
-    </row>
     <row r="93" ht="14" customHeight="1">
-      <c r="B93" s="35" t="n"/>
+      <c r="B93" s="35" cm="1">
+        <f t="array" ref="B93">OAR.SLS(SectionSize,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],$E$37:$F$41,PsiL,PsiS)</f>
+        <v/>
+      </c>
       <c r="C93" s="64" t="n"/>
       <c r="D93" s="66" t="n"/>
       <c r="E93" s="64" t="n"/>
       <c r="F93" s="67" t="n"/>
       <c r="G93" s="68" t="n"/>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>Δ1kN: 1 kN at midspan,</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="14" customHeight="1">
       <c r="B94" s="35" t="n"/>
@@ -6966,18 +6950,44 @@
       <c r="E94" s="64" t="n"/>
       <c r="F94" s="67" t="n"/>
       <c r="G94" s="68" t="n"/>
-    </row>
-    <row r="95" ht="14" customHeight="1"/>
+      <c r="H94" s="6" t="inlineStr">
+        <is>
+          <t>beam alone</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="14" customHeight="1">
+      <c r="B95" s="35" t="n"/>
+      <c r="C95" s="64" t="n"/>
+      <c r="D95" s="66" t="n"/>
+      <c r="E95" s="64" t="n"/>
+      <c r="F95" s="67" t="n"/>
+      <c r="G95" s="68" t="n"/>
+    </row>
     <row r="96" ht="14" customHeight="1">
-      <c r="B96" s="69" t="inlineStr">
+      <c r="B96" s="35" t="n"/>
+      <c r="C96" s="64" t="n"/>
+      <c r="D96" s="66" t="n"/>
+      <c r="E96" s="64" t="n"/>
+      <c r="F96" s="67" t="n"/>
+      <c r="G96" s="68" t="n"/>
+    </row>
+    <row r="97" ht="14" customHeight="1">
+      <c r="B97" s="35" t="n"/>
+      <c r="C97" s="64" t="n"/>
+      <c r="D97" s="66" t="n"/>
+      <c r="E97" s="64" t="n"/>
+      <c r="F97" s="67" t="n"/>
+      <c r="G97" s="68" t="n"/>
+    </row>
+    <row r="98" ht="14" customHeight="1"/>
+    <row r="99" ht="14" customHeight="1">
+      <c r="B99" s="69" t="inlineStr">
         <is>
           <t>Deflected shapes (mm, plotted downward;  x in m)</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="14" customHeight="1"/>
-    <row r="98" ht="14" customHeight="1"/>
-    <row r="99" ht="14" customHeight="1"/>
     <row r="100" ht="14" customHeight="1"/>
     <row r="101" ht="14" customHeight="1"/>
     <row r="102" ht="14" customHeight="1"/>
@@ -6987,31 +6997,31 @@
     <row r="106" ht="14" customHeight="1"/>
     <row r="107" ht="14" customHeight="1"/>
     <row r="108" ht="14" customHeight="1"/>
-    <row r="109" ht="20" customHeight="1">
-      <c r="B109" s="10" t="inlineStr">
+    <row r="109" ht="14" customHeight="1"/>
+    <row r="110" ht="14" customHeight="1"/>
+    <row r="111" ht="14" customHeight="1"/>
+    <row r="112" ht="20" customHeight="1">
+      <c r="B112" s="10" t="inlineStr">
         <is>
           <t>ULS Strength Checks – Bending (AS 4100 Cl. 5.6)</t>
         </is>
       </c>
-      <c r="C109" s="11" t="n"/>
-      <c r="D109" s="11" t="n"/>
-      <c r="E109" s="11" t="n"/>
-      <c r="F109" s="11" t="n"/>
-      <c r="G109" s="11" t="n"/>
-      <c r="H109" s="11" t="n"/>
-      <c r="I109" s="11" t="n"/>
-      <c r="J109" s="11" t="n"/>
-    </row>
-    <row r="110" ht="14" customHeight="1">
-      <c r="B110" s="69" t="inlineStr">
+      <c r="C112" s="11" t="n"/>
+      <c r="D112" s="11" t="n"/>
+      <c r="E112" s="11" t="n"/>
+      <c r="F112" s="11" t="n"/>
+      <c r="G112" s="11" t="n"/>
+      <c r="H112" s="11" t="n"/>
+      <c r="I112" s="11" t="n"/>
+      <c r="J112" s="11" t="n"/>
+    </row>
+    <row r="113" ht="14" customHeight="1">
+      <c r="B113" s="69" t="inlineStr">
         <is>
           <t>Bending moment envelope, all active combinations (kN·m, sagging plotted down;  x in m)</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="14" customHeight="1"/>
-    <row r="112" ht="14" customHeight="1"/>
-    <row r="113" ht="14" customHeight="1"/>
     <row r="114" ht="14" customHeight="1"/>
     <row r="115" ht="14" customHeight="1"/>
     <row r="116" ht="14" customHeight="1"/>
@@ -7021,91 +7031,61 @@
     <row r="120" ht="14" customHeight="1"/>
     <row r="121" ht="14" customHeight="1"/>
     <row r="122" ht="14" customHeight="1"/>
-    <row r="123" ht="16" customHeight="1">
-      <c r="B123" s="60" t="inlineStr">
+    <row r="123" ht="14" customHeight="1"/>
+    <row r="124" ht="14" customHeight="1"/>
+    <row r="125" ht="14" customHeight="1"/>
+    <row r="126" ht="16" customHeight="1">
+      <c r="B126" s="60" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="C123" s="60" t="inlineStr">
+      <c r="C126" s="60" t="inlineStr">
         <is>
           <t>Segment (m)</t>
         </is>
       </c>
-      <c r="D123" s="60" t="inlineStr">
+      <c r="D126" s="60" t="inlineStr">
         <is>
           <t>Ends</t>
         </is>
       </c>
-      <c r="E123" s="60" t="inlineStr">
+      <c r="E126" s="60" t="inlineStr">
         <is>
           <t>Le (m)</t>
         </is>
       </c>
-      <c r="F123" s="60" t="inlineStr">
+      <c r="F126" s="60" t="inlineStr">
         <is>
           <t>αm</t>
         </is>
       </c>
-      <c r="G123" s="60" t="inlineStr">
+      <c r="G126" s="60" t="inlineStr">
         <is>
           <t>αs</t>
         </is>
       </c>
-      <c r="H123" s="60" t="inlineStr">
+      <c r="H126" s="60" t="inlineStr">
         <is>
           <t>φMb (kN·m)</t>
         </is>
       </c>
-      <c r="I123" s="60" t="inlineStr">
+      <c r="I126" s="60" t="inlineStr">
         <is>
           <t>M* (kN·m)</t>
         </is>
       </c>
-      <c r="J123" s="60" t="inlineStr">
+      <c r="J126" s="60" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="14" customHeight="1">
-      <c r="B124" s="35" cm="1">
-        <f t="array" ref="B124">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$F$85:$G$86)</f>
-        <v/>
-      </c>
-      <c r="C124" s="35" t="n"/>
-      <c r="D124" s="35" t="n"/>
-      <c r="E124" s="64" t="n"/>
-      <c r="F124" s="70" t="n"/>
-      <c r="G124" s="70" t="n"/>
-      <c r="H124" s="71" t="n"/>
-      <c r="I124" s="71" t="n"/>
-      <c r="J124" s="68" t="n"/>
-    </row>
-    <row r="125" ht="14" customHeight="1">
-      <c r="B125" s="35" t="n"/>
-      <c r="C125" s="35" t="n"/>
-      <c r="D125" s="35" t="n"/>
-      <c r="E125" s="64" t="n"/>
-      <c r="F125" s="70" t="n"/>
-      <c r="G125" s="70" t="n"/>
-      <c r="H125" s="71" t="n"/>
-      <c r="I125" s="71" t="n"/>
-      <c r="J125" s="68" t="n"/>
-    </row>
-    <row r="126" ht="14" customHeight="1">
-      <c r="B126" s="35" t="n"/>
-      <c r="C126" s="35" t="n"/>
-      <c r="D126" s="35" t="n"/>
-      <c r="E126" s="64" t="n"/>
-      <c r="F126" s="70" t="n"/>
-      <c r="G126" s="70" t="n"/>
-      <c r="H126" s="71" t="n"/>
-      <c r="I126" s="71" t="n"/>
-      <c r="J126" s="68" t="n"/>
-    </row>
     <row r="127" ht="14" customHeight="1">
-      <c r="B127" s="35" t="n"/>
+      <c r="B127" s="35" cm="1">
+        <f t="array" ref="B127">OAR.ULS(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$F$87:$G$89)</f>
+        <v/>
+      </c>
       <c r="C127" s="35" t="n"/>
       <c r="D127" s="35" t="n"/>
       <c r="E127" s="64" t="n"/>
@@ -7248,54 +7228,72 @@
       <c r="J139" s="68" t="n"/>
     </row>
     <row r="140">
-      <c r="B140" s="15" t="inlineStr">
-        <is>
-          <t>* αm overridden in the restraints table.  Full working for the governing segment follows.</t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="20" customHeight="1">
-      <c r="B142" s="10" t="inlineStr">
-        <is>
-          <t>Governing Segment – Working</t>
-        </is>
-      </c>
-      <c r="C142" s="11" t="n"/>
-      <c r="D142" s="11" t="n"/>
-      <c r="E142" s="11" t="n"/>
-      <c r="F142" s="11" t="n"/>
-      <c r="G142" s="11" t="n"/>
-      <c r="H142" s="11" t="n"/>
-      <c r="I142" s="11" t="n"/>
-      <c r="J142" s="11" t="n"/>
+      <c r="B140" s="35" t="n"/>
+      <c r="C140" s="35" t="n"/>
+      <c r="D140" s="35" t="n"/>
+      <c r="E140" s="64" t="n"/>
+      <c r="F140" s="70" t="n"/>
+      <c r="G140" s="70" t="n"/>
+      <c r="H140" s="71" t="n"/>
+      <c r="I140" s="71" t="n"/>
+      <c r="J140" s="68" t="n"/>
+    </row>
+    <row r="141">
+      <c r="B141" s="35" t="n"/>
+      <c r="C141" s="35" t="n"/>
+      <c r="D141" s="35" t="n"/>
+      <c r="E141" s="64" t="n"/>
+      <c r="F141" s="70" t="n"/>
+      <c r="G141" s="70" t="n"/>
+      <c r="H141" s="71" t="n"/>
+      <c r="I141" s="71" t="n"/>
+      <c r="J141" s="68" t="n"/>
+    </row>
+    <row r="142">
+      <c r="B142" s="35" t="n"/>
+      <c r="C142" s="35" t="n"/>
+      <c r="D142" s="35" t="n"/>
+      <c r="E142" s="64" t="n"/>
+      <c r="F142" s="70" t="n"/>
+      <c r="G142" s="70" t="n"/>
+      <c r="H142" s="71" t="n"/>
+      <c r="I142" s="71" t="n"/>
+      <c r="J142" s="68" t="n"/>
     </row>
     <row r="143">
       <c r="B143" s="15" t="inlineStr">
         <is>
+          <t>* αm overridden in the restraints table.  Full working for the governing segment follows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="20" customHeight="1">
+      <c r="B145" s="10" t="inlineStr">
+        <is>
+          <t>Governing Segment – Working</t>
+        </is>
+      </c>
+      <c r="C145" s="11" t="n"/>
+      <c r="D145" s="11" t="n"/>
+      <c r="E145" s="11" t="n"/>
+      <c r="F145" s="11" t="n"/>
+      <c r="G145" s="11" t="n"/>
+      <c r="H145" s="11" t="n"/>
+      <c r="I145" s="11" t="n"/>
+      <c r="J145" s="11" t="n"/>
+    </row>
+    <row r="146">
+      <c r="B146" s="15" t="inlineStr">
+        <is>
           <t>OAR.ULSDETAIL: change the comboId / segment arguments to show any other segment.</t>
         </is>
       </c>
     </row>
-    <row r="144">
-      <c r="D144" s="72" cm="1">
-        <f t="array" ref="D144">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$F$85:$G$86)</f>
-        <v/>
-      </c>
-      <c r="E144" s="73" t="n"/>
-      <c r="F144" s="36" t="n"/>
-    </row>
-    <row r="145">
-      <c r="D145" s="72" t="n"/>
-      <c r="E145" s="73" t="n"/>
-      <c r="F145" s="36" t="n"/>
-    </row>
-    <row r="146">
-      <c r="D146" s="72" t="n"/>
-      <c r="E146" s="73" t="n"/>
-      <c r="F146" s="36" t="n"/>
-    </row>
     <row r="147">
-      <c r="D147" s="72" t="n"/>
+      <c r="D147" s="72" cm="1">
+        <f t="array" ref="D147">OAR.ULSDETAIL(SectionSize,Grade,Span,E_mod,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66),Restraints_B1[#Data],$F$87:$G$89)</f>
+        <v/>
+      </c>
       <c r="E147" s="73" t="n"/>
       <c r="F147" s="36" t="n"/>
     </row>
@@ -7389,82 +7387,73 @@
       <c r="E165" s="73" t="n"/>
       <c r="F165" s="36" t="n"/>
     </row>
-    <row r="167" ht="20" customHeight="1">
-      <c r="B167" s="10" t="inlineStr">
+    <row r="166">
+      <c r="D166" s="72" t="n"/>
+      <c r="E166" s="73" t="n"/>
+      <c r="F166" s="36" t="n"/>
+    </row>
+    <row r="167">
+      <c r="D167" s="72" t="n"/>
+      <c r="E167" s="73" t="n"/>
+      <c r="F167" s="36" t="n"/>
+    </row>
+    <row r="168">
+      <c r="D168" s="72" t="n"/>
+      <c r="E168" s="73" t="n"/>
+      <c r="F168" s="36" t="n"/>
+    </row>
+    <row r="170" ht="20" customHeight="1">
+      <c r="B170" s="10" t="inlineStr">
         <is>
           <t>Shear (AS 4100 Cl. 5.11)</t>
         </is>
       </c>
-      <c r="C167" s="11" t="n"/>
-      <c r="D167" s="11" t="n"/>
-      <c r="E167" s="11" t="n"/>
-      <c r="F167" s="11" t="n"/>
-      <c r="G167" s="11" t="n"/>
-      <c r="H167" s="11" t="n"/>
-      <c r="I167" s="11" t="n"/>
-      <c r="J167" s="11" t="n"/>
-    </row>
-    <row r="168">
-      <c r="B168" s="60" t="inlineStr">
+      <c r="C170" s="11" t="n"/>
+      <c r="D170" s="11" t="n"/>
+      <c r="E170" s="11" t="n"/>
+      <c r="F170" s="11" t="n"/>
+      <c r="G170" s="11" t="n"/>
+      <c r="H170" s="11" t="n"/>
+      <c r="I170" s="11" t="n"/>
+      <c r="J170" s="11" t="n"/>
+    </row>
+    <row r="171">
+      <c r="B171" s="60" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="C168" s="60" t="inlineStr">
+      <c r="C171" s="60" t="inlineStr">
         <is>
           <t>V* (kN)</t>
         </is>
       </c>
-      <c r="D168" s="60" t="inlineStr">
+      <c r="D171" s="60" t="inlineStr">
         <is>
           <t>at x (m)</t>
         </is>
       </c>
-      <c r="E168" s="60" t="inlineStr">
+      <c r="E171" s="60" t="inlineStr">
         <is>
           <t>φVv (kN)</t>
         </is>
       </c>
-      <c r="F168" s="60" t="inlineStr">
+      <c r="F171" s="60" t="inlineStr">
         <is>
           <t>Utilisation</t>
         </is>
       </c>
-      <c r="G168" s="60" t="inlineStr">
+      <c r="G171" s="60" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="169">
-      <c r="B169" s="35" cm="1">
-        <f t="array" ref="B169">OAR.SHEAR(SectionSize,Grade,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
-        <v/>
-      </c>
-      <c r="C169" s="71" t="n"/>
-      <c r="D169" s="64" t="n"/>
-      <c r="E169" s="71" t="n"/>
-      <c r="F169" s="68" t="n"/>
-      <c r="G169" s="74" t="n"/>
-    </row>
-    <row r="170">
-      <c r="B170" s="35" t="n"/>
-      <c r="C170" s="71" t="n"/>
-      <c r="D170" s="64" t="n"/>
-      <c r="E170" s="71" t="n"/>
-      <c r="F170" s="68" t="n"/>
-      <c r="G170" s="74" t="n"/>
-    </row>
-    <row r="171">
-      <c r="B171" s="35" t="n"/>
-      <c r="C171" s="71" t="n"/>
-      <c r="D171" s="64" t="n"/>
-      <c r="E171" s="71" t="n"/>
-      <c r="F171" s="68" t="n"/>
-      <c r="G171" s="74" t="n"/>
-    </row>
     <row r="172">
-      <c r="B172" s="35" t="n"/>
+      <c r="B172" s="35" cm="1">
+        <f t="array" ref="B172">OAR.SHEAR(SectionSize,Grade,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
+        <v/>
+      </c>
       <c r="C172" s="71" t="n"/>
       <c r="D172" s="64" t="n"/>
       <c r="E172" s="71" t="n"/>
@@ -7503,220 +7492,229 @@
       <c r="F176" s="68" t="n"/>
       <c r="G176" s="74" t="n"/>
     </row>
-    <row r="178" ht="20" customHeight="1">
-      <c r="B178" s="10" t="inlineStr">
+    <row r="177">
+      <c r="B177" s="35" t="n"/>
+      <c r="C177" s="71" t="n"/>
+      <c r="D177" s="64" t="n"/>
+      <c r="E177" s="71" t="n"/>
+      <c r="F177" s="68" t="n"/>
+      <c r="G177" s="74" t="n"/>
+    </row>
+    <row r="178">
+      <c r="B178" s="35" t="n"/>
+      <c r="C178" s="71" t="n"/>
+      <c r="D178" s="64" t="n"/>
+      <c r="E178" s="71" t="n"/>
+      <c r="F178" s="68" t="n"/>
+      <c r="G178" s="74" t="n"/>
+    </row>
+    <row r="179">
+      <c r="B179" s="35" t="n"/>
+      <c r="C179" s="71" t="n"/>
+      <c r="D179" s="64" t="n"/>
+      <c r="E179" s="71" t="n"/>
+      <c r="F179" s="68" t="n"/>
+      <c r="G179" s="74" t="n"/>
+    </row>
+    <row r="181" ht="20" customHeight="1">
+      <c r="B181" s="10" t="inlineStr">
         <is>
           <t>Support Reactions</t>
         </is>
       </c>
-      <c r="C178" s="11" t="n"/>
-      <c r="D178" s="11" t="n"/>
-      <c r="E178" s="11" t="n"/>
-      <c r="F178" s="11" t="n"/>
-      <c r="G178" s="11" t="n"/>
-      <c r="H178" s="11" t="n"/>
-      <c r="I178" s="11" t="n"/>
-      <c r="J178" s="11" t="n"/>
-    </row>
-    <row r="179">
-      <c r="B179" s="15" t="inlineStr">
+      <c r="C181" s="11" t="n"/>
+      <c r="D181" s="11" t="n"/>
+      <c r="E181" s="11" t="n"/>
+      <c r="F181" s="11" t="n"/>
+      <c r="G181" s="11" t="n"/>
+      <c r="H181" s="11" t="n"/>
+      <c r="I181" s="11" t="n"/>
+      <c r="J181" s="11" t="n"/>
+    </row>
+    <row r="182">
+      <c r="B182" s="15" t="inlineStr">
         <is>
           <t>Unfactored, per case, positive in the case direction (Wu/Wiu = uplift). Self-weight is in G.  To load another beam: add a Point row with the same case and set Direct to e.g. ='B1'!RxnR_G</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="B180" s="25" t="inlineStr">
+    <row r="183">
+      <c r="B183" s="25" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="D180" s="25" t="inlineStr">
+      <c r="D183" s="25" t="inlineStr">
         <is>
           <t>Left (kN)</t>
         </is>
       </c>
-      <c r="E180" s="25" t="inlineStr">
+      <c r="E183" s="25" t="inlineStr">
         <is>
           <t>Right (kN)</t>
         </is>
       </c>
-      <c r="F180" s="25" t="inlineStr">
+      <c r="F183" s="25" t="inlineStr">
         <is>
           <t>Transfer names</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="B181" s="52" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="C181" s="53" t="n"/>
-      <c r="D181" s="37" cm="1">
-        <f t="array" ref="D181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,2)</f>
-        <v/>
-      </c>
-      <c r="E181" s="37" cm="1">
-        <f t="array" ref="E181">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,3)</f>
-        <v/>
-      </c>
-      <c r="F181" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_G  ·  RxnR_G</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="B182" s="52" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="C182" s="53" t="n"/>
-      <c r="D182" s="37" cm="1">
-        <f t="array" ref="D182">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,2)</f>
-        <v/>
-      </c>
-      <c r="E182" s="37" cm="1">
-        <f t="array" ref="E182">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,3)</f>
-        <v/>
-      </c>
-      <c r="F182" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_Q  ·  RxnR_Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="B183" s="52" t="inlineStr">
-        <is>
-          <t>Wd</t>
-        </is>
-      </c>
-      <c r="C183" s="53" t="n"/>
-      <c r="D183" s="37" cm="1">
-        <f t="array" ref="D183">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,2)</f>
-        <v/>
-      </c>
-      <c r="E183" s="37" cm="1">
-        <f t="array" ref="E183">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,3)</f>
-        <v/>
-      </c>
-      <c r="F183" s="21" t="inlineStr">
-        <is>
-          <t>RxnL_Wd  ·  RxnR_Wd</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="B184" s="52" t="inlineStr">
         <is>
-          <t>Wu</t>
+          <t>G</t>
         </is>
       </c>
       <c r="C184" s="53" t="n"/>
       <c r="D184" s="37" cm="1">
-        <f t="array" ref="D184">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,2)</f>
+        <f t="array" ref="D184">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,2)</f>
         <v/>
       </c>
       <c r="E184" s="37" cm="1">
-        <f t="array" ref="E184">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,3)</f>
+        <f t="array" ref="E184">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),1,3)</f>
         <v/>
       </c>
       <c r="F184" s="21" t="inlineStr">
         <is>
-          <t>RxnL_Wu  ·  RxnR_Wu</t>
+          <t>RxnL_G  ·  RxnR_G</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="B185" s="52" t="inlineStr">
         <is>
-          <t>Wid</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="C185" s="53" t="n"/>
       <c r="D185" s="37" cm="1">
-        <f t="array" ref="D185">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,2)</f>
+        <f t="array" ref="D185">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,2)</f>
         <v/>
       </c>
       <c r="E185" s="37" cm="1">
-        <f t="array" ref="E185">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,3)</f>
+        <f t="array" ref="E185">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),2,3)</f>
         <v/>
       </c>
       <c r="F185" s="21" t="inlineStr">
         <is>
-          <t>RxnL_Wid  ·  RxnR_Wid</t>
+          <t>RxnL_Q  ·  RxnR_Q</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="B186" s="52" t="inlineStr">
         <is>
-          <t>Wiu</t>
+          <t>Wd</t>
         </is>
       </c>
       <c r="C186" s="53" t="n"/>
       <c r="D186" s="37" cm="1">
-        <f t="array" ref="D186">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,2)</f>
+        <f t="array" ref="D186">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,2)</f>
         <v/>
       </c>
       <c r="E186" s="37" cm="1">
-        <f t="array" ref="E186">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,3)</f>
+        <f t="array" ref="E186">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),3,3)</f>
         <v/>
       </c>
       <c r="F186" s="21" t="inlineStr">
         <is>
+          <t>RxnL_Wd  ·  RxnR_Wd</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="B187" s="52" t="inlineStr">
+        <is>
+          <t>Wu</t>
+        </is>
+      </c>
+      <c r="C187" s="53" t="n"/>
+      <c r="D187" s="37" cm="1">
+        <f t="array" ref="D187">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,2)</f>
+        <v/>
+      </c>
+      <c r="E187" s="37" cm="1">
+        <f t="array" ref="E187">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),4,3)</f>
+        <v/>
+      </c>
+      <c r="F187" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_Wu  ·  RxnR_Wu</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="B188" s="52" t="inlineStr">
+        <is>
+          <t>Wid</t>
+        </is>
+      </c>
+      <c r="C188" s="53" t="n"/>
+      <c r="D188" s="37" cm="1">
+        <f t="array" ref="D188">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,2)</f>
+        <v/>
+      </c>
+      <c r="E188" s="37" cm="1">
+        <f t="array" ref="E188">INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),5,3)</f>
+        <v/>
+      </c>
+      <c r="F188" s="21" t="inlineStr">
+        <is>
+          <t>RxnL_Wid  ·  RxnR_Wid</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="B189" s="52" t="inlineStr">
+        <is>
+          <t>Wiu</t>
+        </is>
+      </c>
+      <c r="C189" s="53" t="n"/>
+      <c r="D189" s="37" cm="1">
+        <f t="array" ref="D189">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,2)</f>
+        <v/>
+      </c>
+      <c r="E189" s="37" cm="1">
+        <f t="array" ref="E189">-INDEX(OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66)),6,3)</f>
+        <v/>
+      </c>
+      <c r="F189" s="21" t="inlineStr">
+        <is>
           <t>RxnL_Wiu  ·  RxnR_Wiu</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="B188" s="15" t="inlineStr">
+    <row r="191">
+      <c r="B191" s="15" t="inlineStr">
         <is>
           <t>All cases and active combinations (kN, + = upward reaction; uplift cases show negative)</t>
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="B189" s="60" t="inlineStr">
+    <row r="192">
+      <c r="B192" s="60" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C189" s="60" t="inlineStr">
+      <c r="C192" s="60" t="inlineStr">
         <is>
           <t>Left (kN)</t>
         </is>
       </c>
-      <c r="D189" s="60" t="inlineStr">
+      <c r="D192" s="60" t="inlineStr">
         <is>
           <t>Right (kN)</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="B190" s="35" cm="1">
-        <f t="array" ref="B190">OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
-        <v/>
-      </c>
-      <c r="C190" s="64" t="n"/>
-      <c r="D190" s="64" t="n"/>
-    </row>
-    <row r="191">
-      <c r="B191" s="35" t="n"/>
-      <c r="C191" s="64" t="n"/>
-      <c r="D191" s="64" t="n"/>
-    </row>
-    <row r="192">
-      <c r="B192" s="35" t="n"/>
-      <c r="C192" s="64" t="n"/>
-      <c r="D192" s="64" t="n"/>
-    </row>
     <row r="193">
-      <c r="B193" s="35" t="n"/>
+      <c r="B193" s="35" cm="1">
+        <f t="array" ref="B193">OAR.REACTIONS(SectionSize,Span,IncludeSW,Loads_B1[[Case]:[End (mm)]],_xlfn.ANCHORARRAY(B66))</f>
+        <v/>
+      </c>
       <c r="C193" s="64" t="n"/>
       <c r="D193" s="64" t="n"/>
     </row>
@@ -7770,47 +7768,62 @@
       <c r="C203" s="64" t="n"/>
       <c r="D203" s="64" t="n"/>
     </row>
+    <row r="204">
+      <c r="B204" s="35" t="n"/>
+      <c r="C204" s="64" t="n"/>
+      <c r="D204" s="64" t="n"/>
+    </row>
+    <row r="205">
+      <c r="B205" s="35" t="n"/>
+      <c r="C205" s="64" t="n"/>
+      <c r="D205" s="64" t="n"/>
+    </row>
+    <row r="206">
+      <c r="B206" s="35" t="n"/>
+      <c r="C206" s="64" t="n"/>
+      <c r="D206" s="64" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="F182:G182"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B185:C185"/>
     <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F187:G187"/>
     <mergeCell ref="F183:G183"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B184:C184"/>
-    <mergeCell ref="B180:C180"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="M8:T40"/>
+    <mergeCell ref="F189:G189"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="G2:J2"/>
-    <mergeCell ref="B181:C181"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="F181:G181"/>
     <mergeCell ref="B6:J6"/>
+    <mergeCell ref="F188:G188"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B182:C182"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="E30:F30"/>
     <mergeCell ref="F185:G185"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="F180:G180"/>
     <mergeCell ref="B186:C186"/>
     <mergeCell ref="F184:G184"/>
     <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B187:C187"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="B183:C183"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="F186:G186"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="I10:J10"/>
+    <mergeCell ref="B189:C189"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B188:C188"/>
     <mergeCell ref="I9:J9"/>
   </mergeCells>
   <conditionalFormatting sqref="I14:I23">
@@ -7866,47 +7879,47 @@
       <formula>NumUpliftCombos=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B90:G94">
+  <conditionalFormatting sqref="B93:G97">
     <cfRule type="expression" priority="12" dxfId="7">
-      <formula>$B90&lt;&gt;""</formula>
+      <formula>$B93&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G90:G94">
+  <conditionalFormatting sqref="G93:G97">
     <cfRule type="expression" priority="13" dxfId="0">
-      <formula>AND(ISNUMBER(G90),G90&gt;1)</formula>
+      <formula>AND(ISNUMBER(G93),G93&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B124:J139">
+  <conditionalFormatting sqref="B127:J142">
     <cfRule type="expression" priority="14" dxfId="7">
-      <formula>$B124&lt;&gt;""</formula>
+      <formula>$B127&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J124:J139">
+  <conditionalFormatting sqref="J127:J142">
     <cfRule type="expression" priority="15" dxfId="0">
-      <formula>AND(ISNUMBER(J124),J124&gt;1)</formula>
+      <formula>AND(ISNUMBER(J127),J127&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C124:C139">
+  <conditionalFormatting sqref="C127:C142">
     <cfRule type="expression" priority="16" dxfId="9">
-      <formula>RIGHT(C124,1)="*"</formula>
+      <formula>RIGHT(C127,1)="*"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B169:F176">
+  <conditionalFormatting sqref="B172:F179">
     <cfRule type="expression" priority="17" dxfId="7">
-      <formula>$B169&lt;&gt;""</formula>
+      <formula>$B172&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F169:F176">
+  <conditionalFormatting sqref="F172:F179">
     <cfRule type="expression" priority="18" dxfId="0">
-      <formula>AND(ISNUMBER(F169),F169&gt;1)</formula>
+      <formula>AND(ISNUMBER(F172),F172&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B190:D203">
+  <conditionalFormatting sqref="B193:D206">
     <cfRule type="expression" priority="19" dxfId="7">
-      <formula>$B190&lt;&gt;""</formula>
+      <formula>$B193&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="13">
+  <dataValidations count="14">
     <dataValidation sqref="E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"UB,UC,WB,PFC"</formula1>
     </dataValidation>
@@ -7940,8 +7953,11 @@
     <dataValidation sqref="E63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Floor,Roof,All,Custom"</formula1>
     </dataValidation>
-    <dataValidation sqref="E77:F81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E77:F83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"F,P,L,U,–"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F89:G89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="E27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Section size" error="Pick a section from the list for the selected Section type." type="list">
       <formula1>IF(ISERROR($AL$8),$AN$8:$AN$88,OFFSET($AL$8,0,0,MAX(1,COUNTA($AL$8:$AL$300)),1))</formula1>
@@ -7959,8 +7975,8 @@
   </headerFooter>
   <rowBreaks count="3" manualBreakCount="3">
     <brk id="42" min="0" max="16383" man="1"/>
-    <brk id="87" min="0" max="16383" man="1"/>
-    <brk id="141" min="0" max="16383" man="1"/>
+    <brk id="90" min="0" max="16383" man="1"/>
+    <brk id="144" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <tableParts count="4">

</xml_diff>

<commit_message>
Release pipeline: GitHub Actions build/test/release, staff install script, changelog, version on calc sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -439,14 +439,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1719,37 +1719,41 @@
       </c>
     </row>
     <row r="7" ht="14" customHeight="1">
+      <c r="B7" s="13" cm="1">
+        <f t="array" ref="B7">IFERROR("Calculated with "&amp;OAR.VERSION(),"OAR Steel add-in not loaded")</f>
+        <v/>
+      </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
           <t>Legend:</t>
         </is>
       </c>
-      <c r="H7" s="13" t="inlineStr">
+      <c r="H7" s="14" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="I7" s="14" t="inlineStr">
+      <c r="I7" s="15" t="inlineStr">
         <is>
           <t>Calculated</t>
         </is>
       </c>
-      <c r="Z7" s="15" t="inlineStr">
+      <c r="Z7" s="13" t="inlineStr">
         <is>
           <t>Governing (OAR.GOVERNING)</t>
         </is>
       </c>
-      <c r="AL7" s="15" t="inlineStr">
+      <c r="AL7" s="13" t="inlineStr">
         <is>
           <t>Sections (OAR.SECTIONLIST)</t>
         </is>
       </c>
-      <c r="AN7" s="15" t="inlineStr">
+      <c r="AN7" s="13" t="inlineStr">
         <is>
           <t>All sections (fallback)</t>
         </is>
       </c>
-      <c r="AP7" s="15" t="inlineStr">
+      <c r="AP7" s="13" t="inlineStr">
         <is>
           <t>Typical starting values only – verify for each job. Picking a Description in the loads table fills Press. (kPa); type over it to change. Keep rows grouped by case (insert new rows inside the case's block).</t>
         </is>
@@ -1942,12 +1946,12 @@
       <c r="R12" s="23" t="n"/>
       <c r="S12" s="23" t="n"/>
       <c r="T12" s="24" t="n"/>
-      <c r="Z12" s="15" t="inlineStr">
+      <c r="Z12" s="13" t="inlineStr">
         <is>
           <t>Envelope (OAR.ENVELOPE)</t>
         </is>
       </c>
-      <c r="AF12" s="15" t="inlineStr">
+      <c r="AF12" s="13" t="inlineStr">
         <is>
           <t>Deflected shapes (OAR.DEFLECTIONS)</t>
         </is>
@@ -1975,7 +1979,7 @@
           <t>40 kg/m² x 9.81</t>
         </is>
       </c>
-      <c r="AT12" s="15" t="inlineStr">
+      <c r="AT12" s="13" t="inlineStr">
         <is>
           <t>Chart data (fixed copies of the spills above)</t>
         </is>
@@ -4473,12 +4477,12 @@
       </c>
     </row>
     <row r="44" ht="14" customHeight="1">
-      <c r="B44" s="15" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>Load = trib × pressure + direct.  UDL/PUDL: trib in m → kN/m.  Point: trib in m² → kN, start = position.  UDL: start/end blank = full span.</t>
         </is>
       </c>
-      <c r="M44" s="15" t="inlineStr">
+      <c r="M44" s="13" t="inlineStr">
         <is>
           <t>Include: blank = follow the Combination set;  Yes / No = force on or off.  Active rows appear in the calc.</t>
         </is>
@@ -4522,12 +4526,12 @@
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
-      <c r="B45" s="15" t="inlineStr">
+      <c r="B45" s="13" t="inlineStr">
         <is>
           <t>Magnitudes positive; direction set by case: Wd, Wid act down; Wu, Wiu act up.  Wi = internal pressure, combined with the external wind case.</t>
         </is>
       </c>
-      <c r="M45" s="15" t="inlineStr">
+      <c r="M45" s="13" t="inlineStr">
         <is>
           <t>Groups: Gravity (Floor, Roof, All), Wind (Roof, All), Storage (All only), Custom (always, unless Include = No).  Add rows at the bottom for custom combinations.</t>
         </is>
@@ -6046,7 +6050,7 @@
       </c>
     </row>
     <row r="64" ht="14" customHeight="1">
-      <c r="B64" s="15" t="inlineStr">
+      <c r="B64" s="13" t="inlineStr">
         <is>
           <t>Floor = gravity only.  Roof = gravity + wind.  All = every library row.  Custom = only rows set to Yes / Custom.  Edit in the library to the right →</t>
         </is>
@@ -6581,7 +6585,7 @@
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
-      <c r="B75" s="15" t="inlineStr">
+      <c r="B75" s="13" t="inlineStr">
         <is>
           <t>Restraint type at each cross-section for the critical flange: F, P, L or U (– = none). Supports must be F or P.</t>
         </is>
@@ -6771,7 +6775,7 @@
       </c>
     </row>
     <row r="84" ht="14" customHeight="1">
-      <c r="B84" s="15" t="inlineStr">
+      <c r="B84" s="13" t="inlineStr">
         <is>
           <t>αm top / αm bot. → override αm for that flange's segment from this row to the next restraint on that flange (blank = Cl. 5.6.1.1(a)(iii)). Flagged * in the output.</t>
         </is>
@@ -6823,7 +6827,7 @@
       <c r="G87" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="H87" s="15" t="inlineStr">
+      <c r="H87" s="13" t="inlineStr">
         <is>
           <t>kl: load height, Table 5.6.3(2)</t>
         </is>
@@ -6846,7 +6850,7 @@
       <c r="G88" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="H88" s="15" t="inlineStr">
+      <c r="H88" s="13" t="inlineStr">
         <is>
           <t>kr: rotation, Table 5.6.3(3); kt from restraints</t>
         </is>
@@ -6873,7 +6877,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H89" s="15" t="inlineStr">
+      <c r="H89" s="13" t="inlineStr">
         <is>
           <t>Yes = flange continuously restrained: φMb = φMsx</t>
         </is>
@@ -7261,7 +7265,7 @@
       <c r="J142" s="68" t="n"/>
     </row>
     <row r="143">
-      <c r="B143" s="15" t="inlineStr">
+      <c r="B143" s="13" t="inlineStr">
         <is>
           <t>* αm overridden in the restraints table.  Full working for the governing segment follows.</t>
         </is>
@@ -7283,7 +7287,7 @@
       <c r="J145" s="11" t="n"/>
     </row>
     <row r="146">
-      <c r="B146" s="15" t="inlineStr">
+      <c r="B146" s="13" t="inlineStr">
         <is>
           <t>OAR.ULSDETAIL: change the comboId / segment arguments to show any other segment.</t>
         </is>
@@ -7532,7 +7536,7 @@
       <c r="J181" s="11" t="n"/>
     </row>
     <row r="182">
-      <c r="B182" s="15" t="inlineStr">
+      <c r="B182" s="13" t="inlineStr">
         <is>
           <t>Unfactored, per case, positive in the case direction (Wu/Wiu = uplift). Self-weight is in G.  To load another beam: add a Point row with the same case and set Direct to e.g. ='B1'!RxnR_G</t>
         </is>
@@ -7687,7 +7691,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="B191" s="15" t="inlineStr">
+      <c r="B191" s="13" t="inlineStr">
         <is>
           <t>All cases and active combinations (kN, + = upward reaction; uplift cases show negative)</t>
         </is>

</xml_diff>

<commit_message>
Print tidy-up: hide unused rows of flex blocks on print / PDF; OAR ribbon tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014sNUvFZnmKLVfgfYiGEFoW
</commit_message>
<xml_diff>
--- a/template/Steel Beam Design - Base.xlsx
+++ b/template/Steel Beam Design - Base.xlsx
@@ -45,6 +45,7 @@
     <definedName name="DeflCriteria" localSheetId="0">'B1'!$B$37:$G$41</definedName>
     <definedName name="PsiL" localSheetId="0">'B1'!$G$38</definedName>
     <definedName name="PsiS" localSheetId="0">'B1'!$G$39</definedName>
+    <definedName name="OAR_Flex_Loads" localSheetId="0">Loads_B1[Case]</definedName>
     <definedName name="w_G" localSheetId="0">'B1'!$E$60</definedName>
     <definedName name="w_Q" localSheetId="0">'B1'!$F$60</definedName>
     <definedName name="w_Wd" localSheetId="0">'B1'!$G$60</definedName>
@@ -54,12 +55,16 @@
     <definedName name="NumUpliftCombos" localSheetId="0">'B1'!$S$56</definedName>
     <definedName name="CombSet" localSheetId="0">'B1'!$E$63</definedName>
     <definedName name="PsiC" localSheetId="0">'B1'!$G$63</definedName>
+    <definedName name="OAR_Flex_Combos" localSheetId="0">'B1'!$B$66:$B$73</definedName>
+    <definedName name="OAR_Flex_Restraints" localSheetId="0">Restraints_B1[x (mm)]</definedName>
     <definedName name="kl_Top" localSheetId="0">'B1'!$F$87</definedName>
     <definedName name="kl_Bot" localSheetId="0">'B1'!$G$87</definedName>
     <definedName name="kr_Top" localSheetId="0">'B1'!$F$88</definedName>
     <definedName name="kr_Bot" localSheetId="0">'B1'!$G$88</definedName>
     <definedName name="Cont_Top" localSheetId="0">'B1'!$F$89</definedName>
     <definedName name="Cont_Bot" localSheetId="0">'B1'!$G$89</definedName>
+    <definedName name="OAR_Flex_ULS" localSheetId="0">'B1'!$B$127:$B$142</definedName>
+    <definedName name="OAR_Flex_Shear" localSheetId="0">'B1'!$B$172:$B$179</definedName>
     <definedName name="RxnL_G" localSheetId="0">'B1'!$D$184</definedName>
     <definedName name="RxnR_G" localSheetId="0">'B1'!$E$184</definedName>
     <definedName name="RxnL_Q" localSheetId="0">'B1'!$D$185</definedName>
@@ -72,6 +77,7 @@
     <definedName name="RxnR_Wid" localSheetId="0">'B1'!$E$188</definedName>
     <definedName name="RxnL_Wiu" localSheetId="0">'B1'!$D$189</definedName>
     <definedName name="RxnR_Wiu" localSheetId="0">'B1'!$E$189</definedName>
+    <definedName name="OAR_Flex_Reactions" localSheetId="0">'B1'!$B$193:$B$206</definedName>
     <definedName name="Out_Reactions" localSheetId="0">'B1'!$B$193</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'B1'!$A$1:$K$207</definedName>
   </definedNames>

</xml_diff>